<commit_message>
Update trading data 2026-04-12 14:51:13.585187
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY21"/>
+  <dimension ref="A1:AY23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -696,7 +696,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -708,106 +708,106 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>43866.41666666666</v>
+        <v>43852.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>43879.41666666666</v>
+        <v>43891.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>0.36</v>
+        <v>3.59</v>
       </c>
       <c r="G2" t="n">
-        <v>-21.3</v>
+        <v>-19.5</v>
       </c>
       <c r="H2" t="n">
-        <v>0.33</v>
+        <v>3.31</v>
       </c>
       <c r="I2" t="n">
-        <v>0.38</v>
+        <v>3.1</v>
       </c>
       <c r="J2" t="n">
-        <v>5.22</v>
+        <v>-13.65</v>
       </c>
       <c r="K2" t="n">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="L2" t="n">
-        <v>0.28</v>
+        <v>2.89</v>
       </c>
       <c r="M2" t="n">
-        <v>0.35</v>
+        <v>3.57</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
       </c>
       <c r="O2" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="P2" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>113942</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>96.55</v>
+      </c>
+      <c r="V2" t="n">
+        <v>-14.72</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="X2" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="Y2" t="n">
         <v>0.39</v>
       </c>
-      <c r="P2" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
-        <v>53623856</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U2" t="n">
-        <v>80.93000000000001</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="W2" t="n">
-        <v>4.16</v>
-      </c>
-      <c r="X2" t="n">
-        <v>4.31</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>1.51</v>
-      </c>
       <c r="Z2" t="n">
-        <v>2.22</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AA2" t="n">
-        <v>1.21</v>
+        <v>1.16</v>
       </c>
       <c r="AB2" t="n">
-        <v>6.93</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" t="n">
-        <v>7.69</v>
+        <v>4.22</v>
       </c>
       <c r="AD2" t="n">
-        <v>21.67</v>
+        <v>21.05</v>
       </c>
       <c r="AE2" t="n">
-        <v>4.9</v>
+        <v>2.57</v>
       </c>
       <c r="AF2" t="n">
-        <v>12.61</v>
+        <v>4.74</v>
       </c>
       <c r="AG2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>43874.41666666666</v>
+        <v>43863.41666666666</v>
       </c>
       <c r="AI2" t="n">
-        <v>0</v>
+        <v>-13.65</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -819,13 +819,13 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.37</v>
+        <v>4.13</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.32</v>
+        <v>3.41</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.37</v>
+        <v>3.53</v>
       </c>
       <c r="AP2" t="b">
         <v>0</v>
@@ -840,10 +840,10 @@
         <v>1</v>
       </c>
       <c r="AT2" t="n">
-        <v>84.12697579502198</v>
+        <v>98.59154929577461</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.36</v>
+        <v>3.57</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
@@ -855,7 +855,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -867,43 +867,43 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>43884.41666666666</v>
+        <v>44017.45833333334</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>43899.41666666666</v>
+        <v>44021.45833333334</v>
       </c>
       <c r="F3" t="n">
-        <v>0.42</v>
+        <v>3.6</v>
       </c>
       <c r="G3" t="n">
-        <v>-10.38</v>
+        <v>-41.94</v>
       </c>
       <c r="H3" t="n">
-        <v>0.37</v>
+        <v>3.35</v>
       </c>
       <c r="I3" t="n">
-        <v>0.39</v>
+        <v>3.31</v>
       </c>
       <c r="J3" t="n">
-        <v>-5.75</v>
+        <v>-8.06</v>
       </c>
       <c r="K3" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="L3" t="n">
-        <v>0.37</v>
+        <v>2.09</v>
       </c>
       <c r="M3" t="n">
-        <v>0.42</v>
+        <v>3.55</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>0.39</v>
+        <v>3.35</v>
       </c>
       <c r="P3" t="n">
-        <v>0.47</v>
+        <v>3.74</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>13126590</v>
+        <v>1260399</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -924,49 +924,49 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>87.28</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="V3" t="n">
-        <v>1.58</v>
+        <v>3.74</v>
       </c>
       <c r="W3" t="n">
-        <v>0.59</v>
+        <v>1.96</v>
       </c>
       <c r="X3" t="n">
-        <v>5.15</v>
+        <v>4.56</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.63</v>
+        <v>1.94</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.09</v>
+        <v>1.41</v>
       </c>
       <c r="AA3" t="n">
-        <v>8.19</v>
+        <v>4.66</v>
       </c>
       <c r="AB3" t="n">
-        <v>15.66</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="AC3" t="n">
-        <v>9.92</v>
+        <v>7.02</v>
       </c>
       <c r="AD3" t="n">
-        <v>10.85</v>
+        <v>51.77</v>
       </c>
       <c r="AE3" t="n">
-        <v>1.15</v>
+        <v>3.15</v>
       </c>
       <c r="AF3" t="n">
-        <v>10.85</v>
+        <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>43887.41666666666</v>
+        <v>44017.45833333334</v>
       </c>
       <c r="AI3" t="n">
-        <v>-5.75</v>
+        <v>-8.06</v>
       </c>
       <c r="AJ3" t="b">
         <v>1</v>
@@ -978,13 +978,13 @@
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.42</v>
+        <v>3.6</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.32</v>
+        <v>3.28</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.41</v>
+        <v>3.56</v>
       </c>
       <c r="AP3" t="b">
         <v>0</v>
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="AT3" t="n">
-        <v>93.24894745739515</v>
+        <v>78.12499999999999</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.42</v>
+        <v>3.55</v>
       </c>
       <c r="AV3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW3" t="inlineStr"/>
       <c r="AX3" t="inlineStr"/>
@@ -1014,7 +1014,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1026,106 +1026,106 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>43935.41666666666</v>
+        <v>44040.45833333334</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>44266.41666666666</v>
+        <v>44082.45833333334</v>
       </c>
       <c r="F4" t="n">
-        <v>0.46</v>
+        <v>3.5</v>
       </c>
       <c r="G4" t="n">
-        <v>-35.2</v>
+        <v>-16.86</v>
       </c>
       <c r="H4" t="n">
-        <v>0.31</v>
+        <v>2.91</v>
       </c>
       <c r="I4" t="n">
-        <v>0.98</v>
+        <v>3.49</v>
       </c>
       <c r="J4" t="n">
-        <v>114.84</v>
+        <v>-0.29</v>
       </c>
       <c r="K4" t="n">
-        <v>331</v>
+        <v>42</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3</v>
+        <v>2.91</v>
       </c>
       <c r="M4" t="n">
-        <v>0.45</v>
+        <v>3.47</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
       </c>
       <c r="O4" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="P4" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>3078417</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>85.51000000000001</v>
+      </c>
+      <c r="V4" t="n">
+        <v>-3.89</v>
+      </c>
+      <c r="W4" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="X4" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="Y4" t="n">
         <v>1.03</v>
       </c>
-      <c r="P4" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
-        <v>43473801</v>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U4" t="n">
-        <v>93.33</v>
-      </c>
-      <c r="V4" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="X4" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>3.2</v>
-      </c>
       <c r="Z4" t="n">
-        <v>0.78</v>
+        <v>0.86</v>
       </c>
       <c r="AA4" t="n">
-        <v>7.33</v>
+        <v>5.19</v>
       </c>
       <c r="AB4" t="n">
-        <v>24.94</v>
+        <v>6.57</v>
       </c>
       <c r="AC4" t="n">
-        <v>24.12</v>
+        <v>6.29</v>
       </c>
       <c r="AD4" t="n">
-        <v>41.98</v>
+        <v>17.55</v>
       </c>
       <c r="AE4" t="n">
-        <v>7.51</v>
+        <v>4.48</v>
       </c>
       <c r="AF4" t="n">
-        <v>190.77</v>
+        <v>14.57</v>
       </c>
       <c r="AG4" t="n">
-        <v>314</v>
+        <v>34</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>44249.41666666666</v>
+        <v>44074.45833333334</v>
       </c>
       <c r="AI4" t="n">
-        <v>0</v>
+        <v>-2.57</v>
       </c>
       <c r="AJ4" t="b">
         <v>1</v>
@@ -1137,31 +1137,31 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.44</v>
+        <v>3.74</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.38</v>
+        <v>3.03</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.43</v>
+        <v>3.55</v>
       </c>
       <c r="AP4" t="b">
         <v>0</v>
       </c>
       <c r="AQ4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS4" t="b">
         <v>1</v>
       </c>
       <c r="AT4" t="n">
-        <v>93.41772177984936</v>
+        <v>85.50724637681158</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.45</v>
+        <v>3.47</v>
       </c>
       <c r="AV4" t="b">
         <v>1</v>
@@ -1173,7 +1173,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1185,43 +1185,43 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>44320.45833333334</v>
+        <v>44147.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>44348.45833333334</v>
+        <v>44175.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>0.58</v>
+        <v>3.2</v>
       </c>
       <c r="G5" t="n">
-        <v>-19.8</v>
+        <v>-12.5</v>
       </c>
       <c r="H5" t="n">
-        <v>0.54</v>
+        <v>2.8</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5600000000000001</v>
+        <v>3.21</v>
       </c>
       <c r="J5" t="n">
-        <v>-4.2</v>
+        <v>0.31</v>
       </c>
       <c r="K5" t="n">
         <v>28</v>
       </c>
       <c r="L5" t="n">
-        <v>0.47</v>
+        <v>2.8</v>
       </c>
       <c r="M5" t="n">
-        <v>0.57</v>
+        <v>3.15</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>0.57</v>
+        <v>3.23</v>
       </c>
       <c r="P5" t="n">
-        <v>0.74</v>
+        <v>3.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>117164343</v>
+        <v>2506229</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -1242,49 +1242,49 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>67.8</v>
+        <v>83.33</v>
       </c>
       <c r="V5" t="n">
-        <v>-108.28</v>
+        <v>-25</v>
       </c>
       <c r="W5" t="n">
-        <v>1.34</v>
+        <v>3.09</v>
       </c>
       <c r="X5" t="n">
-        <v>4.81</v>
+        <v>3.88</v>
       </c>
       <c r="Y5" t="n">
-        <v>-3.59</v>
+        <v>-0.73</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.08</v>
+        <v>1.59</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.14</v>
+        <v>3.34</v>
       </c>
       <c r="AB5" t="n">
-        <v>-14.74</v>
+        <v>-2.74</v>
       </c>
       <c r="AC5" t="n">
-        <v>3.1</v>
+        <v>2.19</v>
       </c>
       <c r="AD5" t="n">
-        <v>19.94</v>
+        <v>11.76</v>
       </c>
       <c r="AE5" t="n">
-        <v>6.58</v>
+        <v>2.56</v>
       </c>
       <c r="AF5" t="n">
-        <v>22.37</v>
+        <v>8.44</v>
       </c>
       <c r="AG5" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>44336.45833333334</v>
+        <v>44166.41666666666</v>
       </c>
       <c r="AI5" t="n">
-        <v>-4.2</v>
+        <v>-3.13</v>
       </c>
       <c r="AJ5" t="b">
         <v>1</v>
@@ -1296,13 +1296,13 @@
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>1.25</v>
+        <v>4.1</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.52</v>
+        <v>2.97</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.5600000000000001</v>
+        <v>3.46</v>
       </c>
       <c r="AP5" t="b">
         <v>0</v>
@@ -1317,10 +1317,10 @@
         <v>1</v>
       </c>
       <c r="AT5" t="n">
-        <v>86.21700569120193</v>
+        <v>84.90566037735854</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.57</v>
+        <v>3.17</v>
       </c>
       <c r="AV5" t="b">
         <v>1</v>
@@ -1332,7 +1332,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1344,43 +1344,43 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>44416.45833333334</v>
+        <v>44208.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>44445.45833333334</v>
+        <v>44258.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>0.54</v>
+        <v>3.54</v>
       </c>
       <c r="G6" t="n">
-        <v>-13.62</v>
+        <v>-14.97</v>
       </c>
       <c r="H6" t="n">
-        <v>0.48</v>
+        <v>3.13</v>
       </c>
       <c r="I6" t="n">
-        <v>0.46</v>
+        <v>3.05</v>
       </c>
       <c r="J6" t="n">
-        <v>-15.08</v>
+        <v>-13.84</v>
       </c>
       <c r="K6" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L6" t="n">
-        <v>0.46</v>
+        <v>3.01</v>
       </c>
       <c r="M6" t="n">
-        <v>0.52</v>
+        <v>3.41</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>0.48</v>
+        <v>3.13</v>
       </c>
       <c r="P6" t="n">
-        <v>0.55</v>
+        <v>3.74</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>82672340</v>
+        <v>9793276</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1401,85 +1401,85 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>80.81999999999999</v>
+        <v>78.84</v>
       </c>
       <c r="V6" t="n">
-        <v>-33.57</v>
+        <v>6.03</v>
       </c>
       <c r="W6" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="X6" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>8</v>
+      </c>
+      <c r="AH6" s="2" t="n">
+        <v>44216.41666666666</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>-13.84</v>
+      </c>
+      <c r="AJ6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="AP6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>81.35593220338986</v>
+      </c>
+      <c r="AU6" t="n">
         <v>3.41</v>
-      </c>
-      <c r="X6" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>6.92</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>11.65</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>5.65</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH6" s="2" t="n">
-        <v>44416.45833333334</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>-15.08</v>
-      </c>
-      <c r="AJ6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="AP6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AS6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT6" t="n">
-        <v>81.49999949123762</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>0.52</v>
       </c>
       <c r="AV6" t="b">
         <v>1</v>
@@ -1491,7 +1491,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1503,43 +1503,43 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>44641.41666666666</v>
+        <v>44294.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>44668.41666666666</v>
+        <v>44349.45833333334</v>
       </c>
       <c r="F7" t="n">
-        <v>0.23</v>
+        <v>3.32</v>
       </c>
       <c r="G7" t="n">
-        <v>-14.8</v>
+        <v>-18.67</v>
       </c>
       <c r="H7" t="n">
-        <v>0.21</v>
+        <v>2.7</v>
       </c>
       <c r="I7" t="n">
-        <v>0.19</v>
+        <v>4.28</v>
       </c>
       <c r="J7" t="n">
-        <v>-19.22</v>
+        <v>28.92</v>
       </c>
       <c r="K7" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2</v>
+        <v>2.7</v>
       </c>
       <c r="M7" t="n">
-        <v>0.23</v>
+        <v>3.16</v>
       </c>
       <c r="N7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>0.21</v>
+        <v>4.32</v>
       </c>
       <c r="P7" t="n">
-        <v>0.24</v>
+        <v>4.84</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>12012168</v>
+        <v>3957625</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1560,49 +1560,49 @@
         </is>
       </c>
       <c r="U7" t="n">
-        <v>87.64</v>
+        <v>95.38</v>
       </c>
       <c r="V7" t="n">
-        <v>-112.4</v>
+        <v>2.09</v>
       </c>
       <c r="W7" t="n">
-        <v>2.44</v>
+        <v>5.98</v>
       </c>
       <c r="X7" t="n">
-        <v>4.31</v>
+        <v>6.55</v>
       </c>
       <c r="Y7" t="n">
-        <v>-2.6</v>
+        <v>1.05</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.34</v>
+        <v>5.06</v>
       </c>
       <c r="AA7" t="n">
-        <v>7.59</v>
+        <v>2.39</v>
       </c>
       <c r="AB7" t="n">
-        <v>-10.07</v>
+        <v>7.42</v>
       </c>
       <c r="AC7" t="n">
-        <v>-0.72</v>
+        <v>11.54</v>
       </c>
       <c r="AD7" t="n">
-        <v>15.64</v>
+        <v>15.7</v>
       </c>
       <c r="AE7" t="n">
-        <v>2.44</v>
+        <v>8.85</v>
       </c>
       <c r="AF7" t="n">
-        <v>2.04</v>
+        <v>42.47</v>
       </c>
       <c r="AG7" t="n">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>44643.41666666666</v>
+        <v>44339.45833333334</v>
       </c>
       <c r="AI7" t="n">
-        <v>-19.22</v>
+        <v>0</v>
       </c>
       <c r="AJ7" t="b">
         <v>1</v>
@@ -1614,13 +1614,13 @@
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.5</v>
+        <v>3.28</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.22</v>
+        <v>2.98</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.31</v>
+        <v>3.34</v>
       </c>
       <c r="AP7" t="b">
         <v>0</v>
@@ -1635,10 +1635,10 @@
         <v>1</v>
       </c>
       <c r="AT7" t="n">
-        <v>82.85715185566262</v>
+        <v>96.20253164556958</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.23</v>
+        <v>3.16</v>
       </c>
       <c r="AV7" t="b">
         <v>1</v>
@@ -1650,7 +1650,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1662,106 +1662,106 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>44703.45833333334</v>
+        <v>44353.45833333334</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>44706.45833333334</v>
+        <v>44444.45833333334</v>
       </c>
       <c r="F8" t="n">
-        <v>0.24</v>
+        <v>4.66</v>
       </c>
       <c r="G8" t="n">
-        <v>-28.38</v>
+        <v>-12.02</v>
       </c>
       <c r="H8" t="n">
-        <v>0.21</v>
+        <v>4.09</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2</v>
+        <v>4.6</v>
       </c>
       <c r="J8" t="n">
-        <v>-15.03</v>
+        <v>-1.29</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>91</v>
       </c>
       <c r="L8" t="n">
-        <v>0.17</v>
+        <v>4.1</v>
       </c>
       <c r="M8" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="P8" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>2292545</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>91.93000000000001</v>
+      </c>
+      <c r="V8" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="W8" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="X8" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="Z8" t="n">
         <v>0.22</v>
       </c>
-      <c r="N8" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S8" t="n">
-        <v>87965589</v>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U8" t="n">
-        <v>90.59</v>
-      </c>
-      <c r="V8" t="n">
-        <v>5.79</v>
-      </c>
-      <c r="W8" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="X8" t="n">
-        <v>5.74</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>5.09</v>
-      </c>
       <c r="AA8" t="n">
-        <v>1.16</v>
+        <v>6.28</v>
       </c>
       <c r="AB8" t="n">
-        <v>4.24</v>
+        <v>20.83</v>
       </c>
       <c r="AC8" t="n">
-        <v>8.470000000000001</v>
+        <v>9.49</v>
       </c>
       <c r="AD8" t="n">
-        <v>28.23</v>
+        <v>12.57</v>
       </c>
       <c r="AE8" t="n">
-        <v>7.54</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="AF8" t="n">
-        <v>0</v>
+        <v>26.82</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>44703.45833333334</v>
+        <v>44418.45833333334</v>
       </c>
       <c r="AI8" t="n">
-        <v>-15.03</v>
+        <v>-7.51</v>
       </c>
       <c r="AJ8" t="b">
         <v>1</v>
@@ -1773,13 +1773,13 @@
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.22</v>
+        <v>4.65</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.21</v>
+        <v>3.37</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.24</v>
+        <v>4.51</v>
       </c>
       <c r="AP8" t="b">
         <v>0</v>
@@ -1788,16 +1788,16 @@
         <v>0</v>
       </c>
       <c r="AR8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT8" t="n">
-        <v>92.94116133094631</v>
+        <v>76.00000000000004</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.23</v>
+        <v>4.65</v>
       </c>
       <c r="AV8" t="b">
         <v>1</v>
@@ -1809,7 +1809,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1821,43 +1821,43 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>44763.45833333334</v>
+        <v>44551.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>44795.45833333334</v>
+        <v>44577.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2</v>
+        <v>4.32</v>
       </c>
       <c r="G9" t="n">
-        <v>-15.74</v>
+        <v>-25.93</v>
       </c>
       <c r="H9" t="n">
-        <v>0.19</v>
+        <v>3.67</v>
       </c>
       <c r="I9" t="n">
-        <v>0.21</v>
+        <v>4.25</v>
       </c>
       <c r="J9" t="n">
-        <v>3.93</v>
+        <v>-1.62</v>
       </c>
       <c r="K9" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="L9" t="n">
-        <v>0.17</v>
+        <v>3.2</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2</v>
+        <v>4.29</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>0.21</v>
+        <v>4.5</v>
       </c>
       <c r="P9" t="n">
-        <v>0.25</v>
+        <v>4.7</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1870,57 +1870,57 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>40238124</v>
+        <v>1089232</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BULLISH_TREND</t>
         </is>
       </c>
       <c r="U9" t="n">
-        <v>93.06</v>
+        <v>95.59</v>
       </c>
       <c r="V9" t="n">
-        <v>-16.2</v>
+        <v>-19.54</v>
       </c>
       <c r="W9" t="n">
-        <v>2.5</v>
+        <v>4.51</v>
       </c>
       <c r="X9" t="n">
-        <v>5.09</v>
+        <v>4.15</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.43</v>
+        <v>1.85</v>
       </c>
       <c r="Z9" t="n">
-        <v>2.69</v>
+        <v>0.7</v>
       </c>
       <c r="AA9" t="n">
-        <v>2.47</v>
+        <v>3.86</v>
       </c>
       <c r="AB9" t="n">
-        <v>2.22</v>
+        <v>8.32</v>
       </c>
       <c r="AC9" t="n">
-        <v>6.98</v>
+        <v>7.71</v>
       </c>
       <c r="AD9" t="n">
-        <v>14.44</v>
+        <v>29.11</v>
       </c>
       <c r="AE9" t="n">
-        <v>6.64</v>
+        <v>1.89</v>
       </c>
       <c r="AF9" t="n">
-        <v>16.39</v>
+        <v>7.41</v>
       </c>
       <c r="AG9" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>44787.45833333334</v>
+        <v>44566.41666666666</v>
       </c>
       <c r="AI9" t="n">
-        <v>-0.66</v>
+        <v>-1.62</v>
       </c>
       <c r="AJ9" t="b">
         <v>1</v>
@@ -1932,13 +1932,13 @@
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.24</v>
+        <v>5.2</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.18</v>
+        <v>4.08</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.2</v>
+        <v>4.4</v>
       </c>
       <c r="AP9" t="b">
         <v>0</v>
@@ -1953,13 +1953,13 @@
         <v>1</v>
       </c>
       <c r="AT9" t="n">
-        <v>97.01491133883241</v>
+        <v>89.04109589041094</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.2</v>
+        <v>4.41</v>
       </c>
       <c r="AV9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW9" t="inlineStr"/>
       <c r="AX9" t="inlineStr"/>
@@ -1968,7 +1968,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1980,106 +1980,106 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>44801.45833333334</v>
+        <v>44594.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>44822.45833333334</v>
+        <v>44627.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>0.25</v>
+        <v>4.31</v>
       </c>
       <c r="G10" t="n">
-        <v>-22.96</v>
+        <v>-5.57</v>
       </c>
       <c r="H10" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-6.73</v>
+      </c>
+      <c r="K10" t="n">
+        <v>33</v>
+      </c>
+      <c r="L10" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="M10" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="P10" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>128046</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>45.71</v>
+      </c>
+      <c r="V10" t="n">
+        <v>-4.44</v>
+      </c>
+      <c r="W10" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="X10" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Z10" t="n">
         <v>0.23</v>
       </c>
-      <c r="I10" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="J10" t="n">
-        <v>-10.03</v>
-      </c>
-      <c r="K10" t="n">
-        <v>21</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N10" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S10" t="n">
-        <v>261018733</v>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U10" t="n">
-        <v>99.95999999999999</v>
-      </c>
-      <c r="V10" t="n">
-        <v>2.37</v>
-      </c>
-      <c r="W10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="X10" t="n">
-        <v>7.83</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>2.43</v>
-      </c>
       <c r="AA10" t="n">
-        <v>3.06</v>
+        <v>2.53</v>
       </c>
       <c r="AB10" t="n">
-        <v>18.41</v>
+        <v>2.01</v>
       </c>
       <c r="AC10" t="n">
-        <v>13.68</v>
+        <v>0.61</v>
       </c>
       <c r="AD10" t="n">
-        <v>23.56</v>
+        <v>5.5</v>
       </c>
       <c r="AE10" t="n">
-        <v>9.859999999999999</v>
+        <v>1.41</v>
       </c>
       <c r="AF10" t="n">
-        <v>12.66</v>
+        <v>7.66</v>
       </c>
       <c r="AG10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>44810.45833333334</v>
+        <v>44598.41666666666</v>
       </c>
       <c r="AI10" t="n">
-        <v>-10.03</v>
+        <v>-6.73</v>
       </c>
       <c r="AJ10" t="b">
         <v>1</v>
@@ -2091,13 +2091,13 @@
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.25</v>
+        <v>4.7</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.19</v>
+        <v>4.11</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.25</v>
+        <v>4.69</v>
       </c>
       <c r="AP10" t="b">
         <v>0</v>
@@ -2106,16 +2106,16 @@
         <v>0</v>
       </c>
       <c r="AR10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT10" t="n">
-        <v>100</v>
+        <v>52.17391304347812</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.25</v>
+        <v>4.3</v>
       </c>
       <c r="AV10" t="b">
         <v>1</v>
@@ -2127,7 +2127,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2139,43 +2139,43 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>44903.41666666666</v>
+        <v>44643.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>44957.41666666666</v>
+        <v>44661.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>0.3</v>
+        <v>4.31</v>
       </c>
       <c r="G11" t="n">
-        <v>-26.13</v>
+        <v>-9.050000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>0.26</v>
+        <v>3.9</v>
       </c>
       <c r="I11" t="n">
-        <v>0.32</v>
+        <v>3.75</v>
       </c>
       <c r="J11" t="n">
-        <v>8.56</v>
+        <v>-12.99</v>
       </c>
       <c r="K11" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="L11" t="n">
-        <v>0.22</v>
+        <v>3.92</v>
       </c>
       <c r="M11" t="n">
-        <v>0.29</v>
+        <v>4.3</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>0.32</v>
+        <v>3.9</v>
       </c>
       <c r="P11" t="n">
-        <v>0.37</v>
+        <v>4.45</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -2188,75 +2188,75 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>173388368</v>
+        <v>293154</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BULLISH_TREND</t>
         </is>
       </c>
       <c r="U11" t="n">
-        <v>87.12</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="V11" t="n">
-        <v>4.64</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>1.56</v>
+        <v>0.71</v>
       </c>
       <c r="X11" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="2" t="n">
+        <v>44643.41666666666</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>-12.99</v>
+      </c>
+      <c r="AJ11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="AN11" t="n">
         <v>4.07</v>
       </c>
-      <c r="Y11" t="n">
-        <v>4.06</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>2.78</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>7.29</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>19.78</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>13.86</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>27.37</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>25.45</v>
-      </c>
-      <c r="AG11" t="n">
-        <v>41</v>
-      </c>
-      <c r="AH11" s="2" t="n">
-        <v>44944.41666666666</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>0.18</v>
-      </c>
       <c r="AO11" t="n">
-        <v>0.29</v>
+        <v>4.66</v>
       </c>
       <c r="AP11" t="b">
         <v>0</v>
@@ -2271,13 +2271,13 @@
         <v>1</v>
       </c>
       <c r="AT11" t="n">
-        <v>89.65515873960044</v>
+        <v>74.54545454545446</v>
       </c>
       <c r="AU11" t="n">
-        <v>0.29</v>
+        <v>4.53</v>
       </c>
       <c r="AV11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW11" t="inlineStr"/>
       <c r="AX11" t="inlineStr"/>
@@ -2286,7 +2286,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2298,43 +2298,43 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45067.41666666666</v>
+        <v>44747.45833333334</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45266.41666666666</v>
+        <v>44822.45833333334</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3</v>
+        <v>3.3</v>
       </c>
       <c r="G12" t="n">
-        <v>-30.77</v>
+        <v>-6.06</v>
       </c>
       <c r="H12" t="n">
-        <v>0.26</v>
+        <v>3.07</v>
       </c>
       <c r="I12" t="n">
-        <v>0.58</v>
+        <v>4.7</v>
       </c>
       <c r="J12" t="n">
-        <v>91.87</v>
+        <v>42.42</v>
       </c>
       <c r="K12" t="n">
-        <v>199</v>
+        <v>75</v>
       </c>
       <c r="L12" t="n">
-        <v>0.21</v>
+        <v>3.1</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3</v>
+        <v>3.27</v>
       </c>
       <c r="N12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>0.59</v>
+        <v>4.85</v>
       </c>
       <c r="P12" t="n">
-        <v>0.65</v>
+        <v>5.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -2347,57 +2347,57 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>107687795</v>
+        <v>310094</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BEARISH_BREAK</t>
         </is>
       </c>
       <c r="U12" t="n">
-        <v>98.45999999999999</v>
+        <v>100</v>
       </c>
       <c r="V12" t="n">
-        <v>-16.89</v>
+        <v>-33.33</v>
       </c>
       <c r="W12" t="n">
-        <v>4.37</v>
+        <v>0.41</v>
       </c>
       <c r="X12" t="n">
-        <v>4.42</v>
+        <v>5.32</v>
       </c>
       <c r="Y12" t="n">
-        <v>1.33</v>
+        <v>-1.26</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.44</v>
+        <v>0.92</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.23</v>
+        <v>4.33</v>
       </c>
       <c r="AB12" t="n">
-        <v>6.25</v>
+        <v>-6.26</v>
       </c>
       <c r="AC12" t="n">
-        <v>6.9</v>
+        <v>-0.29</v>
       </c>
       <c r="AD12" t="n">
-        <v>35.94</v>
+        <v>5.34</v>
       </c>
       <c r="AE12" t="n">
-        <v>9.109999999999999</v>
+        <v>3.77</v>
       </c>
       <c r="AF12" t="n">
-        <v>108.57</v>
+        <v>58.18</v>
       </c>
       <c r="AG12" t="n">
-        <v>192</v>
+        <v>65</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>45259.41666666666</v>
+        <v>44812.45833333334</v>
       </c>
       <c r="AI12" t="n">
-        <v>-2.86</v>
+        <v>-0.3</v>
       </c>
       <c r="AJ12" t="b">
         <v>1</v>
@@ -2409,34 +2409,32 @@
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>0.27</v>
-      </c>
+        <v>4.4</v>
+      </c>
+      <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="n">
-        <v>0.3</v>
+        <v>3.6</v>
       </c>
       <c r="AP12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ12" t="b">
         <v>1</v>
       </c>
       <c r="AR12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS12" t="b">
         <v>1</v>
       </c>
       <c r="AT12" t="n">
-        <v>98.48484159779932</v>
+        <v>50.00000000000001</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.3</v>
+        <v>3.27</v>
       </c>
       <c r="AV12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW12" t="inlineStr"/>
       <c r="AX12" t="inlineStr"/>
@@ -2445,7 +2443,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2457,43 +2455,43 @@
         <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45302.41666666666</v>
+        <v>44872.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45349.41666666666</v>
+        <v>44936.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>0.75</v>
+        <v>5.44</v>
       </c>
       <c r="G13" t="n">
-        <v>-29.33</v>
+        <v>-18.2</v>
       </c>
       <c r="H13" t="n">
-        <v>0.62</v>
+        <v>4.5</v>
       </c>
       <c r="I13" t="n">
-        <v>0.85</v>
+        <v>6.84</v>
       </c>
       <c r="J13" t="n">
-        <v>12.19</v>
+        <v>25.74</v>
       </c>
       <c r="K13" t="n">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="L13" t="n">
-        <v>0.53</v>
+        <v>4.45</v>
       </c>
       <c r="M13" t="n">
-        <v>0.65</v>
+        <v>5.4</v>
       </c>
       <c r="N13" t="b">
         <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0.87</v>
+        <v>7.12</v>
       </c>
       <c r="P13" t="n">
-        <v>1.12</v>
+        <v>7.74</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -2506,7 +2504,7 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>85279318</v>
+        <v>439840</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -2514,49 +2512,49 @@
         </is>
       </c>
       <c r="U13" t="n">
-        <v>99.98999999999999</v>
+        <v>96.91</v>
       </c>
       <c r="V13" t="n">
-        <v>13.43</v>
+        <v>1.28</v>
       </c>
       <c r="W13" t="n">
-        <v>7.67</v>
+        <v>2.33</v>
       </c>
       <c r="X13" t="n">
-        <v>5.55</v>
+        <v>3.64</v>
       </c>
       <c r="Y13" t="n">
-        <v>4.44</v>
+        <v>3.64</v>
       </c>
       <c r="Z13" t="n">
-        <v>15.51</v>
+        <v>0.74</v>
       </c>
       <c r="AA13" t="n">
-        <v>5.28</v>
+        <v>5.18</v>
       </c>
       <c r="AB13" t="n">
-        <v>32.63</v>
+        <v>15.27</v>
       </c>
       <c r="AC13" t="n">
-        <v>22.8</v>
+        <v>11.06</v>
       </c>
       <c r="AD13" t="n">
-        <v>20.22</v>
+        <v>19.29</v>
       </c>
       <c r="AE13" t="n">
-        <v>19.92</v>
+        <v>6.67</v>
       </c>
       <c r="AF13" t="n">
-        <v>40.55</v>
+        <v>39.89</v>
       </c>
       <c r="AG13" t="n">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>45321.41666666666</v>
+        <v>44935.41666666666</v>
       </c>
       <c r="AI13" t="n">
-        <v>0</v>
+        <v>-4.41</v>
       </c>
       <c r="AJ13" t="b">
         <v>1</v>
@@ -2568,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.65</v>
+        <v>5.4</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.34</v>
+        <v>4.6</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.63</v>
+        <v>5.2</v>
       </c>
       <c r="AP13" t="b">
         <v>0</v>
@@ -2589,10 +2587,10 @@
         <v>1</v>
       </c>
       <c r="AT13" t="n">
-        <v>100</v>
+        <v>96.90721649484543</v>
       </c>
       <c r="AU13" t="n">
-        <v>0.65</v>
+        <v>5.4</v>
       </c>
       <c r="AV13" t="b">
         <v>1</v>
@@ -2604,7 +2602,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2613,46 +2611,46 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45365.41666666666</v>
+        <v>44983.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45412.41666666666</v>
+        <v>45004.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>0.92</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>-16.96</v>
+        <v>-25.4</v>
       </c>
       <c r="H14" t="n">
-        <v>0.77</v>
+        <v>6.7</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8</v>
+        <v>6.6</v>
       </c>
       <c r="J14" t="n">
-        <v>-13.35</v>
+        <v>-18.62</v>
       </c>
       <c r="K14" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="L14" t="n">
-        <v>0.77</v>
+        <v>6.05</v>
       </c>
       <c r="M14" t="n">
-        <v>0.9</v>
+        <v>7.74</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>0.82</v>
+        <v>6.7</v>
       </c>
       <c r="P14" t="n">
-        <v>1.01</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -2665,7 +2663,7 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>24747619</v>
+        <v>603833</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -2673,49 +2671,49 @@
         </is>
       </c>
       <c r="U14" t="n">
-        <v>91.12</v>
+        <v>88.68000000000001</v>
       </c>
       <c r="V14" t="n">
-        <v>4.47</v>
+        <v>6.63</v>
       </c>
       <c r="W14" t="n">
-        <v>1.56</v>
+        <v>2.91</v>
       </c>
       <c r="X14" t="n">
-        <v>8.08</v>
+        <v>5.18</v>
       </c>
       <c r="Y14" t="n">
-        <v>1.23</v>
+        <v>3.66</v>
       </c>
       <c r="Z14" t="n">
-        <v>3.05</v>
+        <v>4.78</v>
       </c>
       <c r="AA14" t="n">
-        <v>4.19</v>
+        <v>1.96</v>
       </c>
       <c r="AB14" t="n">
-        <v>10.99</v>
+        <v>23.39</v>
       </c>
       <c r="AC14" t="n">
-        <v>6.76</v>
+        <v>18.38</v>
       </c>
       <c r="AD14" t="n">
-        <v>15.54</v>
+        <v>24.51</v>
       </c>
       <c r="AE14" t="n">
-        <v>6.53</v>
+        <v>17.37</v>
       </c>
       <c r="AF14" t="n">
-        <v>8.300000000000001</v>
+        <v>0</v>
       </c>
       <c r="AG14" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>45403.41666666666</v>
+        <v>44983.41666666666</v>
       </c>
       <c r="AI14" t="n">
-        <v>-13.35</v>
+        <v>-18.62</v>
       </c>
       <c r="AJ14" t="b">
         <v>1</v>
@@ -2727,31 +2725,31 @@
         <v>0</v>
       </c>
       <c r="AM14" t="n">
-        <v>0.9</v>
+        <v>7.74</v>
       </c>
       <c r="AN14" t="n">
-        <v>0.76</v>
+        <v>4.4</v>
       </c>
       <c r="AO14" t="n">
-        <v>0.9</v>
+        <v>7.48</v>
       </c>
       <c r="AP14" t="b">
         <v>0</v>
       </c>
       <c r="AQ14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS14" t="b">
         <v>1</v>
       </c>
       <c r="AT14" t="n">
-        <v>91.79104022332528</v>
+        <v>89.34911242603552</v>
       </c>
       <c r="AU14" t="n">
-        <v>0.91</v>
+        <v>7.74</v>
       </c>
       <c r="AV14" t="b">
         <v>1</v>
@@ -2763,7 +2761,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2775,43 +2773,43 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45431.41666666666</v>
+        <v>45006.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45446.41666666666</v>
+        <v>45067.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>0.9</v>
+        <v>7.2</v>
       </c>
       <c r="G15" t="n">
-        <v>-11.31</v>
+        <v>-9.44</v>
       </c>
       <c r="H15" t="n">
-        <v>0.78</v>
+        <v>6.52</v>
       </c>
       <c r="I15" t="n">
-        <v>0.85</v>
+        <v>7.45</v>
       </c>
       <c r="J15" t="n">
-        <v>-5.91</v>
+        <v>3.47</v>
       </c>
       <c r="K15" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="L15" t="n">
-        <v>0.8</v>
+        <v>6.52</v>
       </c>
       <c r="M15" t="n">
-        <v>0.89</v>
+        <v>7.13</v>
       </c>
       <c r="N15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>0.89</v>
+        <v>7.6</v>
       </c>
       <c r="P15" t="n">
-        <v>0.97</v>
+        <v>8.67</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -2824,7 +2822,7 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>25928938</v>
+        <v>676323</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -2832,49 +2830,49 @@
         </is>
       </c>
       <c r="U15" t="n">
-        <v>87.55</v>
+        <v>69.39</v>
       </c>
       <c r="V15" t="n">
-        <v>3.55</v>
+        <v>4.93</v>
       </c>
       <c r="W15" t="n">
-        <v>1.63</v>
+        <v>5.5</v>
       </c>
       <c r="X15" t="n">
-        <v>4.99</v>
+        <v>7.11</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.55</v>
+        <v>0.42</v>
       </c>
       <c r="Z15" t="n">
-        <v>1.73</v>
+        <v>0.98</v>
       </c>
       <c r="AA15" t="n">
-        <v>5.54</v>
+        <v>5.43</v>
       </c>
       <c r="AB15" t="n">
-        <v>2.83</v>
+        <v>3.06</v>
       </c>
       <c r="AC15" t="n">
-        <v>3.98</v>
+        <v>-0.24</v>
       </c>
       <c r="AD15" t="n">
-        <v>10.28</v>
+        <v>8.94</v>
       </c>
       <c r="AE15" t="n">
-        <v>3.28</v>
+        <v>2.86</v>
       </c>
       <c r="AF15" t="n">
-        <v>6.06</v>
+        <v>19.44</v>
       </c>
       <c r="AG15" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>45441.41666666666</v>
+        <v>45046.41666666666</v>
       </c>
       <c r="AI15" t="n">
-        <v>-5.91</v>
+        <v>-0.14</v>
       </c>
       <c r="AJ15" t="b">
         <v>1</v>
@@ -2886,31 +2884,31 @@
         <v>0</v>
       </c>
       <c r="AM15" t="n">
-        <v>0.89</v>
+        <v>7.13</v>
       </c>
       <c r="AN15" t="n">
-        <v>0.8</v>
+        <v>6.14</v>
       </c>
       <c r="AO15" t="n">
-        <v>0.9</v>
+        <v>7.63</v>
       </c>
       <c r="AP15" t="b">
         <v>0</v>
       </c>
       <c r="AQ15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR15" t="b">
         <v>0</v>
       </c>
       <c r="AS15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT15" t="n">
-        <v>87.55980888715901</v>
+        <v>44.30379746835444</v>
       </c>
       <c r="AU15" t="n">
-        <v>0.89</v>
+        <v>7.13</v>
       </c>
       <c r="AV15" t="b">
         <v>1</v>
@@ -2922,7 +2920,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2934,43 +2932,43 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45522.41666666666</v>
+        <v>45103.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45567.41666666666</v>
+        <v>45132.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>1.1</v>
+        <v>8.5</v>
       </c>
       <c r="G16" t="n">
-        <v>-27.76</v>
+        <v>-14.71</v>
       </c>
       <c r="H16" t="n">
-        <v>0.88</v>
+        <v>7.56</v>
       </c>
       <c r="I16" t="n">
-        <v>1.05</v>
+        <v>7.41</v>
       </c>
       <c r="J16" t="n">
-        <v>-4.24</v>
+        <v>-12.82</v>
       </c>
       <c r="K16" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="L16" t="n">
-        <v>0.79</v>
+        <v>7.25</v>
       </c>
       <c r="M16" t="n">
-        <v>1</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N16" t="b">
         <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>1.09</v>
+        <v>7.56</v>
       </c>
       <c r="P16" t="n">
-        <v>1.3</v>
+        <v>8.5</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -2983,7 +2981,7 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>186144552</v>
+        <v>204050</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
@@ -2991,49 +2989,49 @@
         </is>
       </c>
       <c r="U16" t="n">
-        <v>97.05</v>
+        <v>100</v>
       </c>
       <c r="V16" t="n">
-        <v>9.640000000000001</v>
+        <v>2.47</v>
       </c>
       <c r="W16" t="n">
-        <v>6.43</v>
+        <v>1.39</v>
       </c>
       <c r="X16" t="n">
-        <v>6.39</v>
+        <v>5.12</v>
       </c>
       <c r="Y16" t="n">
-        <v>2.86</v>
+        <v>1.78</v>
       </c>
       <c r="Z16" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB16" t="n">
         <v>10</v>
       </c>
-      <c r="AA16" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>22.36</v>
-      </c>
       <c r="AC16" t="n">
-        <v>20.04</v>
+        <v>9.32</v>
       </c>
       <c r="AD16" t="n">
-        <v>22.88</v>
+        <v>13.38</v>
       </c>
       <c r="AE16" t="n">
-        <v>17.86</v>
+        <v>6.92</v>
       </c>
       <c r="AF16" t="n">
-        <v>15.76</v>
+        <v>0</v>
       </c>
       <c r="AG16" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>45538.41666666666</v>
+        <v>45103.41666666666</v>
       </c>
       <c r="AI16" t="n">
-        <v>-4.24</v>
+        <v>-12.82</v>
       </c>
       <c r="AJ16" t="b">
         <v>1</v>
@@ -3045,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="AM16" t="n">
-        <v>1</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="AN16" t="n">
-        <v>0.84</v>
+        <v>7.2</v>
       </c>
       <c r="AO16" t="n">
-        <v>0.9399999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AP16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ16" t="b">
         <v>0</v>
@@ -3066,10 +3064,10 @@
         <v>1</v>
       </c>
       <c r="AT16" t="n">
-        <v>97.82608986294797</v>
+        <v>99.99999999999999</v>
       </c>
       <c r="AU16" t="n">
-        <v>1</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="AV16" t="b">
         <v>1</v>
@@ -3081,7 +3079,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3093,43 +3091,43 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45587.41666666666</v>
+        <v>45162.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45620.41666666666</v>
+        <v>45172.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>1.11</v>
+        <v>7.39</v>
       </c>
       <c r="G17" t="n">
-        <v>-10.24</v>
+        <v>-5.41</v>
       </c>
       <c r="H17" t="n">
-        <v>0.97</v>
+        <v>7.07</v>
       </c>
       <c r="I17" t="n">
-        <v>1.32</v>
+        <v>7.15</v>
       </c>
       <c r="J17" t="n">
-        <v>19.28</v>
+        <v>-3.25</v>
       </c>
       <c r="K17" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="L17" t="n">
-        <v>0.99</v>
+        <v>6.99</v>
       </c>
       <c r="M17" t="n">
-        <v>1.09</v>
+        <v>7.35</v>
       </c>
       <c r="N17" t="b">
         <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>1.35</v>
+        <v>7.28</v>
       </c>
       <c r="P17" t="n">
-        <v>1.47</v>
+        <v>7.87</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -3142,57 +3140,57 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>37405059</v>
+        <v>335317</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BULLISH_TREND</t>
         </is>
       </c>
       <c r="U17" t="n">
-        <v>95.45</v>
+        <v>74.42</v>
       </c>
       <c r="V17" t="n">
-        <v>-9.58</v>
+        <v>-5.07</v>
       </c>
       <c r="W17" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="X17" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="AF17" t="n">
         <v>2.03</v>
       </c>
-      <c r="X17" t="n">
-        <v>5.31</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="AB17" t="n">
-        <v>3.45</v>
-      </c>
-      <c r="AC17" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>9.58</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>5.06</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>32.53</v>
-      </c>
       <c r="AG17" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>45614.41666666666</v>
+        <v>45168.41666666666</v>
       </c>
       <c r="AI17" t="n">
-        <v>0</v>
+        <v>-3.25</v>
       </c>
       <c r="AJ17" t="b">
         <v>1</v>
@@ -3204,34 +3202,34 @@
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>1.22</v>
+        <v>7.88</v>
       </c>
       <c r="AN17" t="n">
-        <v>0.99</v>
+        <v>6.98</v>
       </c>
       <c r="AO17" t="n">
-        <v>1.12</v>
+        <v>7.5</v>
       </c>
       <c r="AP17" t="b">
         <v>0</v>
       </c>
       <c r="AQ17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS17" t="b">
         <v>1</v>
       </c>
       <c r="AT17" t="n">
-        <v>95.45454483471097</v>
+        <v>77.99999999999994</v>
       </c>
       <c r="AU17" t="n">
-        <v>1.09</v>
+        <v>7.88</v>
       </c>
       <c r="AV17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW17" t="inlineStr"/>
       <c r="AX17" t="inlineStr"/>
@@ -3240,7 +3238,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3249,46 +3247,46 @@
         </is>
       </c>
       <c r="C18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45628.41666666666</v>
+        <v>45176.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45648.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>1.52</v>
+        <v>8</v>
       </c>
       <c r="G18" t="n">
-        <v>-14.04</v>
+        <v>-10.62</v>
       </c>
       <c r="H18" t="n">
-        <v>1.33</v>
+        <v>7.13</v>
       </c>
       <c r="I18" t="n">
-        <v>1.53</v>
+        <v>10.03</v>
       </c>
       <c r="J18" t="n">
-        <v>0.88</v>
+        <v>25.37</v>
       </c>
       <c r="K18" t="n">
-        <v>20</v>
+        <v>249</v>
       </c>
       <c r="L18" t="n">
-        <v>1.31</v>
+        <v>7.15</v>
       </c>
       <c r="M18" t="n">
-        <v>1.47</v>
+        <v>7.87</v>
       </c>
       <c r="N18" t="b">
         <v>1</v>
       </c>
       <c r="O18" t="n">
-        <v>1.54</v>
+        <v>10.15</v>
       </c>
       <c r="P18" t="n">
-        <v>1.69</v>
+        <v>17.9</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -3301,7 +3299,7 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>109962794</v>
+        <v>339665</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -3309,49 +3307,49 @@
         </is>
       </c>
       <c r="U18" t="n">
-        <v>85.29000000000001</v>
+        <v>94.56</v>
       </c>
       <c r="V18" t="n">
-        <v>5.15</v>
+        <v>2.24</v>
       </c>
       <c r="W18" t="n">
-        <v>1.82</v>
+        <v>1.29</v>
       </c>
       <c r="X18" t="n">
-        <v>5.46</v>
+        <v>5.12</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.12</v>
+        <v>1.39</v>
       </c>
       <c r="Z18" t="n">
-        <v>3.17</v>
+        <v>1.65</v>
       </c>
       <c r="AA18" t="n">
-        <v>2.39</v>
+        <v>1.91</v>
       </c>
       <c r="AB18" t="n">
-        <v>20.51</v>
+        <v>7.65</v>
       </c>
       <c r="AC18" t="n">
-        <v>11.3</v>
+        <v>7.9</v>
       </c>
       <c r="AD18" t="n">
-        <v>11.99</v>
+        <v>9.59</v>
       </c>
       <c r="AE18" t="n">
-        <v>7.04</v>
+        <v>2.43</v>
       </c>
       <c r="AF18" t="n">
-        <v>9.65</v>
+        <v>100.5</v>
       </c>
       <c r="AG18" t="n">
-        <v>6</v>
+        <v>175</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>45634.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="AI18" t="n">
-        <v>0</v>
+        <v>-9.5</v>
       </c>
       <c r="AJ18" t="b">
         <v>1</v>
@@ -3363,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>1.47</v>
+        <v>7.87</v>
       </c>
       <c r="AN18" t="n">
-        <v>0.8</v>
+        <v>7.06</v>
       </c>
       <c r="AO18" t="n">
-        <v>1.46</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AP18" t="b">
         <v>0</v>
@@ -3378,16 +3376,16 @@
         <v>0</v>
       </c>
       <c r="AR18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT18" t="n">
-        <v>86.48648484295163</v>
+        <v>94.89795918367339</v>
       </c>
       <c r="AU18" t="n">
-        <v>1.47</v>
+        <v>7.97</v>
       </c>
       <c r="AV18" t="b">
         <v>1</v>
@@ -3399,7 +3397,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3408,109 +3406,109 @@
         </is>
       </c>
       <c r="C19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45662.41666666666</v>
+        <v>45496.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45508.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>1.67</v>
+        <v>10.5</v>
       </c>
       <c r="G19" t="n">
-        <v>-13.2</v>
+        <v>-11.71</v>
       </c>
       <c r="H19" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="I19" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-11.43</v>
+      </c>
+      <c r="K19" t="n">
+        <v>12</v>
+      </c>
+      <c r="L19" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="M19" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="N19" t="b">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="P19" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>2229943</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>80.28</v>
+      </c>
+      <c r="V19" t="n">
+        <v>-13.72</v>
+      </c>
+      <c r="W19" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="X19" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="Z19" t="n">
         <v>1.45</v>
       </c>
-      <c r="I19" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="J19" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="K19" t="n">
-        <v>79</v>
-      </c>
-      <c r="L19" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="M19" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="N19" t="b">
-        <v>1</v>
-      </c>
-      <c r="O19" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="P19" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S19" t="n">
-        <v>54533734</v>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U19" t="n">
-        <v>100</v>
-      </c>
-      <c r="V19" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="W19" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="X19" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>2.46</v>
-      </c>
       <c r="AA19" t="n">
-        <v>2.14</v>
+        <v>0.95</v>
       </c>
       <c r="AB19" t="n">
-        <v>14.7</v>
+        <v>1.53</v>
       </c>
       <c r="AC19" t="n">
-        <v>7.44</v>
+        <v>4.32</v>
       </c>
       <c r="AD19" t="n">
-        <v>11.71</v>
+        <v>11.01</v>
       </c>
       <c r="AE19" t="n">
-        <v>5.04</v>
+        <v>2.34</v>
       </c>
       <c r="AF19" t="n">
-        <v>13.2</v>
+        <v>0</v>
       </c>
       <c r="AG19" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>45732.41666666666</v>
+        <v>45496.41666666666</v>
       </c>
       <c r="AI19" t="n">
-        <v>-8.4</v>
+        <v>-11.43</v>
       </c>
       <c r="AJ19" t="b">
         <v>1</v>
@@ -3522,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>1.61</v>
+        <v>12.1</v>
       </c>
       <c r="AN19" t="n">
-        <v>1.49</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="AO19" t="n">
-        <v>1.63</v>
+        <v>10.75</v>
       </c>
       <c r="AP19" t="b">
         <v>0</v>
@@ -3537,19 +3535,19 @@
         <v>0</v>
       </c>
       <c r="AR19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT19" t="n">
-        <v>82.50000112499961</v>
+        <v>76.1904761904762</v>
       </c>
       <c r="AU19" t="n">
-        <v>1.63</v>
+        <v>10.97</v>
       </c>
       <c r="AV19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW19" t="inlineStr"/>
       <c r="AX19" t="inlineStr"/>
@@ -3558,7 +3556,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3570,43 +3568,43 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45820.41666666666</v>
+        <v>45525.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45915.41666666666</v>
+        <v>45656.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>1.74</v>
+        <v>11.3</v>
       </c>
       <c r="G20" t="n">
-        <v>-10.73</v>
+        <v>-23.01</v>
       </c>
       <c r="H20" t="n">
-        <v>1.55</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>1.61</v>
+        <v>16.29</v>
       </c>
       <c r="J20" t="n">
-        <v>-7.28</v>
+        <v>44.16</v>
       </c>
       <c r="K20" t="n">
-        <v>95</v>
+        <v>131</v>
       </c>
       <c r="L20" t="n">
-        <v>1.55</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>1.73</v>
+        <v>10.28</v>
       </c>
       <c r="N20" t="b">
         <v>1</v>
       </c>
       <c r="O20" t="n">
-        <v>1.63</v>
+        <v>16.3</v>
       </c>
       <c r="P20" t="n">
-        <v>2.19</v>
+        <v>17.77</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -3619,7 +3617,7 @@
         </is>
       </c>
       <c r="S20" t="n">
-        <v>93623145</v>
+        <v>10826324</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -3627,49 +3625,49 @@
         </is>
       </c>
       <c r="U20" t="n">
-        <v>93.33</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="V20" t="n">
-        <v>-11.79</v>
+        <v>11.99</v>
       </c>
       <c r="W20" t="n">
-        <v>3</v>
+        <v>4.82</v>
       </c>
       <c r="X20" t="n">
-        <v>3.62</v>
+        <v>5.76</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.87</v>
+        <v>1.96</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.38</v>
+        <v>9.92</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.85</v>
+        <v>0.4</v>
       </c>
       <c r="AB20" t="n">
-        <v>3.26</v>
+        <v>12.72</v>
       </c>
       <c r="AC20" t="n">
-        <v>4.37</v>
+        <v>14.68</v>
       </c>
       <c r="AD20" t="n">
-        <v>10.95</v>
+        <v>16.65</v>
       </c>
       <c r="AE20" t="n">
-        <v>1.95</v>
+        <v>11.22</v>
       </c>
       <c r="AF20" t="n">
-        <v>24.52</v>
+        <v>57.26</v>
       </c>
       <c r="AG20" t="n">
-        <v>24</v>
+        <v>123</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>45844.41666666666</v>
+        <v>45648.41666666666</v>
       </c>
       <c r="AI20" t="n">
-        <v>-7.28</v>
+        <v>-4.34</v>
       </c>
       <c r="AJ20" t="b">
         <v>1</v>
@@ -3681,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>1.96</v>
+        <v>10.28</v>
       </c>
       <c r="AN20" t="n">
-        <v>1.64</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="AO20" t="n">
-        <v>1.78</v>
+        <v>10.46</v>
       </c>
       <c r="AP20" t="b">
         <v>0</v>
@@ -3702,10 +3700,10 @@
         <v>1</v>
       </c>
       <c r="AT20" t="n">
-        <v>93.33333233333369</v>
+        <v>87.24832214765104</v>
       </c>
       <c r="AU20" t="n">
-        <v>1.73</v>
+        <v>10.49</v>
       </c>
       <c r="AV20" t="b">
         <v>1</v>
@@ -3717,7 +3715,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3729,43 +3727,43 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45938.41666666666</v>
+        <v>45662.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45979.41666666666</v>
+        <v>45665.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>1.76</v>
+        <v>17.2</v>
       </c>
       <c r="G21" t="n">
-        <v>-11.74</v>
+        <v>-6.28</v>
       </c>
       <c r="H21" t="n">
-        <v>1.66</v>
+        <v>16.02</v>
       </c>
       <c r="I21" t="n">
-        <v>1.83</v>
+        <v>15.8</v>
       </c>
       <c r="J21" t="n">
-        <v>3.98</v>
+        <v>-8.140000000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>1.55</v>
+        <v>16.12</v>
       </c>
       <c r="M21" t="n">
-        <v>1.71</v>
+        <v>17</v>
       </c>
       <c r="N21" t="b">
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>1.84</v>
+        <v>16.02</v>
       </c>
       <c r="P21" t="n">
-        <v>2.05</v>
+        <v>17.47</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -3778,7 +3776,7 @@
         </is>
       </c>
       <c r="S21" t="n">
-        <v>55814432</v>
+        <v>801972</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
@@ -3786,49 +3784,49 @@
         </is>
       </c>
       <c r="U21" t="n">
-        <v>88.23</v>
+        <v>81.38</v>
       </c>
       <c r="V21" t="n">
-        <v>3.38</v>
+        <v>2.69</v>
       </c>
       <c r="W21" t="n">
-        <v>2.07</v>
+        <v>0.98</v>
       </c>
       <c r="X21" t="n">
-        <v>2.74</v>
+        <v>3.97</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.19</v>
+        <v>2.48</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.72</v>
+        <v>1.18</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.71</v>
+        <v>1.53</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.54</v>
+        <v>10.94</v>
       </c>
       <c r="AC21" t="n">
-        <v>3.73</v>
+        <v>4.22</v>
       </c>
       <c r="AD21" t="n">
-        <v>9.800000000000001</v>
+        <v>5.31</v>
       </c>
       <c r="AE21" t="n">
-        <v>3.94</v>
+        <v>1.78</v>
       </c>
       <c r="AF21" t="n">
-        <v>12.5</v>
+        <v>0.52</v>
       </c>
       <c r="AG21" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>45967.41666666666</v>
+        <v>45663.41666666666</v>
       </c>
       <c r="AI21" t="n">
-        <v>-1.89</v>
+        <v>-8.140000000000001</v>
       </c>
       <c r="AJ21" t="b">
         <v>1</v>
@@ -3840,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>1.71</v>
+        <v>17</v>
       </c>
       <c r="AN21" t="n">
-        <v>1.64</v>
+        <v>14.66</v>
       </c>
       <c r="AO21" t="n">
-        <v>1.73</v>
+        <v>17.74</v>
       </c>
       <c r="AP21" t="b">
         <v>0</v>
@@ -3855,16 +3853,16 @@
         <v>0</v>
       </c>
       <c r="AR21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT21" t="n">
-        <v>93.10345237811985</v>
+        <v>67.42857142857142</v>
       </c>
       <c r="AU21" t="n">
-        <v>1.82</v>
+        <v>17.6</v>
       </c>
       <c r="AV21" t="b">
         <v>0</v>
@@ -3872,6 +3870,324 @@
       <c r="AW21" t="inlineStr"/>
       <c r="AX21" t="inlineStr"/>
       <c r="AY21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C22" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>45678.41666666666</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>45753.41666666666</v>
+      </c>
+      <c r="F22" t="n">
+        <v>17.95</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-21.89</v>
+      </c>
+      <c r="H22" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="I22" t="n">
+        <v>21</v>
+      </c>
+      <c r="J22" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="K22" t="n">
+        <v>75</v>
+      </c>
+      <c r="L22" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="M22" t="n">
+        <v>17.47</v>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="P22" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>7215730</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>82.39</v>
+      </c>
+      <c r="V22" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="W22" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="X22" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>14.28</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>33.48</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>48</v>
+      </c>
+      <c r="AH22" s="2" t="n">
+        <v>45726.41666666666</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="AJ22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>17.47</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>14.64</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="AP22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>82.38993710691824</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="AV22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C23" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>45761.41666666666</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>45907.41666666666</v>
+      </c>
+      <c r="F23" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-13.45</v>
+      </c>
+      <c r="H23" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="I23" t="n">
+        <v>37</v>
+      </c>
+      <c r="J23" t="n">
+        <v>63.72</v>
+      </c>
+      <c r="K23" t="n">
+        <v>146</v>
+      </c>
+      <c r="L23" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="M23" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="P23" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>581928</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>97.12</v>
+      </c>
+      <c r="V23" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="W23" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="X23" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>127</v>
+      </c>
+      <c r="AH23" s="2" t="n">
+        <v>45888.41666666666</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>-3.23</v>
+      </c>
+      <c r="AJ23" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>23</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="AO23" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="AP23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>83.33333333333333</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="AV23" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4147,7 +4463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4156,46 +4472,46 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46089.41666666666</v>
+        <v>45942.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46121.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>1.78</v>
+        <v>47.7</v>
       </c>
       <c r="G2" t="n">
-        <v>-18.54</v>
+        <v>-23.48</v>
       </c>
       <c r="H2" t="n">
-        <v>1.45</v>
+        <v>38.03</v>
       </c>
       <c r="I2" t="n">
-        <v>1.99</v>
+        <v>57.95</v>
       </c>
       <c r="J2" t="n">
-        <v>11.8</v>
+        <v>21.49</v>
       </c>
       <c r="K2" t="n">
-        <v>32</v>
+        <v>179</v>
       </c>
       <c r="L2" t="n">
-        <v>1.45</v>
+        <v>36.5</v>
       </c>
       <c r="M2" t="n">
-        <v>1.69</v>
+        <v>41.6</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>1.73</v>
+        <v>44.92</v>
       </c>
       <c r="P2" t="n">
-        <v>1.91</v>
+        <v>58.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -4208,7 +4524,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>42719294</v>
+        <v>3766781</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -4216,49 +4532,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>94.28</v>
+        <v>100</v>
       </c>
       <c r="V2" t="n">
-        <v>-6.67</v>
+        <v>12.79</v>
       </c>
       <c r="W2" t="n">
-        <v>3.64</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>3.89</v>
+        <v>5.27</v>
       </c>
       <c r="Y2" t="n">
-        <v>1.01</v>
+        <v>3.69</v>
       </c>
       <c r="Z2" t="n">
-        <v>5.33</v>
+        <v>14.66</v>
       </c>
       <c r="AA2" t="n">
-        <v>3.03</v>
+        <v>1.7</v>
       </c>
       <c r="AB2" t="n">
-        <v>4.11</v>
+        <v>24.15</v>
       </c>
       <c r="AC2" t="n">
-        <v>5.66</v>
+        <v>20.5</v>
       </c>
       <c r="AD2" t="n">
-        <v>15.29</v>
+        <v>13.06</v>
       </c>
       <c r="AE2" t="n">
-        <v>5.33</v>
+        <v>20</v>
       </c>
       <c r="AF2" t="n">
-        <v>11.8</v>
+        <v>21.49</v>
       </c>
       <c r="AG2" t="n">
-        <v>32</v>
+        <v>179</v>
       </c>
       <c r="AH2" s="2" t="n">
         <v>46121.41666666666</v>
       </c>
       <c r="AI2" t="n">
-        <v>-4.49</v>
+        <v>-5.62</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -4270,16 +4586,16 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>1.92</v>
+        <v>41.6</v>
       </c>
       <c r="AN2" t="n">
-        <v>1.61</v>
+        <v>39</v>
       </c>
       <c r="AO2" t="n">
-        <v>1.79</v>
+        <v>41.17</v>
       </c>
       <c r="AP2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ2" t="b">
         <v>0</v>
@@ -4291,16 +4607,16 @@
         <v>1</v>
       </c>
       <c r="AT2" t="n">
-        <v>94.28571428571428</v>
+        <v>100</v>
       </c>
       <c r="AU2" t="n">
-        <v>1.72</v>
+        <v>41.6</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
       </c>
       <c r="AW2" t="n">
-        <v>1.99</v>
+        <v>57.95</v>
       </c>
       <c r="AX2" t="b">
         <v>1</v>
@@ -4433,7 +4749,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4442,55 +4758,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
         <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>45</v>
+        <v>40.91</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.9</v>
+        <v>-1.46</v>
       </c>
       <c r="H2" t="n">
-        <v>7.95</v>
+        <v>6.29</v>
       </c>
       <c r="I2" t="n">
-        <v>159.06</v>
+        <v>138.37</v>
       </c>
       <c r="J2" t="n">
-        <v>114.84</v>
+        <v>63.72</v>
       </c>
       <c r="K2" t="n">
-        <v>-19.22</v>
+        <v>-18.62</v>
       </c>
       <c r="L2" t="n">
-        <v>34.24</v>
+        <v>22.64</v>
       </c>
       <c r="M2" t="n">
-        <v>2.56</v>
+        <v>2.23</v>
       </c>
       <c r="N2" t="n">
-        <v>28.97</v>
+        <v>27.9</v>
       </c>
       <c r="O2" t="n">
-        <v>9.24</v>
+        <v>8.67</v>
       </c>
       <c r="P2" t="n">
-        <v>7.95</v>
+        <v>6.29</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.497594211123723</v>
+        <v>0.474350296108291</v>
       </c>
       <c r="R2" t="n">
-        <v>0.484</v>
+        <v>0.5416</v>
       </c>
       <c r="S2" t="n">
-        <v>0.4894376844494892</v>
+        <v>0.5147001184433164</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -4498,7 +4814,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.4894376844494892</v>
+        <v>0.5147001184433164</v>
       </c>
     </row>
   </sheetData>
@@ -4560,7 +4876,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DSCW</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4569,22 +4885,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
-        <v>45</v>
+        <v>40.91</v>
       </c>
       <c r="F2" t="n">
-        <v>2.56</v>
+        <v>2.23</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.9</v>
+        <v>-1.46</v>
       </c>
       <c r="H2" t="n">
-        <v>7.95</v>
+        <v>6.29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-12 19:34:55.925968
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY9"/>
+  <dimension ref="A1:AY22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -705,46 +705,46 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>44333.45833333334</v>
+        <v>43852.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>44349.45833333334</v>
+        <v>43891.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>4.25</v>
+        <v>3.59</v>
       </c>
       <c r="G2" t="n">
-        <v>-22.35</v>
+        <v>-19.5</v>
       </c>
       <c r="H2" t="n">
-        <v>3.3</v>
+        <v>3.31</v>
       </c>
       <c r="I2" t="n">
-        <v>4.28</v>
+        <v>3.1</v>
       </c>
       <c r="J2" t="n">
-        <v>0.71</v>
+        <v>-13.65</v>
       </c>
       <c r="K2" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="L2" t="n">
-        <v>3.3</v>
+        <v>2.89</v>
       </c>
       <c r="M2" t="n">
-        <v>4.01</v>
+        <v>3.57</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>4.32</v>
+        <v>3.31</v>
       </c>
       <c r="P2" t="n">
-        <v>4.84</v>
+        <v>3.78</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>3468414</v>
+        <v>113942</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -765,49 +765,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>89.62</v>
+        <v>96.55</v>
       </c>
       <c r="V2" t="n">
-        <v>11.24</v>
+        <v>-14.72</v>
       </c>
       <c r="W2" t="n">
-        <v>6.05</v>
+        <v>0.97</v>
       </c>
       <c r="X2" t="n">
-        <v>6.43</v>
+        <v>3.07</v>
       </c>
       <c r="Y2" t="n">
-        <v>3.15</v>
+        <v>0.39</v>
       </c>
       <c r="Z2" t="n">
-        <v>5.99</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AA2" t="n">
-        <v>3.92</v>
+        <v>1.16</v>
       </c>
       <c r="AB2" t="n">
-        <v>25.46</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" t="n">
-        <v>18.8</v>
+        <v>4.22</v>
       </c>
       <c r="AD2" t="n">
-        <v>19.43</v>
+        <v>21.05</v>
       </c>
       <c r="AE2" t="n">
-        <v>7.05</v>
+        <v>2.57</v>
       </c>
       <c r="AF2" t="n">
-        <v>11.29</v>
+        <v>4.74</v>
       </c>
       <c r="AG2" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>44339.45833333334</v>
+        <v>43863.41666666666</v>
       </c>
       <c r="AI2" t="n">
-        <v>0</v>
+        <v>-13.65</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -819,13 +819,13 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>3.87</v>
+        <v>4.13</v>
       </c>
       <c r="AN2" t="n">
-        <v>3.42</v>
+        <v>3.41</v>
       </c>
       <c r="AO2" t="n">
-        <v>4.01</v>
+        <v>3.53</v>
       </c>
       <c r="AP2" t="b">
         <v>0</v>
@@ -840,10 +840,10 @@
         <v>1</v>
       </c>
       <c r="AT2" t="n">
-        <v>89.62264150943393</v>
+        <v>98.59154929577461</v>
       </c>
       <c r="AU2" t="n">
-        <v>4.01</v>
+        <v>3.57</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
@@ -864,46 +864,46 @@
         </is>
       </c>
       <c r="C3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>44377.45833333334</v>
+        <v>44040.45833333334</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>44444.45833333334</v>
+        <v>44082.45833333334</v>
       </c>
       <c r="F3" t="n">
-        <v>5.27</v>
+        <v>3.5</v>
       </c>
       <c r="G3" t="n">
-        <v>-18.41</v>
+        <v>-16.86</v>
       </c>
       <c r="H3" t="n">
-        <v>4.52</v>
+        <v>2.91</v>
       </c>
       <c r="I3" t="n">
-        <v>4.6</v>
+        <v>3.49</v>
       </c>
       <c r="J3" t="n">
-        <v>-12.71</v>
+        <v>-0.29</v>
       </c>
       <c r="K3" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="L3" t="n">
-        <v>4.3</v>
+        <v>2.91</v>
       </c>
       <c r="M3" t="n">
-        <v>4.98</v>
+        <v>3.47</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>4.8</v>
+        <v>3.67</v>
       </c>
       <c r="P3" t="n">
-        <v>6.18</v>
+        <v>4.14</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>4553564</v>
+        <v>3078417</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -924,49 +924,49 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>91.45999999999999</v>
+        <v>85.51000000000001</v>
       </c>
       <c r="V3" t="n">
-        <v>12.92</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>5.05</v>
+        <v>5.28</v>
       </c>
       <c r="X3" t="n">
-        <v>6.65</v>
+        <v>5.99</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.83</v>
+        <v>1.03</v>
       </c>
       <c r="Z3" t="n">
-        <v>5.82</v>
+        <v>0.86</v>
       </c>
       <c r="AA3" t="n">
-        <v>4.4</v>
+        <v>5.19</v>
       </c>
       <c r="AB3" t="n">
-        <v>23.22</v>
+        <v>6.57</v>
       </c>
       <c r="AC3" t="n">
-        <v>13.4</v>
+        <v>6.29</v>
       </c>
       <c r="AD3" t="n">
-        <v>14.66</v>
+        <v>17.55</v>
       </c>
       <c r="AE3" t="n">
-        <v>8.44</v>
+        <v>4.48</v>
       </c>
       <c r="AF3" t="n">
-        <v>12.14</v>
+        <v>14.57</v>
       </c>
       <c r="AG3" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>44418.45833333334</v>
+        <v>44074.45833333334</v>
       </c>
       <c r="AI3" t="n">
-        <v>-12.71</v>
+        <v>-2.57</v>
       </c>
       <c r="AJ3" t="b">
         <v>1</v>
@@ -978,31 +978,31 @@
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>4.65</v>
+        <v>3.6</v>
       </c>
       <c r="AN3" t="n">
-        <v>4.09</v>
+        <v>3.03</v>
       </c>
       <c r="AO3" t="n">
-        <v>5.04</v>
+        <v>3.55</v>
       </c>
       <c r="AP3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ3" t="b">
         <v>1</v>
       </c>
       <c r="AR3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS3" t="b">
         <v>1</v>
       </c>
       <c r="AT3" t="n">
-        <v>93.26923076923075</v>
+        <v>85.50724637681158</v>
       </c>
       <c r="AU3" t="n">
-        <v>5.12</v>
+        <v>3.47</v>
       </c>
       <c r="AV3" t="b">
         <v>1</v>
@@ -1023,46 +1023,46 @@
         </is>
       </c>
       <c r="C4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>44896.41666666666</v>
+        <v>44147.41666666666</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>44936.41666666666</v>
+        <v>44175.41666666666</v>
       </c>
       <c r="F4" t="n">
-        <v>6.08</v>
+        <v>3.2</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.62</v>
+        <v>-12.5</v>
       </c>
       <c r="H4" t="n">
-        <v>5.76</v>
+        <v>2.8</v>
       </c>
       <c r="I4" t="n">
-        <v>6.84</v>
+        <v>3.21</v>
       </c>
       <c r="J4" t="n">
-        <v>12.5</v>
+        <v>0.31</v>
       </c>
       <c r="K4" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="L4" t="n">
-        <v>5.86</v>
+        <v>2.8</v>
       </c>
       <c r="M4" t="n">
-        <v>6.05</v>
+        <v>3.15</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>7.12</v>
+        <v>3.23</v>
       </c>
       <c r="P4" t="n">
-        <v>7.74</v>
+        <v>3.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -1075,57 +1075,57 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>7973</v>
+        <v>2506229</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>BULLISH_TREND</t>
+          <t>BULLISH_BREAK</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>96.97</v>
+        <v>83.33</v>
       </c>
       <c r="V4" t="n">
-        <v>14.61</v>
+        <v>-25</v>
       </c>
       <c r="W4" t="n">
-        <v>0.07000000000000001</v>
+        <v>3.09</v>
       </c>
       <c r="X4" t="n">
-        <v>3.09</v>
+        <v>3.88</v>
       </c>
       <c r="Y4" t="n">
-        <v>4.49</v>
+        <v>-0.73</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.5</v>
+        <v>1.59</v>
       </c>
       <c r="AA4" t="n">
-        <v>7</v>
+        <v>3.34</v>
       </c>
       <c r="AB4" t="n">
-        <v>16.12</v>
+        <v>-2.74</v>
       </c>
       <c r="AC4" t="n">
-        <v>7.64</v>
+        <v>2.19</v>
       </c>
       <c r="AD4" t="n">
-        <v>3.19</v>
+        <v>11.76</v>
       </c>
       <c r="AE4" t="n">
-        <v>1.33</v>
+        <v>2.56</v>
       </c>
       <c r="AF4" t="n">
-        <v>25.16</v>
+        <v>8.44</v>
       </c>
       <c r="AG4" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>44935.41666666666</v>
+        <v>44166.41666666666</v>
       </c>
       <c r="AI4" t="n">
-        <v>-2.14</v>
+        <v>-3.13</v>
       </c>
       <c r="AJ4" t="b">
         <v>1</v>
@@ -1137,13 +1137,13 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>5.2</v>
+        <v>4.1</v>
       </c>
       <c r="AN4" t="n">
-        <v>3.1</v>
+        <v>2.97</v>
       </c>
       <c r="AO4" t="n">
-        <v>6.08</v>
+        <v>3.46</v>
       </c>
       <c r="AP4" t="b">
         <v>0</v>
@@ -1158,13 +1158,13 @@
         <v>1</v>
       </c>
       <c r="AT4" t="n">
-        <v>98.82352941176472</v>
+        <v>84.90566037735854</v>
       </c>
       <c r="AU4" t="n">
-        <v>6.13</v>
+        <v>3.17</v>
       </c>
       <c r="AV4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="inlineStr"/>
@@ -1182,46 +1182,46 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>44983.41666666666</v>
+        <v>44208.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45004.41666666666</v>
+        <v>44258.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>8.109999999999999</v>
+        <v>3.54</v>
       </c>
       <c r="G5" t="n">
-        <v>-25.4</v>
+        <v>-14.97</v>
       </c>
       <c r="H5" t="n">
-        <v>6.7</v>
+        <v>3.13</v>
       </c>
       <c r="I5" t="n">
-        <v>6.6</v>
+        <v>3.05</v>
       </c>
       <c r="J5" t="n">
-        <v>-18.62</v>
+        <v>-13.84</v>
       </c>
       <c r="K5" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="L5" t="n">
-        <v>6.05</v>
+        <v>3.01</v>
       </c>
       <c r="M5" t="n">
-        <v>7.74</v>
+        <v>3.41</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>6.7</v>
+        <v>3.13</v>
       </c>
       <c r="P5" t="n">
-        <v>8.289999999999999</v>
+        <v>3.74</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>603833</v>
+        <v>9793276</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -1242,49 +1242,49 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>88.68000000000001</v>
+        <v>78.84</v>
       </c>
       <c r="V5" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="W5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="X5" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="AE5" t="n">
         <v>6.63</v>
       </c>
-      <c r="W5" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="X5" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>23.39</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>18.38</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>24.51</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>17.37</v>
-      </c>
       <c r="AF5" t="n">
-        <v>0</v>
+        <v>3.67</v>
       </c>
       <c r="AG5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>44983.41666666666</v>
+        <v>44216.41666666666</v>
       </c>
       <c r="AI5" t="n">
-        <v>-18.62</v>
+        <v>-13.84</v>
       </c>
       <c r="AJ5" t="b">
         <v>1</v>
@@ -1296,13 +1296,13 @@
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>7.74</v>
+        <v>3.43</v>
       </c>
       <c r="AN5" t="n">
-        <v>4.4</v>
+        <v>3.32</v>
       </c>
       <c r="AO5" t="n">
-        <v>7.48</v>
+        <v>3.34</v>
       </c>
       <c r="AP5" t="b">
         <v>0</v>
@@ -1317,10 +1317,10 @@
         <v>1</v>
       </c>
       <c r="AT5" t="n">
-        <v>89.34911242603552</v>
+        <v>81.35593220338986</v>
       </c>
       <c r="AU5" t="n">
-        <v>7.74</v>
+        <v>3.41</v>
       </c>
       <c r="AV5" t="b">
         <v>1</v>
@@ -1341,46 +1341,46 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45224.41666666666</v>
+        <v>44294.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>44349.45833333334</v>
       </c>
       <c r="F6" t="n">
-        <v>9.359999999999999</v>
+        <v>3.32</v>
       </c>
       <c r="G6" t="n">
-        <v>-23.82</v>
+        <v>-18.67</v>
       </c>
       <c r="H6" t="n">
-        <v>7.7</v>
+        <v>2.7</v>
       </c>
       <c r="I6" t="n">
-        <v>10.03</v>
+        <v>4.28</v>
       </c>
       <c r="J6" t="n">
-        <v>7.16</v>
+        <v>28.92</v>
       </c>
       <c r="K6" t="n">
-        <v>201</v>
+        <v>55</v>
       </c>
       <c r="L6" t="n">
-        <v>7.13</v>
+        <v>2.7</v>
       </c>
       <c r="M6" t="n">
-        <v>8.050000000000001</v>
+        <v>3.16</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>10.15</v>
+        <v>4.32</v>
       </c>
       <c r="P6" t="n">
-        <v>17.9</v>
+        <v>4.84</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>636643</v>
+        <v>3957625</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1401,49 +1401,49 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>100</v>
+        <v>95.38</v>
       </c>
       <c r="V6" t="n">
-        <v>23.82</v>
+        <v>2.09</v>
       </c>
       <c r="W6" t="n">
-        <v>5.64</v>
+        <v>5.98</v>
       </c>
       <c r="X6" t="n">
-        <v>6.06</v>
+        <v>6.55</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.94</v>
+        <v>1.05</v>
       </c>
       <c r="Z6" t="n">
-        <v>16.27</v>
+        <v>5.06</v>
       </c>
       <c r="AA6" t="n">
-        <v>2.79</v>
+        <v>2.39</v>
       </c>
       <c r="AB6" t="n">
-        <v>21.7</v>
+        <v>7.42</v>
       </c>
       <c r="AC6" t="n">
-        <v>19.01</v>
+        <v>11.54</v>
       </c>
       <c r="AD6" t="n">
-        <v>12.12</v>
+        <v>15.7</v>
       </c>
       <c r="AE6" t="n">
-        <v>20</v>
+        <v>8.85</v>
       </c>
       <c r="AF6" t="n">
-        <v>71.37</v>
+        <v>42.47</v>
       </c>
       <c r="AG6" t="n">
-        <v>127</v>
+        <v>45</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>44339.45833333334</v>
       </c>
       <c r="AI6" t="n">
-        <v>-2.24</v>
+        <v>0</v>
       </c>
       <c r="AJ6" t="b">
         <v>1</v>
@@ -1455,13 +1455,13 @@
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>7.13</v>
+        <v>3.28</v>
       </c>
       <c r="AN6" t="n">
-        <v>7.12</v>
+        <v>2.98</v>
       </c>
       <c r="AO6" t="n">
-        <v>8.07</v>
+        <v>3.34</v>
       </c>
       <c r="AP6" t="b">
         <v>0</v>
@@ -1476,10 +1476,10 @@
         <v>1</v>
       </c>
       <c r="AT6" t="n">
-        <v>100</v>
+        <v>96.20253164556958</v>
       </c>
       <c r="AU6" t="n">
-        <v>8.4</v>
+        <v>3.16</v>
       </c>
       <c r="AV6" t="b">
         <v>1</v>
@@ -1500,46 +1500,46 @@
         </is>
       </c>
       <c r="C7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45641.41666666666</v>
+        <v>44353.45833333334</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45656.41666666666</v>
+        <v>44444.45833333334</v>
       </c>
       <c r="F7" t="n">
-        <v>17.01</v>
+        <v>4.66</v>
       </c>
       <c r="G7" t="n">
-        <v>-13.29</v>
+        <v>-12.02</v>
       </c>
       <c r="H7" t="n">
-        <v>15.15</v>
+        <v>4.09</v>
       </c>
       <c r="I7" t="n">
-        <v>16.29</v>
+        <v>4.6</v>
       </c>
       <c r="J7" t="n">
-        <v>-4.23</v>
+        <v>-1.29</v>
       </c>
       <c r="K7" t="n">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="L7" t="n">
-        <v>14.75</v>
+        <v>4.1</v>
       </c>
       <c r="M7" t="n">
-        <v>16.6</v>
+        <v>4.65</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>16.3</v>
+        <v>4.8</v>
       </c>
       <c r="P7" t="n">
-        <v>17.77</v>
+        <v>6.18</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>2026310</v>
+        <v>2292545</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1560,49 +1560,49 @@
         </is>
       </c>
       <c r="U7" t="n">
-        <v>91.63</v>
+        <v>91.93000000000001</v>
       </c>
       <c r="V7" t="n">
-        <v>29.57</v>
+        <v>1.27</v>
       </c>
       <c r="W7" t="n">
-        <v>2.2</v>
+        <v>2.04</v>
       </c>
       <c r="X7" t="n">
-        <v>3.63</v>
+        <v>7.8</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.12</v>
+        <v>2.21</v>
       </c>
       <c r="Z7" t="n">
-        <v>2.47</v>
+        <v>0.22</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.46</v>
+        <v>6.28</v>
       </c>
       <c r="AB7" t="n">
-        <v>17.54</v>
+        <v>20.83</v>
       </c>
       <c r="AC7" t="n">
-        <v>10.38</v>
+        <v>9.49</v>
       </c>
       <c r="AD7" t="n">
-        <v>11.8</v>
+        <v>12.57</v>
       </c>
       <c r="AE7" t="n">
-        <v>3.97</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="AF7" t="n">
-        <v>4.47</v>
+        <v>26.82</v>
       </c>
       <c r="AG7" t="n">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>45648.41666666666</v>
+        <v>44418.45833333334</v>
       </c>
       <c r="AI7" t="n">
-        <v>-4.23</v>
+        <v>-7.51</v>
       </c>
       <c r="AJ7" t="b">
         <v>1</v>
@@ -1614,13 +1614,13 @@
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>12.1</v>
+        <v>4.65</v>
       </c>
       <c r="AN7" t="n">
-        <v>14.66</v>
+        <v>3.37</v>
       </c>
       <c r="AO7" t="n">
-        <v>16.6</v>
+        <v>4.51</v>
       </c>
       <c r="AP7" t="b">
         <v>0</v>
@@ -1629,16 +1629,16 @@
         <v>0</v>
       </c>
       <c r="AR7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT7" t="n">
-        <v>93.41085271317837</v>
+        <v>76.00000000000004</v>
       </c>
       <c r="AU7" t="n">
-        <v>16.6</v>
+        <v>4.65</v>
       </c>
       <c r="AV7" t="b">
         <v>1</v>
@@ -1659,46 +1659,46 @@
         </is>
       </c>
       <c r="C8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45678.41666666666</v>
+        <v>44551.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45753.41666666666</v>
+        <v>44577.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>17.95</v>
+        <v>4.32</v>
       </c>
       <c r="G8" t="n">
-        <v>-21.89</v>
+        <v>-25.93</v>
       </c>
       <c r="H8" t="n">
-        <v>14.02</v>
+        <v>3.67</v>
       </c>
       <c r="I8" t="n">
-        <v>21</v>
+        <v>4.25</v>
       </c>
       <c r="J8" t="n">
-        <v>16.99</v>
+        <v>-1.62</v>
       </c>
       <c r="K8" t="n">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="L8" t="n">
-        <v>14.02</v>
+        <v>3.2</v>
       </c>
       <c r="M8" t="n">
-        <v>17.47</v>
+        <v>4.29</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
       </c>
       <c r="O8" t="n">
-        <v>22.25</v>
+        <v>4.5</v>
       </c>
       <c r="P8" t="n">
-        <v>23.96</v>
+        <v>4.7</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1711,57 +1711,57 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>7215730</v>
+        <v>1089232</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BULLISH_TREND</t>
         </is>
       </c>
       <c r="U8" t="n">
-        <v>82.39</v>
+        <v>95.59</v>
       </c>
       <c r="V8" t="n">
-        <v>9.529999999999999</v>
+        <v>-19.54</v>
       </c>
       <c r="W8" t="n">
-        <v>4.95</v>
+        <v>4.51</v>
       </c>
       <c r="X8" t="n">
-        <v>7.21</v>
+        <v>4.15</v>
       </c>
       <c r="Y8" t="n">
-        <v>1.73</v>
+        <v>1.85</v>
       </c>
       <c r="Z8" t="n">
-        <v>2.75</v>
+        <v>0.7</v>
       </c>
       <c r="AA8" t="n">
-        <v>2.76</v>
+        <v>3.86</v>
       </c>
       <c r="AB8" t="n">
-        <v>14.28</v>
+        <v>8.32</v>
       </c>
       <c r="AC8" t="n">
-        <v>10.17</v>
+        <v>7.71</v>
       </c>
       <c r="AD8" t="n">
-        <v>21.91</v>
+        <v>29.11</v>
       </c>
       <c r="AE8" t="n">
-        <v>8.130000000000001</v>
+        <v>1.89</v>
       </c>
       <c r="AF8" t="n">
-        <v>33.48</v>
+        <v>7.41</v>
       </c>
       <c r="AG8" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>45726.41666666666</v>
+        <v>44566.41666666666</v>
       </c>
       <c r="AI8" t="n">
-        <v>-1.78</v>
+        <v>-1.62</v>
       </c>
       <c r="AJ8" t="b">
         <v>1</v>
@@ -1773,16 +1773,16 @@
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>17</v>
+        <v>5.2</v>
       </c>
       <c r="AN8" t="n">
-        <v>14.64</v>
+        <v>4.08</v>
       </c>
       <c r="AO8" t="n">
-        <v>17.6</v>
+        <v>4.4</v>
       </c>
       <c r="AP8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ8" t="b">
         <v>0</v>
@@ -1794,13 +1794,13 @@
         <v>1</v>
       </c>
       <c r="AT8" t="n">
-        <v>82.38993710691824</v>
+        <v>89.04109589041094</v>
       </c>
       <c r="AU8" t="n">
-        <v>17.72</v>
+        <v>4.41</v>
       </c>
       <c r="AV8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW8" t="inlineStr"/>
       <c r="AX8" t="inlineStr"/>
@@ -1818,46 +1818,46 @@
         </is>
       </c>
       <c r="C9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45775.41666666666</v>
+        <v>44598.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45907.41666666666</v>
+        <v>44627.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>24</v>
+        <v>4.64</v>
       </c>
       <c r="G9" t="n">
-        <v>-9.17</v>
+        <v>-10.56</v>
       </c>
       <c r="H9" t="n">
-        <v>21.8</v>
+        <v>4.15</v>
       </c>
       <c r="I9" t="n">
-        <v>37</v>
+        <v>4.02</v>
       </c>
       <c r="J9" t="n">
-        <v>54.17</v>
+        <v>-13.36</v>
       </c>
       <c r="K9" t="n">
-        <v>132</v>
+        <v>29</v>
       </c>
       <c r="L9" t="n">
-        <v>21.8</v>
+        <v>4.15</v>
       </c>
       <c r="M9" t="n">
-        <v>23.18</v>
+        <v>4.5</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>37.5</v>
+        <v>4.15</v>
       </c>
       <c r="P9" t="n">
-        <v>48.89</v>
+        <v>4.64</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>552715</v>
+        <v>158602</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -1878,49 +1878,49 @@
         </is>
       </c>
       <c r="U9" t="n">
-        <v>95.65000000000001</v>
+        <v>100</v>
       </c>
       <c r="V9" t="n">
-        <v>4.56</v>
+        <v>-1.29</v>
       </c>
       <c r="W9" t="n">
-        <v>1.21</v>
+        <v>3.59</v>
       </c>
       <c r="X9" t="n">
-        <v>4.09</v>
+        <v>4.27</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.47</v>
+        <v>1.96</v>
       </c>
       <c r="Z9" t="n">
-        <v>3.54</v>
+        <v>3.11</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.14</v>
+        <v>0.65</v>
       </c>
       <c r="AB9" t="n">
-        <v>11.25</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="AC9" t="n">
-        <v>7.69</v>
+        <v>7</v>
       </c>
       <c r="AD9" t="n">
-        <v>6.14</v>
+        <v>8.09</v>
       </c>
       <c r="AE9" t="n">
-        <v>3.99</v>
+        <v>7.41</v>
       </c>
       <c r="AF9" t="n">
-        <v>90.54000000000001</v>
+        <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>113</v>
+        <v>0</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>45888.41666666666</v>
+        <v>44598.41666666666</v>
       </c>
       <c r="AI9" t="n">
-        <v>-0.75</v>
+        <v>-13.36</v>
       </c>
       <c r="AJ9" t="b">
         <v>1</v>
@@ -1932,16 +1932,16 @@
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>23</v>
+        <v>4.7</v>
       </c>
       <c r="AN9" t="n">
-        <v>22.08</v>
+        <v>4.11</v>
       </c>
       <c r="AO9" t="n">
-        <v>23.67</v>
+        <v>4.68</v>
       </c>
       <c r="AP9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ9" t="b">
         <v>0</v>
@@ -1953,17 +1953,2082 @@
         <v>1</v>
       </c>
       <c r="AT9" t="n">
-        <v>97.87234042553187</v>
+        <v>100</v>
       </c>
       <c r="AU9" t="n">
-        <v>23.18</v>
+        <v>4.68</v>
       </c>
       <c r="AV9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW9" t="inlineStr"/>
       <c r="AX9" t="inlineStr"/>
       <c r="AY9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>44643.41666666666</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>44661.41666666666</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-9.050000000000001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-12.99</v>
+      </c>
+      <c r="K10" t="n">
+        <v>18</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="M10" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="P10" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>293154</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>BULLISH_TREND</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>74.54000000000001</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="X10" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="2" t="n">
+        <v>44643.41666666666</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>-12.99</v>
+      </c>
+      <c r="AJ10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="AP10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>74.54545454545446</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="AV10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>44747.45833333334</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>44822.45833333334</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-6.06</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J11" t="n">
+        <v>42.42</v>
+      </c>
+      <c r="K11" t="n">
+        <v>75</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="P11" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>310094</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>BEARISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>100</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-33.33</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="X11" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>-1.26</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>-6.26</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>58.18</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>65</v>
+      </c>
+      <c r="AH11" s="2" t="n">
+        <v>44812.45833333334</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="AJ11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>50.00000000000001</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="AV11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>44872.41666666666</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>44936.41666666666</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-18.2</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="J12" t="n">
+        <v>25.74</v>
+      </c>
+      <c r="K12" t="n">
+        <v>64</v>
+      </c>
+      <c r="L12" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="M12" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="N12" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="P12" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>439840</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>96.91</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="W12" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="X12" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>15.27</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>19.29</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>39.89</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>63</v>
+      </c>
+      <c r="AH12" s="2" t="n">
+        <v>44935.41666666666</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>-4.41</v>
+      </c>
+      <c r="AJ12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="AP12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>96.90721649484543</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="AV12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>44983.41666666666</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>45004.41666666666</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8.109999999999999</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="I13" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-18.62</v>
+      </c>
+      <c r="K13" t="n">
+        <v>21</v>
+      </c>
+      <c r="L13" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="M13" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="P13" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>603833</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>88.68000000000001</v>
+      </c>
+      <c r="V13" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="W13" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="X13" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="2" t="n">
+        <v>44983.41666666666</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>-18.62</v>
+      </c>
+      <c r="AJ13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="AP13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>89.34911242603552</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="AV13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>45011.41666666666</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>45067.41666666666</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-15.21</v>
+      </c>
+      <c r="H14" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="I14" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="K14" t="n">
+        <v>56</v>
+      </c>
+      <c r="L14" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="M14" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="P14" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>1034727</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>98.91</v>
+      </c>
+      <c r="V14" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="W14" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="X14" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>13.98</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>11.83</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>35</v>
+      </c>
+      <c r="AH14" s="2" t="n">
+        <v>45046.41666666666</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="AJ14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="AP14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>85.00000000000001</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="AV14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>45103.41666666666</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>45132.41666666666</v>
+      </c>
+      <c r="F15" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-14.71</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-12.82</v>
+      </c>
+      <c r="K15" t="n">
+        <v>29</v>
+      </c>
+      <c r="L15" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="M15" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="P15" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>204050</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>100</v>
+      </c>
+      <c r="V15" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="W15" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="X15" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="2" t="n">
+        <v>45103.41666666666</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>-12.82</v>
+      </c>
+      <c r="AJ15" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="AP15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR15" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS15" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>99.99999999999999</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="AV15" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>45162.41666666666</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>45172.41666666666</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-5.41</v>
+      </c>
+      <c r="H16" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="J16" t="n">
+        <v>-3.25</v>
+      </c>
+      <c r="K16" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="M16" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="N16" t="b">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="P16" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>335317</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>BULLISH_TREND</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>74.42</v>
+      </c>
+      <c r="V16" t="n">
+        <v>-5.07</v>
+      </c>
+      <c r="W16" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="X16" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH16" s="2" t="n">
+        <v>45168.41666666666</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>-3.25</v>
+      </c>
+      <c r="AJ16" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="AP16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR16" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS16" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>77.99999999999994</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="AV16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>45176.41666666666</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>45425.41666666666</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-10.62</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="I17" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="J17" t="n">
+        <v>25.37</v>
+      </c>
+      <c r="K17" t="n">
+        <v>249</v>
+      </c>
+      <c r="L17" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="M17" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="P17" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>339665</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>94.56</v>
+      </c>
+      <c r="V17" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="W17" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="X17" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>175</v>
+      </c>
+      <c r="AH17" s="2" t="n">
+        <v>45351.41666666666</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="AJ17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="AP17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>94.89795918367339</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="AV17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>45496.41666666666</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>45508.41666666666</v>
+      </c>
+      <c r="F18" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-11.71</v>
+      </c>
+      <c r="H18" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="I18" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-11.43</v>
+      </c>
+      <c r="K18" t="n">
+        <v>12</v>
+      </c>
+      <c r="L18" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="M18" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="N18" t="b">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="P18" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>2229943</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>80.28</v>
+      </c>
+      <c r="V18" t="n">
+        <v>-13.72</v>
+      </c>
+      <c r="W18" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="X18" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="2" t="n">
+        <v>45496.41666666666</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>-11.43</v>
+      </c>
+      <c r="AJ18" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="AP18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR18" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS18" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>76.1904761904762</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="AV18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>45525.41666666666</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>45656.41666666666</v>
+      </c>
+      <c r="F19" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-23.01</v>
+      </c>
+      <c r="H19" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="I19" t="n">
+        <v>16.29</v>
+      </c>
+      <c r="J19" t="n">
+        <v>44.16</v>
+      </c>
+      <c r="K19" t="n">
+        <v>131</v>
+      </c>
+      <c r="L19" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="M19" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="N19" t="b">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="P19" t="n">
+        <v>17.77</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>10826324</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="V19" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="W19" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="X19" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>14.68</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>16.65</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>57.26</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>123</v>
+      </c>
+      <c r="AH19" s="2" t="n">
+        <v>45648.41666666666</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>-4.34</v>
+      </c>
+      <c r="AJ19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="AP19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>87.24832214765104</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="AV19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>45662.41666666666</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>45665.41666666666</v>
+      </c>
+      <c r="F20" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-6.28</v>
+      </c>
+      <c r="H20" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="I20" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-8.140000000000001</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" t="n">
+        <v>16.12</v>
+      </c>
+      <c r="M20" t="n">
+        <v>17</v>
+      </c>
+      <c r="N20" t="b">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="P20" t="n">
+        <v>17.47</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>801972</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>81.38</v>
+      </c>
+      <c r="V20" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="X20" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH20" s="2" t="n">
+        <v>45663.41666666666</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>-8.140000000000001</v>
+      </c>
+      <c r="AJ20" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>17</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>14.66</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="AP20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>67.42857142857142</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="AV20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C21" t="b">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>45678.41666666666</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>45753.41666666666</v>
+      </c>
+      <c r="F21" t="n">
+        <v>17.95</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-21.89</v>
+      </c>
+      <c r="H21" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="I21" t="n">
+        <v>21</v>
+      </c>
+      <c r="J21" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="K21" t="n">
+        <v>75</v>
+      </c>
+      <c r="L21" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="M21" t="n">
+        <v>17.47</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="P21" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>7215730</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>82.39</v>
+      </c>
+      <c r="V21" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="W21" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="X21" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>14.28</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>33.48</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>48</v>
+      </c>
+      <c r="AH21" s="2" t="n">
+        <v>45726.41666666666</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="AJ21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>17.47</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>14.64</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="AP21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>82.38993710691824</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="AV21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C22" t="b">
+        <v>0</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>45761.41666666666</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>45907.41666666666</v>
+      </c>
+      <c r="F22" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-13.45</v>
+      </c>
+      <c r="H22" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="I22" t="n">
+        <v>37</v>
+      </c>
+      <c r="J22" t="n">
+        <v>63.72</v>
+      </c>
+      <c r="K22" t="n">
+        <v>146</v>
+      </c>
+      <c r="L22" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="M22" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="P22" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>581928</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>97.12</v>
+      </c>
+      <c r="V22" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="W22" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="X22" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>127</v>
+      </c>
+      <c r="AH22" s="2" t="n">
+        <v>45888.41666666666</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>-3.23</v>
+      </c>
+      <c r="AJ22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>23</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="AP22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>83.33333333333333</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="AV22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2534,55 +4599,55 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2" t="n">
         <v>8</v>
       </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>62.5</v>
+        <v>38.1</v>
       </c>
       <c r="G2" t="n">
-        <v>3.94</v>
+        <v>-1.62</v>
       </c>
       <c r="H2" t="n">
-        <v>7</v>
+        <v>6.34</v>
       </c>
       <c r="I2" t="n">
-        <v>55.97</v>
+        <v>133.21</v>
       </c>
       <c r="J2" t="n">
-        <v>54.17</v>
+        <v>63.72</v>
       </c>
       <c r="K2" t="n">
         <v>-18.62</v>
       </c>
       <c r="L2" t="n">
-        <v>22.57</v>
+        <v>23.3</v>
       </c>
       <c r="M2" t="n">
-        <v>2.57</v>
+        <v>2.16</v>
       </c>
       <c r="N2" t="n">
-        <v>18.31</v>
+        <v>30.95</v>
       </c>
       <c r="O2" t="n">
-        <v>11.85</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>7</v>
+        <v>6.34</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.5453567034365719</v>
+        <v>0.4635380658436214</v>
       </c>
       <c r="R2" t="n">
-        <v>0.44551</v>
+        <v>0.5351999999999999</v>
       </c>
       <c r="S2" t="n">
-        <v>0.4854486813746288</v>
+        <v>0.5065352263374485</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -2590,7 +4655,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.4854486813746288</v>
+        <v>0.5065352263374485</v>
       </c>
     </row>
   </sheetData>
@@ -2661,22 +4726,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E2" t="n">
-        <v>62.5</v>
+        <v>38.1</v>
       </c>
       <c r="F2" t="n">
-        <v>2.57</v>
+        <v>2.16</v>
       </c>
       <c r="G2" t="n">
-        <v>3.94</v>
+        <v>-1.62</v>
       </c>
       <c r="H2" t="n">
-        <v>7</v>
+        <v>6.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-12 20:19:44.442226
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1038,7 +1038,7 @@
         <v>-16.29</v>
       </c>
       <c r="H4" t="n">
-        <v>2.91</v>
+        <v>2.93</v>
       </c>
       <c r="I4" t="n">
         <v>3.49</v>
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>85.51000000000001</v>
+        <v>85.06999999999999</v>
       </c>
       <c r="V4" t="n">
         <v>-3.89</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-12 20:22:08.432982
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY22"/>
+  <dimension ref="A1:AY23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1035,10 +1035,10 @@
         <v>3.5</v>
       </c>
       <c r="G4" t="n">
-        <v>-16.29</v>
+        <v>-16.86</v>
       </c>
       <c r="H4" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="I4" t="n">
         <v>3.49</v>
@@ -1050,10 +1050,10 @@
         <v>42</v>
       </c>
       <c r="L4" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="M4" t="n">
-        <v>3.45</v>
+        <v>3.47</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>85.06999999999999</v>
+        <v>85.51000000000001</v>
       </c>
       <c r="V4" t="n">
         <v>-3.89</v>
@@ -1098,7 +1098,7 @@
         <v>1.03</v>
       </c>
       <c r="Z4" t="n">
-        <v>1.45</v>
+        <v>0.86</v>
       </c>
       <c r="AA4" t="n">
         <v>5.19</v>
@@ -1110,7 +1110,7 @@
         <v>6.29</v>
       </c>
       <c r="AD4" t="n">
-        <v>16.3</v>
+        <v>17.55</v>
       </c>
       <c r="AE4" t="n">
         <v>4.48</v>
@@ -1161,7 +1161,7 @@
         <v>85.50724637681158</v>
       </c>
       <c r="AU4" t="n">
-        <v>3.45</v>
+        <v>3.47</v>
       </c>
       <c r="AV4" t="b">
         <v>1</v>
@@ -1194,10 +1194,10 @@
         <v>3.2</v>
       </c>
       <c r="G5" t="n">
-        <v>-11.88</v>
+        <v>-12.5</v>
       </c>
       <c r="H5" t="n">
-        <v>2.82</v>
+        <v>2.8</v>
       </c>
       <c r="I5" t="n">
         <v>3.21</v>
@@ -1209,7 +1209,7 @@
         <v>28</v>
       </c>
       <c r="L5" t="n">
-        <v>2.82</v>
+        <v>2.8</v>
       </c>
       <c r="M5" t="n">
         <v>3.15</v>
@@ -1242,7 +1242,7 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>82.61</v>
+        <v>83.33</v>
       </c>
       <c r="V5" t="n">
         <v>-25</v>
@@ -1269,7 +1269,7 @@
         <v>2.19</v>
       </c>
       <c r="AD5" t="n">
-        <v>11.06</v>
+        <v>11.76</v>
       </c>
       <c r="AE5" t="n">
         <v>2.56</v>
@@ -1404,7 +1404,7 @@
         <v>78.84</v>
       </c>
       <c r="V6" t="n">
-        <v>1.37</v>
+        <v>6.03</v>
       </c>
       <c r="W6" t="n">
         <v>7.08</v>
@@ -1455,7 +1455,7 @@
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>3.6</v>
+        <v>3.43</v>
       </c>
       <c r="AN6" t="n">
         <v>3.32</v>
@@ -1530,7 +1530,7 @@
         <v>2.7</v>
       </c>
       <c r="M7" t="n">
-        <v>3.25</v>
+        <v>3.16</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
@@ -1575,7 +1575,7 @@
         <v>1.05</v>
       </c>
       <c r="Z7" t="n">
-        <v>2.15</v>
+        <v>5.06</v>
       </c>
       <c r="AA7" t="n">
         <v>2.39</v>
@@ -1587,7 +1587,7 @@
         <v>11.54</v>
       </c>
       <c r="AD7" t="n">
-        <v>18.49</v>
+        <v>15.7</v>
       </c>
       <c r="AE7" t="n">
         <v>8.85</v>
@@ -1638,7 +1638,7 @@
         <v>96.20253164556958</v>
       </c>
       <c r="AU7" t="n">
-        <v>3.25</v>
+        <v>3.16</v>
       </c>
       <c r="AV7" t="b">
         <v>1</v>
@@ -2782,10 +2782,10 @@
         <v>7.2</v>
       </c>
       <c r="G15" t="n">
-        <v>-8.33</v>
+        <v>-9.44</v>
       </c>
       <c r="H15" t="n">
-        <v>6.6</v>
+        <v>6.52</v>
       </c>
       <c r="I15" t="n">
         <v>7.45</v>
@@ -2797,7 +2797,7 @@
         <v>61</v>
       </c>
       <c r="L15" t="n">
-        <v>6.6</v>
+        <v>6.52</v>
       </c>
       <c r="M15" t="n">
         <v>7.13</v>
@@ -2830,7 +2830,7 @@
         </is>
       </c>
       <c r="U15" t="n">
-        <v>66.67</v>
+        <v>69.39</v>
       </c>
       <c r="V15" t="n">
         <v>4.93</v>
@@ -2857,7 +2857,7 @@
         <v>-0.24</v>
       </c>
       <c r="AD15" t="n">
-        <v>7.72</v>
+        <v>8.94</v>
       </c>
       <c r="AE15" t="n">
         <v>2.86</v>
@@ -2935,7 +2935,7 @@
         <v>45103.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45133.41666666666</v>
+        <v>45132.41666666666</v>
       </c>
       <c r="F16" t="n">
         <v>8.5</v>
@@ -2944,16 +2944,16 @@
         <v>-14.71</v>
       </c>
       <c r="H16" t="n">
-        <v>7.2</v>
+        <v>7.56</v>
       </c>
       <c r="I16" t="n">
-        <v>7.17</v>
+        <v>7.41</v>
       </c>
       <c r="J16" t="n">
-        <v>-15.65</v>
+        <v>-12.82</v>
       </c>
       <c r="K16" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L16" t="n">
         <v>7.25</v>
@@ -2965,7 +2965,7 @@
         <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>7.2</v>
+        <v>7.56</v>
       </c>
       <c r="P16" t="n">
         <v>8.5</v>
@@ -3031,7 +3031,7 @@
         <v>45103.41666666666</v>
       </c>
       <c r="AI16" t="n">
-        <v>-15.65</v>
+        <v>-12.82</v>
       </c>
       <c r="AJ16" t="b">
         <v>1</v>
@@ -3151,7 +3151,7 @@
         <v>74.42</v>
       </c>
       <c r="V17" t="n">
-        <v>-9.33</v>
+        <v>-5.07</v>
       </c>
       <c r="W17" t="n">
         <v>2.56</v>
@@ -3202,7 +3202,7 @@
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>8.199999999999999</v>
+        <v>7.88</v>
       </c>
       <c r="AN17" t="n">
         <v>6.98</v>
@@ -3571,7 +3571,7 @@
         <v>45525.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45649.41666666666</v>
+        <v>45656.41666666666</v>
       </c>
       <c r="F20" t="n">
         <v>11.3</v>
@@ -3583,13 +3583,13 @@
         <v>9.130000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>16.5</v>
+        <v>16.29</v>
       </c>
       <c r="J20" t="n">
-        <v>46.02</v>
+        <v>44.16</v>
       </c>
       <c r="K20" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="L20" t="n">
         <v>8.699999999999999</v>
@@ -3601,7 +3601,7 @@
         <v>1</v>
       </c>
       <c r="O20" t="n">
-        <v>16.57</v>
+        <v>16.3</v>
       </c>
       <c r="P20" t="n">
         <v>17.77</v>
@@ -3724,47 +3724,47 @@
         </is>
       </c>
       <c r="C21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45678.41666666666</v>
+        <v>45662.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45753.41666666666</v>
+        <v>45665.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>17.95</v>
+        <v>17.2</v>
       </c>
       <c r="G21" t="n">
-        <v>-21.89</v>
+        <v>-6.28</v>
       </c>
       <c r="H21" t="n">
-        <v>14.02</v>
+        <v>16.02</v>
       </c>
       <c r="I21" t="n">
-        <v>21</v>
+        <v>15.8</v>
       </c>
       <c r="J21" t="n">
-        <v>16.99</v>
+        <v>-8.140000000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>14.02</v>
+        <v>16.12</v>
       </c>
       <c r="M21" t="n">
+        <v>17</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="P21" t="n">
         <v>17.47</v>
       </c>
-      <c r="N21" t="b">
-        <v>1</v>
-      </c>
-      <c r="O21" t="n">
-        <v>22.25</v>
-      </c>
-      <c r="P21" t="n">
-        <v>23.96</v>
-      </c>
       <c r="Q21" t="inlineStr">
         <is>
           <t>RANGE_BREAKDOWN</t>
@@ -3776,7 +3776,7 @@
         </is>
       </c>
       <c r="S21" t="n">
-        <v>7215730</v>
+        <v>801972</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
@@ -3784,49 +3784,49 @@
         </is>
       </c>
       <c r="U21" t="n">
-        <v>82.39</v>
+        <v>81.38</v>
       </c>
       <c r="V21" t="n">
-        <v>5.43</v>
+        <v>2.69</v>
       </c>
       <c r="W21" t="n">
-        <v>4.95</v>
+        <v>0.98</v>
       </c>
       <c r="X21" t="n">
-        <v>7.21</v>
+        <v>3.97</v>
       </c>
       <c r="Y21" t="n">
-        <v>1.73</v>
+        <v>2.48</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.75</v>
+        <v>1.18</v>
       </c>
       <c r="AA21" t="n">
-        <v>2.76</v>
+        <v>1.53</v>
       </c>
       <c r="AB21" t="n">
-        <v>14.28</v>
+        <v>10.94</v>
       </c>
       <c r="AC21" t="n">
-        <v>10.17</v>
+        <v>4.22</v>
       </c>
       <c r="AD21" t="n">
-        <v>21.91</v>
+        <v>5.31</v>
       </c>
       <c r="AE21" t="n">
-        <v>8.130000000000001</v>
+        <v>1.78</v>
       </c>
       <c r="AF21" t="n">
-        <v>33.48</v>
+        <v>0.52</v>
       </c>
       <c r="AG21" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>45726.41666666666</v>
+        <v>45663.41666666666</v>
       </c>
       <c r="AI21" t="n">
-        <v>-1.78</v>
+        <v>-8.140000000000001</v>
       </c>
       <c r="AJ21" t="b">
         <v>1</v>
@@ -3838,34 +3838,34 @@
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>17.77</v>
+        <v>17</v>
       </c>
       <c r="AN21" t="n">
-        <v>14.64</v>
+        <v>14.66</v>
       </c>
       <c r="AO21" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="AP21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>67.42857142857142</v>
+      </c>
+      <c r="AU21" t="n">
         <v>17.6</v>
       </c>
-      <c r="AP21" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ21" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR21" t="b">
-        <v>1</v>
-      </c>
-      <c r="AS21" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT21" t="n">
-        <v>82.38993710691824</v>
-      </c>
-      <c r="AU21" t="n">
-        <v>17.72</v>
-      </c>
       <c r="AV21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW21" t="inlineStr"/>
       <c r="AX21" t="inlineStr"/>
@@ -3883,46 +3883,46 @@
         </is>
       </c>
       <c r="C22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45761.41666666666</v>
+        <v>45678.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45907.41666666666</v>
+        <v>45753.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>22.6</v>
+        <v>17.95</v>
       </c>
       <c r="G22" t="n">
-        <v>-13.45</v>
+        <v>-21.89</v>
       </c>
       <c r="H22" t="n">
-        <v>19.56</v>
+        <v>14.02</v>
       </c>
       <c r="I22" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="J22" t="n">
-        <v>63.72</v>
+        <v>16.99</v>
       </c>
       <c r="K22" t="n">
-        <v>146</v>
+        <v>75</v>
       </c>
       <c r="L22" t="n">
-        <v>19.56</v>
+        <v>14.02</v>
       </c>
       <c r="M22" t="n">
-        <v>21.98</v>
+        <v>17.47</v>
       </c>
       <c r="N22" t="b">
         <v>1</v>
       </c>
       <c r="O22" t="n">
-        <v>37.5</v>
+        <v>22.25</v>
       </c>
       <c r="P22" t="n">
-        <v>48.89</v>
+        <v>23.96</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="S22" t="n">
-        <v>581928</v>
+        <v>7215730</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
@@ -3943,49 +3943,49 @@
         </is>
       </c>
       <c r="U22" t="n">
-        <v>97.12</v>
+        <v>82.39</v>
       </c>
       <c r="V22" t="n">
-        <v>-1.37</v>
+        <v>7.03</v>
       </c>
       <c r="W22" t="n">
-        <v>1.3</v>
+        <v>4.95</v>
       </c>
       <c r="X22" t="n">
-        <v>5.79</v>
+        <v>7.21</v>
       </c>
       <c r="Y22" t="n">
-        <v>1.03</v>
+        <v>1.73</v>
       </c>
       <c r="Z22" t="n">
-        <v>2.82</v>
+        <v>2.75</v>
       </c>
       <c r="AA22" t="n">
-        <v>4.78</v>
+        <v>2.76</v>
       </c>
       <c r="AB22" t="n">
-        <v>6.38</v>
+        <v>14.28</v>
       </c>
       <c r="AC22" t="n">
-        <v>3.1</v>
+        <v>10.17</v>
       </c>
       <c r="AD22" t="n">
-        <v>11.65</v>
+        <v>21.91</v>
       </c>
       <c r="AE22" t="n">
-        <v>4.78</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="AF22" t="n">
-        <v>102.35</v>
+        <v>33.48</v>
       </c>
       <c r="AG22" t="n">
-        <v>127</v>
+        <v>48</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>45888.41666666666</v>
+        <v>45726.41666666666</v>
       </c>
       <c r="AI22" t="n">
-        <v>-3.23</v>
+        <v>-1.78</v>
       </c>
       <c r="AJ22" t="b">
         <v>1</v>
@@ -3997,31 +3997,31 @@
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>23</v>
+        <v>17.47</v>
       </c>
       <c r="AN22" t="n">
-        <v>18.5</v>
+        <v>14.64</v>
       </c>
       <c r="AO22" t="n">
-        <v>23.58</v>
+        <v>17.6</v>
       </c>
       <c r="AP22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ22" t="b">
         <v>0</v>
       </c>
       <c r="AR22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT22" t="n">
-        <v>83.33333333333333</v>
+        <v>82.38993710691824</v>
       </c>
       <c r="AU22" t="n">
-        <v>21.98</v>
+        <v>17.72</v>
       </c>
       <c r="AV22" t="b">
         <v>1</v>
@@ -4029,6 +4029,165 @@
       <c r="AW22" t="inlineStr"/>
       <c r="AX22" t="inlineStr"/>
       <c r="AY22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C23" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>45761.41666666666</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>45907.41666666666</v>
+      </c>
+      <c r="F23" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-13.45</v>
+      </c>
+      <c r="H23" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="I23" t="n">
+        <v>37</v>
+      </c>
+      <c r="J23" t="n">
+        <v>63.72</v>
+      </c>
+      <c r="K23" t="n">
+        <v>146</v>
+      </c>
+      <c r="L23" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="M23" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="P23" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>581928</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>97.12</v>
+      </c>
+      <c r="V23" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="W23" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="X23" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>127</v>
+      </c>
+      <c r="AH23" s="2" t="n">
+        <v>45888.41666666666</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>-3.23</v>
+      </c>
+      <c r="AJ23" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>23</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="AO23" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="AP23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>83.33333333333333</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="AV23" t="b">
+        <v>1</v>
+      </c>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4343,7 +4502,7 @@
         <v>36.5</v>
       </c>
       <c r="M2" t="n">
-        <v>41.28</v>
+        <v>41.6</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -4376,7 +4535,7 @@
         <v>100</v>
       </c>
       <c r="V2" t="n">
-        <v>13.46</v>
+        <v>12.79</v>
       </c>
       <c r="W2" t="n">
         <v>8.960000000000001</v>
@@ -4388,7 +4547,7 @@
         <v>3.69</v>
       </c>
       <c r="Z2" t="n">
-        <v>15.55</v>
+        <v>14.66</v>
       </c>
       <c r="AA2" t="n">
         <v>1.7</v>
@@ -4400,7 +4559,7 @@
         <v>20.5</v>
       </c>
       <c r="AD2" t="n">
-        <v>12.29</v>
+        <v>13.06</v>
       </c>
       <c r="AE2" t="n">
         <v>20</v>
@@ -4427,7 +4586,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>41.28</v>
+        <v>41.6</v>
       </c>
       <c r="AN2" t="n">
         <v>39</v>
@@ -4451,7 +4610,7 @@
         <v>100</v>
       </c>
       <c r="AU2" t="n">
-        <v>41.42</v>
+        <v>41.6</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
@@ -4599,25 +4758,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
         <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>42.86</v>
+        <v>40.91</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.29</v>
+        <v>-1.46</v>
       </c>
       <c r="H2" t="n">
-        <v>6.93</v>
+        <v>6.29</v>
       </c>
       <c r="I2" t="n">
-        <v>145.54</v>
+        <v>138.37</v>
       </c>
       <c r="J2" t="n">
         <v>63.72</v>
@@ -4626,28 +4785,28 @@
         <v>-18.62</v>
       </c>
       <c r="L2" t="n">
-        <v>23.24</v>
+        <v>22.64</v>
       </c>
       <c r="M2" t="n">
-        <v>2.35</v>
+        <v>2.23</v>
       </c>
       <c r="N2" t="n">
-        <v>28.11</v>
+        <v>27.9</v>
       </c>
       <c r="O2" t="n">
-        <v>8.949999999999999</v>
+        <v>8.67</v>
       </c>
       <c r="P2" t="n">
-        <v>6.93</v>
+        <v>6.29</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4849635313531353</v>
+        <v>0.474350296108291</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5484</v>
+        <v>0.5416</v>
       </c>
       <c r="S2" t="n">
-        <v>0.5230254125412541</v>
+        <v>0.5147001184433164</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -4655,7 +4814,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.5230254125412541</v>
+        <v>0.5147001184433164</v>
       </c>
     </row>
   </sheetData>
@@ -4726,22 +4885,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
-        <v>42.86</v>
+        <v>40.91</v>
       </c>
       <c r="F2" t="n">
-        <v>2.35</v>
+        <v>2.23</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.29</v>
+        <v>-1.46</v>
       </c>
       <c r="H2" t="n">
-        <v>6.93</v>
+        <v>6.29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 10:33:14.687563
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1123,10 +1123,10 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>24.23</v>
+        <v>23.25</v>
       </c>
       <c r="AV4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1669,10 +1669,10 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>55.06</v>
+        <v>80.33</v>
       </c>
       <c r="V8" t="n">
-        <v>-10.91</v>
+        <v>-11.71</v>
       </c>
       <c r="W8" t="n">
         <v>0.51</v>
@@ -1747,10 +1747,10 @@
         <v>42.88164665523157</v>
       </c>
       <c r="AU8" t="n">
-        <v>40.79</v>
+        <v>38.64</v>
       </c>
       <c r="AV8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2059,10 +2059,10 @@
         <v>69.19917864476385</v>
       </c>
       <c r="AU10" t="n">
-        <v>48.07</v>
+        <v>46.95</v>
       </c>
       <c r="AV10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2683,7 +2683,7 @@
         <v>70.54545454545459</v>
       </c>
       <c r="AU14" t="n">
-        <v>48.08</v>
+        <v>47.88</v>
       </c>
       <c r="AV14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 10:35:21.785792
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1123,10 +1123,10 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>23.25</v>
+        <v>24.23</v>
       </c>
       <c r="AV4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1669,10 +1669,10 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>80.33</v>
+        <v>55.06</v>
       </c>
       <c r="V8" t="n">
-        <v>-11.71</v>
+        <v>-10.91</v>
       </c>
       <c r="W8" t="n">
         <v>0.51</v>
@@ -1747,10 +1747,10 @@
         <v>42.88164665523157</v>
       </c>
       <c r="AU8" t="n">
-        <v>38.64</v>
+        <v>40.79</v>
       </c>
       <c r="AV8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2059,10 +2059,10 @@
         <v>69.19917864476385</v>
       </c>
       <c r="AU10" t="n">
-        <v>46.95</v>
+        <v>48.07</v>
       </c>
       <c r="AV10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2683,7 +2683,7 @@
         <v>70.54545454545459</v>
       </c>
       <c r="AU14" t="n">
-        <v>47.88</v>
+        <v>48.08</v>
       </c>
       <c r="AV14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 10:37:51.039327
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1669,10 +1669,10 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>55.06</v>
+        <v>80.33</v>
       </c>
       <c r="V8" t="n">
-        <v>-10.91</v>
+        <v>-11.71</v>
       </c>
       <c r="W8" t="n">
         <v>0.51</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 10:41:08.348688
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1123,10 +1123,10 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>24.23</v>
+        <v>23.25</v>
       </c>
       <c r="AV4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1279,10 +1279,10 @@
         <v>51.86567164179107</v>
       </c>
       <c r="AU5" t="n">
-        <v>22.99</v>
+        <v>23.47</v>
       </c>
       <c r="AV5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1747,7 +1747,7 @@
         <v>42.88164665523157</v>
       </c>
       <c r="AU8" t="n">
-        <v>40.79</v>
+        <v>39.4</v>
       </c>
       <c r="AV8" t="b">
         <v>0</v>
@@ -2059,7 +2059,7 @@
         <v>69.19917864476385</v>
       </c>
       <c r="AU10" t="n">
-        <v>48.07</v>
+        <v>50.62</v>
       </c>
       <c r="AV10" t="b">
         <v>0</v>
@@ -2371,10 +2371,10 @@
         <v>54.11954765751216</v>
       </c>
       <c r="AU12" t="n">
-        <v>48.24</v>
+        <v>49</v>
       </c>
       <c r="AV12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2683,7 +2683,7 @@
         <v>70.54545454545459</v>
       </c>
       <c r="AU14" t="n">
-        <v>48.08</v>
+        <v>47.88</v>
       </c>
       <c r="AV14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 10:58:39.253029
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1279,10 +1279,10 @@
         <v>51.86567164179107</v>
       </c>
       <c r="AU5" t="n">
-        <v>23.47</v>
+        <v>22.99</v>
       </c>
       <c r="AV5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1747,10 +1747,10 @@
         <v>42.88164665523157</v>
       </c>
       <c r="AU8" t="n">
-        <v>39.4</v>
+        <v>38.64</v>
       </c>
       <c r="AV8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2059,10 +2059,10 @@
         <v>69.19917864476385</v>
       </c>
       <c r="AU10" t="n">
-        <v>50.62</v>
+        <v>46.95</v>
       </c>
       <c r="AV10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2371,10 +2371,10 @@
         <v>54.11954765751216</v>
       </c>
       <c r="AU12" t="n">
-        <v>49</v>
+        <v>48.24</v>
       </c>
       <c r="AV12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Update trading data 2026-04-17 11:00:47.993548
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -815,7 +815,7 @@
         <v>75.68134171907757</v>
       </c>
       <c r="AU2" t="n">
-        <v>14.8</v>
+        <v>14.36</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
@@ -967,7 +967,7 @@
         <v>89.3648449039882</v>
       </c>
       <c r="AU3" t="n">
-        <v>19.07</v>
+        <v>18.21</v>
       </c>
       <c r="AV3" t="b">
         <v>1</v>
@@ -1123,7 +1123,7 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>23.25</v>
+        <v>22.71</v>
       </c>
       <c r="AV4" t="b">
         <v>1</v>
@@ -1279,7 +1279,7 @@
         <v>51.86567164179107</v>
       </c>
       <c r="AU5" t="n">
-        <v>22.99</v>
+        <v>22.75</v>
       </c>
       <c r="AV5" t="b">
         <v>1</v>
@@ -1591,7 +1591,7 @@
         <v>58.28220858895707</v>
       </c>
       <c r="AU7" t="n">
-        <v>34.89</v>
+        <v>34.34</v>
       </c>
       <c r="AV7" t="b">
         <v>1</v>
@@ -1747,7 +1747,7 @@
         <v>42.88164665523157</v>
       </c>
       <c r="AU8" t="n">
-        <v>38.64</v>
+        <v>35.68</v>
       </c>
       <c r="AV8" t="b">
         <v>1</v>
@@ -1903,7 +1903,7 @@
         <v>60.99173553719012</v>
       </c>
       <c r="AU9" t="n">
-        <v>37.98</v>
+        <v>36.94</v>
       </c>
       <c r="AV9" t="b">
         <v>1</v>
@@ -2059,7 +2059,7 @@
         <v>69.19917864476385</v>
       </c>
       <c r="AU10" t="n">
-        <v>46.95</v>
+        <v>44.6</v>
       </c>
       <c r="AV10" t="b">
         <v>1</v>
@@ -2215,7 +2215,7 @@
         <v>44.26494345718907</v>
       </c>
       <c r="AU11" t="n">
-        <v>47.65</v>
+        <v>46.13</v>
       </c>
       <c r="AV11" t="b">
         <v>1</v>
@@ -2527,7 +2527,7 @@
         <v>54.16666666666669</v>
       </c>
       <c r="AU13" t="n">
-        <v>50.5</v>
+        <v>47.83</v>
       </c>
       <c r="AV13" t="b">
         <v>1</v>
@@ -2683,7 +2683,7 @@
         <v>70.54545454545459</v>
       </c>
       <c r="AU14" t="n">
-        <v>47.88</v>
+        <v>44.5</v>
       </c>
       <c r="AV14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 11:04:51.815730
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1123,7 +1123,7 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>22.71</v>
+        <v>22.17</v>
       </c>
       <c r="AV4" t="b">
         <v>1</v>
@@ -1591,7 +1591,7 @@
         <v>58.28220858895707</v>
       </c>
       <c r="AU7" t="n">
-        <v>34.34</v>
+        <v>34.89</v>
       </c>
       <c r="AV7" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 11:08:00.559550
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -719,7 +719,7 @@
         <v>14.02</v>
       </c>
       <c r="M2" t="n">
-        <v>14.8</v>
+        <v>15.96</v>
       </c>
       <c r="N2" t="b">
         <v>0</v>
@@ -728,7 +728,7 @@
         <v>18.26</v>
       </c>
       <c r="P2" t="n">
-        <v>19.93</v>
+        <v>20.79</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -758,7 +758,7 @@
         <v>-4.63</v>
       </c>
       <c r="Z2" t="n">
-        <v>5</v>
+        <v>-2.63</v>
       </c>
       <c r="AA2" t="n">
         <v>16.89</v>
@@ -770,7 +770,7 @@
         <v>-9.24</v>
       </c>
       <c r="AD2" t="n">
-        <v>5.41</v>
+        <v>12.94</v>
       </c>
       <c r="AE2" t="n">
         <v>8.75</v>
@@ -788,7 +788,7 @@
         <v>0</v>
       </c>
       <c r="AJ2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK2" t="b">
         <v>0</v>
@@ -815,7 +815,7 @@
         <v>75.68134171907757</v>
       </c>
       <c r="AU2" t="n">
-        <v>14.36</v>
+        <v>14.8</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
@@ -863,7 +863,7 @@
         <v>18.07</v>
       </c>
       <c r="M3" t="n">
-        <v>19.07</v>
+        <v>20.6</v>
       </c>
       <c r="N3" t="b">
         <v>0</v>
@@ -872,7 +872,7 @@
         <v>22.66</v>
       </c>
       <c r="P3" t="n">
-        <v>23.8</v>
+        <v>23.79</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
         <v>0.12</v>
       </c>
       <c r="Z3" t="n">
-        <v>5.24</v>
+        <v>-2.57</v>
       </c>
       <c r="AA3" t="n">
         <v>16.89</v>
@@ -920,7 +920,7 @@
         <v>17.22</v>
       </c>
       <c r="AD3" t="n">
-        <v>5.39</v>
+        <v>13.09</v>
       </c>
       <c r="AE3" t="n">
         <v>10.27</v>
@@ -938,7 +938,7 @@
         <v>-7.17</v>
       </c>
       <c r="AJ3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK3" t="b">
         <v>0</v>
@@ -967,7 +967,7 @@
         <v>89.3648449039882</v>
       </c>
       <c r="AU3" t="n">
-        <v>18.21</v>
+        <v>19.07</v>
       </c>
       <c r="AV3" t="b">
         <v>1</v>
@@ -1015,7 +1015,7 @@
         <v>22.25</v>
       </c>
       <c r="M4" t="n">
-        <v>23.25</v>
+        <v>23.96</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1024,7 +1024,7 @@
         <v>22.67</v>
       </c>
       <c r="P4" t="n">
-        <v>23.96</v>
+        <v>24.7</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>3.69</v>
       </c>
       <c r="Z4" t="n">
-        <v>3.05</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
         <v>5.5</v>
@@ -1072,7 +1072,7 @@
         <v>7.93</v>
       </c>
       <c r="AD4" t="n">
-        <v>4.4</v>
+        <v>7.4</v>
       </c>
       <c r="AE4" t="n">
         <v>5.69</v>
@@ -1090,7 +1090,7 @@
         <v>-5.68</v>
       </c>
       <c r="AJ4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK4" t="b">
         <v>0</v>
@@ -1123,7 +1123,7 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>22.17</v>
+        <v>23.25</v>
       </c>
       <c r="AV4" t="b">
         <v>1</v>
@@ -1171,7 +1171,7 @@
         <v>22.2</v>
       </c>
       <c r="M5" t="n">
-        <v>22.99</v>
+        <v>23.47</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
@@ -1180,7 +1180,7 @@
         <v>22.02</v>
       </c>
       <c r="P5" t="n">
-        <v>23.47</v>
+        <v>23</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>3.04</v>
       </c>
       <c r="Z5" t="n">
-        <v>1.83</v>
+        <v>-0.26</v>
       </c>
       <c r="AA5" t="n">
         <v>1.17</v>
@@ -1228,7 +1228,7 @@
         <v>3.87</v>
       </c>
       <c r="AD5" t="n">
-        <v>3.5</v>
+        <v>5.56</v>
       </c>
       <c r="AE5" t="n">
         <v>5.07</v>
@@ -1246,7 +1246,7 @@
         <v>-10.29</v>
       </c>
       <c r="AJ5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK5" t="b">
         <v>0</v>
@@ -1279,10 +1279,10 @@
         <v>51.86567164179107</v>
       </c>
       <c r="AU5" t="n">
-        <v>22.75</v>
+        <v>23.47</v>
       </c>
       <c r="AV5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1327,7 +1327,7 @@
         <v>19.56</v>
       </c>
       <c r="M6" t="n">
-        <v>21.7</v>
+        <v>22.69</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
@@ -1336,7 +1336,7 @@
         <v>36.6</v>
       </c>
       <c r="P6" t="n">
-        <v>38</v>
+        <v>37.55</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1372,7 +1372,7 @@
         <v>1.25</v>
       </c>
       <c r="Z6" t="n">
-        <v>4.15</v>
+        <v>-0.4</v>
       </c>
       <c r="AA6" t="n">
         <v>4.77</v>
@@ -1384,7 +1384,7 @@
         <v>3.12</v>
       </c>
       <c r="AD6" t="n">
-        <v>10.37</v>
+        <v>14.82</v>
       </c>
       <c r="AE6" t="n">
         <v>4.78</v>
@@ -1402,7 +1402,7 @@
         <v>-3.23</v>
       </c>
       <c r="AJ6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK6" t="b">
         <v>0</v>
@@ -1483,7 +1483,7 @@
         <v>32.66</v>
       </c>
       <c r="M7" t="n">
-        <v>34.89</v>
+        <v>35.88</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
@@ -1528,7 +1528,7 @@
         <v>2.39</v>
       </c>
       <c r="Z7" t="n">
-        <v>1.78</v>
+        <v>-1.03</v>
       </c>
       <c r="AA7" t="n">
         <v>1.55</v>
@@ -1540,7 +1540,7 @@
         <v>4.61</v>
       </c>
       <c r="AD7" t="n">
-        <v>6.6</v>
+        <v>9.4</v>
       </c>
       <c r="AE7" t="n">
         <v>6</v>
@@ -1558,7 +1558,7 @@
         <v>0</v>
       </c>
       <c r="AJ7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK7" t="b">
         <v>0</v>
@@ -1639,7 +1639,7 @@
         <v>36.5</v>
       </c>
       <c r="M8" t="n">
-        <v>38.64</v>
+        <v>39.4</v>
       </c>
       <c r="N8" t="b">
         <v>0</v>
@@ -1648,7 +1648,7 @@
         <v>39</v>
       </c>
       <c r="P8" t="n">
-        <v>40.77</v>
+        <v>41.06</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1684,7 +1684,7 @@
         <v>1.05</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.93</v>
+        <v>-1.02</v>
       </c>
       <c r="AA8" t="n">
         <v>5.03</v>
@@ -1696,7 +1696,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="AD8" t="n">
-        <v>5.7</v>
+        <v>7.64</v>
       </c>
       <c r="AE8" t="n">
         <v>0.96</v>
@@ -1714,7 +1714,7 @@
         <v>-0.26</v>
       </c>
       <c r="AJ8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK8" t="b">
         <v>0</v>
@@ -1747,10 +1747,10 @@
         <v>42.88164665523157</v>
       </c>
       <c r="AU8" t="n">
-        <v>35.68</v>
+        <v>39.4</v>
       </c>
       <c r="AV8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1795,7 +1795,7 @@
         <v>35.01</v>
       </c>
       <c r="M9" t="n">
-        <v>37.98</v>
+        <v>38.7</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
@@ -1840,7 +1840,7 @@
         <v>0.63</v>
       </c>
       <c r="Z9" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="AA9" t="n">
         <v>2.11</v>
@@ -1852,7 +1852,7 @@
         <v>0.89</v>
       </c>
       <c r="AD9" t="n">
-        <v>8.140000000000001</v>
+        <v>10.01</v>
       </c>
       <c r="AE9" t="n">
         <v>5.02</v>
@@ -1870,7 +1870,7 @@
         <v>-0.52</v>
       </c>
       <c r="AJ9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK9" t="b">
         <v>0</v>
@@ -1903,7 +1903,7 @@
         <v>60.99173553719012</v>
       </c>
       <c r="AU9" t="n">
-        <v>36.94</v>
+        <v>37.98</v>
       </c>
       <c r="AV9" t="b">
         <v>1</v>
@@ -1951,7 +1951,7 @@
         <v>44.75</v>
       </c>
       <c r="M10" t="n">
-        <v>46.95</v>
+        <v>47.5</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
@@ -1960,7 +1960,7 @@
         <v>48.5</v>
       </c>
       <c r="P10" t="n">
-        <v>58.2</v>
+        <v>51.19</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1996,7 +1996,7 @@
         <v>2.49</v>
       </c>
       <c r="Z10" t="n">
-        <v>1.17</v>
+        <v>0</v>
       </c>
       <c r="AA10" t="n">
         <v>0.35</v>
@@ -2008,7 +2008,7 @@
         <v>4.02</v>
       </c>
       <c r="AD10" t="n">
-        <v>4.8</v>
+        <v>5.96</v>
       </c>
       <c r="AE10" t="n">
         <v>4.9</v>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="AJ10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK10" t="b">
         <v>0</v>
@@ -2059,10 +2059,10 @@
         <v>69.19917864476385</v>
       </c>
       <c r="AU10" t="n">
-        <v>44.6</v>
+        <v>50.62</v>
       </c>
       <c r="AV10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2107,7 +2107,7 @@
         <v>45</v>
       </c>
       <c r="M11" t="n">
-        <v>47.65</v>
+        <v>47.88</v>
       </c>
       <c r="N11" t="b">
         <v>0</v>
@@ -2116,7 +2116,7 @@
         <v>47.03</v>
       </c>
       <c r="P11" t="n">
-        <v>47.88</v>
+        <v>48.24</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -2152,7 +2152,7 @@
         <v>-0.64</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.19</v>
+        <v>-0.29</v>
       </c>
       <c r="AA11" t="n">
         <v>3.98</v>
@@ -2164,7 +2164,7 @@
         <v>-1.8</v>
       </c>
       <c r="AD11" t="n">
-        <v>5.72</v>
+        <v>6.2</v>
       </c>
       <c r="AE11" t="n">
         <v>1.29</v>
@@ -2182,7 +2182,7 @@
         <v>-1.78</v>
       </c>
       <c r="AJ11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK11" t="b">
         <v>0</v>
@@ -2215,7 +2215,7 @@
         <v>44.26494345718907</v>
       </c>
       <c r="AU11" t="n">
-        <v>46.13</v>
+        <v>47.65</v>
       </c>
       <c r="AV11" t="b">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         <v>46.5</v>
       </c>
       <c r="M12" t="n">
-        <v>48.24</v>
+        <v>49</v>
       </c>
       <c r="N12" t="b">
         <v>0</v>
@@ -2272,7 +2272,7 @@
         <v>49.15</v>
       </c>
       <c r="P12" t="n">
-        <v>52.11</v>
+        <v>52.5</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
         <v>-0.11</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.23</v>
+        <v>-1.33</v>
       </c>
       <c r="AA12" t="n">
         <v>4.19</v>
@@ -2320,7 +2320,7 @@
         <v>-0.19</v>
       </c>
       <c r="AD12" t="n">
-        <v>3.67</v>
+        <v>5.24</v>
       </c>
       <c r="AE12" t="n">
         <v>3.11</v>
@@ -2338,7 +2338,7 @@
         <v>-4.03</v>
       </c>
       <c r="AJ12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK12" t="b">
         <v>0</v>
@@ -2371,10 +2371,10 @@
         <v>54.11954765751216</v>
       </c>
       <c r="AU12" t="n">
-        <v>48.24</v>
+        <v>49</v>
       </c>
       <c r="AV12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2419,7 +2419,7 @@
         <v>48.02</v>
       </c>
       <c r="M13" t="n">
-        <v>50.5</v>
+        <v>53.5</v>
       </c>
       <c r="N13" t="b">
         <v>0</v>
@@ -2428,7 +2428,7 @@
         <v>49.02</v>
       </c>
       <c r="P13" t="n">
-        <v>53.5</v>
+        <v>51.78</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -2464,7 +2464,7 @@
         <v>0.88</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.28</v>
+        <v>-5.35</v>
       </c>
       <c r="AA13" t="n">
         <v>2.91</v>
@@ -2476,7 +2476,7 @@
         <v>2.85</v>
       </c>
       <c r="AD13" t="n">
-        <v>5.03</v>
+        <v>10.8</v>
       </c>
       <c r="AE13" t="n">
         <v>2.51</v>
@@ -2494,7 +2494,7 @@
         <v>-4.13</v>
       </c>
       <c r="AJ13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK13" t="b">
         <v>0</v>
@@ -2527,7 +2527,7 @@
         <v>54.16666666666669</v>
       </c>
       <c r="AU13" t="n">
-        <v>47.83</v>
+        <v>50.5</v>
       </c>
       <c r="AV13" t="b">
         <v>1</v>
@@ -2575,7 +2575,7 @@
         <v>45.51</v>
       </c>
       <c r="M14" t="n">
-        <v>47.88</v>
+        <v>51</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
@@ -2584,7 +2584,7 @@
         <v>55.79</v>
       </c>
       <c r="P14" t="n">
-        <v>58.4</v>
+        <v>59</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         <v>0.46</v>
       </c>
       <c r="Z14" t="n">
-        <v>3.13</v>
+        <v>-3.18</v>
       </c>
       <c r="AA14" t="n">
         <v>3.89</v>
@@ -2632,7 +2632,7 @@
         <v>2.37</v>
       </c>
       <c r="AD14" t="n">
-        <v>5.08</v>
+        <v>11.38</v>
       </c>
       <c r="AE14" t="n">
         <v>5.27</v>
@@ -2650,7 +2650,7 @@
         <v>-0.63</v>
       </c>
       <c r="AJ14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK14" t="b">
         <v>0</v>
@@ -2683,10 +2683,10 @@
         <v>70.54545454545459</v>
       </c>
       <c r="AU14" t="n">
-        <v>44.5</v>
+        <v>79.16</v>
       </c>
       <c r="AV14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 11:11:16.432597
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV14"/>
+  <dimension ref="A1:AV10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,37 +689,37 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45672.41666666666</v>
+        <v>45678.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>45686.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>15.54</v>
+        <v>17.95</v>
       </c>
       <c r="G2" t="n">
-        <v>-9.779999999999999</v>
+        <v>-21.89</v>
       </c>
       <c r="H2" t="n">
-        <v>14.29</v>
+        <v>16.6</v>
       </c>
       <c r="I2" t="n">
         <v>18.2</v>
       </c>
       <c r="J2" t="n">
-        <v>17.12</v>
+        <v>1.39</v>
       </c>
       <c r="K2" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="L2" t="n">
         <v>14.02</v>
       </c>
       <c r="M2" t="n">
-        <v>15.96</v>
+        <v>17.47</v>
       </c>
       <c r="N2" t="b">
         <v>0</v>
@@ -728,7 +728,7 @@
         <v>18.26</v>
       </c>
       <c r="P2" t="n">
-        <v>20.79</v>
+        <v>19.93</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -741,54 +741,58 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>2912989</v>
-      </c>
-      <c r="T2" t="inlineStr"/>
+        <v>7215730</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>74.84999999999999</v>
+        <v>61.64</v>
       </c>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="n">
-        <v>1.07</v>
+        <v>2.66</v>
       </c>
       <c r="X2" t="n">
-        <v>6.05</v>
+        <v>7.19</v>
       </c>
       <c r="Y2" t="n">
-        <v>-4.63</v>
+        <v>-1.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>-2.63</v>
+        <v>2.75</v>
       </c>
       <c r="AA2" t="n">
         <v>16.89</v>
       </c>
       <c r="AB2" t="n">
-        <v>-21.88</v>
+        <v>-9.77</v>
       </c>
       <c r="AC2" t="n">
-        <v>-9.24</v>
+        <v>4.84</v>
       </c>
       <c r="AD2" t="n">
-        <v>12.94</v>
+        <v>21.91</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.75</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>24.58</v>
+        <v>7.86</v>
       </c>
       <c r="AG2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="AH2" s="2" t="n">
         <v>45684.41666666666</v>
       </c>
       <c r="AI2" t="n">
-        <v>0</v>
+        <v>-1.78</v>
       </c>
       <c r="AJ2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK2" t="b">
         <v>0</v>
@@ -815,7 +819,7 @@
         <v>75.68134171907757</v>
       </c>
       <c r="AU2" t="n">
-        <v>14.8</v>
+        <v>17.72</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
@@ -836,43 +840,43 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45687.41666666666</v>
+        <v>45705.41666666666</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>45722.41666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>20.07</v>
+        <v>21.53</v>
       </c>
       <c r="G3" t="n">
-        <v>-9.970000000000001</v>
+        <v>-16.07</v>
       </c>
       <c r="H3" t="n">
-        <v>18.2</v>
+        <v>20.59</v>
       </c>
       <c r="I3" t="n">
         <v>22.6</v>
       </c>
       <c r="J3" t="n">
-        <v>12.61</v>
+        <v>4.97</v>
       </c>
       <c r="K3" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="L3" t="n">
         <v>18.07</v>
       </c>
       <c r="M3" t="n">
-        <v>20.6</v>
+        <v>20.79</v>
       </c>
       <c r="N3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O3" t="n">
         <v>22.66</v>
       </c>
       <c r="P3" t="n">
-        <v>23.79</v>
+        <v>23.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -885,60 +889,60 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>5186111</v>
+        <v>3914369</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>BULLISH_TREND</t>
+          <t>BULLISH_BREAK</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>77.92</v>
+        <v>52.22</v>
       </c>
       <c r="V3" t="n">
-        <v>7.43</v>
+        <v>7.15</v>
       </c>
       <c r="W3" t="n">
-        <v>1.91</v>
+        <v>1.28</v>
       </c>
       <c r="X3" t="n">
-        <v>7.66</v>
+        <v>5.63</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.12</v>
+        <v>1.35</v>
       </c>
       <c r="Z3" t="n">
-        <v>-2.57</v>
+        <v>3.56</v>
       </c>
       <c r="AA3" t="n">
-        <v>16.89</v>
+        <v>6.13</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.89</v>
+        <v>8.23</v>
       </c>
       <c r="AC3" t="n">
-        <v>17.22</v>
+        <v>12.06</v>
       </c>
       <c r="AD3" t="n">
-        <v>13.09</v>
+        <v>14</v>
       </c>
       <c r="AE3" t="n">
-        <v>10.27</v>
+        <v>4.57</v>
       </c>
       <c r="AF3" t="n">
-        <v>18.24</v>
+        <v>10.22</v>
       </c>
       <c r="AG3" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="AH3" s="2" t="n">
         <v>45720.41666666666</v>
       </c>
       <c r="AI3" t="n">
-        <v>-7.17</v>
+        <v>-0.33</v>
       </c>
       <c r="AJ3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK3" t="b">
         <v>0</v>
@@ -947,30 +951,34 @@
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>19.07</v>
-      </c>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
+        <v>20.79</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>21.13</v>
+      </c>
       <c r="AP3" t="b">
         <v>0</v>
       </c>
       <c r="AQ3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT3" t="n">
-        <v>89.3648449039882</v>
+        <v>80.09259259259261</v>
       </c>
       <c r="AU3" t="n">
-        <v>19.07</v>
+        <v>22.52</v>
       </c>
       <c r="AV3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1015,7 +1023,7 @@
         <v>22.25</v>
       </c>
       <c r="M4" t="n">
-        <v>23.96</v>
+        <v>23.79</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1024,7 +1032,7 @@
         <v>22.67</v>
       </c>
       <c r="P4" t="n">
-        <v>24.7</v>
+        <v>23.96</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -1048,7 +1056,7 @@
         <v>100</v>
       </c>
       <c r="V4" t="n">
-        <v>2.96</v>
+        <v>0.71</v>
       </c>
       <c r="W4" t="n">
         <v>1.12</v>
@@ -1060,7 +1068,7 @@
         <v>3.69</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>0.71</v>
       </c>
       <c r="AA4" t="n">
         <v>5.5</v>
@@ -1072,7 +1080,7 @@
         <v>7.93</v>
       </c>
       <c r="AD4" t="n">
-        <v>7.4</v>
+        <v>6.69</v>
       </c>
       <c r="AE4" t="n">
         <v>5.69</v>
@@ -1090,7 +1098,7 @@
         <v>-5.68</v>
       </c>
       <c r="AJ4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK4" t="b">
         <v>0</v>
@@ -1099,7 +1107,7 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>23.25</v>
+        <v>23.79</v>
       </c>
       <c r="AN4" t="n">
         <v>22.25</v>
@@ -1123,7 +1131,7 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>23.25</v>
+        <v>23.79</v>
       </c>
       <c r="AV4" t="b">
         <v>1</v>
@@ -1144,43 +1152,43 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45735.41666666666</v>
+        <v>45761.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45753.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>23.41</v>
+        <v>22.6</v>
       </c>
       <c r="G5" t="n">
-        <v>-5.17</v>
+        <v>-13.45</v>
       </c>
       <c r="H5" t="n">
-        <v>22.02</v>
+        <v>21.57</v>
       </c>
       <c r="I5" t="n">
-        <v>21</v>
+        <v>36.21</v>
       </c>
       <c r="J5" t="n">
-        <v>-10.29</v>
+        <v>60.22</v>
       </c>
       <c r="K5" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="L5" t="n">
-        <v>22.2</v>
+        <v>19.56</v>
       </c>
       <c r="M5" t="n">
-        <v>23.47</v>
+        <v>21.98</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>22.02</v>
+        <v>36.6</v>
       </c>
       <c r="P5" t="n">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1193,60 +1201,60 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>448788</v>
+        <v>581928</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>BEARISH_BREAK</t>
+          <t>BULLISH_BREAK</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>95.86</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="V5" t="n">
-        <v>-5.24</v>
+        <v>-8.859999999999999</v>
       </c>
       <c r="W5" t="n">
-        <v>0.54</v>
+        <v>1.3</v>
       </c>
       <c r="X5" t="n">
-        <v>4.34</v>
+        <v>5.79</v>
       </c>
       <c r="Y5" t="n">
-        <v>3.04</v>
+        <v>1.25</v>
       </c>
       <c r="Z5" t="n">
-        <v>-0.26</v>
+        <v>2.82</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.17</v>
+        <v>4.77</v>
       </c>
       <c r="AB5" t="n">
-        <v>15.2</v>
+        <v>7.83</v>
       </c>
       <c r="AC5" t="n">
-        <v>3.87</v>
+        <v>3.12</v>
       </c>
       <c r="AD5" t="n">
-        <v>5.56</v>
+        <v>11.65</v>
       </c>
       <c r="AE5" t="n">
-        <v>5.07</v>
+        <v>4.78</v>
       </c>
       <c r="AF5" t="n">
-        <v>0</v>
+        <v>64.69</v>
       </c>
       <c r="AG5" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>45735.41666666666</v>
+        <v>45837.41666666666</v>
       </c>
       <c r="AI5" t="n">
-        <v>-10.29</v>
+        <v>-3.23</v>
       </c>
       <c r="AJ5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK5" t="b">
         <v>0</v>
@@ -1258,10 +1266,10 @@
         <v>24.7</v>
       </c>
       <c r="AN5" t="n">
-        <v>22.22</v>
+        <v>18.5</v>
       </c>
       <c r="AO5" t="n">
-        <v>23.79</v>
+        <v>23.64</v>
       </c>
       <c r="AP5" t="b">
         <v>0</v>
@@ -1276,13 +1284,13 @@
         <v>0</v>
       </c>
       <c r="AT5" t="n">
-        <v>51.86567164179107</v>
+        <v>83.33333333333333</v>
       </c>
       <c r="AU5" t="n">
-        <v>23.47</v>
+        <v>21.98</v>
       </c>
       <c r="AV5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1300,124 +1308,124 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45761.41666666666</v>
+        <v>45861.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>45890.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>22.6</v>
+        <v>36.92</v>
       </c>
       <c r="G6" t="n">
-        <v>-13.45</v>
+        <v>-11.54</v>
       </c>
       <c r="H6" t="n">
-        <v>21.57</v>
+        <v>35.51</v>
       </c>
       <c r="I6" t="n">
-        <v>36.21</v>
+        <v>41.93</v>
       </c>
       <c r="J6" t="n">
-        <v>60.22</v>
+        <v>13.57</v>
       </c>
       <c r="K6" t="n">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="L6" t="n">
-        <v>19.56</v>
+        <v>32.66</v>
       </c>
       <c r="M6" t="n">
-        <v>22.69</v>
+        <v>36</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>36.6</v>
+        <v>42.8</v>
       </c>
       <c r="P6" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>3527162</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>75.81</v>
+      </c>
+      <c r="V6" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="W6" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="X6" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>17.11</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>23.86</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>27</v>
+      </c>
+      <c r="AH6" s="2" t="n">
+        <v>45888.41666666666</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="AJ6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="n">
         <v>37.55</v>
       </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S6" t="n">
-        <v>581928</v>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U6" t="n">
-        <v>91.95999999999999</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="W6" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="X6" t="n">
-        <v>5.79</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>4.77</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>7.83</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>14.82</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>64.69</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>76</v>
-      </c>
-      <c r="AH6" s="2" t="n">
-        <v>45837.41666666666</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>-3.23</v>
-      </c>
-      <c r="AJ6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>22.6</v>
-      </c>
       <c r="AN6" t="n">
-        <v>18.5</v>
+        <v>32.77</v>
       </c>
       <c r="AO6" t="n">
-        <v>23.64</v>
+        <v>37</v>
       </c>
       <c r="AP6" t="b">
         <v>0</v>
@@ -1432,10 +1440,10 @@
         <v>0</v>
       </c>
       <c r="AT6" t="n">
-        <v>83.33333333333333</v>
+        <v>90.44585987261156</v>
       </c>
       <c r="AU6" t="n">
-        <v>21.7</v>
+        <v>36</v>
       </c>
       <c r="AV6" t="b">
         <v>1</v>
@@ -1453,127 +1461,127 @@
         </is>
       </c>
       <c r="C7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45942.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45890.41666666666</v>
+        <v>45944.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>35.51</v>
+        <v>47.7</v>
       </c>
       <c r="G7" t="n">
-        <v>-8.029999999999999</v>
+        <v>-23.48</v>
       </c>
       <c r="H7" t="n">
-        <v>33.5</v>
+        <v>39.75</v>
       </c>
       <c r="I7" t="n">
-        <v>41.93</v>
+        <v>47.44</v>
       </c>
       <c r="J7" t="n">
-        <v>18.08</v>
+        <v>-0.55</v>
       </c>
       <c r="K7" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>32.66</v>
+        <v>36.5</v>
       </c>
       <c r="M7" t="n">
-        <v>35.88</v>
+        <v>41.6</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>42.8</v>
+        <v>47.7</v>
       </c>
       <c r="P7" t="n">
+        <v>54.95</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>3766781</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>100</v>
+      </c>
+      <c r="V7" t="n">
+        <v>-2.49</v>
+      </c>
+      <c r="W7" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="X7" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>14.66</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>24.16</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>13.06</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH7" s="2" t="n">
+        <v>45943.41666666666</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="AJ7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="n">
         <v>48.89</v>
       </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S7" t="n">
-        <v>2216102</v>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U7" t="n">
-        <v>84.45</v>
-      </c>
-      <c r="V7" t="n">
-        <v>-4.65</v>
-      </c>
-      <c r="W7" t="n">
-        <v>4.96</v>
-      </c>
-      <c r="X7" t="n">
-        <v>4.94</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>-1.03</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>13.43</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>4.61</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>28.78</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>28</v>
-      </c>
-      <c r="AH7" s="2" t="n">
-        <v>45888.41666666666</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>37.55</v>
-      </c>
       <c r="AN7" t="n">
-        <v>32.77</v>
+        <v>39</v>
       </c>
       <c r="AO7" t="n">
-        <v>37</v>
+        <v>41.17</v>
       </c>
       <c r="AP7" t="b">
         <v>0</v>
@@ -1582,16 +1590,16 @@
         <v>0</v>
       </c>
       <c r="AR7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT7" t="n">
-        <v>58.28220858895707</v>
+        <v>100</v>
       </c>
       <c r="AU7" t="n">
-        <v>34.89</v>
+        <v>41.6</v>
       </c>
       <c r="AV7" t="b">
         <v>1</v>
@@ -1612,109 +1620,109 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45914.41666666666</v>
+        <v>45971.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45916.41666666666</v>
+        <v>46035.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>39</v>
+        <v>48.52</v>
       </c>
       <c r="G8" t="n">
-        <v>-6.41</v>
+        <v>-7.77</v>
       </c>
       <c r="H8" t="n">
-        <v>38.51</v>
+        <v>47.5</v>
       </c>
       <c r="I8" t="n">
-        <v>38.9</v>
+        <v>47.53</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.26</v>
+        <v>-2.04</v>
       </c>
       <c r="K8" t="n">
+        <v>64</v>
+      </c>
+      <c r="L8" t="n">
+        <v>44.75</v>
+      </c>
+      <c r="M8" t="n">
+        <v>47.89</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="P8" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>1429713</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>56.98</v>
+      </c>
+      <c r="V8" t="n">
+        <v>-11.48</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="X8" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="AG8" t="n">
         <v>2</v>
       </c>
-      <c r="L8" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="M8" t="n">
-        <v>39.4</v>
-      </c>
-      <c r="N8" t="b">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>39</v>
-      </c>
-      <c r="P8" t="n">
-        <v>41.06</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S8" t="n">
-        <v>212755</v>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>BULLISH_TREND</t>
-        </is>
-      </c>
-      <c r="U8" t="n">
-        <v>80.33</v>
-      </c>
-      <c r="V8" t="n">
-        <v>-11.71</v>
-      </c>
-      <c r="W8" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="X8" t="n">
-        <v>3.64</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>-1.02</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>7.64</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>1</v>
-      </c>
       <c r="AH8" s="2" t="n">
-        <v>45915.41666666666</v>
+        <v>45973.41666666666</v>
       </c>
       <c r="AI8" t="n">
-        <v>-0.26</v>
+        <v>-2.04</v>
       </c>
       <c r="AJ8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK8" t="b">
         <v>0</v>
@@ -1723,13 +1731,13 @@
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>43.7</v>
+        <v>54.95</v>
       </c>
       <c r="AN8" t="n">
-        <v>36.5</v>
+        <v>44.34</v>
       </c>
       <c r="AO8" t="n">
-        <v>39.64</v>
+        <v>47.7</v>
       </c>
       <c r="AP8" t="b">
         <v>0</v>
@@ -1744,13 +1752,13 @@
         <v>0</v>
       </c>
       <c r="AT8" t="n">
-        <v>42.88164665523157</v>
+        <v>85.07751937984503</v>
       </c>
       <c r="AU8" t="n">
-        <v>39.4</v>
+        <v>47.89</v>
       </c>
       <c r="AV8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1768,43 +1776,43 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45925.41666666666</v>
+        <v>46070.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45944.41666666666</v>
+        <v>46072.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>38.7</v>
+        <v>51.8</v>
       </c>
       <c r="G9" t="n">
-        <v>-9.529999999999999</v>
+        <v>-13.13</v>
       </c>
       <c r="H9" t="n">
-        <v>36.85</v>
+        <v>50.4</v>
       </c>
       <c r="I9" t="n">
-        <v>47.44</v>
+        <v>49.9</v>
       </c>
       <c r="J9" t="n">
-        <v>22.58</v>
+        <v>-3.67</v>
       </c>
       <c r="K9" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>35.01</v>
+        <v>45</v>
       </c>
       <c r="M9" t="n">
-        <v>38.7</v>
+        <v>51.19</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>47.7</v>
+        <v>50.4</v>
       </c>
       <c r="P9" t="n">
-        <v>54.95</v>
+        <v>52.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1817,60 +1825,60 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>300539</v>
+        <v>1667107</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>BULLISH_TREND</t>
+          <t>BULLISH_BREAK</t>
         </is>
       </c>
       <c r="U9" t="n">
-        <v>100</v>
+        <v>66.67</v>
       </c>
       <c r="V9" t="n">
-        <v>-6.1</v>
+        <v>2.5</v>
       </c>
       <c r="W9" t="n">
-        <v>1.11</v>
+        <v>2.15</v>
       </c>
       <c r="X9" t="n">
-        <v>4.27</v>
+        <v>3.24</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.63</v>
+        <v>2.07</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>1.19</v>
       </c>
       <c r="AA9" t="n">
-        <v>2.11</v>
+        <v>1.58</v>
       </c>
       <c r="AB9" t="n">
-        <v>2.78</v>
+        <v>7.18</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.89</v>
+        <v>6.85</v>
       </c>
       <c r="AD9" t="n">
-        <v>10.01</v>
+        <v>12.87</v>
       </c>
       <c r="AE9" t="n">
-        <v>5.02</v>
+        <v>1.53</v>
       </c>
       <c r="AF9" t="n">
-        <v>27.21</v>
+        <v>0.19</v>
       </c>
       <c r="AG9" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>45943.41666666666</v>
+        <v>46071.41666666666</v>
       </c>
       <c r="AI9" t="n">
-        <v>-0.52</v>
+        <v>-3.67</v>
       </c>
       <c r="AJ9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK9" t="b">
         <v>0</v>
@@ -1879,13 +1887,13 @@
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>41.06</v>
+        <v>51.19</v>
       </c>
       <c r="AN9" t="n">
-        <v>32.77</v>
+        <v>47.57</v>
       </c>
       <c r="AO9" t="n">
-        <v>37.43</v>
+        <v>54.54</v>
       </c>
       <c r="AP9" t="b">
         <v>0</v>
@@ -1894,19 +1902,19 @@
         <v>0</v>
       </c>
       <c r="AR9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT9" t="n">
-        <v>60.99173553719012</v>
+        <v>88.69143780290787</v>
       </c>
       <c r="AU9" t="n">
-        <v>37.98</v>
+        <v>52.14</v>
       </c>
       <c r="AV9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1924,43 +1932,43 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45970.41666666666</v>
+        <v>46112.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>46035.41666666666</v>
+        <v>46126.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>47.5</v>
+        <v>51.85</v>
       </c>
       <c r="G10" t="n">
-        <v>-5.79</v>
+        <v>-12.23</v>
       </c>
       <c r="H10" t="n">
-        <v>45.28</v>
+        <v>49.07</v>
       </c>
       <c r="I10" t="n">
-        <v>47.53</v>
+        <v>54.9</v>
       </c>
       <c r="J10" t="n">
-        <v>0.06</v>
+        <v>5.88</v>
       </c>
       <c r="K10" t="n">
-        <v>65</v>
+        <v>14</v>
       </c>
       <c r="L10" t="n">
-        <v>44.75</v>
+        <v>45.51</v>
       </c>
       <c r="M10" t="n">
-        <v>47.5</v>
+        <v>49.91</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>48.5</v>
+        <v>55.79</v>
       </c>
       <c r="P10" t="n">
-        <v>51.19</v>
+        <v>58.4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1973,7 +1981,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>403885</v>
+        <v>2394589</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1981,52 +1989,52 @@
         </is>
       </c>
       <c r="U10" t="n">
-        <v>100</v>
+        <v>97.54000000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>-7.37</v>
+        <v>-1.12</v>
       </c>
       <c r="W10" t="n">
-        <v>0.25</v>
+        <v>2.77</v>
       </c>
       <c r="X10" t="n">
-        <v>3.77</v>
+        <v>3.86</v>
       </c>
       <c r="Y10" t="n">
-        <v>2.49</v>
+        <v>1.57</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.35</v>
+        <v>1.3</v>
       </c>
       <c r="AB10" t="n">
-        <v>10.38</v>
+        <v>6.46</v>
       </c>
       <c r="AC10" t="n">
-        <v>4.02</v>
+        <v>6.33</v>
       </c>
       <c r="AD10" t="n">
-        <v>5.96</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="AE10" t="n">
-        <v>4.9</v>
+        <v>5.67</v>
       </c>
       <c r="AF10" t="n">
-        <v>15.83</v>
+        <v>11.76</v>
       </c>
       <c r="AG10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>45973.41666666666</v>
+        <v>46121.41666666666</v>
       </c>
       <c r="AI10" t="n">
         <v>0</v>
       </c>
       <c r="AJ10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK10" t="b">
         <v>0</v>
@@ -2035,13 +2043,13 @@
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>51</v>
+        <v>52.5</v>
       </c>
       <c r="AN10" t="n">
-        <v>44.34</v>
+        <v>47.33</v>
       </c>
       <c r="AO10" t="n">
-        <v>47.7</v>
+        <v>52.37</v>
       </c>
       <c r="AP10" t="b">
         <v>0</v>
@@ -2050,643 +2058,19 @@
         <v>0</v>
       </c>
       <c r="AR10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT10" t="n">
-        <v>69.19917864476385</v>
+        <v>98.90965732087227</v>
       </c>
       <c r="AU10" t="n">
-        <v>50.62</v>
+        <v>51.41</v>
       </c>
       <c r="AV10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C11" t="b">
-        <v>0</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>46041.41666666666</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>46042.41666666666</v>
-      </c>
-      <c r="F11" t="n">
-        <v>47.74</v>
-      </c>
-      <c r="G11" t="n">
-        <v>-5.74</v>
-      </c>
-      <c r="H11" t="n">
-        <v>47.03</v>
-      </c>
-      <c r="I11" t="n">
-        <v>46.89</v>
-      </c>
-      <c r="J11" t="n">
-        <v>-1.78</v>
-      </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="n">
-        <v>45</v>
-      </c>
-      <c r="M11" t="n">
-        <v>47.88</v>
-      </c>
-      <c r="N11" t="b">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>47.03</v>
-      </c>
-      <c r="P11" t="n">
-        <v>48.24</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S11" t="n">
-        <v>250069</v>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>BULLISH_TREND</t>
-        </is>
-      </c>
-      <c r="U11" t="n">
-        <v>83.53</v>
-      </c>
-      <c r="V11" t="n">
-        <v>-2.34</v>
-      </c>
-      <c r="W11" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="X11" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>-0.64</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>-0.29</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>3.98</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>-1.79</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="2" t="n">
-        <v>46041.41666666666</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>-1.78</v>
-      </c>
-      <c r="AJ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>49</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>44.34</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="AP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT11" t="n">
-        <v>44.26494345718907</v>
-      </c>
-      <c r="AU11" t="n">
-        <v>47.65</v>
-      </c>
-      <c r="AV11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C12" t="b">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>46043.41666666666</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>46075.41666666666</v>
-      </c>
-      <c r="F12" t="n">
-        <v>48.35</v>
-      </c>
-      <c r="G12" t="n">
-        <v>-3.83</v>
-      </c>
-      <c r="H12" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="I12" t="n">
-        <v>48.39</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="K12" t="n">
-        <v>32</v>
-      </c>
-      <c r="L12" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="M12" t="n">
-        <v>49</v>
-      </c>
-      <c r="N12" t="b">
-        <v>0</v>
-      </c>
-      <c r="O12" t="n">
-        <v>49.15</v>
-      </c>
-      <c r="P12" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S12" t="n">
-        <v>1463983</v>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U12" t="n">
-        <v>77.59</v>
-      </c>
-      <c r="V12" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="W12" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="X12" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>-1.33</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>-0.38</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>-0.19</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="AE12" t="n">
-        <v>3.11</v>
-      </c>
-      <c r="AF12" t="n">
-        <v>7.34</v>
-      </c>
-      <c r="AG12" t="n">
-        <v>28</v>
-      </c>
-      <c r="AH12" s="2" t="n">
-        <v>46071.41666666666</v>
-      </c>
-      <c r="AI12" t="n">
-        <v>-4.03</v>
-      </c>
-      <c r="AJ12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>48.24</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>44.34</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="AP12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT12" t="n">
-        <v>54.11954765751216</v>
-      </c>
-      <c r="AU12" t="n">
-        <v>49</v>
-      </c>
-      <c r="AV12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C13" t="b">
-        <v>0</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>46079.41666666666</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>46090.41666666666</v>
-      </c>
-      <c r="F13" t="n">
-        <v>50.64</v>
-      </c>
-      <c r="G13" t="n">
-        <v>-5.17</v>
-      </c>
-      <c r="H13" t="n">
-        <v>49.02</v>
-      </c>
-      <c r="I13" t="n">
-        <v>48.55</v>
-      </c>
-      <c r="J13" t="n">
-        <v>-4.13</v>
-      </c>
-      <c r="K13" t="n">
-        <v>11</v>
-      </c>
-      <c r="L13" t="n">
-        <v>48.02</v>
-      </c>
-      <c r="M13" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="N13" t="b">
-        <v>0</v>
-      </c>
-      <c r="O13" t="n">
-        <v>49.02</v>
-      </c>
-      <c r="P13" t="n">
-        <v>51.78</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S13" t="n">
-        <v>1689183</v>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U13" t="n">
-        <v>36.16</v>
-      </c>
-      <c r="V13" t="n">
-        <v>5.61</v>
-      </c>
-      <c r="W13" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="X13" t="n">
-        <v>4.29</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>-5.35</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>2.51</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>4</v>
-      </c>
-      <c r="AH13" s="2" t="n">
-        <v>46083.41666666666</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>-4.13</v>
-      </c>
-      <c r="AJ13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>44.65</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>52.37</v>
-      </c>
-      <c r="AP13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR13" t="b">
-        <v>1</v>
-      </c>
-      <c r="AS13" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>54.16666666666669</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="AV13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>46107.41666666666</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>46126.41666666666</v>
-      </c>
-      <c r="F14" t="n">
-        <v>49.38</v>
-      </c>
-      <c r="G14" t="n">
-        <v>-7.84</v>
-      </c>
-      <c r="H14" t="n">
-        <v>46.91</v>
-      </c>
-      <c r="I14" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="J14" t="n">
-        <v>11.18</v>
-      </c>
-      <c r="K14" t="n">
-        <v>19</v>
-      </c>
-      <c r="L14" t="n">
-        <v>45.51</v>
-      </c>
-      <c r="M14" t="n">
-        <v>51</v>
-      </c>
-      <c r="N14" t="b">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
-        <v>55.79</v>
-      </c>
-      <c r="P14" t="n">
-        <v>59</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S14" t="n">
-        <v>3000298</v>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U14" t="n">
-        <v>60.39</v>
-      </c>
-      <c r="V14" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="W14" t="n">
-        <v>3.93</v>
-      </c>
-      <c r="X14" t="n">
-        <v>3.79</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>-3.18</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>2.37</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>11.38</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>17.36</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>14</v>
-      </c>
-      <c r="AH14" s="2" t="n">
-        <v>46121.41666666666</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>-0.63</v>
-      </c>
-      <c r="AJ14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>49.46</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>45.39</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>49.53</v>
-      </c>
-      <c r="AP14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>70.54545454545459</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>79.16</v>
-      </c>
-      <c r="AV14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2822,55 +2206,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>61.54</v>
+        <v>55.56</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08</v>
+        <v>1.39</v>
       </c>
       <c r="H2" t="n">
-        <v>9.210000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="I2" t="n">
-        <v>119.79</v>
+        <v>74.09</v>
       </c>
       <c r="J2" t="n">
         <v>60.22</v>
       </c>
       <c r="K2" t="n">
-        <v>-10.29</v>
+        <v>-5.68</v>
       </c>
       <c r="L2" t="n">
-        <v>18.47</v>
+        <v>20.35</v>
       </c>
       <c r="M2" t="n">
         <v>5</v>
       </c>
       <c r="N2" t="n">
-        <v>17.74</v>
+        <v>17.21</v>
       </c>
       <c r="O2" t="n">
-        <v>4.43</v>
+        <v>2.98</v>
       </c>
       <c r="P2" t="n">
-        <v>9.210000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6666902670775552</v>
+        <v>0.6506096018735363</v>
       </c>
       <c r="R2" t="n">
-        <v>0.4982</v>
+        <v>0.41287</v>
       </c>
       <c r="S2" t="n">
-        <v>0.565596106831022</v>
+        <v>0.5079658407494145</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -2878,7 +2262,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.565596106831022</v>
+        <v>0.5079658407494145</v>
       </c>
     </row>
   </sheetData>
@@ -2949,22 +2333,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.57</v>
+        <v>0.51</v>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>61.54</v>
+        <v>55.56</v>
       </c>
       <c r="F2" t="n">
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08</v>
+        <v>1.39</v>
       </c>
       <c r="H2" t="n">
-        <v>9.210000000000001</v>
+        <v>8.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 11:12:48.170716
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV10"/>
+  <dimension ref="A1:AV14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,37 +689,37 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45678.41666666666</v>
+        <v>45672.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>45686.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>17.95</v>
+        <v>15.54</v>
       </c>
       <c r="G2" t="n">
-        <v>-21.89</v>
+        <v>-9.779999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>16.6</v>
+        <v>14.29</v>
       </c>
       <c r="I2" t="n">
         <v>18.2</v>
       </c>
       <c r="J2" t="n">
-        <v>1.39</v>
+        <v>17.12</v>
       </c>
       <c r="K2" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="L2" t="n">
         <v>14.02</v>
       </c>
       <c r="M2" t="n">
-        <v>17.47</v>
+        <v>14.8</v>
       </c>
       <c r="N2" t="b">
         <v>0</v>
@@ -741,55 +741,51 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>7215730</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
+        <v>2912989</v>
+      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>61.64</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="n">
-        <v>2.66</v>
+        <v>1.07</v>
       </c>
       <c r="X2" t="n">
-        <v>7.19</v>
+        <v>6.05</v>
       </c>
       <c r="Y2" t="n">
-        <v>-1.5</v>
+        <v>-4.63</v>
       </c>
       <c r="Z2" t="n">
-        <v>2.75</v>
+        <v>5</v>
       </c>
       <c r="AA2" t="n">
         <v>16.89</v>
       </c>
       <c r="AB2" t="n">
-        <v>-9.77</v>
+        <v>-21.88</v>
       </c>
       <c r="AC2" t="n">
-        <v>4.84</v>
+        <v>-9.24</v>
       </c>
       <c r="AD2" t="n">
-        <v>21.91</v>
+        <v>5.41</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.130000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="AF2" t="n">
-        <v>7.86</v>
+        <v>24.58</v>
       </c>
       <c r="AG2" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="AH2" s="2" t="n">
         <v>45684.41666666666</v>
       </c>
       <c r="AI2" t="n">
-        <v>-1.78</v>
+        <v>0</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -819,7 +815,7 @@
         <v>75.68134171907757</v>
       </c>
       <c r="AU2" t="n">
-        <v>17.72</v>
+        <v>14.8</v>
       </c>
       <c r="AV2" t="b">
         <v>1</v>
@@ -840,37 +836,37 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45705.41666666666</v>
+        <v>45687.41666666666</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>45722.41666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>21.53</v>
+        <v>20.07</v>
       </c>
       <c r="G3" t="n">
-        <v>-16.07</v>
+        <v>-9.970000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>20.59</v>
+        <v>18.2</v>
       </c>
       <c r="I3" t="n">
         <v>22.6</v>
       </c>
       <c r="J3" t="n">
-        <v>4.97</v>
+        <v>12.61</v>
       </c>
       <c r="K3" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="L3" t="n">
         <v>18.07</v>
       </c>
       <c r="M3" t="n">
-        <v>20.79</v>
+        <v>19.07</v>
       </c>
       <c r="N3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
         <v>22.66</v>
@@ -889,57 +885,57 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>3914369</v>
+        <v>5186111</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BULLISH_TREND</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>52.22</v>
+        <v>77.92</v>
       </c>
       <c r="V3" t="n">
-        <v>7.15</v>
+        <v>7.43</v>
       </c>
       <c r="W3" t="n">
-        <v>1.28</v>
+        <v>1.91</v>
       </c>
       <c r="X3" t="n">
-        <v>5.63</v>
+        <v>7.66</v>
       </c>
       <c r="Y3" t="n">
-        <v>1.35</v>
+        <v>0.12</v>
       </c>
       <c r="Z3" t="n">
-        <v>3.56</v>
+        <v>5.24</v>
       </c>
       <c r="AA3" t="n">
-        <v>6.13</v>
+        <v>16.89</v>
       </c>
       <c r="AB3" t="n">
-        <v>8.23</v>
+        <v>0.89</v>
       </c>
       <c r="AC3" t="n">
-        <v>12.06</v>
+        <v>17.22</v>
       </c>
       <c r="AD3" t="n">
-        <v>14</v>
+        <v>5.39</v>
       </c>
       <c r="AE3" t="n">
-        <v>4.57</v>
+        <v>10.27</v>
       </c>
       <c r="AF3" t="n">
-        <v>10.22</v>
+        <v>18.24</v>
       </c>
       <c r="AG3" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="AH3" s="2" t="n">
         <v>45720.41666666666</v>
       </c>
       <c r="AI3" t="n">
-        <v>-0.33</v>
+        <v>-7.17</v>
       </c>
       <c r="AJ3" t="b">
         <v>1</v>
@@ -951,34 +947,30 @@
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>20.79</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>14.14</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>21.13</v>
-      </c>
+        <v>19.07</v>
+      </c>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="b">
         <v>0</v>
       </c>
       <c r="AQ3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT3" t="n">
-        <v>80.09259259259261</v>
+        <v>89.3648449039882</v>
       </c>
       <c r="AU3" t="n">
-        <v>22.52</v>
+        <v>19.07</v>
       </c>
       <c r="AV3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1023,7 +1015,7 @@
         <v>22.25</v>
       </c>
       <c r="M4" t="n">
-        <v>23.79</v>
+        <v>23.25</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1056,7 +1048,7 @@
         <v>100</v>
       </c>
       <c r="V4" t="n">
-        <v>0.71</v>
+        <v>2.96</v>
       </c>
       <c r="W4" t="n">
         <v>1.12</v>
@@ -1068,7 +1060,7 @@
         <v>3.69</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.71</v>
+        <v>3.05</v>
       </c>
       <c r="AA4" t="n">
         <v>5.5</v>
@@ -1080,7 +1072,7 @@
         <v>7.93</v>
       </c>
       <c r="AD4" t="n">
-        <v>6.69</v>
+        <v>4.4</v>
       </c>
       <c r="AE4" t="n">
         <v>5.69</v>
@@ -1107,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>23.79</v>
+        <v>23.25</v>
       </c>
       <c r="AN4" t="n">
         <v>22.25</v>
@@ -1131,10 +1123,10 @@
         <v>98.61111111111114</v>
       </c>
       <c r="AU4" t="n">
-        <v>23.79</v>
+        <v>24.23</v>
       </c>
       <c r="AV4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1152,43 +1144,43 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45761.41666666666</v>
+        <v>45735.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>45753.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>22.6</v>
+        <v>23.41</v>
       </c>
       <c r="G5" t="n">
-        <v>-13.45</v>
+        <v>-5.17</v>
       </c>
       <c r="H5" t="n">
-        <v>21.57</v>
+        <v>22.02</v>
       </c>
       <c r="I5" t="n">
-        <v>36.21</v>
+        <v>21</v>
       </c>
       <c r="J5" t="n">
-        <v>60.22</v>
+        <v>-10.29</v>
       </c>
       <c r="K5" t="n">
-        <v>78</v>
+        <v>18</v>
       </c>
       <c r="L5" t="n">
-        <v>19.56</v>
+        <v>22.2</v>
       </c>
       <c r="M5" t="n">
-        <v>21.98</v>
+        <v>22.99</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>36.6</v>
+        <v>22.02</v>
       </c>
       <c r="P5" t="n">
-        <v>38</v>
+        <v>23.47</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1201,57 +1193,57 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>581928</v>
+        <v>448788</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BEARISH_BREAK</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>91.95999999999999</v>
+        <v>95.86</v>
       </c>
       <c r="V5" t="n">
-        <v>-8.859999999999999</v>
+        <v>-5.24</v>
       </c>
       <c r="W5" t="n">
-        <v>1.3</v>
+        <v>0.54</v>
       </c>
       <c r="X5" t="n">
-        <v>5.79</v>
+        <v>4.34</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.25</v>
+        <v>3.04</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.82</v>
+        <v>1.83</v>
       </c>
       <c r="AA5" t="n">
-        <v>4.77</v>
+        <v>1.17</v>
       </c>
       <c r="AB5" t="n">
-        <v>7.83</v>
+        <v>15.2</v>
       </c>
       <c r="AC5" t="n">
-        <v>3.12</v>
+        <v>3.87</v>
       </c>
       <c r="AD5" t="n">
-        <v>11.65</v>
+        <v>3.5</v>
       </c>
       <c r="AE5" t="n">
-        <v>4.78</v>
+        <v>5.07</v>
       </c>
       <c r="AF5" t="n">
-        <v>64.69</v>
+        <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>45837.41666666666</v>
+        <v>45735.41666666666</v>
       </c>
       <c r="AI5" t="n">
-        <v>-3.23</v>
+        <v>-10.29</v>
       </c>
       <c r="AJ5" t="b">
         <v>1</v>
@@ -1266,10 +1258,10 @@
         <v>24.7</v>
       </c>
       <c r="AN5" t="n">
-        <v>18.5</v>
+        <v>22.22</v>
       </c>
       <c r="AO5" t="n">
-        <v>23.64</v>
+        <v>23.79</v>
       </c>
       <c r="AP5" t="b">
         <v>0</v>
@@ -1284,10 +1276,10 @@
         <v>0</v>
       </c>
       <c r="AT5" t="n">
-        <v>83.33333333333333</v>
+        <v>51.86567164179107</v>
       </c>
       <c r="AU5" t="n">
-        <v>21.98</v>
+        <v>22.99</v>
       </c>
       <c r="AV5" t="b">
         <v>1</v>
@@ -1308,43 +1300,43 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45861.41666666666</v>
+        <v>45761.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45890.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>36.92</v>
+        <v>22.6</v>
       </c>
       <c r="G6" t="n">
-        <v>-11.54</v>
+        <v>-13.45</v>
       </c>
       <c r="H6" t="n">
-        <v>35.51</v>
+        <v>21.57</v>
       </c>
       <c r="I6" t="n">
-        <v>41.93</v>
+        <v>36.21</v>
       </c>
       <c r="J6" t="n">
-        <v>13.57</v>
+        <v>60.22</v>
       </c>
       <c r="K6" t="n">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="L6" t="n">
-        <v>32.66</v>
+        <v>19.56</v>
       </c>
       <c r="M6" t="n">
-        <v>36</v>
+        <v>21.7</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>42.8</v>
+        <v>36.6</v>
       </c>
       <c r="P6" t="n">
-        <v>48.89</v>
+        <v>38</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1357,7 +1349,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>3527162</v>
+        <v>581928</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1365,49 +1357,49 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>75.81</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="V6" t="n">
-        <v>-0.48</v>
+        <v>0.4</v>
       </c>
       <c r="W6" t="n">
-        <v>5.77</v>
+        <v>1.3</v>
       </c>
       <c r="X6" t="n">
-        <v>4.81</v>
+        <v>5.79</v>
       </c>
       <c r="Y6" t="n">
-        <v>3.04</v>
+        <v>1.25</v>
       </c>
       <c r="Z6" t="n">
-        <v>2.56</v>
+        <v>4.15</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.28</v>
+        <v>4.77</v>
       </c>
       <c r="AB6" t="n">
-        <v>17.11</v>
+        <v>7.83</v>
       </c>
       <c r="AC6" t="n">
-        <v>7.86</v>
+        <v>3.12</v>
       </c>
       <c r="AD6" t="n">
-        <v>9.73</v>
+        <v>10.37</v>
       </c>
       <c r="AE6" t="n">
-        <v>3.97</v>
+        <v>4.78</v>
       </c>
       <c r="AF6" t="n">
-        <v>23.86</v>
+        <v>64.69</v>
       </c>
       <c r="AG6" t="n">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>45888.41666666666</v>
+        <v>45837.41666666666</v>
       </c>
       <c r="AI6" t="n">
-        <v>-1.14</v>
+        <v>-3.23</v>
       </c>
       <c r="AJ6" t="b">
         <v>1</v>
@@ -1419,13 +1411,13 @@
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>37.55</v>
+        <v>22.6</v>
       </c>
       <c r="AN6" t="n">
-        <v>32.77</v>
+        <v>18.5</v>
       </c>
       <c r="AO6" t="n">
-        <v>37</v>
+        <v>23.64</v>
       </c>
       <c r="AP6" t="b">
         <v>0</v>
@@ -1440,10 +1432,10 @@
         <v>0</v>
       </c>
       <c r="AT6" t="n">
-        <v>90.44585987261156</v>
+        <v>83.33333333333333</v>
       </c>
       <c r="AU6" t="n">
-        <v>36</v>
+        <v>21.7</v>
       </c>
       <c r="AV6" t="b">
         <v>1</v>
@@ -1461,46 +1453,46 @@
         </is>
       </c>
       <c r="C7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45942.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45944.41666666666</v>
+        <v>45890.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>47.7</v>
+        <v>35.51</v>
       </c>
       <c r="G7" t="n">
-        <v>-23.48</v>
+        <v>-8.029999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>39.75</v>
+        <v>33.5</v>
       </c>
       <c r="I7" t="n">
-        <v>47.44</v>
+        <v>41.93</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.55</v>
+        <v>18.08</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="L7" t="n">
-        <v>36.5</v>
+        <v>32.66</v>
       </c>
       <c r="M7" t="n">
-        <v>41.6</v>
+        <v>34.89</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>47.7</v>
+        <v>42.8</v>
       </c>
       <c r="P7" t="n">
-        <v>54.95</v>
+        <v>48.89</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1513,7 +1505,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>3766781</v>
+        <v>2216102</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1521,49 +1513,49 @@
         </is>
       </c>
       <c r="U7" t="n">
-        <v>100</v>
+        <v>84.45</v>
       </c>
       <c r="V7" t="n">
-        <v>-2.49</v>
+        <v>-4.65</v>
       </c>
       <c r="W7" t="n">
-        <v>8.960000000000001</v>
+        <v>4.96</v>
       </c>
       <c r="X7" t="n">
-        <v>5.27</v>
+        <v>4.94</v>
       </c>
       <c r="Y7" t="n">
-        <v>3.69</v>
+        <v>2.39</v>
       </c>
       <c r="Z7" t="n">
-        <v>14.66</v>
+        <v>1.78</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.7</v>
+        <v>1.55</v>
       </c>
       <c r="AB7" t="n">
-        <v>24.16</v>
+        <v>13.43</v>
       </c>
       <c r="AC7" t="n">
-        <v>20.5</v>
+        <v>4.61</v>
       </c>
       <c r="AD7" t="n">
-        <v>13.06</v>
+        <v>6.6</v>
       </c>
       <c r="AE7" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="AF7" t="n">
-        <v>3.21</v>
+        <v>28.78</v>
       </c>
       <c r="AG7" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>45943.41666666666</v>
+        <v>45888.41666666666</v>
       </c>
       <c r="AI7" t="n">
-        <v>-0.55</v>
+        <v>0</v>
       </c>
       <c r="AJ7" t="b">
         <v>1</v>
@@ -1575,13 +1567,13 @@
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>48.89</v>
+        <v>37.55</v>
       </c>
       <c r="AN7" t="n">
-        <v>39</v>
+        <v>32.77</v>
       </c>
       <c r="AO7" t="n">
-        <v>41.17</v>
+        <v>37</v>
       </c>
       <c r="AP7" t="b">
         <v>0</v>
@@ -1590,16 +1582,16 @@
         <v>0</v>
       </c>
       <c r="AR7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT7" t="n">
-        <v>100</v>
+        <v>58.28220858895707</v>
       </c>
       <c r="AU7" t="n">
-        <v>41.6</v>
+        <v>34.89</v>
       </c>
       <c r="AV7" t="b">
         <v>1</v>
@@ -1620,43 +1612,43 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45971.41666666666</v>
+        <v>45914.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46035.41666666666</v>
+        <v>45916.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>48.52</v>
+        <v>39</v>
       </c>
       <c r="G8" t="n">
-        <v>-7.77</v>
+        <v>-6.41</v>
       </c>
       <c r="H8" t="n">
-        <v>47.5</v>
+        <v>38.51</v>
       </c>
       <c r="I8" t="n">
-        <v>47.53</v>
+        <v>38.9</v>
       </c>
       <c r="J8" t="n">
-        <v>-2.04</v>
+        <v>-0.26</v>
       </c>
       <c r="K8" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="L8" t="n">
-        <v>44.75</v>
+        <v>36.5</v>
       </c>
       <c r="M8" t="n">
-        <v>47.89</v>
+        <v>38.64</v>
       </c>
       <c r="N8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>48.5</v>
+        <v>39</v>
       </c>
       <c r="P8" t="n">
-        <v>58.2</v>
+        <v>40.77</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1669,57 +1661,57 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>1429713</v>
+        <v>212755</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BULLISH_TREND</t>
         </is>
       </c>
       <c r="U8" t="n">
-        <v>56.98</v>
+        <v>80.33</v>
       </c>
       <c r="V8" t="n">
-        <v>-11.48</v>
+        <v>-11.71</v>
       </c>
       <c r="W8" t="n">
-        <v>0.95</v>
+        <v>0.51</v>
       </c>
       <c r="X8" t="n">
-        <v>3.69</v>
+        <v>3.64</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.94</v>
+        <v>1.05</v>
       </c>
       <c r="Z8" t="n">
-        <v>1.32</v>
+        <v>0.93</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.27</v>
+        <v>5.03</v>
       </c>
       <c r="AB8" t="n">
-        <v>12.19</v>
+        <v>3.97</v>
       </c>
       <c r="AC8" t="n">
-        <v>5.62</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="AD8" t="n">
-        <v>6.78</v>
+        <v>5.7</v>
       </c>
       <c r="AE8" t="n">
-        <v>2.15</v>
+        <v>0.96</v>
       </c>
       <c r="AF8" t="n">
-        <v>13.4</v>
+        <v>3.41</v>
       </c>
       <c r="AG8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>45973.41666666666</v>
+        <v>45915.41666666666</v>
       </c>
       <c r="AI8" t="n">
-        <v>-2.04</v>
+        <v>-0.26</v>
       </c>
       <c r="AJ8" t="b">
         <v>1</v>
@@ -1731,13 +1723,13 @@
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>54.95</v>
+        <v>43.7</v>
       </c>
       <c r="AN8" t="n">
-        <v>44.34</v>
+        <v>36.5</v>
       </c>
       <c r="AO8" t="n">
-        <v>47.7</v>
+        <v>39.64</v>
       </c>
       <c r="AP8" t="b">
         <v>0</v>
@@ -1752,13 +1744,13 @@
         <v>0</v>
       </c>
       <c r="AT8" t="n">
-        <v>85.07751937984503</v>
+        <v>42.88164665523157</v>
       </c>
       <c r="AU8" t="n">
-        <v>47.89</v>
+        <v>40.79</v>
       </c>
       <c r="AV8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1776,43 +1768,43 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46070.41666666666</v>
+        <v>45925.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>46072.41666666666</v>
+        <v>45944.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>51.8</v>
+        <v>38.7</v>
       </c>
       <c r="G9" t="n">
-        <v>-13.13</v>
+        <v>-9.529999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>50.4</v>
+        <v>36.85</v>
       </c>
       <c r="I9" t="n">
-        <v>49.9</v>
+        <v>47.44</v>
       </c>
       <c r="J9" t="n">
-        <v>-3.67</v>
+        <v>22.58</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="L9" t="n">
-        <v>45</v>
+        <v>35.01</v>
       </c>
       <c r="M9" t="n">
-        <v>51.19</v>
+        <v>37.98</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>50.4</v>
+        <v>47.7</v>
       </c>
       <c r="P9" t="n">
-        <v>52.5</v>
+        <v>54.95</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1825,57 +1817,57 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>1667107</v>
+        <v>300539</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>BULLISH_BREAK</t>
+          <t>BULLISH_TREND</t>
         </is>
       </c>
       <c r="U9" t="n">
-        <v>66.67</v>
+        <v>100</v>
       </c>
       <c r="V9" t="n">
-        <v>2.5</v>
+        <v>-6.1</v>
       </c>
       <c r="W9" t="n">
-        <v>2.15</v>
+        <v>1.11</v>
       </c>
       <c r="X9" t="n">
-        <v>3.24</v>
+        <v>4.27</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.07</v>
+        <v>0.63</v>
       </c>
       <c r="Z9" t="n">
-        <v>1.19</v>
+        <v>1.9</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.58</v>
+        <v>2.11</v>
       </c>
       <c r="AB9" t="n">
-        <v>7.18</v>
+        <v>2.78</v>
       </c>
       <c r="AC9" t="n">
-        <v>6.85</v>
+        <v>0.89</v>
       </c>
       <c r="AD9" t="n">
-        <v>12.87</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="AE9" t="n">
-        <v>1.53</v>
+        <v>5.02</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.19</v>
+        <v>27.21</v>
       </c>
       <c r="AG9" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>46071.41666666666</v>
+        <v>45943.41666666666</v>
       </c>
       <c r="AI9" t="n">
-        <v>-3.67</v>
+        <v>-0.52</v>
       </c>
       <c r="AJ9" t="b">
         <v>1</v>
@@ -1887,13 +1879,13 @@
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>51.19</v>
+        <v>41.06</v>
       </c>
       <c r="AN9" t="n">
-        <v>47.57</v>
+        <v>32.77</v>
       </c>
       <c r="AO9" t="n">
-        <v>54.54</v>
+        <v>37.43</v>
       </c>
       <c r="AP9" t="b">
         <v>0</v>
@@ -1902,19 +1894,19 @@
         <v>0</v>
       </c>
       <c r="AR9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT9" t="n">
-        <v>88.69143780290787</v>
+        <v>60.99173553719012</v>
       </c>
       <c r="AU9" t="n">
-        <v>52.14</v>
+        <v>37.98</v>
       </c>
       <c r="AV9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1932,144 +1924,768 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46112.41666666666</v>
+        <v>45970.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
+        <v>46035.41666666666</v>
+      </c>
+      <c r="F10" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="H10" t="n">
+        <v>45.28</v>
+      </c>
+      <c r="I10" t="n">
+        <v>47.53</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K10" t="n">
+        <v>65</v>
+      </c>
+      <c r="L10" t="n">
+        <v>44.75</v>
+      </c>
+      <c r="M10" t="n">
+        <v>46.95</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="P10" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>403885</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>100</v>
+      </c>
+      <c r="V10" t="n">
+        <v>-7.37</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X10" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>15.83</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH10" s="2" t="n">
+        <v>45973.41666666666</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>51</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>44.34</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AP10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>69.19917864476385</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>48.07</v>
+      </c>
+      <c r="AV10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>46041.41666666666</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>46042.41666666666</v>
+      </c>
+      <c r="F11" t="n">
+        <v>47.74</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-5.74</v>
+      </c>
+      <c r="H11" t="n">
+        <v>47.03</v>
+      </c>
+      <c r="I11" t="n">
+        <v>46.89</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>45</v>
+      </c>
+      <c r="M11" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>47.03</v>
+      </c>
+      <c r="P11" t="n">
+        <v>47.88</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>250069</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>BULLISH_TREND</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>83.53</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-2.34</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="X11" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>-1.79</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="2" t="n">
+        <v>46041.41666666666</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="AJ11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>49</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>44.34</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>44.26494345718907</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="AV11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>46043.41666666666</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>46075.41666666666</v>
+      </c>
+      <c r="F12" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-3.83</v>
+      </c>
+      <c r="H12" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>48.39</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="K12" t="n">
+        <v>32</v>
+      </c>
+      <c r="L12" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>49.15</v>
+      </c>
+      <c r="P12" t="n">
+        <v>52.11</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>1463983</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>77.59</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="W12" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="X12" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>28</v>
+      </c>
+      <c r="AH12" s="2" t="n">
+        <v>46071.41666666666</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>-4.03</v>
+      </c>
+      <c r="AJ12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>44.34</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AP12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>54.11954765751216</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="AV12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>46079.41666666666</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>46090.41666666666</v>
+      </c>
+      <c r="F13" t="n">
+        <v>50.64</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-5.17</v>
+      </c>
+      <c r="H13" t="n">
+        <v>49.02</v>
+      </c>
+      <c r="I13" t="n">
+        <v>48.55</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-4.13</v>
+      </c>
+      <c r="K13" t="n">
+        <v>11</v>
+      </c>
+      <c r="L13" t="n">
+        <v>48.02</v>
+      </c>
+      <c r="M13" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="N13" t="b">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>49.02</v>
+      </c>
+      <c r="P13" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>1689183</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>36.16</v>
+      </c>
+      <c r="V13" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="W13" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="X13" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH13" s="2" t="n">
+        <v>46083.41666666666</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>-4.13</v>
+      </c>
+      <c r="AJ13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>44.65</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>52.37</v>
+      </c>
+      <c r="AP13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>54.16666666666669</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="AV13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>46107.41666666666</v>
+      </c>
+      <c r="E14" s="2" t="n">
         <v>46126.41666666666</v>
       </c>
-      <c r="F10" t="n">
-        <v>51.85</v>
-      </c>
-      <c r="G10" t="n">
-        <v>-12.23</v>
-      </c>
-      <c r="H10" t="n">
-        <v>49.07</v>
-      </c>
-      <c r="I10" t="n">
+      <c r="F14" t="n">
+        <v>49.38</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-7.84</v>
+      </c>
+      <c r="H14" t="n">
+        <v>46.91</v>
+      </c>
+      <c r="I14" t="n">
         <v>54.9</v>
       </c>
-      <c r="J10" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="K10" t="n">
+      <c r="J14" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="K14" t="n">
+        <v>19</v>
+      </c>
+      <c r="L14" t="n">
+        <v>45.51</v>
+      </c>
+      <c r="M14" t="n">
+        <v>47.88</v>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>55.79</v>
+      </c>
+      <c r="P14" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>3000298</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>BULLISH_BREAK</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>60.39</v>
+      </c>
+      <c r="V14" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="W14" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="X14" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>17.36</v>
+      </c>
+      <c r="AG14" t="n">
         <v>14</v>
       </c>
-      <c r="L10" t="n">
-        <v>45.51</v>
-      </c>
-      <c r="M10" t="n">
-        <v>49.91</v>
-      </c>
-      <c r="N10" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" t="n">
-        <v>55.79</v>
-      </c>
-      <c r="P10" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="S10" t="n">
-        <v>2394589</v>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>BULLISH_BREAK</t>
-        </is>
-      </c>
-      <c r="U10" t="n">
-        <v>97.54000000000001</v>
-      </c>
-      <c r="V10" t="n">
-        <v>-1.12</v>
-      </c>
-      <c r="W10" t="n">
-        <v>2.77</v>
-      </c>
-      <c r="X10" t="n">
-        <v>3.86</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>6.46</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>6.33</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>9.220000000000001</v>
-      </c>
-      <c r="AE10" t="n">
-        <v>5.67</v>
-      </c>
-      <c r="AF10" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="AG10" t="n">
-        <v>9</v>
-      </c>
-      <c r="AH10" s="2" t="n">
+      <c r="AH14" s="2" t="n">
         <v>46121.41666666666</v>
       </c>
-      <c r="AI10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>47.33</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>52.37</v>
-      </c>
-      <c r="AP10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AS10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>98.90965732087227</v>
-      </c>
-      <c r="AU10" t="n">
-        <v>51.41</v>
-      </c>
-      <c r="AV10" t="b">
+      <c r="AI14" t="n">
+        <v>-0.63</v>
+      </c>
+      <c r="AJ14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>49.46</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>45.39</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>49.53</v>
+      </c>
+      <c r="AP14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>70.54545454545459</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>48.08</v>
+      </c>
+      <c r="AV14" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2206,55 +2822,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
         <v>5</v>
       </c>
-      <c r="E2" t="n">
-        <v>4</v>
-      </c>
       <c r="F2" t="n">
-        <v>55.56</v>
+        <v>61.54</v>
       </c>
       <c r="G2" t="n">
-        <v>1.39</v>
+        <v>0.08</v>
       </c>
       <c r="H2" t="n">
-        <v>8.23</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>74.09</v>
+        <v>119.79</v>
       </c>
       <c r="J2" t="n">
         <v>60.22</v>
       </c>
       <c r="K2" t="n">
-        <v>-5.68</v>
+        <v>-10.29</v>
       </c>
       <c r="L2" t="n">
-        <v>20.35</v>
+        <v>18.47</v>
       </c>
       <c r="M2" t="n">
         <v>5</v>
       </c>
       <c r="N2" t="n">
-        <v>17.21</v>
+        <v>17.74</v>
       </c>
       <c r="O2" t="n">
-        <v>2.98</v>
+        <v>4.43</v>
       </c>
       <c r="P2" t="n">
-        <v>8.23</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6506096018735363</v>
+        <v>0.6666902670775552</v>
       </c>
       <c r="R2" t="n">
-        <v>0.41287</v>
+        <v>0.4982</v>
       </c>
       <c r="S2" t="n">
-        <v>0.5079658407494145</v>
+        <v>0.565596106831022</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -2262,7 +2878,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.5079658407494145</v>
+        <v>0.565596106831022</v>
       </c>
     </row>
   </sheetData>
@@ -2333,22 +2949,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.51</v>
+        <v>0.57</v>
       </c>
       <c r="D2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>55.56</v>
+        <v>61.54</v>
       </c>
       <c r="F2" t="n">
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>1.39</v>
+        <v>0.08</v>
       </c>
       <c r="H2" t="n">
-        <v>8.23</v>
+        <v>9.210000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:13:45.906083
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -8,10 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Closed_Trades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Open_Trades" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Strategy_Profile" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Best_Strategy_Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="refresh_date" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Strategy_Profile" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Best_Strategy_Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="refresh_date" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +528,14 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Current_Price</t>
+          <t>Anchor_High</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -545,34 +544,34 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45666.41666666666</v>
+        <v>45672.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45699.41666666666</v>
+        <v>45686.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>4.97</v>
+        <v>15.54</v>
       </c>
       <c r="G2" t="n">
-        <v>4.61</v>
+        <v>14.29</v>
       </c>
       <c r="H2" t="n">
-        <v>4.59</v>
+        <v>18.2</v>
       </c>
       <c r="I2" t="n">
-        <v>-7.65</v>
+        <v>17.12</v>
       </c>
       <c r="J2" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="K2" t="n">
-        <v>4.44</v>
+        <v>14.02</v>
       </c>
       <c r="L2" t="n">
-        <v>4.65</v>
+        <v>14.8</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -585,23 +584,25 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>3052353</v>
+        <v>2912989</v>
       </c>
       <c r="P2" t="n">
-        <v>7.81</v>
+        <v>8.75</v>
       </c>
       <c r="Q2" t="n">
-        <v>4.89</v>
+        <v>14.8</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
-      <c r="S2" t="inlineStr"/>
+      <c r="S2" t="n">
+        <v>15.96</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -610,34 +611,34 @@
         </is>
       </c>
       <c r="C3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45769.41666666666</v>
+        <v>45687.41666666666</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45789.41666666666</v>
+        <v>45722.41666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>5.27</v>
+        <v>20.07</v>
       </c>
       <c r="G3" t="n">
-        <v>4.92</v>
+        <v>18.2</v>
       </c>
       <c r="H3" t="n">
-        <v>6</v>
+        <v>22.6</v>
       </c>
       <c r="I3" t="n">
-        <v>13.85</v>
+        <v>12.61</v>
       </c>
       <c r="J3" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="K3" t="n">
-        <v>4.44</v>
+        <v>18.07</v>
       </c>
       <c r="L3" t="n">
-        <v>5.2</v>
+        <v>19.07</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -650,23 +651,25 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>2274184</v>
+        <v>5186111</v>
       </c>
       <c r="P3" t="n">
-        <v>7.11</v>
+        <v>10.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>5.75</v>
+        <v>19.07</v>
       </c>
       <c r="R3" t="b">
-        <v>0</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>20.6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -675,63 +678,65 @@
         </is>
       </c>
       <c r="C4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>45726.41666666666</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>45728.41666666666</v>
+      </c>
+      <c r="F4" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="G4" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="H4" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="L4" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>1305391</v>
+      </c>
+      <c r="P4" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>24.23</v>
+      </c>
+      <c r="R4" t="b">
         <v>0</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>45799.41666666666</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>45819.41666666666</v>
-      </c>
-      <c r="F4" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="G4" t="n">
-        <v>5.52</v>
-      </c>
-      <c r="H4" t="n">
-        <v>5.82</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-1.36</v>
-      </c>
-      <c r="J4" t="n">
-        <v>20</v>
-      </c>
-      <c r="K4" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="L4" t="n">
-        <v>5.69</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O4" t="n">
-        <v>1619883</v>
-      </c>
-      <c r="P4" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>5.69</v>
-      </c>
-      <c r="R4" t="b">
-        <v>1</v>
-      </c>
-      <c r="S4" t="inlineStr"/>
+      <c r="S4" t="n">
+        <v>23.96</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -743,31 +748,31 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>45735.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45865.41666666666</v>
+        <v>45753.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>5.6</v>
+        <v>23.41</v>
       </c>
       <c r="G5" t="n">
-        <v>5.49</v>
+        <v>22.02</v>
       </c>
       <c r="H5" t="n">
-        <v>6.72</v>
+        <v>21</v>
       </c>
       <c r="I5" t="n">
-        <v>20</v>
+        <v>-10.29</v>
       </c>
       <c r="J5" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="K5" t="n">
-        <v>4.6</v>
+        <v>22.2</v>
       </c>
       <c r="L5" t="n">
-        <v>5.57</v>
+        <v>22.99</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -780,23 +785,25 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>1189884</v>
+        <v>448788</v>
       </c>
       <c r="P5" t="n">
-        <v>1.63</v>
+        <v>5.07</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.57</v>
+        <v>22.99</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
-      <c r="S5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>23.47</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -808,31 +815,31 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45873.41666666666</v>
+        <v>45761.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45880.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>6.9</v>
+        <v>22.6</v>
       </c>
       <c r="G6" t="n">
-        <v>6.62</v>
+        <v>21.57</v>
       </c>
       <c r="H6" t="n">
-        <v>6.53</v>
+        <v>36.21</v>
       </c>
       <c r="I6" t="n">
-        <v>-5.36</v>
+        <v>60.22</v>
       </c>
       <c r="J6" t="n">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="K6" t="n">
-        <v>6.48</v>
+        <v>19.56</v>
       </c>
       <c r="L6" t="n">
-        <v>6.73</v>
+        <v>21.7</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -845,23 +852,25 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>1865203</v>
+        <v>581928</v>
       </c>
       <c r="P6" t="n">
-        <v>3.45</v>
+        <v>4.78</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.9</v>
+        <v>21.7</v>
       </c>
       <c r="R6" t="b">
-        <v>0</v>
-      </c>
-      <c r="S6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S6" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -873,60 +882,62 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45888.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45889.41666666666</v>
+        <v>45890.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>6.8</v>
+        <v>35.51</v>
       </c>
       <c r="G7" t="n">
-        <v>6.71</v>
+        <v>33.5</v>
       </c>
       <c r="H7" t="n">
-        <v>6.55</v>
+        <v>41.93</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.68</v>
+        <v>18.08</v>
       </c>
       <c r="J7" t="n">
+        <v>30</v>
+      </c>
+      <c r="K7" t="n">
+        <v>32.66</v>
+      </c>
+      <c r="L7" t="n">
+        <v>34.89</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>2216102</v>
+      </c>
+      <c r="P7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>34.89</v>
+      </c>
+      <c r="R7" t="b">
         <v>1</v>
       </c>
-      <c r="K7" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="L7" t="n">
-        <v>6.73</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O7" t="n">
-        <v>1273591</v>
-      </c>
-      <c r="P7" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>7.63</v>
-      </c>
-      <c r="R7" t="b">
-        <v>0</v>
-      </c>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>35.88</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -938,31 +949,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45922.41666666666</v>
+        <v>45914.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45932.41666666666</v>
+        <v>45916.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>6.4</v>
+        <v>39</v>
       </c>
       <c r="G8" t="n">
-        <v>5.95</v>
+        <v>38.51</v>
       </c>
       <c r="H8" t="n">
-        <v>6.25</v>
+        <v>38.9</v>
       </c>
       <c r="I8" t="n">
-        <v>-2.34</v>
+        <v>-0.26</v>
       </c>
       <c r="J8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>5.93</v>
+        <v>36.5</v>
       </c>
       <c r="L8" t="n">
-        <v>6.19</v>
+        <v>38.64</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -975,23 +986,25 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>1694740</v>
+        <v>212755</v>
       </c>
       <c r="P8" t="n">
-        <v>6.84</v>
+        <v>0.96</v>
       </c>
       <c r="Q8" t="n">
-        <v>6.19</v>
+        <v>40.79</v>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
-      </c>
-      <c r="S8" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>39.4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1003,31 +1016,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45935.41666666666</v>
+        <v>45925.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45958.41666666666</v>
+        <v>45944.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>6.5</v>
+        <v>38.7</v>
       </c>
       <c r="G9" t="n">
-        <v>6.2</v>
+        <v>36.85</v>
       </c>
       <c r="H9" t="n">
-        <v>6.69</v>
+        <v>47.44</v>
       </c>
       <c r="I9" t="n">
-        <v>2.92</v>
+        <v>22.58</v>
       </c>
       <c r="J9" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="K9" t="n">
-        <v>6.23</v>
+        <v>35.01</v>
       </c>
       <c r="L9" t="n">
-        <v>6.45</v>
+        <v>37.98</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1040,23 +1053,25 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>1208314</v>
+        <v>300539</v>
       </c>
       <c r="P9" t="n">
-        <v>4</v>
+        <v>5.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>6.45</v>
+        <v>37.98</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
       </c>
-      <c r="S9" t="inlineStr"/>
+      <c r="S9" t="n">
+        <v>38.7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1068,31 +1083,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45984.41666666666</v>
+        <v>45970.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45986.41666666666</v>
+        <v>46035.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>6.59</v>
+        <v>47.5</v>
       </c>
       <c r="G10" t="n">
-        <v>6.34</v>
+        <v>45.28</v>
       </c>
       <c r="H10" t="n">
-        <v>6.33</v>
+        <v>47.53</v>
       </c>
       <c r="I10" t="n">
-        <v>-3.95</v>
+        <v>0.06</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>65</v>
       </c>
       <c r="K10" t="n">
-        <v>6.2</v>
+        <v>44.75</v>
       </c>
       <c r="L10" t="n">
-        <v>6.37</v>
+        <v>46.95</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1105,23 +1120,25 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>1101047</v>
+        <v>403885</v>
       </c>
       <c r="P10" t="n">
-        <v>3.94</v>
+        <v>4.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.59</v>
+        <v>48.07</v>
       </c>
       <c r="R10" t="b">
         <v>0</v>
       </c>
-      <c r="S10" t="inlineStr"/>
+      <c r="S10" t="n">
+        <v>47.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1133,31 +1150,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46007.41666666666</v>
+        <v>46041.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>46019.41666666666</v>
+        <v>46042.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>6.46</v>
+        <v>47.74</v>
       </c>
       <c r="G11" t="n">
-        <v>6.22</v>
+        <v>47.03</v>
       </c>
       <c r="H11" t="n">
-        <v>6.82</v>
+        <v>46.89</v>
       </c>
       <c r="I11" t="n">
-        <v>5.57</v>
+        <v>-1.78</v>
       </c>
       <c r="J11" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>6.13</v>
+        <v>45</v>
       </c>
       <c r="L11" t="n">
-        <v>6.25</v>
+        <v>47.65</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1170,23 +1187,25 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>1689563</v>
+        <v>250069</v>
       </c>
       <c r="P11" t="n">
-        <v>3.86</v>
+        <v>1.29</v>
       </c>
       <c r="Q11" t="n">
-        <v>6.37</v>
+        <v>47.65</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
-      <c r="S11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>47.88</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1198,31 +1217,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>46033.41666666666</v>
+        <v>46043.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>46035.41666666666</v>
+        <v>46075.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>7.06</v>
+        <v>48.35</v>
       </c>
       <c r="G12" t="n">
-        <v>7.03</v>
+        <v>46.1</v>
       </c>
       <c r="H12" t="n">
-        <v>6.7</v>
+        <v>48.39</v>
       </c>
       <c r="I12" t="n">
-        <v>-5.1</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="K12" t="n">
-        <v>6.41</v>
+        <v>46.5</v>
       </c>
       <c r="L12" t="n">
-        <v>7.04</v>
+        <v>48.24</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1235,23 +1254,25 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>1647282</v>
+        <v>1463983</v>
       </c>
       <c r="P12" t="n">
-        <v>0.43</v>
+        <v>3.11</v>
       </c>
       <c r="Q12" t="n">
-        <v>7.44</v>
+        <v>48.24</v>
       </c>
       <c r="R12" t="b">
-        <v>0</v>
-      </c>
-      <c r="S12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1263,31 +1284,31 @@
         <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>46055.41666666666</v>
+        <v>46079.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>46064.41666666666</v>
+        <v>46090.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>6.48</v>
+        <v>50.64</v>
       </c>
       <c r="G13" t="n">
-        <v>6.17</v>
+        <v>49.02</v>
       </c>
       <c r="H13" t="n">
-        <v>9.699999999999999</v>
+        <v>48.55</v>
       </c>
       <c r="I13" t="n">
-        <v>49.69</v>
+        <v>-4.13</v>
       </c>
       <c r="J13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K13" t="n">
-        <v>6.02</v>
+        <v>48.02</v>
       </c>
       <c r="L13" t="n">
-        <v>6.34</v>
+        <v>50.5</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1300,23 +1321,25 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>318660</v>
+        <v>1689183</v>
       </c>
       <c r="P13" t="n">
-        <v>3.85</v>
+        <v>2.51</v>
       </c>
       <c r="Q13" t="n">
-        <v>6.34</v>
+        <v>50.5</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
-      <c r="S13" t="inlineStr"/>
+      <c r="S13" t="n">
+        <v>53.5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1328,31 +1351,31 @@
         <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>46071.41666666666</v>
+        <v>46107.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>46072.41666666666</v>
+        <v>46126.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>9.85</v>
+        <v>49.38</v>
       </c>
       <c r="G14" t="n">
-        <v>9.42</v>
+        <v>46.91</v>
       </c>
       <c r="H14" t="n">
-        <v>9.26</v>
+        <v>54.9</v>
       </c>
       <c r="I14" t="n">
-        <v>-5.99</v>
+        <v>11.18</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="K14" t="n">
-        <v>9.41</v>
+        <v>45.51</v>
       </c>
       <c r="L14" t="n">
-        <v>9.800000000000001</v>
+        <v>47.88</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1365,83 +1388,20 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>4798270</v>
+        <v>3000298</v>
       </c>
       <c r="P14" t="n">
-        <v>4.56</v>
+        <v>5.27</v>
       </c>
       <c r="Q14" t="n">
-        <v>9.800000000000001</v>
+        <v>48.08</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
-      <c r="S14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>EPCO</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C15" t="b">
-        <v>0</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>46106.41666666666</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>46111.41666666666</v>
-      </c>
-      <c r="F15" t="n">
-        <v>9.02</v>
-      </c>
-      <c r="G15" t="n">
-        <v>8.390000000000001</v>
-      </c>
-      <c r="H15" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="I15" t="n">
-        <v>-7.87</v>
-      </c>
-      <c r="J15" t="n">
-        <v>5</v>
-      </c>
-      <c r="K15" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="L15" t="n">
-        <v>8.84</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O15" t="n">
-        <v>6893557</v>
-      </c>
-      <c r="P15" t="n">
-        <v>7.51</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>8.84</v>
-      </c>
-      <c r="R15" t="b">
-        <v>1</v>
-      </c>
-      <c r="S15" t="inlineStr"/>
+      <c r="S14" t="n">
+        <v>51</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1454,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1470,94 +1430,104 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>All_Time_High</t>
+          <t>total_trades</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Entry_Date</t>
+          <t>winners</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Exit_Date</t>
+          <t>losers</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Entry_Price</t>
+          <t>win_rate</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Entry_Low</t>
+          <t>median_pnl</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Exit_Price</t>
+          <t>avg_pnl</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Trade_PnL_%</t>
+          <t>total_pnl</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Days_Held</t>
+          <t>max_pnl</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Entry_Support</t>
+          <t>min_pnl</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Entry_Resistance</t>
+          <t>std_pnl</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Exit_Reason</t>
+          <t>profit_factor</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>avg_win</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Entry_Volume</t>
+          <t>avg_loss</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Today_%</t>
+          <t>expectancy</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Trendline_Price</t>
+          <t>risk_score</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Breaks_Trendline</t>
+          <t>return_score</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Current_Price</t>
+          <t>composite_score</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Best_Strategy</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>composite_score_best</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1565,60 +1535,64 @@
           <t>RANGE_BREAKOUT</t>
         </is>
       </c>
-      <c r="C2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>46127.41666666666</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>46128.41666666666</v>
+      <c r="C2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>8.74</v>
+        <v>61.54</v>
       </c>
       <c r="G2" t="n">
-        <v>8.539999999999999</v>
+        <v>0.08</v>
       </c>
       <c r="H2" t="n">
-        <v>9.140000000000001</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>4.58</v>
+        <v>119.79</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>60.22</v>
       </c>
       <c r="K2" t="n">
-        <v>8.31</v>
+        <v>-10.29</v>
       </c>
       <c r="L2" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
+        <v>18.47</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N2" t="n">
+        <v>17.74</v>
       </c>
       <c r="O2" t="n">
-        <v>1437309</v>
+        <v>4.43</v>
       </c>
       <c r="P2" t="n">
-        <v>2.1</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>8.960000000000001</v>
-      </c>
-      <c r="R2" t="b">
-        <v>0</v>
+        <v>0.6666902670775552</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.4982</v>
       </c>
       <c r="S2" t="n">
-        <v>9.140000000000001</v>
+        <v>0.565596106831022</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>0.565596106831022</v>
       </c>
     </row>
   </sheetData>
@@ -1632,7 +1606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1643,27 +1617,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>BUY_REASON</t>
+          <t>Best_Strategy</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>composite_score</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>total_trades</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>winners</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>losers</t>
+          <t>win_rate</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>win_rate</t>
+          <t>profit_factor</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1673,79 +1647,14 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>avg_pnl</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>total_pnl</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>max_pnl</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>min_pnl</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>std_pnl</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>profit_factor</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>avg_win</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>avg_loss</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
           <t>expectancy</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>risk_score</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>return_score</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>composite_score</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Best_Strategy</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>composite_score_best</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1754,63 +1663,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>0.57</v>
       </c>
       <c r="D2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E2" t="n">
+        <v>61.54</v>
+      </c>
+      <c r="F2" t="n">
         <v>5</v>
       </c>
-      <c r="E2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F2" t="n">
-        <v>35.71</v>
-      </c>
       <c r="G2" t="n">
-        <v>-3.01</v>
+        <v>0.08</v>
       </c>
       <c r="H2" t="n">
-        <v>3.48</v>
-      </c>
-      <c r="I2" t="n">
-        <v>48.73</v>
-      </c>
-      <c r="J2" t="n">
-        <v>49.69</v>
-      </c>
-      <c r="K2" t="n">
-        <v>-7.87</v>
-      </c>
-      <c r="L2" t="n">
-        <v>15.64</v>
-      </c>
-      <c r="M2" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="N2" t="n">
-        <v>18.41</v>
-      </c>
-      <c r="O2" t="n">
-        <v>4.81</v>
-      </c>
-      <c r="P2" t="n">
-        <v>3.48</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.4607990384615385</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.23579</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.3257936153846154</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="U2" t="n">
-        <v>0.3257936153846154</v>
+        <v>9.210000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1824,92 +1692,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Best_Strategy</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>composite_score</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>total_trades</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>win_rate</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>profit_factor</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>median_pnl</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>expectancy</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>EPCO</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D2" t="n">
-        <v>14</v>
-      </c>
-      <c r="E2" t="n">
-        <v>35.71</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-3.01</v>
-      </c>
-      <c r="H2" t="n">
-        <v>3.48</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:18:32.860562
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>15.96</v>
+        <v>17.47</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +663,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>20.6</v>
+        <v>20.79</v>
       </c>
     </row>
     <row r="4">
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.96</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>22.69</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>35.88</v>
+        <v>34.89</v>
       </c>
     </row>
     <row r="8">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>38.7</v>
+        <v>37.98</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>47.5</v>
+        <v>46.95</v>
       </c>
     </row>
     <row r="11">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>47.88</v>
+        <v>47.65</v>
       </c>
     </row>
     <row r="12">
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>49</v>
+        <v>48.24</v>
       </c>
     </row>
     <row r="13">
@@ -1333,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>53.5</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="14">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>51</v>
+        <v>47.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:25:04.095192
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>16.01</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +663,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>20.79</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="4">
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.74</v>
+        <v>23.96</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>21.7</v>
+        <v>22.69</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>34.89</v>
+        <v>35.88</v>
       </c>
     </row>
     <row r="8">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>37.98</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>46.95</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="11">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>47.65</v>
+        <v>47.88</v>
       </c>
     </row>
     <row r="12">
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>48.24</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
@@ -1333,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>50.5</v>
+        <v>53.5</v>
       </c>
     </row>
     <row r="14">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>47.88</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:28:16.919776
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>15.96</v>
+        <v>17.47</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +663,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>20.6</v>
+        <v>20.79</v>
       </c>
     </row>
     <row r="4">
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.96</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>22.69</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>35.88</v>
+        <v>34.89</v>
       </c>
     </row>
     <row r="8">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>38.7</v>
+        <v>37.98</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>47.5</v>
+        <v>46.95</v>
       </c>
     </row>
     <row r="11">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>47.88</v>
+        <v>47.65</v>
       </c>
     </row>
     <row r="12">
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>49</v>
+        <v>48.24</v>
       </c>
     </row>
     <row r="13">
@@ -1333,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>53.5</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="14">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>51</v>
+        <v>47.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:34:23.941387
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,34 +544,34 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45672.41666666666</v>
+        <v>45678.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>45686.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>15.54</v>
+        <v>17.95</v>
       </c>
       <c r="G2" t="n">
-        <v>14.29</v>
+        <v>16.6</v>
       </c>
       <c r="H2" t="n">
         <v>18.2</v>
       </c>
       <c r="I2" t="n">
-        <v>17.12</v>
+        <v>1.39</v>
       </c>
       <c r="J2" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="K2" t="n">
-        <v>14.02</v>
+        <v>16.9</v>
       </c>
       <c r="L2" t="n">
-        <v>14.8</v>
+        <v>17.47</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -584,19 +584,19 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>2912989</v>
+        <v>7215730</v>
       </c>
       <c r="P2" t="n">
-        <v>8.75</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>14.8</v>
+        <v>17.72</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>17.47</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="3">
@@ -635,10 +635,10 @@
         <v>35</v>
       </c>
       <c r="K3" t="n">
-        <v>18.07</v>
+        <v>18.26</v>
       </c>
       <c r="L3" t="n">
-        <v>19.07</v>
+        <v>19.93</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -657,13 +657,13 @@
         <v>10.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>19.07</v>
+        <v>23.37</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>20.79</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="4">
@@ -702,10 +702,10 @@
         <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>22.25</v>
+        <v>22.66</v>
       </c>
       <c r="L4" t="n">
-        <v>23.25</v>
+        <v>23.8</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -724,13 +724,13 @@
         <v>5.69</v>
       </c>
       <c r="Q4" t="n">
-        <v>24.23</v>
+        <v>25.8</v>
       </c>
       <c r="R4" t="b">
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.74</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="5">
@@ -745,59 +745,59 @@
         </is>
       </c>
       <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>45775.41666666666</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>45839.41666666666</v>
+      </c>
+      <c r="F5" t="n">
+        <v>24</v>
+      </c>
+      <c r="G5" t="n">
+        <v>23</v>
+      </c>
+      <c r="H5" t="n">
+        <v>36.21</v>
+      </c>
+      <c r="I5" t="n">
+        <v>50.88</v>
+      </c>
+      <c r="J5" t="n">
+        <v>64</v>
+      </c>
+      <c r="K5" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="L5" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>552715</v>
+      </c>
+      <c r="P5" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>44.68</v>
+      </c>
+      <c r="R5" t="b">
         <v>0</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>45735.41666666666</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>45753.41666666666</v>
-      </c>
-      <c r="F5" t="n">
-        <v>23.41</v>
-      </c>
-      <c r="G5" t="n">
-        <v>22.02</v>
-      </c>
-      <c r="H5" t="n">
-        <v>21</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-10.29</v>
-      </c>
-      <c r="J5" t="n">
-        <v>18</v>
-      </c>
-      <c r="K5" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="L5" t="n">
-        <v>22.99</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>448788</v>
-      </c>
-      <c r="P5" t="n">
-        <v>5.07</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>22.99</v>
-      </c>
-      <c r="R5" t="b">
-        <v>1</v>
-      </c>
       <c r="S5" t="n">
-        <v>23.47</v>
+        <v>23.96</v>
       </c>
     </row>
     <row r="6">
@@ -812,59 +812,59 @@
         </is>
       </c>
       <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>45869.41666666666</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>45890.41666666666</v>
+      </c>
+      <c r="F6" t="n">
+        <v>39.03</v>
+      </c>
+      <c r="G6" t="n">
+        <v>38</v>
+      </c>
+      <c r="H6" t="n">
+        <v>41.93</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="J6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K6" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="L6" t="n">
+        <v>38</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>1089647</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="R6" t="b">
         <v>0</v>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>45761.41666666666</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>45839.41666666666</v>
-      </c>
-      <c r="F6" t="n">
-        <v>22.6</v>
-      </c>
-      <c r="G6" t="n">
-        <v>21.57</v>
-      </c>
-      <c r="H6" t="n">
-        <v>36.21</v>
-      </c>
-      <c r="I6" t="n">
-        <v>60.22</v>
-      </c>
-      <c r="J6" t="n">
-        <v>78</v>
-      </c>
-      <c r="K6" t="n">
-        <v>19.56</v>
-      </c>
-      <c r="L6" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O6" t="n">
-        <v>581928</v>
-      </c>
-      <c r="P6" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="R6" t="b">
-        <v>1</v>
-      </c>
       <c r="S6" t="n">
-        <v>21.7</v>
+        <v>39.24</v>
       </c>
     </row>
     <row r="7">
@@ -879,34 +879,34 @@
         </is>
       </c>
       <c r="C7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45943.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45890.41666666666</v>
+        <v>45944.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>35.51</v>
+        <v>49.23</v>
       </c>
       <c r="G7" t="n">
-        <v>33.5</v>
+        <v>47.7</v>
       </c>
       <c r="H7" t="n">
-        <v>41.93</v>
+        <v>47.44</v>
       </c>
       <c r="I7" t="n">
-        <v>18.08</v>
+        <v>-3.64</v>
       </c>
       <c r="J7" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>32.66</v>
+        <v>42.8</v>
       </c>
       <c r="L7" t="n">
-        <v>34.89</v>
+        <v>48.89</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -919,19 +919,19 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>2216102</v>
+        <v>3928197</v>
       </c>
       <c r="P7" t="n">
-        <v>6</v>
+        <v>3.21</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.89</v>
+        <v>48.89</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>34.89</v>
+        <v>48.89</v>
       </c>
     </row>
     <row r="8">
@@ -946,34 +946,34 @@
         </is>
       </c>
       <c r="C8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45914.41666666666</v>
+        <v>45973.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45916.41666666666</v>
+        <v>46035.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>39</v>
+        <v>55.02</v>
       </c>
       <c r="G8" t="n">
-        <v>38.51</v>
+        <v>48.5</v>
       </c>
       <c r="H8" t="n">
-        <v>38.9</v>
+        <v>47.53</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.26</v>
+        <v>-13.61</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="K8" t="n">
-        <v>36.5</v>
+        <v>47.7</v>
       </c>
       <c r="L8" t="n">
-        <v>38.64</v>
+        <v>54.95</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -986,421 +986,19 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>212755</v>
+        <v>3596313</v>
       </c>
       <c r="P8" t="n">
-        <v>0.96</v>
+        <v>13.44</v>
       </c>
       <c r="Q8" t="n">
-        <v>40.79</v>
+        <v>54.95</v>
       </c>
       <c r="R8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>39.4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C9" t="b">
-        <v>0</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>45925.41666666666</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>45944.41666666666</v>
-      </c>
-      <c r="F9" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="G9" t="n">
-        <v>36.85</v>
-      </c>
-      <c r="H9" t="n">
-        <v>47.44</v>
-      </c>
-      <c r="I9" t="n">
-        <v>22.58</v>
-      </c>
-      <c r="J9" t="n">
-        <v>19</v>
-      </c>
-      <c r="K9" t="n">
-        <v>35.01</v>
-      </c>
-      <c r="L9" t="n">
-        <v>37.98</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O9" t="n">
-        <v>300539</v>
-      </c>
-      <c r="P9" t="n">
-        <v>5.02</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>37.98</v>
-      </c>
-      <c r="R9" t="b">
-        <v>1</v>
-      </c>
-      <c r="S9" t="n">
-        <v>37.98</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C10" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>45970.41666666666</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>46035.41666666666</v>
-      </c>
-      <c r="F10" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="G10" t="n">
-        <v>45.28</v>
-      </c>
-      <c r="H10" t="n">
-        <v>47.53</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="J10" t="n">
-        <v>65</v>
-      </c>
-      <c r="K10" t="n">
-        <v>44.75</v>
-      </c>
-      <c r="L10" t="n">
-        <v>46.95</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O10" t="n">
-        <v>403885</v>
-      </c>
-      <c r="P10" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>48.07</v>
-      </c>
-      <c r="R10" t="b">
-        <v>0</v>
-      </c>
-      <c r="S10" t="n">
-        <v>46.95</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C11" t="b">
-        <v>0</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>46041.41666666666</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>46042.41666666666</v>
-      </c>
-      <c r="F11" t="n">
-        <v>47.74</v>
-      </c>
-      <c r="G11" t="n">
-        <v>47.03</v>
-      </c>
-      <c r="H11" t="n">
-        <v>46.89</v>
-      </c>
-      <c r="I11" t="n">
-        <v>-1.78</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>45</v>
-      </c>
-      <c r="L11" t="n">
-        <v>47.65</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O11" t="n">
-        <v>250069</v>
-      </c>
-      <c r="P11" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>47.65</v>
-      </c>
-      <c r="R11" t="b">
-        <v>1</v>
-      </c>
-      <c r="S11" t="n">
-        <v>47.65</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C12" t="b">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>46043.41666666666</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>46075.41666666666</v>
-      </c>
-      <c r="F12" t="n">
-        <v>48.35</v>
-      </c>
-      <c r="G12" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="H12" t="n">
-        <v>48.39</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="J12" t="n">
-        <v>32</v>
-      </c>
-      <c r="K12" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="L12" t="n">
-        <v>48.24</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O12" t="n">
-        <v>1463983</v>
-      </c>
-      <c r="P12" t="n">
-        <v>3.11</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>48.24</v>
-      </c>
-      <c r="R12" t="b">
-        <v>1</v>
-      </c>
-      <c r="S12" t="n">
-        <v>48.24</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C13" t="b">
-        <v>0</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>46079.41666666666</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>46090.41666666666</v>
-      </c>
-      <c r="F13" t="n">
-        <v>50.64</v>
-      </c>
-      <c r="G13" t="n">
-        <v>49.02</v>
-      </c>
-      <c r="H13" t="n">
-        <v>48.55</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-4.13</v>
-      </c>
-      <c r="J13" t="n">
-        <v>11</v>
-      </c>
-      <c r="K13" t="n">
-        <v>48.02</v>
-      </c>
-      <c r="L13" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O13" t="n">
-        <v>1689183</v>
-      </c>
-      <c r="P13" t="n">
-        <v>2.51</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="R13" t="b">
-        <v>1</v>
-      </c>
-      <c r="S13" t="n">
-        <v>50.5</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>ARCC</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>46107.41666666666</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>46126.41666666666</v>
-      </c>
-      <c r="F14" t="n">
-        <v>49.38</v>
-      </c>
-      <c r="G14" t="n">
-        <v>46.91</v>
-      </c>
-      <c r="H14" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="I14" t="n">
-        <v>11.18</v>
-      </c>
-      <c r="J14" t="n">
-        <v>19</v>
-      </c>
-      <c r="K14" t="n">
-        <v>45.51</v>
-      </c>
-      <c r="L14" t="n">
-        <v>47.88</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O14" t="n">
-        <v>3000298</v>
-      </c>
-      <c r="P14" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>48.08</v>
-      </c>
-      <c r="R14" t="b">
-        <v>1</v>
-      </c>
-      <c r="S14" t="n">
-        <v>47.88</v>
+        <v>54.95</v>
       </c>
     </row>
   </sheetData>
@@ -1536,55 +1134,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>61.54</v>
+        <v>57.14</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08</v>
+        <v>1.39</v>
       </c>
       <c r="H2" t="n">
-        <v>9.210000000000001</v>
+        <v>7.05</v>
       </c>
       <c r="I2" t="n">
-        <v>119.79</v>
+        <v>49.38</v>
       </c>
       <c r="J2" t="n">
-        <v>60.22</v>
+        <v>50.88</v>
       </c>
       <c r="K2" t="n">
-        <v>-10.29</v>
+        <v>-13.61</v>
       </c>
       <c r="L2" t="n">
-        <v>18.47</v>
+        <v>21.16</v>
       </c>
       <c r="M2" t="n">
-        <v>5</v>
+        <v>3.15</v>
       </c>
       <c r="N2" t="n">
-        <v>17.74</v>
+        <v>18.08</v>
       </c>
       <c r="O2" t="n">
-        <v>4.43</v>
+        <v>7.64</v>
       </c>
       <c r="P2" t="n">
-        <v>9.210000000000001</v>
+        <v>7.05</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6666902670775552</v>
+        <v>0.5616315884476535</v>
       </c>
       <c r="R2" t="n">
-        <v>0.4982</v>
+        <v>0.30874</v>
       </c>
       <c r="S2" t="n">
-        <v>0.565596106831022</v>
+        <v>0.4098966353790614</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -1592,7 +1190,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.565596106831022</v>
+        <v>0.4098966353790614</v>
       </c>
     </row>
   </sheetData>
@@ -1663,22 +1261,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.57</v>
+        <v>0.41</v>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>61.54</v>
+        <v>57.14</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>3.15</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08</v>
+        <v>1.39</v>
       </c>
       <c r="H2" t="n">
-        <v>9.210000000000001</v>
+        <v>7.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:35:32.383536
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,34 +544,34 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45678.41666666666</v>
+        <v>45672.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>45686.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>17.95</v>
+        <v>15.54</v>
       </c>
       <c r="G2" t="n">
-        <v>16.6</v>
+        <v>14.29</v>
       </c>
       <c r="H2" t="n">
         <v>18.2</v>
       </c>
       <c r="I2" t="n">
-        <v>1.39</v>
+        <v>17.12</v>
       </c>
       <c r="J2" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="K2" t="n">
-        <v>16.9</v>
+        <v>14.02</v>
       </c>
       <c r="L2" t="n">
-        <v>17.47</v>
+        <v>14.8</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -584,19 +584,19 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>7215730</v>
+        <v>2912989</v>
       </c>
       <c r="P2" t="n">
-        <v>8.130000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="Q2" t="n">
-        <v>17.72</v>
+        <v>14.8</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>17.7</v>
+        <v>17.47</v>
       </c>
     </row>
     <row r="3">
@@ -635,10 +635,10 @@
         <v>35</v>
       </c>
       <c r="K3" t="n">
-        <v>18.26</v>
+        <v>18.07</v>
       </c>
       <c r="L3" t="n">
-        <v>19.93</v>
+        <v>19.07</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -657,13 +657,13 @@
         <v>10.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>23.37</v>
+        <v>19.07</v>
       </c>
       <c r="R3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>19.93</v>
+        <v>20.79</v>
       </c>
     </row>
     <row r="4">
@@ -702,10 +702,10 @@
         <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>22.66</v>
+        <v>22.25</v>
       </c>
       <c r="L4" t="n">
-        <v>23.8</v>
+        <v>23.25</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -724,13 +724,13 @@
         <v>5.69</v>
       </c>
       <c r="Q4" t="n">
-        <v>25.8</v>
+        <v>24.23</v>
       </c>
       <c r="R4" t="b">
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.8</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="5">
@@ -745,59 +745,59 @@
         </is>
       </c>
       <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>45735.41666666666</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>45753.41666666666</v>
+      </c>
+      <c r="F5" t="n">
+        <v>23.41</v>
+      </c>
+      <c r="G5" t="n">
+        <v>22.02</v>
+      </c>
+      <c r="H5" t="n">
+        <v>21</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-10.29</v>
+      </c>
+      <c r="J5" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="L5" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>448788</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="R5" t="b">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>45775.41666666666</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>45839.41666666666</v>
-      </c>
-      <c r="F5" t="n">
-        <v>24</v>
-      </c>
-      <c r="G5" t="n">
-        <v>23</v>
-      </c>
-      <c r="H5" t="n">
-        <v>36.21</v>
-      </c>
-      <c r="I5" t="n">
-        <v>50.88</v>
-      </c>
-      <c r="J5" t="n">
-        <v>64</v>
-      </c>
-      <c r="K5" t="n">
-        <v>22.67</v>
-      </c>
-      <c r="L5" t="n">
-        <v>23.96</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>552715</v>
-      </c>
-      <c r="P5" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>44.68</v>
-      </c>
-      <c r="R5" t="b">
-        <v>0</v>
-      </c>
       <c r="S5" t="n">
-        <v>23.96</v>
+        <v>23.47</v>
       </c>
     </row>
     <row r="6">
@@ -812,59 +812,59 @@
         </is>
       </c>
       <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>45761.41666666666</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>45839.41666666666</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="H6" t="n">
+        <v>36.21</v>
+      </c>
+      <c r="I6" t="n">
+        <v>60.22</v>
+      </c>
+      <c r="J6" t="n">
+        <v>78</v>
+      </c>
+      <c r="K6" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="L6" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>581928</v>
+      </c>
+      <c r="P6" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="R6" t="b">
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>45869.41666666666</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>45890.41666666666</v>
-      </c>
-      <c r="F6" t="n">
-        <v>39.03</v>
-      </c>
-      <c r="G6" t="n">
-        <v>38</v>
-      </c>
-      <c r="H6" t="n">
-        <v>41.93</v>
-      </c>
-      <c r="I6" t="n">
-        <v>7.43</v>
-      </c>
-      <c r="J6" t="n">
-        <v>21</v>
-      </c>
-      <c r="K6" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="L6" t="n">
-        <v>38</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O6" t="n">
-        <v>1089647</v>
-      </c>
-      <c r="P6" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="R6" t="b">
-        <v>0</v>
-      </c>
       <c r="S6" t="n">
-        <v>39.24</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="7">
@@ -879,34 +879,34 @@
         </is>
       </c>
       <c r="C7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45943.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45944.41666666666</v>
+        <v>45890.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>49.23</v>
+        <v>35.51</v>
       </c>
       <c r="G7" t="n">
-        <v>47.7</v>
+        <v>33.5</v>
       </c>
       <c r="H7" t="n">
-        <v>47.44</v>
+        <v>41.93</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.64</v>
+        <v>18.08</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="K7" t="n">
-        <v>42.8</v>
+        <v>32.66</v>
       </c>
       <c r="L7" t="n">
-        <v>48.89</v>
+        <v>34.89</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -919,19 +919,19 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>3928197</v>
+        <v>2216102</v>
       </c>
       <c r="P7" t="n">
-        <v>3.21</v>
+        <v>6</v>
       </c>
       <c r="Q7" t="n">
-        <v>48.89</v>
+        <v>34.89</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>48.89</v>
+        <v>34.89</v>
       </c>
     </row>
     <row r="8">
@@ -946,59 +946,461 @@
         </is>
       </c>
       <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>45914.41666666666</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>45916.41666666666</v>
+      </c>
+      <c r="F8" t="n">
+        <v>39</v>
+      </c>
+      <c r="G8" t="n">
+        <v>38.51</v>
+      </c>
+      <c r="H8" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="L8" t="n">
+        <v>38.64</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>212755</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>40.79</v>
+      </c>
+      <c r="R8" t="b">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>39.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>45925.41666666666</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>45944.41666666666</v>
+      </c>
+      <c r="F9" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G9" t="n">
+        <v>36.85</v>
+      </c>
+      <c r="H9" t="n">
+        <v>47.44</v>
+      </c>
+      <c r="I9" t="n">
+        <v>22.58</v>
+      </c>
+      <c r="J9" t="n">
+        <v>19</v>
+      </c>
+      <c r="K9" t="n">
+        <v>35.01</v>
+      </c>
+      <c r="L9" t="n">
+        <v>37.98</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>300539</v>
+      </c>
+      <c r="P9" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>37.98</v>
+      </c>
+      <c r="R9" t="b">
         <v>1</v>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>45973.41666666666</v>
-      </c>
-      <c r="E8" s="2" t="n">
+      <c r="S9" t="n">
+        <v>37.98</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>45970.41666666666</v>
+      </c>
+      <c r="E10" s="2" t="n">
         <v>46035.41666666666</v>
       </c>
-      <c r="F8" t="n">
-        <v>55.02</v>
-      </c>
-      <c r="G8" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="H8" t="n">
+      <c r="F10" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>45.28</v>
+      </c>
+      <c r="H10" t="n">
         <v>47.53</v>
       </c>
-      <c r="I8" t="n">
-        <v>-13.61</v>
-      </c>
-      <c r="J8" t="n">
-        <v>62</v>
-      </c>
-      <c r="K8" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="L8" t="n">
-        <v>54.95</v>
-      </c>
-      <c r="M8" t="inlineStr">
+      <c r="I10" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J10" t="n">
+        <v>65</v>
+      </c>
+      <c r="K10" t="n">
+        <v>44.75</v>
+      </c>
+      <c r="L10" t="n">
+        <v>46.95</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>RANGE_BREAKDOWN</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="O8" t="n">
-        <v>3596313</v>
-      </c>
-      <c r="P8" t="n">
-        <v>13.44</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>54.95</v>
-      </c>
-      <c r="R8" t="b">
+      <c r="O10" t="n">
+        <v>403885</v>
+      </c>
+      <c r="P10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>48.07</v>
+      </c>
+      <c r="R10" t="b">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>46.95</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>46041.41666666666</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>46042.41666666666</v>
+      </c>
+      <c r="F11" t="n">
+        <v>47.74</v>
+      </c>
+      <c r="G11" t="n">
+        <v>47.03</v>
+      </c>
+      <c r="H11" t="n">
+        <v>46.89</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="S8" t="n">
-        <v>54.95</v>
+      <c r="K11" t="n">
+        <v>45</v>
+      </c>
+      <c r="L11" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>250069</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="R11" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" t="n">
+        <v>47.65</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>46043.41666666666</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>46075.41666666666</v>
+      </c>
+      <c r="F12" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="G12" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>48.39</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J12" t="n">
+        <v>32</v>
+      </c>
+      <c r="K12" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="L12" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>1463983</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="R12" t="b">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>48.24</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>46079.41666666666</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>46090.41666666666</v>
+      </c>
+      <c r="F13" t="n">
+        <v>50.64</v>
+      </c>
+      <c r="G13" t="n">
+        <v>49.02</v>
+      </c>
+      <c r="H13" t="n">
+        <v>48.55</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-4.13</v>
+      </c>
+      <c r="J13" t="n">
+        <v>11</v>
+      </c>
+      <c r="K13" t="n">
+        <v>48.02</v>
+      </c>
+      <c r="L13" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>1689183</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="R13" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>50.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>46107.41666666666</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>46126.41666666666</v>
+      </c>
+      <c r="F14" t="n">
+        <v>49.38</v>
+      </c>
+      <c r="G14" t="n">
+        <v>46.91</v>
+      </c>
+      <c r="H14" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="I14" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="J14" t="n">
+        <v>19</v>
+      </c>
+      <c r="K14" t="n">
+        <v>45.51</v>
+      </c>
+      <c r="L14" t="n">
+        <v>47.88</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>3000298</v>
+      </c>
+      <c r="P14" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>48.08</v>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>47.88</v>
       </c>
     </row>
   </sheetData>
@@ -1134,55 +1536,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>57.14</v>
+        <v>61.54</v>
       </c>
       <c r="G2" t="n">
-        <v>1.39</v>
+        <v>0.08</v>
       </c>
       <c r="H2" t="n">
-        <v>7.05</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>49.38</v>
+        <v>119.79</v>
       </c>
       <c r="J2" t="n">
-        <v>50.88</v>
+        <v>60.22</v>
       </c>
       <c r="K2" t="n">
-        <v>-13.61</v>
+        <v>-10.29</v>
       </c>
       <c r="L2" t="n">
-        <v>21.16</v>
+        <v>18.47</v>
       </c>
       <c r="M2" t="n">
-        <v>3.15</v>
+        <v>5</v>
       </c>
       <c r="N2" t="n">
-        <v>18.08</v>
+        <v>17.74</v>
       </c>
       <c r="O2" t="n">
-        <v>7.64</v>
+        <v>4.43</v>
       </c>
       <c r="P2" t="n">
-        <v>7.05</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.5616315884476535</v>
+        <v>0.6666902670775552</v>
       </c>
       <c r="R2" t="n">
-        <v>0.30874</v>
+        <v>0.4982</v>
       </c>
       <c r="S2" t="n">
-        <v>0.4098966353790614</v>
+        <v>0.565596106831022</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -1190,7 +1592,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.4098966353790614</v>
+        <v>0.565596106831022</v>
       </c>
     </row>
   </sheetData>
@@ -1261,22 +1663,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.41</v>
+        <v>0.57</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>57.14</v>
+        <v>61.54</v>
       </c>
       <c r="F2" t="n">
-        <v>3.15</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>1.39</v>
+        <v>0.08</v>
       </c>
       <c r="H2" t="n">
-        <v>7.05</v>
+        <v>9.210000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:38:20.069788
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.74</v>
+        <v>23.79</v>
       </c>
     </row>
     <row r="5">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>34.89</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -998,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>39.4</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="9">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>37.98</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>46.95</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="11">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>47.88</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:39:18.508074
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>17.47</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +663,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>20.79</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="4">
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.79</v>
+        <v>23.96</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>21.7</v>
+        <v>22.69</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>36</v>
+        <v>35.88</v>
       </c>
     </row>
     <row r="8">
@@ -998,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>39.5</v>
+        <v>39.12</v>
       </c>
     </row>
     <row r="9">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>38.5</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>47.4</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="11">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>47.65</v>
+        <v>47.88</v>
       </c>
     </row>
     <row r="12">
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>48.24</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
@@ -1333,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>50.5</v>
+        <v>53.5</v>
       </c>
     </row>
     <row r="14">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:43:58.125134
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>15.96</v>
+        <v>17.47</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +663,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>20.6</v>
+        <v>19.07</v>
       </c>
     </row>
     <row r="4">
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.96</v>
+        <v>23.25</v>
       </c>
     </row>
     <row r="5">
@@ -797,7 +797,7 @@
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>23.47</v>
+        <v>22.99</v>
       </c>
     </row>
     <row r="6">
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>22.69</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>35.88</v>
+        <v>34.89</v>
       </c>
     </row>
     <row r="8">
@@ -998,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>39.12</v>
+        <v>38.64</v>
       </c>
     </row>
     <row r="9">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>38.7</v>
+        <v>37.98</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>47.5</v>
+        <v>46.95</v>
       </c>
     </row>
     <row r="11">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>47.88</v>
+        <v>47.65</v>
       </c>
     </row>
     <row r="12">
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>49</v>
+        <v>48.24</v>
       </c>
     </row>
     <row r="13">
@@ -1333,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>53.5</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="14">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>51</v>
+        <v>47.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:50:37.693543
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>17.3</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +663,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>19.07</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="4">
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.25</v>
+        <v>23.96</v>
       </c>
     </row>
     <row r="5">
@@ -797,7 +797,7 @@
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>22.99</v>
+        <v>23.47</v>
       </c>
     </row>
     <row r="6">
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>21.7</v>
+        <v>22.69</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>34.89</v>
+        <v>35.88</v>
       </c>
     </row>
     <row r="8">
@@ -998,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>38.64</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="9">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>37.98</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>46.95</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="11">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>47.65</v>
+        <v>47.88</v>
       </c>
     </row>
     <row r="12">
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>48.24</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
@@ -1333,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>50.5</v>
+        <v>53.5</v>
       </c>
     </row>
     <row r="14">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>47.88</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:52:54.495919
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>15.96</v>
+        <v>17.47</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +663,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>20.6</v>
+        <v>20.79</v>
       </c>
     </row>
     <row r="4">
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>23.96</v>
+        <v>23.79</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>22.69</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>35.88</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -998,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>39.4</v>
+        <v>41.6</v>
       </c>
     </row>
     <row r="9">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>38.7</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="10">
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>47.5</v>
+        <v>47.89</v>
       </c>
     </row>
     <row r="11">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>47.88</v>
+        <v>51.19</v>
       </c>
     </row>
     <row r="12">
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>49</v>
+        <v>48.24</v>
       </c>
     </row>
     <row r="13">
@@ -1333,7 +1333,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>53.5</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="14">
@@ -1400,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>51</v>
+        <v>49.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 14:58:22.229146
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -590,10 +590,10 @@
         <v>8.75</v>
       </c>
       <c r="Q2" t="n">
-        <v>14.8</v>
+        <v>17.47</v>
       </c>
       <c r="R2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
         <v>17.47</v>
@@ -657,10 +657,10 @@
         <v>10.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>19.07</v>
+        <v>20.79</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
         <v>20.79</v>
@@ -724,10 +724,10 @@
         <v>5.69</v>
       </c>
       <c r="Q4" t="n">
-        <v>24.23</v>
+        <v>23.79</v>
       </c>
       <c r="R4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S4" t="n">
         <v>23.79</v>
@@ -791,10 +791,10 @@
         <v>5.07</v>
       </c>
       <c r="Q5" t="n">
-        <v>22.99</v>
+        <v>23.47</v>
       </c>
       <c r="R5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
         <v>23.47</v>
@@ -925,10 +925,10 @@
         <v>6</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.89</v>
+        <v>36</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
         <v>36</v>
@@ -992,7 +992,7 @@
         <v>0.96</v>
       </c>
       <c r="Q8" t="n">
-        <v>40.79</v>
+        <v>41.6</v>
       </c>
       <c r="R8" t="b">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>5.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.98</v>
+        <v>38.5</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
@@ -1126,7 +1126,7 @@
         <v>4.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>48.07</v>
+        <v>47.89</v>
       </c>
       <c r="R10" t="b">
         <v>0</v>
@@ -1193,10 +1193,10 @@
         <v>1.29</v>
       </c>
       <c r="Q11" t="n">
-        <v>47.65</v>
+        <v>51.19</v>
       </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>51.19</v>
@@ -1327,10 +1327,10 @@
         <v>2.51</v>
       </c>
       <c r="Q13" t="n">
-        <v>50.5</v>
+        <v>52.5</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>52.5</v>
@@ -1394,10 +1394,10 @@
         <v>5.27</v>
       </c>
       <c r="Q14" t="n">
-        <v>48.08</v>
+        <v>49.91</v>
       </c>
       <c r="R14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
         <v>49.91</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 15:01:31.205677
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -590,10 +590,10 @@
         <v>8.75</v>
       </c>
       <c r="Q2" t="n">
-        <v>17.47</v>
+        <v>14.36</v>
       </c>
       <c r="R2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2" t="n">
         <v>17.47</v>
@@ -657,10 +657,10 @@
         <v>10.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>20.79</v>
+        <v>18.21</v>
       </c>
       <c r="R3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>20.79</v>
@@ -791,10 +791,10 @@
         <v>5.07</v>
       </c>
       <c r="Q5" t="n">
-        <v>23.47</v>
+        <v>22.75</v>
       </c>
       <c r="R5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
         <v>23.47</v>
@@ -925,10 +925,10 @@
         <v>6</v>
       </c>
       <c r="Q7" t="n">
-        <v>36</v>
+        <v>34.34</v>
       </c>
       <c r="R7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
         <v>36</v>
@@ -992,7 +992,7 @@
         <v>0.96</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.6</v>
+        <v>39.16</v>
       </c>
       <c r="R8" t="b">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>5.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.5</v>
+        <v>36.84</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
@@ -1126,10 +1126,10 @@
         <v>4.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>47.89</v>
+        <v>47.03</v>
       </c>
       <c r="R10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="n">
         <v>47.89</v>
@@ -1193,10 +1193,10 @@
         <v>1.29</v>
       </c>
       <c r="Q11" t="n">
-        <v>51.19</v>
+        <v>46.8</v>
       </c>
       <c r="R11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="n">
         <v>51.19</v>
@@ -1327,10 +1327,10 @@
         <v>2.51</v>
       </c>
       <c r="Q13" t="n">
-        <v>52.5</v>
+        <v>49.88</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="n">
         <v>52.5</v>
@@ -1394,10 +1394,10 @@
         <v>5.27</v>
       </c>
       <c r="Q14" t="n">
-        <v>49.91</v>
+        <v>47.36</v>
       </c>
       <c r="R14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="n">
         <v>49.91</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 15:05:40.027767
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -590,10 +590,10 @@
         <v>8.75</v>
       </c>
       <c r="Q2" t="n">
-        <v>14.36</v>
+        <v>17.47</v>
       </c>
       <c r="R2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
         <v>17.47</v>
@@ -657,10 +657,10 @@
         <v>10.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>18.21</v>
+        <v>20.79</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
         <v>20.79</v>
@@ -791,10 +791,10 @@
         <v>5.07</v>
       </c>
       <c r="Q5" t="n">
-        <v>22.75</v>
+        <v>23.47</v>
       </c>
       <c r="R5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
         <v>23.47</v>
@@ -925,10 +925,10 @@
         <v>6</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.34</v>
+        <v>36</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
         <v>36</v>
@@ -992,7 +992,7 @@
         <v>0.96</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.16</v>
+        <v>41.6</v>
       </c>
       <c r="R8" t="b">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>5.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>36.84</v>
+        <v>38.5</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
@@ -1126,10 +1126,10 @@
         <v>4.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>47.03</v>
+        <v>47.89</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
         <v>47.89</v>
@@ -1193,10 +1193,10 @@
         <v>1.29</v>
       </c>
       <c r="Q11" t="n">
-        <v>46.8</v>
+        <v>51.19</v>
       </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>51.19</v>
@@ -1327,10 +1327,10 @@
         <v>2.51</v>
       </c>
       <c r="Q13" t="n">
-        <v>49.88</v>
+        <v>52.5</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>52.5</v>
@@ -1394,10 +1394,10 @@
         <v>5.27</v>
       </c>
       <c r="Q14" t="n">
-        <v>47.36</v>
+        <v>49.91</v>
       </c>
       <c r="R14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
         <v>49.91</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 15:06:30.903368
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -590,7 +590,7 @@
         <v>8.75</v>
       </c>
       <c r="Q2" t="n">
-        <v>17.47</v>
+        <v>16.98</v>
       </c>
       <c r="R2" t="b">
         <v>0</v>
@@ -657,10 +657,10 @@
         <v>10.27</v>
       </c>
       <c r="Q3" t="n">
-        <v>20.79</v>
+        <v>18.21</v>
       </c>
       <c r="R3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>20.79</v>
@@ -791,10 +791,10 @@
         <v>5.07</v>
       </c>
       <c r="Q5" t="n">
-        <v>23.47</v>
+        <v>22.96</v>
       </c>
       <c r="R5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
         <v>23.47</v>
@@ -925,10 +925,10 @@
         <v>6</v>
       </c>
       <c r="Q7" t="n">
-        <v>36</v>
+        <v>34.34</v>
       </c>
       <c r="R7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
         <v>36</v>
@@ -992,7 +992,7 @@
         <v>0.96</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.6</v>
+        <v>39.16</v>
       </c>
       <c r="R8" t="b">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>5.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.5</v>
+        <v>36.94</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
@@ -1126,10 +1126,10 @@
         <v>4.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>47.89</v>
+        <v>47.03</v>
       </c>
       <c r="R10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="n">
         <v>47.89</v>
@@ -1193,7 +1193,7 @@
         <v>1.29</v>
       </c>
       <c r="Q11" t="n">
-        <v>51.19</v>
+        <v>47.81</v>
       </c>
       <c r="R11" t="b">
         <v>0</v>
@@ -1327,7 +1327,7 @@
         <v>2.51</v>
       </c>
       <c r="Q13" t="n">
-        <v>52.5</v>
+        <v>51.45</v>
       </c>
       <c r="R13" t="b">
         <v>0</v>
@@ -1394,10 +1394,10 @@
         <v>5.27</v>
       </c>
       <c r="Q14" t="n">
-        <v>49.91</v>
+        <v>47.36</v>
       </c>
       <c r="R14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="n">
         <v>49.91</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 15:15:12.477278
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:T14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,6 +531,11 @@
           <t>Anchor_High</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Buffer_Gain</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -598,6 +603,9 @@
       <c r="S2" t="n">
         <v>17.47</v>
       </c>
+      <c r="T2" t="n">
+        <v>12.42</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -665,6 +673,9 @@
       <c r="S3" t="n">
         <v>20.79</v>
       </c>
+      <c r="T3" t="n">
+        <v>3.59</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -732,6 +743,9 @@
       <c r="S4" t="n">
         <v>23.79</v>
       </c>
+      <c r="T4" t="n">
+        <v>-0.71</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -799,6 +813,9 @@
       <c r="S5" t="n">
         <v>23.47</v>
       </c>
+      <c r="T5" t="n">
+        <v>0.26</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -866,6 +883,9 @@
       <c r="S6" t="n">
         <v>21.7</v>
       </c>
+      <c r="T6" t="n">
+        <v>-3.98</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -933,6 +953,9 @@
       <c r="S7" t="n">
         <v>36</v>
       </c>
+      <c r="T7" t="n">
+        <v>1.38</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1000,6 +1023,9 @@
       <c r="S8" t="n">
         <v>41.6</v>
       </c>
+      <c r="T8" t="n">
+        <v>6.67</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1067,6 +1093,9 @@
       <c r="S9" t="n">
         <v>38.5</v>
       </c>
+      <c r="T9" t="n">
+        <v>-0.52</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1134,6 +1163,9 @@
       <c r="S10" t="n">
         <v>47.89</v>
       </c>
+      <c r="T10" t="n">
+        <v>0.82</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1201,6 +1233,9 @@
       <c r="S11" t="n">
         <v>51.19</v>
       </c>
+      <c r="T11" t="n">
+        <v>7.23</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1268,6 +1303,9 @@
       <c r="S12" t="n">
         <v>48.24</v>
       </c>
+      <c r="T12" t="n">
+        <v>-0.23</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1335,6 +1373,9 @@
       <c r="S13" t="n">
         <v>52.5</v>
       </c>
+      <c r="T13" t="n">
+        <v>3.67</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1401,6 +1442,9 @@
       </c>
       <c r="S14" t="n">
         <v>49.91</v>
+      </c>
+      <c r="T14" t="n">
+        <v>1.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 15:19:33.376317
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T14"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,6 +533,11 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>Testing_Anchor</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Buffer_Gain</t>
         </is>
       </c>
@@ -603,7 +608,10 @@
       <c r="S2" t="n">
         <v>17.47</v>
       </c>
-      <c r="T2" t="n">
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
         <v>12.42</v>
       </c>
     </row>
@@ -673,7 +681,10 @@
       <c r="S3" t="n">
         <v>20.79</v>
       </c>
-      <c r="T3" t="n">
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
         <v>3.59</v>
       </c>
     </row>
@@ -743,7 +754,10 @@
       <c r="S4" t="n">
         <v>23.79</v>
       </c>
-      <c r="T4" t="n">
+      <c r="T4" t="b">
+        <v>1</v>
+      </c>
+      <c r="U4" t="n">
         <v>-0.71</v>
       </c>
     </row>
@@ -813,7 +827,10 @@
       <c r="S5" t="n">
         <v>23.47</v>
       </c>
-      <c r="T5" t="n">
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
         <v>0.26</v>
       </c>
     </row>
@@ -883,7 +900,10 @@
       <c r="S6" t="n">
         <v>21.7</v>
       </c>
-      <c r="T6" t="n">
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
         <v>-3.98</v>
       </c>
     </row>
@@ -953,7 +973,10 @@
       <c r="S7" t="n">
         <v>36</v>
       </c>
-      <c r="T7" t="n">
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
         <v>1.38</v>
       </c>
     </row>
@@ -1023,7 +1046,10 @@
       <c r="S8" t="n">
         <v>41.6</v>
       </c>
-      <c r="T8" t="n">
+      <c r="T8" t="b">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
         <v>6.67</v>
       </c>
     </row>
@@ -1093,7 +1119,10 @@
       <c r="S9" t="n">
         <v>38.5</v>
       </c>
-      <c r="T9" t="n">
+      <c r="T9" t="b">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
         <v>-0.52</v>
       </c>
     </row>
@@ -1163,7 +1192,10 @@
       <c r="S10" t="n">
         <v>47.89</v>
       </c>
-      <c r="T10" t="n">
+      <c r="T10" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" t="n">
         <v>0.82</v>
       </c>
     </row>
@@ -1233,7 +1265,10 @@
       <c r="S11" t="n">
         <v>51.19</v>
       </c>
-      <c r="T11" t="n">
+      <c r="T11" t="b">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
         <v>7.23</v>
       </c>
     </row>
@@ -1303,7 +1338,10 @@
       <c r="S12" t="n">
         <v>48.24</v>
       </c>
-      <c r="T12" t="n">
+      <c r="T12" t="b">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
         <v>-0.23</v>
       </c>
     </row>
@@ -1373,7 +1411,10 @@
       <c r="S13" t="n">
         <v>52.5</v>
       </c>
-      <c r="T13" t="n">
+      <c r="T13" t="b">
+        <v>0</v>
+      </c>
+      <c r="U13" t="n">
         <v>3.67</v>
       </c>
     </row>
@@ -1443,7 +1484,10 @@
       <c r="S14" t="n">
         <v>49.91</v>
       </c>
-      <c r="T14" t="n">
+      <c r="T14" t="b">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
         <v>1.07</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trading data 2026-04-17 15:22:00.210135
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
         <v>45672.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45686.41666666666</v>
+        <v>45676.41666666666</v>
       </c>
       <c r="F2" t="n">
         <v>15.54</v>
@@ -569,13 +569,13 @@
         <v>14.29</v>
       </c>
       <c r="H2" t="n">
-        <v>18.2</v>
+        <v>17.34</v>
       </c>
       <c r="I2" t="n">
-        <v>17.12</v>
+        <v>11.58</v>
       </c>
       <c r="J2" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="K2" t="n">
         <v>14.02</v>
@@ -609,7 +609,7 @@
         <v>17.47</v>
       </c>
       <c r="T2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="n">
         <v>12.42</v>
@@ -630,31 +630,31 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45687.41666666666</v>
+        <v>45678.41666666666</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45722.41666666666</v>
+        <v>45686.41666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>20.07</v>
+        <v>17.95</v>
       </c>
       <c r="G3" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H3" t="n">
         <v>18.2</v>
       </c>
-      <c r="H3" t="n">
-        <v>22.6</v>
-      </c>
       <c r="I3" t="n">
-        <v>12.61</v>
+        <v>1.39</v>
       </c>
       <c r="J3" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="K3" t="n">
-        <v>18.07</v>
+        <v>16.3</v>
       </c>
       <c r="L3" t="n">
-        <v>19.07</v>
+        <v>17.59</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -667,25 +667,25 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>5186111</v>
+        <v>7215730</v>
       </c>
       <c r="P3" t="n">
-        <v>10.27</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="Q3" t="n">
-        <v>18.21</v>
+        <v>17.81</v>
       </c>
       <c r="R3" t="b">
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>20.79</v>
+        <v>17.59</v>
       </c>
       <c r="T3" t="b">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>3.59</v>
+        <v>-2.01</v>
       </c>
     </row>
     <row r="4">
@@ -703,31 +703,31 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>45726.41666666666</v>
+        <v>45687.41666666666</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45690.41666666666</v>
       </c>
       <c r="F4" t="n">
-        <v>23.96</v>
+        <v>20.07</v>
       </c>
       <c r="G4" t="n">
-        <v>22.67</v>
+        <v>18.2</v>
       </c>
       <c r="H4" t="n">
-        <v>22.6</v>
+        <v>20.05</v>
       </c>
       <c r="I4" t="n">
-        <v>-5.68</v>
+        <v>-0.1</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>22.25</v>
+        <v>18.07</v>
       </c>
       <c r="L4" t="n">
-        <v>23.25</v>
+        <v>19.07</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -740,25 +740,25 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>1305391</v>
+        <v>5186111</v>
       </c>
       <c r="P4" t="n">
-        <v>5.69</v>
+        <v>10.27</v>
       </c>
       <c r="Q4" t="n">
-        <v>23.79</v>
+        <v>18.21</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>23.79</v>
+        <v>20.79</v>
       </c>
       <c r="T4" t="b">
         <v>1</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.71</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="5">
@@ -773,34 +773,34 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45735.41666666666</v>
+        <v>45705.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45753.41666666666</v>
+        <v>45722.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>23.41</v>
+        <v>21.53</v>
       </c>
       <c r="G5" t="n">
-        <v>22.02</v>
+        <v>20.59</v>
       </c>
       <c r="H5" t="n">
-        <v>21</v>
+        <v>22.6</v>
       </c>
       <c r="I5" t="n">
-        <v>-10.29</v>
+        <v>4.97</v>
       </c>
       <c r="J5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>22.2</v>
+        <v>18.2</v>
       </c>
       <c r="L5" t="n">
-        <v>22.99</v>
+        <v>20.6</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -813,25 +813,25 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>448788</v>
+        <v>3914369</v>
       </c>
       <c r="P5" t="n">
-        <v>5.07</v>
+        <v>4.57</v>
       </c>
       <c r="Q5" t="n">
-        <v>22.96</v>
+        <v>28.4</v>
       </c>
       <c r="R5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>23.47</v>
+        <v>20.6</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>0.26</v>
+        <v>-4.32</v>
       </c>
     </row>
     <row r="6">
@@ -846,34 +846,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45761.41666666666</v>
+        <v>45726.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>45727.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>22.6</v>
+        <v>23.96</v>
       </c>
       <c r="G6" t="n">
-        <v>21.57</v>
+        <v>22.67</v>
       </c>
       <c r="H6" t="n">
-        <v>36.21</v>
+        <v>23.72</v>
       </c>
       <c r="I6" t="n">
-        <v>60.22</v>
+        <v>-1</v>
       </c>
       <c r="J6" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>19.56</v>
+        <v>22.25</v>
       </c>
       <c r="L6" t="n">
-        <v>21.7</v>
+        <v>23.25</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -886,25 +886,25 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>581928</v>
+        <v>1305391</v>
       </c>
       <c r="P6" t="n">
-        <v>4.78</v>
+        <v>5.69</v>
       </c>
       <c r="Q6" t="n">
-        <v>21.7</v>
+        <v>23.79</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>21.7</v>
+        <v>23.79</v>
       </c>
       <c r="T6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>-3.98</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="7">
@@ -922,31 +922,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45735.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45890.41666666666</v>
+        <v>45753.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>35.51</v>
+        <v>23.41</v>
       </c>
       <c r="G7" t="n">
-        <v>33.5</v>
+        <v>22.02</v>
       </c>
       <c r="H7" t="n">
-        <v>41.93</v>
+        <v>21</v>
       </c>
       <c r="I7" t="n">
-        <v>18.08</v>
+        <v>-10.29</v>
       </c>
       <c r="J7" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="K7" t="n">
-        <v>32.66</v>
+        <v>22.2</v>
       </c>
       <c r="L7" t="n">
-        <v>34.89</v>
+        <v>22.99</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -959,25 +959,25 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>2216102</v>
+        <v>448788</v>
       </c>
       <c r="P7" t="n">
-        <v>6</v>
+        <v>5.07</v>
       </c>
       <c r="Q7" t="n">
-        <v>34.34</v>
+        <v>22.96</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>36</v>
+        <v>23.47</v>
       </c>
       <c r="T7" t="b">
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>1.38</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="8">
@@ -995,31 +995,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45914.41666666666</v>
+        <v>45761.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45916.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>39</v>
+        <v>22.6</v>
       </c>
       <c r="G8" t="n">
-        <v>38.51</v>
+        <v>21.57</v>
       </c>
       <c r="H8" t="n">
-        <v>38.9</v>
+        <v>36.21</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.26</v>
+        <v>60.22</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>78</v>
       </c>
       <c r="K8" t="n">
-        <v>36.5</v>
+        <v>19.56</v>
       </c>
       <c r="L8" t="n">
-        <v>38.64</v>
+        <v>21.7</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1032,25 +1032,25 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>212755</v>
+        <v>581928</v>
       </c>
       <c r="P8" t="n">
-        <v>0.96</v>
+        <v>4.78</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.16</v>
+        <v>21.7</v>
       </c>
       <c r="R8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>41.6</v>
+        <v>21.7</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>6.67</v>
+        <v>-3.98</v>
       </c>
     </row>
     <row r="9">
@@ -1068,31 +1068,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45925.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45944.41666666666</v>
+        <v>45890.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>38.7</v>
+        <v>35.51</v>
       </c>
       <c r="G9" t="n">
-        <v>36.85</v>
+        <v>33.5</v>
       </c>
       <c r="H9" t="n">
-        <v>47.44</v>
+        <v>41.93</v>
       </c>
       <c r="I9" t="n">
-        <v>22.58</v>
+        <v>18.08</v>
       </c>
       <c r="J9" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K9" t="n">
-        <v>35.01</v>
+        <v>32.66</v>
       </c>
       <c r="L9" t="n">
-        <v>37.98</v>
+        <v>34.89</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1105,25 +1105,25 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>300539</v>
+        <v>2216102</v>
       </c>
       <c r="P9" t="n">
-        <v>5.02</v>
+        <v>6</v>
       </c>
       <c r="Q9" t="n">
-        <v>36.94</v>
+        <v>34.34</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>38.5</v>
+        <v>36</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.52</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="10">
@@ -1141,31 +1141,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45970.41666666666</v>
+        <v>45914.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>46035.41666666666</v>
+        <v>45916.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>47.5</v>
+        <v>39</v>
       </c>
       <c r="G10" t="n">
-        <v>45.28</v>
+        <v>38.51</v>
       </c>
       <c r="H10" t="n">
-        <v>47.53</v>
+        <v>38.9</v>
       </c>
       <c r="I10" t="n">
-        <v>0.06</v>
+        <v>-0.26</v>
       </c>
       <c r="J10" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>44.75</v>
+        <v>36.5</v>
       </c>
       <c r="L10" t="n">
-        <v>46.95</v>
+        <v>38.64</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1178,25 +1178,25 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>403885</v>
+        <v>212755</v>
       </c>
       <c r="P10" t="n">
-        <v>4.9</v>
+        <v>0.96</v>
       </c>
       <c r="Q10" t="n">
-        <v>47.03</v>
+        <v>39.16</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>47.89</v>
+        <v>41.6</v>
       </c>
       <c r="T10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>0.82</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="11">
@@ -1214,31 +1214,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46041.41666666666</v>
+        <v>45925.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>46042.41666666666</v>
+        <v>45944.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>47.74</v>
+        <v>38.7</v>
       </c>
       <c r="G11" t="n">
-        <v>47.03</v>
+        <v>36.85</v>
       </c>
       <c r="H11" t="n">
-        <v>46.89</v>
+        <v>47.44</v>
       </c>
       <c r="I11" t="n">
-        <v>-1.78</v>
+        <v>22.58</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="K11" t="n">
-        <v>45</v>
+        <v>35.01</v>
       </c>
       <c r="L11" t="n">
-        <v>47.65</v>
+        <v>37.98</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1251,25 +1251,25 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>250069</v>
+        <v>300539</v>
       </c>
       <c r="P11" t="n">
-        <v>1.29</v>
+        <v>5.02</v>
       </c>
       <c r="Q11" t="n">
-        <v>47.81</v>
+        <v>36.94</v>
       </c>
       <c r="R11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>51.19</v>
+        <v>38.5</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>7.23</v>
+        <v>-0.52</v>
       </c>
     </row>
     <row r="12">
@@ -1287,31 +1287,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>46043.41666666666</v>
+        <v>45970.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>46075.41666666666</v>
+        <v>46035.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>48.35</v>
+        <v>47.5</v>
       </c>
       <c r="G12" t="n">
-        <v>46.1</v>
+        <v>45.28</v>
       </c>
       <c r="H12" t="n">
-        <v>48.39</v>
+        <v>47.53</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="J12" t="n">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="K12" t="n">
-        <v>46.5</v>
+        <v>44.75</v>
       </c>
       <c r="L12" t="n">
-        <v>48.24</v>
+        <v>46.95</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1324,25 +1324,25 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>1463983</v>
+        <v>403885</v>
       </c>
       <c r="P12" t="n">
-        <v>3.11</v>
+        <v>4.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>48.24</v>
+        <v>47.03</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>48.24</v>
+        <v>47.89</v>
       </c>
       <c r="T12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.23</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="13">
@@ -1360,31 +1360,31 @@
         <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>46079.41666666666</v>
+        <v>46041.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>46090.41666666666</v>
+        <v>46042.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>50.64</v>
+        <v>47.74</v>
       </c>
       <c r="G13" t="n">
-        <v>49.02</v>
+        <v>47.03</v>
       </c>
       <c r="H13" t="n">
-        <v>48.55</v>
+        <v>46.89</v>
       </c>
       <c r="I13" t="n">
-        <v>-4.13</v>
+        <v>-1.78</v>
       </c>
       <c r="J13" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>48.02</v>
+        <v>45</v>
       </c>
       <c r="L13" t="n">
-        <v>50.5</v>
+        <v>47.65</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>1689183</v>
+        <v>250069</v>
       </c>
       <c r="P13" t="n">
-        <v>2.51</v>
+        <v>1.29</v>
       </c>
       <c r="Q13" t="n">
-        <v>51.45</v>
+        <v>47.81</v>
       </c>
       <c r="R13" t="b">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>52.5</v>
+        <v>51.19</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>3.67</v>
+        <v>7.23</v>
       </c>
     </row>
     <row r="14">
@@ -1433,62 +1433,354 @@
         <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
+        <v>46043.41666666666</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>46044.41666666666</v>
+      </c>
+      <c r="F14" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="G14" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>48</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>1463983</v>
+      </c>
+      <c r="P14" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="T14" t="b">
+        <v>1</v>
+      </c>
+      <c r="U14" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>46068.41666666666</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>46075.41666666666</v>
+      </c>
+      <c r="F15" t="n">
+        <v>49.15</v>
+      </c>
+      <c r="G15" t="n">
+        <v>48.04</v>
+      </c>
+      <c r="H15" t="n">
+        <v>48.39</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>49</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>1584986</v>
+      </c>
+      <c r="P15" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>52.76</v>
+      </c>
+      <c r="R15" t="b">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>49</v>
+      </c>
+      <c r="T15" t="b">
+        <v>1</v>
+      </c>
+      <c r="U15" t="n">
+        <v>-0.31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>46079.41666666666</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>46079.41666666666</v>
+      </c>
+      <c r="F16" t="n">
+        <v>50.64</v>
+      </c>
+      <c r="G16" t="n">
+        <v>49.02</v>
+      </c>
+      <c r="H16" t="n">
+        <v>50.64</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>48.02</v>
+      </c>
+      <c r="L16" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>1689183</v>
+      </c>
+      <c r="P16" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>51.45</v>
+      </c>
+      <c r="R16" t="b">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="T16" t="b">
+        <v>1</v>
+      </c>
+      <c r="U16" t="n">
+        <v>3.67</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2" t="n">
         <v>46107.41666666666</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E17" s="2" t="n">
+        <v>46107.41666666666</v>
+      </c>
+      <c r="F17" t="n">
+        <v>49.38</v>
+      </c>
+      <c r="G17" t="n">
+        <v>46.91</v>
+      </c>
+      <c r="H17" t="n">
+        <v>49.38</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>45.51</v>
+      </c>
+      <c r="L17" t="n">
+        <v>47.88</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>3000298</v>
+      </c>
+      <c r="P17" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>47.36</v>
+      </c>
+      <c r="R17" t="b">
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="T17" t="b">
+        <v>1</v>
+      </c>
+      <c r="U17" t="n">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>46112.41666666666</v>
+      </c>
+      <c r="E18" s="2" t="n">
         <v>46126.41666666666</v>
       </c>
-      <c r="F14" t="n">
-        <v>49.38</v>
-      </c>
-      <c r="G14" t="n">
+      <c r="F18" t="n">
+        <v>51.85</v>
+      </c>
+      <c r="G18" t="n">
+        <v>49.07</v>
+      </c>
+      <c r="H18" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="I18" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J18" t="n">
+        <v>14</v>
+      </c>
+      <c r="K18" t="n">
         <v>46.91</v>
       </c>
-      <c r="H14" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="I14" t="n">
-        <v>11.18</v>
-      </c>
-      <c r="J14" t="n">
-        <v>19</v>
-      </c>
-      <c r="K14" t="n">
-        <v>45.51</v>
-      </c>
-      <c r="L14" t="n">
-        <v>47.88</v>
-      </c>
-      <c r="M14" t="inlineStr">
+      <c r="L18" t="n">
+        <v>51</v>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>RANGE_BREAKDOWN</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="O14" t="n">
-        <v>3000298</v>
-      </c>
-      <c r="P14" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>47.36</v>
-      </c>
-      <c r="R14" t="b">
-        <v>1</v>
-      </c>
-      <c r="S14" t="n">
-        <v>49.91</v>
-      </c>
-      <c r="T14" t="b">
-        <v>0</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1.07</v>
+      <c r="O18" t="n">
+        <v>2394589</v>
+      </c>
+      <c r="P18" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>50.97</v>
+      </c>
+      <c r="R18" t="b">
+        <v>1</v>
+      </c>
+      <c r="S18" t="n">
+        <v>51</v>
+      </c>
+      <c r="T18" t="b">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>-1.64</v>
       </c>
     </row>
   </sheetData>
@@ -1624,25 +1916,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>61.54</v>
+        <v>47.06</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>9.210000000000001</v>
+        <v>6.42</v>
       </c>
       <c r="I2" t="n">
-        <v>119.79</v>
+        <v>109.06</v>
       </c>
       <c r="J2" t="n">
         <v>60.22</v>
@@ -1651,28 +1943,28 @@
         <v>-10.29</v>
       </c>
       <c r="L2" t="n">
-        <v>18.47</v>
+        <v>15.95</v>
       </c>
       <c r="M2" t="n">
         <v>5</v>
       </c>
       <c r="N2" t="n">
-        <v>17.74</v>
+        <v>15.6</v>
       </c>
       <c r="O2" t="n">
-        <v>4.43</v>
+        <v>2.24</v>
       </c>
       <c r="P2" t="n">
-        <v>9.210000000000001</v>
+        <v>6.42</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6666902670775552</v>
+        <v>0.6323992625368732</v>
       </c>
       <c r="R2" t="n">
-        <v>0.4982</v>
+        <v>0.5549999999999999</v>
       </c>
       <c r="S2" t="n">
-        <v>0.565596106831022</v>
+        <v>0.5859597050147493</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -1680,7 +1972,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.565596106831022</v>
+        <v>0.5859597050147493</v>
       </c>
     </row>
   </sheetData>
@@ -1751,22 +2043,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2" t="n">
-        <v>61.54</v>
+        <v>47.06</v>
       </c>
       <c r="F2" t="n">
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>9.210000000000001</v>
+        <v>6.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 15:41:38.559732
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z12"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -580,34 +580,34 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45865.41666666666</v>
+        <v>45819.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>5.6</v>
+        <v>26.79</v>
       </c>
       <c r="G2" t="n">
-        <v>5.49</v>
+        <v>26</v>
       </c>
       <c r="H2" t="n">
-        <v>6.72</v>
+        <v>25.86</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>-3.47</v>
       </c>
       <c r="J2" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="K2" t="n">
-        <v>4.6</v>
+        <v>25.81</v>
       </c>
       <c r="L2" t="n">
-        <v>5.57</v>
+        <v>26.6</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -620,31 +620,31 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>1189884</v>
+        <v>2887899</v>
       </c>
       <c r="P2" t="n">
-        <v>1.63</v>
+        <v>3.04</v>
       </c>
       <c r="Q2" t="n">
-        <v>5.46</v>
+        <v>26.6</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>6.2</v>
+        <v>26.6</v>
       </c>
       <c r="T2" t="b">
         <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>10.71</v>
+        <v>-0.71</v>
       </c>
       <c r="W2" t="n">
-        <v>-2.5</v>
+        <v>-0.71</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
@@ -655,7 +655,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -667,31 +667,31 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45873.41666666666</v>
+        <v>45832.41666666666</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45880.41666666666</v>
+        <v>45855.41666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>6.9</v>
+        <v>23.52</v>
       </c>
       <c r="G3" t="n">
-        <v>6.62</v>
+        <v>22.8</v>
       </c>
       <c r="H3" t="n">
-        <v>6.53</v>
+        <v>26.03</v>
       </c>
       <c r="I3" t="n">
-        <v>-5.36</v>
+        <v>10.67</v>
       </c>
       <c r="J3" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="K3" t="n">
-        <v>6.48</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
-        <v>6.73</v>
+        <v>23.1</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -704,19 +704,19 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>1865203</v>
+        <v>928406</v>
       </c>
       <c r="P3" t="n">
-        <v>3.45</v>
+        <v>3.16</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.72</v>
+        <v>25.87</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>7.19</v>
+        <v>27.43</v>
       </c>
       <c r="T3" t="b">
         <v>0</v>
@@ -725,10 +725,10 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>4.2</v>
+        <v>16.62</v>
       </c>
       <c r="W3" t="n">
-        <v>-2.61</v>
+        <v>9.99</v>
       </c>
       <c r="X3" t="b">
         <v>1</v>
@@ -739,7 +739,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -751,31 +751,31 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>45888.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>45889.41666666666</v>
+        <v>45874.41666666666</v>
       </c>
       <c r="F4" t="n">
-        <v>6.8</v>
+        <v>25.74</v>
       </c>
       <c r="G4" t="n">
-        <v>6.71</v>
+        <v>25.49</v>
       </c>
       <c r="H4" t="n">
-        <v>6.55</v>
+        <v>25.4</v>
       </c>
       <c r="I4" t="n">
-        <v>-3.68</v>
+        <v>-1.32</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>6.5</v>
+        <v>24.7</v>
       </c>
       <c r="L4" t="n">
-        <v>6.73</v>
+        <v>25.69</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -788,19 +788,19 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>1273591</v>
+        <v>485199</v>
       </c>
       <c r="P4" t="n">
-        <v>1.34</v>
+        <v>0.98</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.68</v>
+        <v>25.11</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>7.39</v>
+        <v>26.64</v>
       </c>
       <c r="T4" t="b">
         <v>0</v>
@@ -809,10 +809,10 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>8.68</v>
+        <v>3.5</v>
       </c>
       <c r="W4" t="n">
-        <v>-1.76</v>
+        <v>-2.45</v>
       </c>
       <c r="X4" t="b">
         <v>0</v>
@@ -823,7 +823,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -835,31 +835,31 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45922.41666666666</v>
+        <v>45893.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45932.41666666666</v>
+        <v>45895.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>6.4</v>
+        <v>26</v>
       </c>
       <c r="G5" t="n">
-        <v>5.95</v>
+        <v>24.26</v>
       </c>
       <c r="H5" t="n">
-        <v>6.25</v>
+        <v>25.8</v>
       </c>
       <c r="I5" t="n">
-        <v>-2.34</v>
+        <v>-0.77</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>5.93</v>
+        <v>23.9</v>
       </c>
       <c r="L5" t="n">
-        <v>6.19</v>
+        <v>24.85</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -872,19 +872,19 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>1694740</v>
+        <v>1688191</v>
       </c>
       <c r="P5" t="n">
-        <v>6.84</v>
+        <v>6.47</v>
       </c>
       <c r="Q5" t="n">
-        <v>6.1</v>
+        <v>24.71</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>6.28</v>
+        <v>25.88</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
@@ -893,10 +893,10 @@
         <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>-1.88</v>
+        <v>-0.46</v>
       </c>
       <c r="W5" t="n">
-        <v>-4.69</v>
+        <v>-4.96</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
@@ -907,7 +907,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -919,31 +919,31 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45935.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45958.41666666666</v>
+        <v>45917.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>6.5</v>
+        <v>26.86</v>
       </c>
       <c r="G6" t="n">
-        <v>6.2</v>
+        <v>26.15</v>
       </c>
       <c r="H6" t="n">
-        <v>6.69</v>
+        <v>25.64</v>
       </c>
       <c r="I6" t="n">
-        <v>2.92</v>
+        <v>-4.54</v>
       </c>
       <c r="J6" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="K6" t="n">
-        <v>6.23</v>
+        <v>25.4</v>
       </c>
       <c r="L6" t="n">
-        <v>6.45</v>
+        <v>26.5</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -956,31 +956,31 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>1208314</v>
+        <v>1350366</v>
       </c>
       <c r="P6" t="n">
-        <v>4</v>
+        <v>2.72</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.24</v>
+        <v>28.21</v>
       </c>
       <c r="R6" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>26.68</v>
+      </c>
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" t="b">
         <v>1</v>
       </c>
-      <c r="S6" t="n">
-        <v>6.87</v>
-      </c>
-      <c r="T6" t="b">
-        <v>0</v>
-      </c>
-      <c r="U6" t="b">
-        <v>0</v>
-      </c>
       <c r="V6" t="n">
-        <v>5.69</v>
+        <v>-0.67</v>
       </c>
       <c r="W6" t="n">
-        <v>-4</v>
+        <v>5.03</v>
       </c>
       <c r="X6" t="b">
         <v>1</v>
@@ -991,7 +991,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1003,31 +1003,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45984.41666666666</v>
+        <v>45928.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45986.41666666666</v>
+        <v>45951.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>6.59</v>
+        <v>24.97</v>
       </c>
       <c r="G7" t="n">
-        <v>6.34</v>
+        <v>24.63</v>
       </c>
       <c r="H7" t="n">
-        <v>6.33</v>
+        <v>26.6</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.95</v>
+        <v>6.53</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K7" t="n">
-        <v>6.2</v>
+        <v>24.12</v>
       </c>
       <c r="L7" t="n">
-        <v>6.37</v>
+        <v>24.78</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1040,31 +1040,31 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>1101047</v>
+        <v>370152</v>
       </c>
       <c r="P7" t="n">
-        <v>3.94</v>
+        <v>1.38</v>
       </c>
       <c r="Q7" t="n">
-        <v>6.45</v>
+        <v>26.95</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>6.57</v>
+        <v>27.25</v>
       </c>
       <c r="T7" t="b">
         <v>0</v>
       </c>
       <c r="U7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.3</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="W7" t="n">
-        <v>-2.12</v>
+        <v>7.93</v>
       </c>
       <c r="X7" t="b">
         <v>1</v>
@@ -1075,7 +1075,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1087,31 +1087,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46007.41666666666</v>
+        <v>45952.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46019.41666666666</v>
+        <v>45963.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>6.46</v>
+        <v>27.25</v>
       </c>
       <c r="G8" t="n">
-        <v>6.22</v>
+        <v>26.6</v>
       </c>
       <c r="H8" t="n">
-        <v>6.82</v>
+        <v>27.08</v>
       </c>
       <c r="I8" t="n">
-        <v>5.57</v>
+        <v>-0.62</v>
       </c>
       <c r="J8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K8" t="n">
-        <v>6.13</v>
+        <v>26.5</v>
       </c>
       <c r="L8" t="n">
-        <v>6.25</v>
+        <v>27.09</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1124,31 +1124,31 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>1689563</v>
+        <v>1411464</v>
       </c>
       <c r="P8" t="n">
-        <v>3.86</v>
+        <v>2.44</v>
       </c>
       <c r="Q8" t="n">
-        <v>6.32</v>
+        <v>27.38</v>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>6.28</v>
+        <v>27.96</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
       </c>
       <c r="U8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>-2.79</v>
+        <v>2.61</v>
       </c>
       <c r="W8" t="n">
-        <v>-2.17</v>
+        <v>0.48</v>
       </c>
       <c r="X8" t="b">
         <v>1</v>
@@ -1159,7 +1159,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1171,31 +1171,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46033.41666666666</v>
+        <v>45991.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>46035.41666666666</v>
+        <v>46007.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>7.06</v>
+        <v>25.79</v>
       </c>
       <c r="G9" t="n">
-        <v>7.03</v>
+        <v>25</v>
       </c>
       <c r="H9" t="n">
-        <v>6.7</v>
+        <v>25.53</v>
       </c>
       <c r="I9" t="n">
-        <v>-5.1</v>
+        <v>-1.01</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="K9" t="n">
-        <v>6.41</v>
+        <v>25.2</v>
       </c>
       <c r="L9" t="n">
-        <v>7.04</v>
+        <v>25.78</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1208,19 +1208,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>1647282</v>
+        <v>442438</v>
       </c>
       <c r="P9" t="n">
-        <v>0.43</v>
+        <v>2.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>7.25</v>
+        <v>25.06</v>
       </c>
       <c r="R9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>7.68</v>
+        <v>26.17</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>8.779999999999999</v>
+        <v>1.47</v>
       </c>
       <c r="W9" t="n">
-        <v>2.69</v>
+        <v>-2.83</v>
       </c>
       <c r="X9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
@@ -1243,7 +1243,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1255,31 +1255,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46055.41666666666</v>
+        <v>46012.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>46064.41666666666</v>
+        <v>46016.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>6.48</v>
+        <v>25.95</v>
       </c>
       <c r="G10" t="n">
-        <v>6.17</v>
+        <v>25.51</v>
       </c>
       <c r="H10" t="n">
-        <v>9.699999999999999</v>
+        <v>25.33</v>
       </c>
       <c r="I10" t="n">
-        <v>49.69</v>
+        <v>-2.39</v>
       </c>
       <c r="J10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>6.02</v>
+        <v>25.51</v>
       </c>
       <c r="L10" t="n">
-        <v>6.34</v>
+        <v>25.89</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1292,19 +1292,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>318660</v>
+        <v>197579</v>
       </c>
       <c r="P10" t="n">
-        <v>3.85</v>
+        <v>0.66</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.24</v>
+        <v>25.62</v>
       </c>
       <c r="R10" t="b">
         <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>6.54</v>
+        <v>26.84</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1313,13 +1313,13 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>0.93</v>
+        <v>3.43</v>
       </c>
       <c r="W10" t="n">
-        <v>-3.7</v>
+        <v>-1.27</v>
       </c>
       <c r="X10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
@@ -1327,7 +1327,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1339,158 +1339,74 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46071.41666666666</v>
+        <v>46056.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>46072.41666666666</v>
+        <v>46070.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>9.85</v>
+        <v>25.67</v>
       </c>
       <c r="G11" t="n">
-        <v>9.42</v>
+        <v>23.54</v>
       </c>
       <c r="H11" t="n">
-        <v>9.26</v>
+        <v>27.48</v>
       </c>
       <c r="I11" t="n">
-        <v>-5.99</v>
+        <v>7.05</v>
       </c>
       <c r="J11" t="n">
+        <v>14</v>
+      </c>
+      <c r="K11" t="n">
+        <v>23.44</v>
+      </c>
+      <c r="L11" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>1796699</v>
+      </c>
+      <c r="P11" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>24.37</v>
+      </c>
+      <c r="R11" t="b">
         <v>1</v>
       </c>
-      <c r="K11" t="n">
-        <v>9.41</v>
-      </c>
-      <c r="L11" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O11" t="n">
-        <v>4798270</v>
-      </c>
-      <c r="P11" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>10.36</v>
-      </c>
-      <c r="R11" t="b">
-        <v>0</v>
-      </c>
       <c r="S11" t="n">
-        <v>12.25</v>
+        <v>25.19</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
       </c>
       <c r="U11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>24.37</v>
+        <v>-1.87</v>
       </c>
       <c r="W11" t="n">
-        <v>5.18</v>
+        <v>-5.06</v>
       </c>
       <c r="X11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>EPCO</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C12" t="b">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>46106.41666666666</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>46111.41666666666</v>
-      </c>
-      <c r="F12" t="n">
-        <v>9.02</v>
-      </c>
-      <c r="G12" t="n">
-        <v>8.390000000000001</v>
-      </c>
-      <c r="H12" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-7.87</v>
-      </c>
-      <c r="J12" t="n">
-        <v>5</v>
-      </c>
-      <c r="K12" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="L12" t="n">
-        <v>8.84</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O12" t="n">
-        <v>6893557</v>
-      </c>
-      <c r="P12" t="n">
-        <v>7.51</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="R12" t="b">
-        <v>1</v>
-      </c>
-      <c r="S12" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="T12" t="b">
-        <v>0</v>
-      </c>
-      <c r="U12" t="b">
-        <v>0</v>
-      </c>
-      <c r="V12" t="n">
-        <v>8.09</v>
-      </c>
-      <c r="W12" t="n">
-        <v>-6.76</v>
-      </c>
-      <c r="X12" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1641,7 +1557,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1653,31 +1569,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46127.41666666666</v>
+        <v>46128.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46128.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>8.74</v>
+        <v>26.3</v>
       </c>
       <c r="G2" t="n">
-        <v>8.539999999999999</v>
+        <v>25.03</v>
       </c>
       <c r="H2" t="n">
-        <v>9.140000000000001</v>
+        <v>26.3</v>
       </c>
       <c r="I2" t="n">
-        <v>4.58</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>8.31</v>
+        <v>23.35</v>
       </c>
       <c r="L2" t="n">
-        <v>8.609999999999999</v>
+        <v>25.91</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -1690,19 +1606,19 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>1437309</v>
+        <v>2038762</v>
       </c>
       <c r="P2" t="n">
-        <v>2.1</v>
+        <v>4.74</v>
       </c>
       <c r="Q2" t="n">
-        <v>8.57</v>
+        <v>26.8</v>
       </c>
       <c r="R2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>9.35</v>
+        <v>27.79</v>
       </c>
       <c r="T2" t="b">
         <v>0</v>
@@ -1711,16 +1627,16 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>6.98</v>
+        <v>5.67</v>
       </c>
       <c r="W2" t="n">
-        <v>-1.95</v>
+        <v>1.9</v>
       </c>
       <c r="X2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y2" t="n">
-        <v>9.140000000000001</v>
+        <v>26.3</v>
       </c>
       <c r="Z2" t="b">
         <v>0</v>
@@ -1850,7 +1766,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1859,55 +1775,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>36.36</v>
+        <v>30</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.68</v>
+        <v>-0.89</v>
       </c>
       <c r="H2" t="n">
-        <v>3.99</v>
+        <v>1.01</v>
       </c>
       <c r="I2" t="n">
-        <v>43.89</v>
+        <v>10.13</v>
       </c>
       <c r="J2" t="n">
-        <v>49.69</v>
+        <v>10.67</v>
       </c>
       <c r="K2" t="n">
-        <v>-7.87</v>
+        <v>-4.54</v>
       </c>
       <c r="L2" t="n">
-        <v>17.09</v>
+        <v>5.14</v>
       </c>
       <c r="M2" t="n">
-        <v>2.28</v>
+        <v>1.72</v>
       </c>
       <c r="N2" t="n">
-        <v>19.55</v>
+        <v>8.08</v>
       </c>
       <c r="O2" t="n">
-        <v>4.9</v>
+        <v>2.02</v>
       </c>
       <c r="P2" t="n">
-        <v>3.99</v>
+        <v>1.01</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4687197899391929</v>
+        <v>0.4517166123778502</v>
       </c>
       <c r="R2" t="n">
-        <v>0.14947</v>
+        <v>0.14479</v>
       </c>
       <c r="S2" t="n">
-        <v>0.2771699159756772</v>
+        <v>0.2675606449511401</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -1915,7 +1831,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.2771699159756772</v>
+        <v>0.2675606449511401</v>
       </c>
     </row>
   </sheetData>
@@ -1977,7 +1893,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1986,22 +1902,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>36.36</v>
+        <v>30</v>
       </c>
       <c r="F2" t="n">
-        <v>2.28</v>
+        <v>1.72</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.68</v>
+        <v>-0.89</v>
       </c>
       <c r="H2" t="n">
-        <v>3.99</v>
+        <v>1.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:08:42.127906
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,10 +564,15 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>Bars_To_Target</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Current_Clears_Anchor</t>
         </is>
@@ -657,8 +662,11 @@
       <c r="Y2" s="2" t="n">
         <v>45833.41666666666</v>
       </c>
-      <c r="Z2" t="inlineStr"/>
+      <c r="Z2" t="n">
+        <v>2</v>
+      </c>
       <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -744,8 +752,11 @@
       <c r="Y3" s="2" t="n">
         <v>45875.41666666666</v>
       </c>
-      <c r="Z3" t="inlineStr"/>
+      <c r="Z3" t="n">
+        <v>2</v>
+      </c>
       <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -831,6 +842,7 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -910,12 +922,11 @@
       <c r="W5" t="n">
         <v>-4.69</v>
       </c>
-      <c r="X5" t="b">
-        <v>1</v>
-      </c>
+      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1001,8 +1012,11 @@
       <c r="Y6" s="2" t="n">
         <v>45952.41666666666</v>
       </c>
-      <c r="Z6" t="inlineStr"/>
+      <c r="Z6" t="n">
+        <v>12</v>
+      </c>
       <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1082,12 +1096,11 @@
       <c r="W7" t="n">
         <v>-2.12</v>
       </c>
-      <c r="X7" t="b">
-        <v>1</v>
-      </c>
+      <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1167,12 +1180,11 @@
       <c r="W8" t="n">
         <v>-2.17</v>
       </c>
-      <c r="X8" t="b">
-        <v>1</v>
-      </c>
+      <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1258,6 +1270,7 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1343,8 +1356,11 @@
       <c r="Y10" s="2" t="n">
         <v>46056.41666666666</v>
       </c>
-      <c r="Z10" t="inlineStr"/>
+      <c r="Z10" t="n">
+        <v>1</v>
+      </c>
       <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1430,6 +1446,7 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1515,6 +1532,7 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1527,7 +1545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1658,10 +1676,15 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>Bars_To_Target</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Current_Clears_Anchor</t>
         </is>
@@ -1748,11 +1771,16 @@
       <c r="X2" t="b">
         <v>1</v>
       </c>
-      <c r="Y2" t="inlineStr"/>
+      <c r="Y2" s="2" t="n">
+        <v>46128.41666666666</v>
+      </c>
       <c r="Z2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="n">
         <v>9.140000000000001</v>
       </c>
-      <c r="AA2" t="b">
+      <c r="AB2" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:13:03.966312
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,10 +569,25 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
+          <t>Trendline_Hit</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Trendline_Hit_Date</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Bars_To_Trendline</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Current_Clears_Anchor</t>
         </is>
@@ -667,6 +682,9 @@
       </c>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -757,6 +775,9 @@
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -843,6 +864,9 @@
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -927,6 +951,9 @@
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1017,6 +1044,9 @@
       </c>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1101,6 +1131,9 @@
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1185,6 +1218,9 @@
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1269,8 +1305,13 @@
       </c>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
       <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1361,6 +1402,9 @@
       </c>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1445,8 +1489,13 @@
       </c>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
       <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1533,6 +1582,9 @@
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1545,7 +1597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1681,10 +1733,25 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
+          <t>Trendline_Hit</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Trendline_Hit_Date</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Bars_To_Trendline</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Current_Clears_Anchor</t>
         </is>
@@ -1777,10 +1844,13 @@
       <c r="Z2" t="n">
         <v>1</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="n">
         <v>9.140000000000001</v>
       </c>
-      <c r="AB2" t="b">
+      <c r="AE2" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:13:55.878198
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -605,34 +605,34 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45865.41666666666</v>
+        <v>45819.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>5.6</v>
+        <v>26.79</v>
       </c>
       <c r="G2" t="n">
-        <v>5.49</v>
+        <v>26</v>
       </c>
       <c r="H2" t="n">
-        <v>6.72</v>
+        <v>25.86</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>-3.47</v>
       </c>
       <c r="J2" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="K2" t="n">
-        <v>4.6</v>
+        <v>25.81</v>
       </c>
       <c r="L2" t="n">
-        <v>5.57</v>
+        <v>26.6</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -645,41 +645,35 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>1189884</v>
+        <v>2887899</v>
       </c>
       <c r="P2" t="n">
-        <v>1.63</v>
+        <v>3.04</v>
       </c>
       <c r="Q2" t="n">
-        <v>5.46</v>
+        <v>26.6</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>6.2</v>
+        <v>26.6</v>
       </c>
       <c r="T2" t="b">
         <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>10.71</v>
+        <v>-0.71</v>
       </c>
       <c r="W2" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="X2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y2" s="2" t="n">
-        <v>45833.41666666666</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>2</v>
-      </c>
+        <v>-0.71</v>
+      </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -689,7 +683,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -701,31 +695,31 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45873.41666666666</v>
+        <v>45832.41666666666</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45880.41666666666</v>
+        <v>45855.41666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>6.9</v>
+        <v>23.52</v>
       </c>
       <c r="G3" t="n">
-        <v>6.62</v>
+        <v>22.8</v>
       </c>
       <c r="H3" t="n">
-        <v>6.53</v>
+        <v>26.03</v>
       </c>
       <c r="I3" t="n">
-        <v>-5.36</v>
+        <v>10.67</v>
       </c>
       <c r="J3" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="K3" t="n">
-        <v>6.48</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
-        <v>6.73</v>
+        <v>23.1</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -738,19 +732,19 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>1865203</v>
+        <v>928406</v>
       </c>
       <c r="P3" t="n">
-        <v>3.45</v>
+        <v>3.16</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.72</v>
+        <v>25.87</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>7.19</v>
+        <v>27.43</v>
       </c>
       <c r="T3" t="b">
         <v>0</v>
@@ -759,30 +753,36 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>4.2</v>
+        <v>16.62</v>
       </c>
       <c r="W3" t="n">
-        <v>-2.61</v>
+        <v>9.99</v>
       </c>
       <c r="X3" t="b">
         <v>1</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>45875.41666666666</v>
+        <v>45844.41666666666</v>
       </c>
       <c r="Z3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="2" t="n">
+        <v>45840.41666666666</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>5</v>
+      </c>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -794,31 +794,31 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>45888.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>45889.41666666666</v>
+        <v>45874.41666666666</v>
       </c>
       <c r="F4" t="n">
-        <v>6.8</v>
+        <v>25.74</v>
       </c>
       <c r="G4" t="n">
-        <v>6.71</v>
+        <v>25.49</v>
       </c>
       <c r="H4" t="n">
-        <v>6.55</v>
+        <v>25.4</v>
       </c>
       <c r="I4" t="n">
-        <v>-3.68</v>
+        <v>-1.32</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>6.5</v>
+        <v>24.7</v>
       </c>
       <c r="L4" t="n">
-        <v>6.73</v>
+        <v>25.69</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -831,19 +831,19 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>1273591</v>
+        <v>485199</v>
       </c>
       <c r="P4" t="n">
-        <v>1.34</v>
+        <v>0.98</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.68</v>
+        <v>25.11</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>7.39</v>
+        <v>26.64</v>
       </c>
       <c r="T4" t="b">
         <v>0</v>
@@ -852,10 +852,10 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>8.68</v>
+        <v>3.5</v>
       </c>
       <c r="W4" t="n">
-        <v>-1.76</v>
+        <v>-2.45</v>
       </c>
       <c r="X4" t="b">
         <v>0</v>
@@ -871,7 +871,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -883,31 +883,31 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45922.41666666666</v>
+        <v>45893.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45932.41666666666</v>
+        <v>45895.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>6.4</v>
+        <v>26</v>
       </c>
       <c r="G5" t="n">
-        <v>5.95</v>
+        <v>24.26</v>
       </c>
       <c r="H5" t="n">
-        <v>6.25</v>
+        <v>25.8</v>
       </c>
       <c r="I5" t="n">
-        <v>-2.34</v>
+        <v>-0.77</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>5.93</v>
+        <v>23.9</v>
       </c>
       <c r="L5" t="n">
-        <v>6.19</v>
+        <v>24.85</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -920,19 +920,19 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>1694740</v>
+        <v>1688191</v>
       </c>
       <c r="P5" t="n">
-        <v>6.84</v>
+        <v>6.47</v>
       </c>
       <c r="Q5" t="n">
-        <v>6.1</v>
+        <v>24.71</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>6.28</v>
+        <v>25.88</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
@@ -941,10 +941,10 @@
         <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>-1.88</v>
+        <v>-0.46</v>
       </c>
       <c r="W5" t="n">
-        <v>-4.69</v>
+        <v>-4.96</v>
       </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
@@ -958,7 +958,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -970,31 +970,31 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45935.41666666666</v>
+        <v>45908.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45958.41666666666</v>
+        <v>45917.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>6.5</v>
+        <v>26.86</v>
       </c>
       <c r="G6" t="n">
-        <v>6.2</v>
+        <v>26.15</v>
       </c>
       <c r="H6" t="n">
-        <v>6.69</v>
+        <v>25.64</v>
       </c>
       <c r="I6" t="n">
-        <v>2.92</v>
+        <v>-4.54</v>
       </c>
       <c r="J6" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="K6" t="n">
-        <v>6.23</v>
+        <v>25.4</v>
       </c>
       <c r="L6" t="n">
-        <v>6.45</v>
+        <v>26.5</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1007,42 +1007,38 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>1208314</v>
+        <v>1350366</v>
       </c>
       <c r="P6" t="n">
-        <v>4</v>
+        <v>2.72</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.24</v>
+        <v>28.21</v>
       </c>
       <c r="R6" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>26.68</v>
+      </c>
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" t="b">
         <v>1</v>
       </c>
-      <c r="S6" t="n">
-        <v>6.87</v>
-      </c>
-      <c r="T6" t="b">
-        <v>0</v>
-      </c>
-      <c r="U6" t="b">
-        <v>0</v>
-      </c>
       <c r="V6" t="n">
-        <v>5.69</v>
+        <v>-0.67</v>
       </c>
       <c r="W6" t="n">
-        <v>-4</v>
-      </c>
-      <c r="X6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="2" t="n">
-        <v>45952.41666666666</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>12</v>
-      </c>
-      <c r="AA6" t="inlineStr"/>
+        <v>5.03</v>
+      </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -1051,7 +1047,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1063,31 +1059,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45984.41666666666</v>
+        <v>45928.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45986.41666666666</v>
+        <v>45951.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>6.59</v>
+        <v>24.97</v>
       </c>
       <c r="G7" t="n">
-        <v>6.34</v>
+        <v>24.63</v>
       </c>
       <c r="H7" t="n">
-        <v>6.33</v>
+        <v>26.6</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.95</v>
+        <v>6.53</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K7" t="n">
-        <v>6.2</v>
+        <v>24.12</v>
       </c>
       <c r="L7" t="n">
-        <v>6.37</v>
+        <v>24.78</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1100,45 +1096,57 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>1101047</v>
+        <v>370152</v>
       </c>
       <c r="P7" t="n">
-        <v>3.94</v>
+        <v>1.38</v>
       </c>
       <c r="Q7" t="n">
-        <v>6.45</v>
+        <v>26.95</v>
       </c>
       <c r="R7" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>27.25</v>
+      </c>
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" t="b">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="W7" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="X7" t="b">
         <v>1</v>
       </c>
-      <c r="S7" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="T7" t="b">
-        <v>0</v>
-      </c>
-      <c r="U7" t="b">
+      <c r="Y7" s="2" t="n">
+        <v>45945.41666666666</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA7" t="b">
         <v>1</v>
       </c>
-      <c r="V7" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="W7" t="n">
-        <v>-2.12</v>
-      </c>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
+      <c r="AB7" s="2" t="n">
+        <v>45945.41666666666</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>12</v>
+      </c>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1150,31 +1158,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46007.41666666666</v>
+        <v>45952.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46019.41666666666</v>
+        <v>45963.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>6.46</v>
+        <v>27.25</v>
       </c>
       <c r="G8" t="n">
-        <v>6.22</v>
+        <v>26.6</v>
       </c>
       <c r="H8" t="n">
-        <v>6.82</v>
+        <v>27.08</v>
       </c>
       <c r="I8" t="n">
-        <v>5.57</v>
+        <v>-0.62</v>
       </c>
       <c r="J8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K8" t="n">
-        <v>6.13</v>
+        <v>26.5</v>
       </c>
       <c r="L8" t="n">
-        <v>6.25</v>
+        <v>27.09</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1187,45 +1195,57 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>1689563</v>
+        <v>1411464</v>
       </c>
       <c r="P8" t="n">
-        <v>3.86</v>
+        <v>2.44</v>
       </c>
       <c r="Q8" t="n">
-        <v>6.32</v>
+        <v>27.38</v>
       </c>
       <c r="R8" t="b">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>27.96</v>
+      </c>
+      <c r="T8" t="b">
+        <v>0</v>
+      </c>
+      <c r="U8" t="b">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="X8" t="b">
         <v>1</v>
       </c>
-      <c r="S8" t="n">
-        <v>6.28</v>
-      </c>
-      <c r="T8" t="b">
-        <v>0</v>
-      </c>
-      <c r="U8" t="b">
+      <c r="Y8" s="2" t="n">
+        <v>45958.41666666666</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA8" t="b">
         <v>1</v>
       </c>
-      <c r="V8" t="n">
-        <v>-2.79</v>
-      </c>
-      <c r="W8" t="n">
-        <v>-2.17</v>
-      </c>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
+      <c r="AB8" s="2" t="n">
+        <v>45957.41666666666</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>3</v>
+      </c>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1237,31 +1257,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46033.41666666666</v>
+        <v>45991.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>46035.41666666666</v>
+        <v>46007.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>7.06</v>
+        <v>25.79</v>
       </c>
       <c r="G9" t="n">
-        <v>7.03</v>
+        <v>25</v>
       </c>
       <c r="H9" t="n">
-        <v>6.7</v>
+        <v>25.53</v>
       </c>
       <c r="I9" t="n">
-        <v>-5.1</v>
+        <v>-1.01</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="K9" t="n">
-        <v>6.41</v>
+        <v>25.2</v>
       </c>
       <c r="L9" t="n">
-        <v>7.04</v>
+        <v>25.78</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1274,19 +1294,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>1647282</v>
+        <v>442438</v>
       </c>
       <c r="P9" t="n">
-        <v>0.43</v>
+        <v>2.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>7.25</v>
+        <v>25.06</v>
       </c>
       <c r="R9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>7.68</v>
+        <v>26.17</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1295,19 +1315,21 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>8.779999999999999</v>
+        <v>1.47</v>
       </c>
       <c r="W9" t="n">
-        <v>2.69</v>
+        <v>-2.83</v>
       </c>
       <c r="X9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="b">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>46000.41666666666</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
@@ -1316,7 +1338,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1328,31 +1350,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46055.41666666666</v>
+        <v>46012.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>46064.41666666666</v>
+        <v>46016.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>6.48</v>
+        <v>25.95</v>
       </c>
       <c r="G10" t="n">
-        <v>6.17</v>
+        <v>25.51</v>
       </c>
       <c r="H10" t="n">
-        <v>9.699999999999999</v>
+        <v>25.33</v>
       </c>
       <c r="I10" t="n">
-        <v>49.69</v>
+        <v>-2.39</v>
       </c>
       <c r="J10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>6.02</v>
+        <v>25.51</v>
       </c>
       <c r="L10" t="n">
-        <v>6.34</v>
+        <v>25.89</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1365,19 +1387,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>318660</v>
+        <v>197579</v>
       </c>
       <c r="P10" t="n">
-        <v>3.85</v>
+        <v>0.66</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.24</v>
+        <v>25.62</v>
       </c>
       <c r="R10" t="b">
         <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>6.54</v>
+        <v>26.84</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1386,20 +1408,16 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>0.93</v>
+        <v>3.43</v>
       </c>
       <c r="W10" t="n">
-        <v>-3.7</v>
+        <v>-1.27</v>
       </c>
       <c r="X10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="2" t="n">
-        <v>46056.41666666666</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
@@ -1409,7 +1427,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1421,170 +1439,77 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46071.41666666666</v>
+        <v>46056.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>46072.41666666666</v>
+        <v>46070.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>9.85</v>
+        <v>25.67</v>
       </c>
       <c r="G11" t="n">
-        <v>9.42</v>
+        <v>23.54</v>
       </c>
       <c r="H11" t="n">
-        <v>9.26</v>
+        <v>27.48</v>
       </c>
       <c r="I11" t="n">
-        <v>-5.99</v>
+        <v>7.05</v>
       </c>
       <c r="J11" t="n">
+        <v>14</v>
+      </c>
+      <c r="K11" t="n">
+        <v>23.44</v>
+      </c>
+      <c r="L11" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>1796699</v>
+      </c>
+      <c r="P11" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>24.37</v>
+      </c>
+      <c r="R11" t="b">
         <v>1</v>
       </c>
-      <c r="K11" t="n">
-        <v>9.41</v>
-      </c>
-      <c r="L11" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O11" t="n">
-        <v>4798270</v>
-      </c>
-      <c r="P11" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>10.36</v>
-      </c>
-      <c r="R11" t="b">
-        <v>0</v>
-      </c>
       <c r="S11" t="n">
-        <v>12.25</v>
+        <v>25.19</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
       </c>
       <c r="U11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>24.37</v>
+        <v>-1.87</v>
       </c>
       <c r="W11" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="X11" t="b">
-        <v>0</v>
-      </c>
+        <v>-5.06</v>
+      </c>
+      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="b">
-        <v>0</v>
-      </c>
+      <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>EPCO</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C12" t="b">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>46106.41666666666</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>46111.41666666666</v>
-      </c>
-      <c r="F12" t="n">
-        <v>9.02</v>
-      </c>
-      <c r="G12" t="n">
-        <v>8.390000000000001</v>
-      </c>
-      <c r="H12" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-7.87</v>
-      </c>
-      <c r="J12" t="n">
-        <v>5</v>
-      </c>
-      <c r="K12" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="L12" t="n">
-        <v>8.84</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O12" t="n">
-        <v>6893557</v>
-      </c>
-      <c r="P12" t="n">
-        <v>7.51</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="R12" t="b">
-        <v>1</v>
-      </c>
-      <c r="S12" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="T12" t="b">
-        <v>0</v>
-      </c>
-      <c r="U12" t="b">
-        <v>0</v>
-      </c>
-      <c r="V12" t="n">
-        <v>8.09</v>
-      </c>
-      <c r="W12" t="n">
-        <v>-6.76</v>
-      </c>
-      <c r="X12" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1760,7 +1685,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1772,31 +1697,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46127.41666666666</v>
+        <v>46128.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46128.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>8.74</v>
+        <v>26.3</v>
       </c>
       <c r="G2" t="n">
-        <v>8.539999999999999</v>
+        <v>25.03</v>
       </c>
       <c r="H2" t="n">
-        <v>9.140000000000001</v>
+        <v>26.3</v>
       </c>
       <c r="I2" t="n">
-        <v>4.58</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>8.31</v>
+        <v>23.35</v>
       </c>
       <c r="L2" t="n">
-        <v>8.609999999999999</v>
+        <v>25.91</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -1809,19 +1734,19 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>1437309</v>
+        <v>2038762</v>
       </c>
       <c r="P2" t="n">
-        <v>2.1</v>
+        <v>4.74</v>
       </c>
       <c r="Q2" t="n">
-        <v>8.57</v>
+        <v>26.8</v>
       </c>
       <c r="R2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>9.35</v>
+        <v>27.79</v>
       </c>
       <c r="T2" t="b">
         <v>0</v>
@@ -1830,25 +1755,23 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>6.98</v>
+        <v>5.67</v>
       </c>
       <c r="W2" t="n">
-        <v>-1.95</v>
+        <v>1.9</v>
       </c>
       <c r="X2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y2" s="2" t="n">
-        <v>46128.41666666666</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="b">
+        <v>0</v>
+      </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="n">
-        <v>9.140000000000001</v>
+        <v>26.3</v>
       </c>
       <c r="AE2" t="b">
         <v>0</v>
@@ -1978,7 +1901,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1987,55 +1910,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>36.36</v>
+        <v>30</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.68</v>
+        <v>-0.89</v>
       </c>
       <c r="H2" t="n">
-        <v>3.99</v>
+        <v>1.01</v>
       </c>
       <c r="I2" t="n">
-        <v>43.89</v>
+        <v>10.13</v>
       </c>
       <c r="J2" t="n">
-        <v>49.69</v>
+        <v>10.67</v>
       </c>
       <c r="K2" t="n">
-        <v>-7.87</v>
+        <v>-4.54</v>
       </c>
       <c r="L2" t="n">
-        <v>17.09</v>
+        <v>5.14</v>
       </c>
       <c r="M2" t="n">
-        <v>2.28</v>
+        <v>1.72</v>
       </c>
       <c r="N2" t="n">
-        <v>19.55</v>
+        <v>8.08</v>
       </c>
       <c r="O2" t="n">
-        <v>4.9</v>
+        <v>2.02</v>
       </c>
       <c r="P2" t="n">
-        <v>3.99</v>
+        <v>1.01</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4687197899391929</v>
+        <v>0.4517166123778502</v>
       </c>
       <c r="R2" t="n">
-        <v>0.14947</v>
+        <v>0.14479</v>
       </c>
       <c r="S2" t="n">
-        <v>0.2771699159756772</v>
+        <v>0.2675606449511401</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -2043,7 +1966,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.2771699159756772</v>
+        <v>0.2675606449511401</v>
       </c>
     </row>
   </sheetData>
@@ -2105,7 +2028,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EPCO</t>
+          <t>LCSW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2114,22 +2037,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>36.36</v>
+        <v>30</v>
       </c>
       <c r="F2" t="n">
-        <v>2.28</v>
+        <v>1.72</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.68</v>
+        <v>-0.89</v>
       </c>
       <c r="H2" t="n">
-        <v>3.99</v>
+        <v>1.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:29:38.180957
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AJ11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,10 +584,35 @@
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
+          <t>Stop_Loss</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Target_Price</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Risk_%</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Reward_%</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>RR_Ratio</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Current_Clears_Anchor</t>
         </is>
@@ -677,8 +702,23 @@
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AD2" t="n">
+        <v>25.81</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -776,8 +816,23 @@
       <c r="AC3" t="n">
         <v>5</v>
       </c>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AD3" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>-1.79</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -865,8 +920,23 @@
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AD4" t="n">
+        <v>24.79</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -952,8 +1022,23 @@
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
+      <c r="AD5" t="n">
+        <v>24.22</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>-4.42</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1041,8 +1126,23 @@
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
+      <c r="AD6" t="n">
+        <v>25.81</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>-1.34</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1140,8 +1240,23 @@
       <c r="AC7" t="n">
         <v>12</v>
       </c>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
+      <c r="AD7" t="n">
+        <v>24.57</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>24.78</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1239,8 +1354,23 @@
       <c r="AC8" t="n">
         <v>3</v>
       </c>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AD8" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>27.09</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>-0.21</v>
+      </c>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1332,8 +1462,23 @@
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
+      <c r="AD9" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>25.78</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1421,8 +1566,23 @@
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
+      <c r="AD10" t="n">
+        <v>25.47</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1508,8 +1668,23 @@
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr"/>
+      <c r="AD11" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>-4.95</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1522,7 +1697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AJ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1673,10 +1848,35 @@
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
+          <t>Stop_Loss</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Target_Price</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Risk_%</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Reward_%</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>RR_Ratio</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Current_Clears_Anchor</t>
         </is>
@@ -1771,9 +1971,24 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="n">
+        <v>24.89</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>25.91</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>-1.48</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="AI2" t="n">
         <v>26.3</v>
       </c>
-      <c r="AE2" t="b">
+      <c r="AJ2" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:34:26.716818
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -705,18 +705,12 @@
       <c r="AD2" t="n">
         <v>25.81</v>
       </c>
-      <c r="AE2" t="n">
-        <v>26.6</v>
-      </c>
+      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="n">
         <v>3.66</v>
       </c>
-      <c r="AG2" t="n">
-        <v>-0.71</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>-0.19</v>
-      </c>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
     </row>
@@ -820,16 +814,16 @@
         <v>22.4</v>
       </c>
       <c r="AE3" t="n">
-        <v>23.1</v>
+        <v>27.43</v>
       </c>
       <c r="AF3" t="n">
         <v>4.76</v>
       </c>
       <c r="AG3" t="n">
-        <v>-1.79</v>
+        <v>16.62</v>
       </c>
       <c r="AH3" t="n">
-        <v>-0.38</v>
+        <v>3.49</v>
       </c>
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
@@ -924,16 +918,16 @@
         <v>24.79</v>
       </c>
       <c r="AE4" t="n">
-        <v>25.69</v>
+        <v>26.64</v>
       </c>
       <c r="AF4" t="n">
         <v>3.69</v>
       </c>
       <c r="AG4" t="n">
-        <v>-0.19</v>
+        <v>3.5</v>
       </c>
       <c r="AH4" t="n">
-        <v>-0.05</v>
+        <v>0.95</v>
       </c>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
@@ -1025,18 +1019,12 @@
       <c r="AD5" t="n">
         <v>24.22</v>
       </c>
-      <c r="AE5" t="n">
-        <v>24.85</v>
-      </c>
+      <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="n">
         <v>6.85</v>
       </c>
-      <c r="AG5" t="n">
-        <v>-4.42</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>-0.65</v>
-      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
     </row>
@@ -1129,18 +1117,12 @@
       <c r="AD6" t="n">
         <v>25.81</v>
       </c>
-      <c r="AE6" t="n">
-        <v>26.5</v>
-      </c>
+      <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="n">
         <v>3.91</v>
       </c>
-      <c r="AG6" t="n">
-        <v>-1.34</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>-0.34</v>
-      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
     </row>
@@ -1244,16 +1226,16 @@
         <v>24.57</v>
       </c>
       <c r="AE7" t="n">
-        <v>24.78</v>
+        <v>27.25</v>
       </c>
       <c r="AF7" t="n">
         <v>1.6</v>
       </c>
       <c r="AG7" t="n">
-        <v>-0.76</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="AH7" t="n">
-        <v>-0.48</v>
+        <v>5.71</v>
       </c>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
@@ -1358,16 +1340,16 @@
         <v>26.5</v>
       </c>
       <c r="AE8" t="n">
-        <v>27.09</v>
+        <v>27.96</v>
       </c>
       <c r="AF8" t="n">
         <v>2.75</v>
       </c>
       <c r="AG8" t="n">
-        <v>-0.59</v>
+        <v>2.61</v>
       </c>
       <c r="AH8" t="n">
-        <v>-0.21</v>
+        <v>0.95</v>
       </c>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
@@ -1466,16 +1448,16 @@
         <v>24.7</v>
       </c>
       <c r="AE9" t="n">
-        <v>25.78</v>
+        <v>26.17</v>
       </c>
       <c r="AF9" t="n">
         <v>4.23</v>
       </c>
       <c r="AG9" t="n">
-        <v>-0.04</v>
+        <v>1.47</v>
       </c>
       <c r="AH9" t="n">
-        <v>-0.01</v>
+        <v>0.35</v>
       </c>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
@@ -1570,16 +1552,16 @@
         <v>25.47</v>
       </c>
       <c r="AE10" t="n">
-        <v>25.89</v>
+        <v>26.84</v>
       </c>
       <c r="AF10" t="n">
         <v>1.85</v>
       </c>
       <c r="AG10" t="n">
-        <v>-0.23</v>
+        <v>3.43</v>
       </c>
       <c r="AH10" t="n">
-        <v>-0.12</v>
+        <v>1.85</v>
       </c>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
@@ -1671,18 +1653,12 @@
       <c r="AD11" t="n">
         <v>23.2</v>
       </c>
-      <c r="AE11" t="n">
-        <v>24.4</v>
-      </c>
+      <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="n">
         <v>9.619999999999999</v>
       </c>
-      <c r="AG11" t="n">
-        <v>-4.95</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>-0.51</v>
-      </c>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
     </row>
@@ -1974,16 +1950,16 @@
         <v>24.89</v>
       </c>
       <c r="AE2" t="n">
-        <v>25.91</v>
+        <v>27.79</v>
       </c>
       <c r="AF2" t="n">
         <v>5.36</v>
       </c>
       <c r="AG2" t="n">
-        <v>-1.48</v>
+        <v>5.67</v>
       </c>
       <c r="AH2" t="n">
-        <v>-0.28</v>
+        <v>1.06</v>
       </c>
       <c r="AI2" t="n">
         <v>26.3</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:34:57.161998
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -703,11 +703,11 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="n">
-        <v>25.81</v>
+        <v>26</v>
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="n">
-        <v>3.66</v>
+        <v>2.95</v>
       </c>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr"/>
@@ -811,19 +811,19 @@
         <v>5</v>
       </c>
       <c r="AD3" t="n">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
       <c r="AE3" t="n">
         <v>27.43</v>
       </c>
       <c r="AF3" t="n">
-        <v>4.76</v>
+        <v>3.06</v>
       </c>
       <c r="AG3" t="n">
         <v>16.62</v>
       </c>
       <c r="AH3" t="n">
-        <v>3.49</v>
+        <v>5.43</v>
       </c>
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
@@ -915,19 +915,19 @@
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="n">
-        <v>24.79</v>
+        <v>25.49</v>
       </c>
       <c r="AE4" t="n">
         <v>26.64</v>
       </c>
       <c r="AF4" t="n">
-        <v>3.69</v>
+        <v>0.97</v>
       </c>
       <c r="AG4" t="n">
         <v>3.5</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.95</v>
+        <v>3.61</v>
       </c>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
@@ -1017,11 +1017,11 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="n">
-        <v>24.22</v>
+        <v>24.26</v>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="n">
-        <v>6.85</v>
+        <v>6.69</v>
       </c>
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
@@ -1115,11 +1115,11 @@
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="n">
-        <v>25.81</v>
+        <v>26.15</v>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="n">
-        <v>3.91</v>
+        <v>2.64</v>
       </c>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
@@ -1223,19 +1223,19 @@
         <v>12</v>
       </c>
       <c r="AD7" t="n">
-        <v>24.57</v>
+        <v>24.63</v>
       </c>
       <c r="AE7" t="n">
         <v>27.25</v>
       </c>
       <c r="AF7" t="n">
-        <v>1.6</v>
+        <v>1.36</v>
       </c>
       <c r="AG7" t="n">
         <v>9.130000000000001</v>
       </c>
       <c r="AH7" t="n">
-        <v>5.71</v>
+        <v>6.71</v>
       </c>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
@@ -1337,19 +1337,19 @@
         <v>3</v>
       </c>
       <c r="AD8" t="n">
-        <v>26.5</v>
+        <v>26.6</v>
       </c>
       <c r="AE8" t="n">
         <v>27.96</v>
       </c>
       <c r="AF8" t="n">
-        <v>2.75</v>
+        <v>2.39</v>
       </c>
       <c r="AG8" t="n">
         <v>2.61</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.95</v>
+        <v>1.09</v>
       </c>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
@@ -1445,19 +1445,19 @@
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
-        <v>24.7</v>
+        <v>25</v>
       </c>
       <c r="AE9" t="n">
         <v>26.17</v>
       </c>
       <c r="AF9" t="n">
-        <v>4.23</v>
+        <v>3.06</v>
       </c>
       <c r="AG9" t="n">
         <v>1.47</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.35</v>
+        <v>0.48</v>
       </c>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
@@ -1549,19 +1549,19 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
-        <v>25.47</v>
+        <v>25.51</v>
       </c>
       <c r="AE10" t="n">
         <v>26.84</v>
       </c>
       <c r="AF10" t="n">
-        <v>1.85</v>
+        <v>1.7</v>
       </c>
       <c r="AG10" t="n">
         <v>3.43</v>
       </c>
       <c r="AH10" t="n">
-        <v>1.85</v>
+        <v>2.02</v>
       </c>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
@@ -1651,11 +1651,11 @@
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="n">
-        <v>23.2</v>
+        <v>23.54</v>
       </c>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="n">
-        <v>9.619999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
@@ -1947,19 +1947,19 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="n">
-        <v>24.89</v>
+        <v>25.03</v>
       </c>
       <c r="AE2" t="n">
         <v>27.79</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.36</v>
+        <v>4.83</v>
       </c>
       <c r="AG2" t="n">
         <v>5.67</v>
       </c>
       <c r="AH2" t="n">
-        <v>1.06</v>
+        <v>1.17</v>
       </c>
       <c r="AI2" t="n">
         <v>26.3</v>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:39:34.690562
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -705,12 +705,18 @@
       <c r="AD2" t="n">
         <v>26</v>
       </c>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AE2" t="n">
+        <v>26.6</v>
+      </c>
       <c r="AF2" t="n">
         <v>2.95</v>
       </c>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
+      <c r="AG2" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>1</v>
+      </c>
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
     </row>
@@ -1019,12 +1025,18 @@
       <c r="AD5" t="n">
         <v>24.26</v>
       </c>
-      <c r="AE5" t="inlineStr"/>
+      <c r="AE5" t="n">
+        <v>24.85</v>
+      </c>
       <c r="AF5" t="n">
         <v>6.69</v>
       </c>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
+      <c r="AG5" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0.55</v>
+      </c>
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
     </row>
@@ -1117,12 +1129,18 @@
       <c r="AD6" t="n">
         <v>26.15</v>
       </c>
-      <c r="AE6" t="inlineStr"/>
+      <c r="AE6" t="n">
+        <v>26.5</v>
+      </c>
       <c r="AF6" t="n">
         <v>2.64</v>
       </c>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
+      <c r="AG6" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
     </row>
@@ -1653,12 +1671,18 @@
       <c r="AD11" t="n">
         <v>23.54</v>
       </c>
-      <c r="AE11" t="inlineStr"/>
+      <c r="AE11" t="n">
+        <v>24.4</v>
+      </c>
       <c r="AF11" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr"/>
+      <c r="AG11" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0.45</v>
+      </c>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:46:45.574011
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -706,7 +706,7 @@
         <v>26</v>
       </c>
       <c r="AE2" t="n">
-        <v>26.6</v>
+        <v>27.58</v>
       </c>
       <c r="AF2" t="n">
         <v>2.95</v>
@@ -1026,16 +1026,16 @@
         <v>24.26</v>
       </c>
       <c r="AE5" t="n">
-        <v>24.85</v>
+        <v>27.98</v>
       </c>
       <c r="AF5" t="n">
         <v>6.69</v>
       </c>
       <c r="AG5" t="n">
-        <v>3.65</v>
+        <v>7.62</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.55</v>
+        <v>1.14</v>
       </c>
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
@@ -1130,16 +1130,16 @@
         <v>26.15</v>
       </c>
       <c r="AE6" t="n">
-        <v>26.5</v>
+        <v>28.14</v>
       </c>
       <c r="AF6" t="n">
         <v>2.64</v>
       </c>
       <c r="AG6" t="n">
-        <v>4.1</v>
+        <v>4.77</v>
       </c>
       <c r="AH6" t="n">
-        <v>1.55</v>
+        <v>1.81</v>
       </c>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
@@ -1672,16 +1672,16 @@
         <v>23.54</v>
       </c>
       <c r="AE11" t="n">
-        <v>24.4</v>
+        <v>27.42</v>
       </c>
       <c r="AF11" t="n">
         <v>8.300000000000001</v>
       </c>
       <c r="AG11" t="n">
-        <v>3.74</v>
+        <v>6.82</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.45</v>
+        <v>0.82</v>
       </c>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:49:42.266901
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -696,7 +696,9 @@
       <c r="W2" t="n">
         <v>-0.71</v>
       </c>
-      <c r="X2" t="inlineStr"/>
+      <c r="X2" t="b">
+        <v>0</v>
+      </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
@@ -811,10 +813,10 @@
         <v>1</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>45840.41666666666</v>
+        <v>45838.41666666666</v>
       </c>
       <c r="AC3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AD3" t="n">
         <v>22.8</v>
@@ -1016,7 +1018,9 @@
       <c r="W5" t="n">
         <v>-4.96</v>
       </c>
-      <c r="X5" t="inlineStr"/>
+      <c r="X5" t="b">
+        <v>0</v>
+      </c>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
@@ -1118,7 +1122,9 @@
       <c r="W6" t="n">
         <v>5.03</v>
       </c>
-      <c r="X6" t="inlineStr"/>
+      <c r="X6" t="b">
+        <v>0</v>
+      </c>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="b">
@@ -1235,10 +1241,10 @@
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45945.41666666666</v>
+        <v>45944.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AD7" t="n">
         <v>24.63</v>
@@ -1349,10 +1355,10 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45957.41666666666</v>
+        <v>45953.41666666666</v>
       </c>
       <c r="AC8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD8" t="n">
         <v>26.6</v>
@@ -1662,9 +1668,15 @@
       <c r="W11" t="n">
         <v>-5.06</v>
       </c>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
+      <c r="X11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="2" t="n">
+        <v>46061.41666666666</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>3</v>
+      </c>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:51:59.743025
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -696,9 +696,7 @@
       <c r="W2" t="n">
         <v>-0.71</v>
       </c>
-      <c r="X2" t="b">
-        <v>0</v>
-      </c>
+      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
@@ -813,10 +811,10 @@
         <v>1</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>45838.41666666666</v>
+        <v>45840.41666666666</v>
       </c>
       <c r="AC3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AD3" t="n">
         <v>22.8</v>
@@ -1018,9 +1016,7 @@
       <c r="W5" t="n">
         <v>-4.96</v>
       </c>
-      <c r="X5" t="b">
-        <v>0</v>
-      </c>
+      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
@@ -1122,9 +1118,7 @@
       <c r="W6" t="n">
         <v>5.03</v>
       </c>
-      <c r="X6" t="b">
-        <v>0</v>
-      </c>
+      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="b">
@@ -1241,10 +1235,10 @@
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45944.41666666666</v>
+        <v>45945.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AD7" t="n">
         <v>24.63</v>
@@ -1355,10 +1349,10 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45953.41666666666</v>
+        <v>45957.41666666666</v>
       </c>
       <c r="AC8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD8" t="n">
         <v>26.6</v>
@@ -1668,15 +1662,9 @@
       <c r="W11" t="n">
         <v>-5.06</v>
       </c>
-      <c r="X11" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y11" s="2" t="n">
-        <v>46061.41666666666</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3</v>
-      </c>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:52:29.629890
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -798,15 +798,9 @@
       <c r="W3" t="n">
         <v>9.99</v>
       </c>
-      <c r="X3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y3" s="2" t="n">
-        <v>45844.41666666666</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>6</v>
-      </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="b">
         <v>1</v>
       </c>
@@ -912,9 +906,7 @@
       <c r="W4" t="n">
         <v>-2.45</v>
       </c>
-      <c r="X4" t="b">
-        <v>0</v>
-      </c>
+      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
@@ -1222,15 +1214,9 @@
       <c r="W7" t="n">
         <v>7.93</v>
       </c>
-      <c r="X7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="2" t="n">
-        <v>45945.41666666666</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>12</v>
-      </c>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
@@ -1336,15 +1322,9 @@
       <c r="W8" t="n">
         <v>0.48</v>
       </c>
-      <c r="X8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y8" s="2" t="n">
-        <v>45958.41666666666</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>4</v>
-      </c>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="b">
         <v>1</v>
       </c>
@@ -1450,15 +1430,9 @@
       <c r="W9" t="n">
         <v>-2.83</v>
       </c>
-      <c r="X9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="2" t="n">
-        <v>46000.41666666666</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>7</v>
-      </c>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -1558,9 +1532,7 @@
       <c r="W10" t="n">
         <v>-1.27</v>
       </c>
-      <c r="X10" t="b">
-        <v>0</v>
-      </c>
+      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:52:47.786208
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -696,7 +696,9 @@
       <c r="W2" t="n">
         <v>-0.71</v>
       </c>
-      <c r="X2" t="inlineStr"/>
+      <c r="X2" t="b">
+        <v>0</v>
+      </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
@@ -1008,7 +1010,9 @@
       <c r="W5" t="n">
         <v>-4.96</v>
       </c>
-      <c r="X5" t="inlineStr"/>
+      <c r="X5" t="b">
+        <v>0</v>
+      </c>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
@@ -1110,7 +1114,9 @@
       <c r="W6" t="n">
         <v>5.03</v>
       </c>
-      <c r="X6" t="inlineStr"/>
+      <c r="X6" t="b">
+        <v>0</v>
+      </c>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="b">
@@ -1634,9 +1640,15 @@
       <c r="W11" t="n">
         <v>-5.06</v>
       </c>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
+      <c r="X11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="2" t="n">
+        <v>46061.41666666666</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>3</v>
+      </c>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:53:50.246828
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -800,9 +800,15 @@
       <c r="W3" t="n">
         <v>9.99</v>
       </c>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
+      <c r="X3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>45844.41666666666</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>6</v>
+      </c>
       <c r="AA3" t="b">
         <v>1</v>
       </c>
@@ -908,7 +914,9 @@
       <c r="W4" t="n">
         <v>-2.45</v>
       </c>
-      <c r="X4" t="inlineStr"/>
+      <c r="X4" t="b">
+        <v>0</v>
+      </c>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
@@ -1220,9 +1228,15 @@
       <c r="W7" t="n">
         <v>7.93</v>
       </c>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+      <c r="X7" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>45945.41666666666</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>12</v>
+      </c>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
@@ -1328,9 +1342,15 @@
       <c r="W8" t="n">
         <v>0.48</v>
       </c>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
+      <c r="X8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="2" t="n">
+        <v>45958.41666666666</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>4</v>
+      </c>
       <c r="AA8" t="b">
         <v>1</v>
       </c>
@@ -1436,9 +1456,15 @@
       <c r="W9" t="n">
         <v>-2.83</v>
       </c>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
+      <c r="X9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>46000.41666666666</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>7</v>
+      </c>
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -1538,7 +1564,9 @@
       <c r="W10" t="n">
         <v>-1.27</v>
       </c>
-      <c r="X10" t="inlineStr"/>
+      <c r="X10" t="b">
+        <v>0</v>
+      </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-18 16:55:56.441984
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -701,9 +701,15 @@
       </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+      <c r="AA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="2" t="n">
+        <v>45811.41666666666</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
       <c r="AD2" t="n">
         <v>26</v>
       </c>
@@ -919,9 +925,15 @@
       </c>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AA4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="2" t="n">
+        <v>45872.41666666666</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD4" t="n">
         <v>25.49</v>
       </c>
@@ -1023,9 +1035,15 @@
       </c>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
+      <c r="AA5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="2" t="n">
+        <v>45893.41666666666</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
       <c r="AD5" t="n">
         <v>24.26</v>
       </c>
@@ -1465,9 +1483,15 @@
       <c r="Z9" t="n">
         <v>7</v>
       </c>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+      <c r="AA9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2" t="n">
+        <v>45991.41666666666</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0</v>
+      </c>
       <c r="AD9" t="n">
         <v>25</v>
       </c>
@@ -1569,9 +1593,15 @@
       </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB10" s="2" t="n">
+        <v>46012.41666666666</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
       <c r="AD10" t="n">
         <v>25.51</v>
       </c>
@@ -1677,9 +1707,15 @@
       <c r="Z11" t="n">
         <v>3</v>
       </c>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
+      <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB11" s="2" t="n">
+        <v>46056.41666666666</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0</v>
+      </c>
       <c r="AD11" t="n">
         <v>23.54</v>
       </c>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:02:54.594439
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Closed_Trades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Strategy_Profile" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Best_Strategy_Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="refresh_date" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Open_Trades" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Strategy_Profile" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Best_Strategy_Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="refresh_date" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI24"/>
+  <dimension ref="A1:AK27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -611,11 +612,21 @@
           <t>RR_Ratio</t>
         </is>
       </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Current_Price</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Current_Clears_Anchor</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -627,31 +638,31 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45295.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>45322.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>13.43</v>
+        <v>51.31</v>
       </c>
       <c r="G2" t="n">
-        <v>12.66</v>
+        <v>45.11</v>
       </c>
       <c r="H2" t="n">
-        <v>13.26</v>
+        <v>44</v>
       </c>
       <c r="I2" t="n">
-        <v>-1.25</v>
+        <v>-14.25</v>
       </c>
       <c r="J2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K2" t="n">
-        <v>12.54</v>
+        <v>46</v>
       </c>
       <c r="L2" t="n">
-        <v>13.42</v>
+        <v>48</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -664,19 +675,19 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>3180532</v>
+        <v>103663</v>
       </c>
       <c r="P2" t="n">
-        <v>3.32</v>
+        <v>10.11</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.98</v>
+        <v>48</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>13.42</v>
+        <v>48</v>
       </c>
       <c r="T2" t="b">
         <v>0</v>
@@ -685,40 +696,40 @@
         <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>-0.09</v>
+        <v>-6.45</v>
       </c>
       <c r="W2" t="n">
-        <v>-3.37</v>
+        <v>-6.45</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45313.41666666666</v>
+        <v>45295.41666666666</v>
       </c>
       <c r="Z2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45295.41666666666</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>12.66</v>
+        <v>45.11</v>
       </c>
       <c r="AE2" t="n">
-        <v>14.32</v>
+        <v>53.31</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.78</v>
+        <v>12.08</v>
       </c>
       <c r="AG2" t="n">
-        <v>6.61</v>
+        <v>3.9</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
@@ -726,13 +737,15 @@
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>1.14</v>
-      </c>
+        <v>0.32</v>
+      </c>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -741,34 +754,34 @@
         </is>
       </c>
       <c r="C3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45340.41666666666</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45347.41666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>15.59</v>
+        <v>50.52</v>
       </c>
       <c r="G3" t="n">
-        <v>13.66</v>
+        <v>45.03</v>
       </c>
       <c r="H3" t="n">
-        <v>16</v>
+        <v>51.12</v>
       </c>
       <c r="I3" t="n">
-        <v>2.62</v>
+        <v>1.19</v>
       </c>
       <c r="J3" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="K3" t="n">
-        <v>12.64</v>
+        <v>44</v>
       </c>
       <c r="L3" t="n">
-        <v>14.56</v>
+        <v>49.75</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -781,75 +794,77 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>708583</v>
+        <v>92034</v>
       </c>
       <c r="P3" t="n">
-        <v>10.05</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>13.78</v>
+        <v>47.53</v>
       </c>
       <c r="R3" t="b">
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>15.04</v>
+        <v>52.6</v>
       </c>
       <c r="T3" t="b">
         <v>0</v>
       </c>
       <c r="U3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>-3.54</v>
+        <v>4.12</v>
       </c>
       <c r="W3" t="n">
-        <v>-11.62</v>
+        <v>-5.92</v>
       </c>
       <c r="X3" t="b">
         <v>1</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>45336.41666666666</v>
+        <v>45341.41666666666</v>
       </c>
       <c r="Z3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45340.41666666666</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
       </c>
       <c r="AD3" t="n">
-        <v>13.66</v>
+        <v>45.03</v>
       </c>
       <c r="AE3" t="n">
-        <v>17.99</v>
+        <v>52.6</v>
       </c>
       <c r="AF3" t="n">
-        <v>12.37</v>
+        <v>10.87</v>
       </c>
       <c r="AG3" t="n">
-        <v>15.39</v>
+        <v>4.12</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>1.24</v>
-      </c>
+        <v>0.38</v>
+      </c>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -861,31 +876,31 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45489.41666666666</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>45379.41666666666</v>
+        <v>45543.41666666666</v>
       </c>
       <c r="F4" t="n">
-        <v>15.92</v>
+        <v>39.11</v>
       </c>
       <c r="G4" t="n">
-        <v>14.54</v>
+        <v>33.5</v>
       </c>
       <c r="H4" t="n">
-        <v>14.11</v>
+        <v>43.99</v>
       </c>
       <c r="I4" t="n">
-        <v>-11.36</v>
+        <v>12.48</v>
       </c>
       <c r="J4" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="K4" t="n">
-        <v>14.54</v>
+        <v>30.03</v>
       </c>
       <c r="L4" t="n">
-        <v>15.68</v>
+        <v>37.5</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -898,61 +913,61 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>2359660</v>
+        <v>69611</v>
       </c>
       <c r="P4" t="n">
-        <v>3.65</v>
+        <v>12.94</v>
       </c>
       <c r="Q4" t="n">
-        <v>15.3</v>
+        <v>34.74</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>16.22</v>
+        <v>40.29</v>
       </c>
       <c r="T4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U4" t="b">
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>1.88</v>
+        <v>3.02</v>
       </c>
       <c r="W4" t="n">
-        <v>-3.89</v>
+        <v>-11.17</v>
       </c>
       <c r="X4" t="b">
         <v>1</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45494.41666666666</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45489.41666666666</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
       </c>
       <c r="AD4" t="n">
-        <v>14.54</v>
+        <v>33.5</v>
       </c>
       <c r="AE4" t="n">
-        <v>16.22</v>
+        <v>40.29</v>
       </c>
       <c r="AF4" t="n">
-        <v>8.69</v>
+        <v>14.34</v>
       </c>
       <c r="AG4" t="n">
-        <v>1.91</v>
+        <v>3.02</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
@@ -960,8 +975,10 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.22</v>
-      </c>
+        <v>0.21</v>
+      </c>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -975,34 +992,34 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>13.08</v>
+        <v>13.43</v>
       </c>
       <c r="G5" t="n">
-        <v>12.76</v>
+        <v>12.66</v>
       </c>
       <c r="H5" t="n">
-        <v>12.39</v>
+        <v>13.26</v>
       </c>
       <c r="I5" t="n">
-        <v>-5.26</v>
+        <v>-1.25</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="K5" t="n">
-        <v>12.22</v>
+        <v>12.54</v>
       </c>
       <c r="L5" t="n">
-        <v>13.04</v>
+        <v>13.42</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1015,66 +1032,72 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>5618577</v>
+        <v>3180532</v>
       </c>
       <c r="P5" t="n">
-        <v>2.06</v>
+        <v>3.32</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.72</v>
+        <v>12.98</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>14.15</v>
+        <v>13.42</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
       </c>
       <c r="U5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>8.18</v>
+        <v>-0.09</v>
       </c>
       <c r="W5" t="n">
-        <v>-2.75</v>
+        <v>-3.37</v>
       </c>
       <c r="X5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>45313.41666666666</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>8</v>
+      </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>12.76</v>
+        <v>12.66</v>
       </c>
       <c r="AE5" t="n">
-        <v>14.15</v>
+        <v>14.32</v>
       </c>
       <c r="AF5" t="n">
-        <v>2.45</v>
+        <v>5.78</v>
       </c>
       <c r="AG5" t="n">
-        <v>8.199999999999999</v>
+        <v>6.61</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>3.35</v>
-      </c>
+        <v>1.14</v>
+      </c>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1088,34 +1111,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>11.44</v>
+        <v>15.59</v>
       </c>
       <c r="G6" t="n">
-        <v>10.23</v>
+        <v>13.66</v>
       </c>
       <c r="H6" t="n">
-        <v>11.76</v>
+        <v>16</v>
       </c>
       <c r="I6" t="n">
-        <v>2.8</v>
+        <v>2.62</v>
       </c>
       <c r="J6" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="K6" t="n">
-        <v>10.01</v>
+        <v>12.64</v>
       </c>
       <c r="L6" t="n">
-        <v>11.2</v>
+        <v>14.56</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1128,62 +1151,72 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>3697242</v>
+        <v>708583</v>
       </c>
       <c r="P6" t="n">
-        <v>10</v>
+        <v>10.05</v>
       </c>
       <c r="Q6" t="n">
-        <v>13.1</v>
+        <v>13.78</v>
       </c>
       <c r="R6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>13.42</v>
+        <v>15.04</v>
       </c>
       <c r="T6" t="b">
         <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>17.31</v>
+        <v>-3.54</v>
       </c>
       <c r="W6" t="n">
-        <v>14.51</v>
+        <v>-11.62</v>
       </c>
       <c r="X6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>45336.41666666666</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>8</v>
+      </c>
       <c r="AA6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB6" s="2" t="n">
+        <v>45326.41666666666</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
       <c r="AD6" t="n">
-        <v>10.23</v>
+        <v>13.66</v>
       </c>
       <c r="AE6" t="n">
-        <v>13.42</v>
+        <v>17.99</v>
       </c>
       <c r="AF6" t="n">
-        <v>10.56</v>
+        <v>12.37</v>
       </c>
       <c r="AG6" t="n">
-        <v>17.34</v>
+        <v>15.39</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>1.64</v>
-      </c>
+        <v>1.24</v>
+      </c>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1200,31 +1233,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45434.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>12.1</v>
+        <v>15.92</v>
       </c>
       <c r="G7" t="n">
-        <v>11.68</v>
+        <v>14.54</v>
       </c>
       <c r="H7" t="n">
-        <v>12.4</v>
+        <v>14.11</v>
       </c>
       <c r="I7" t="n">
-        <v>2.51</v>
+        <v>-11.36</v>
       </c>
       <c r="J7" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>11.68</v>
+        <v>14.54</v>
       </c>
       <c r="L7" t="n">
-        <v>12.08</v>
+        <v>15.68</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1237,61 +1270,61 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>719120</v>
+        <v>2359660</v>
       </c>
       <c r="P7" t="n">
-        <v>2.86</v>
+        <v>3.65</v>
       </c>
       <c r="Q7" t="n">
-        <v>11.92</v>
+        <v>15.3</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>12.39</v>
+        <v>16.22</v>
       </c>
       <c r="T7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>2.43</v>
+        <v>1.88</v>
       </c>
       <c r="W7" t="n">
-        <v>-1.46</v>
+        <v>-3.89</v>
       </c>
       <c r="X7" t="b">
         <v>1</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>45426.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="Z7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="AC7" t="n">
         <v>0</v>
       </c>
       <c r="AD7" t="n">
-        <v>11.68</v>
+        <v>14.54</v>
       </c>
       <c r="AE7" t="n">
-        <v>12.39</v>
+        <v>16.22</v>
       </c>
       <c r="AF7" t="n">
-        <v>3.44</v>
+        <v>8.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>2.45</v>
+        <v>1.91</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1299,8 +1332,10 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.71</v>
-      </c>
+        <v>0.22</v>
+      </c>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1317,31 +1352,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>13.23</v>
+        <v>13.08</v>
       </c>
       <c r="G8" t="n">
-        <v>12.37</v>
+        <v>12.76</v>
       </c>
       <c r="H8" t="n">
-        <v>15.11</v>
+        <v>12.39</v>
       </c>
       <c r="I8" t="n">
-        <v>14.21</v>
+        <v>-5.26</v>
       </c>
       <c r="J8" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>12.37</v>
+        <v>12.22</v>
       </c>
       <c r="L8" t="n">
-        <v>12.68</v>
+        <v>13.04</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1354,70 +1389,68 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>2872871</v>
+        <v>5618577</v>
       </c>
       <c r="P8" t="n">
-        <v>4.75</v>
+        <v>2.06</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.61</v>
+        <v>12.72</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>13.12</v>
+        <v>14.15</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
       </c>
       <c r="U8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.85</v>
+        <v>8.18</v>
       </c>
       <c r="W8" t="n">
-        <v>-4.7</v>
+        <v>-2.75</v>
       </c>
       <c r="X8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y8" s="2" t="n">
-        <v>45454.41666666666</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="b">
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>12.37</v>
+        <v>12.76</v>
       </c>
       <c r="AE8" t="n">
-        <v>13.98</v>
+        <v>14.15</v>
       </c>
       <c r="AF8" t="n">
-        <v>6.53</v>
+        <v>2.45</v>
       </c>
       <c r="AG8" t="n">
-        <v>5.68</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>0.87</v>
-      </c>
+        <v>3.35</v>
+      </c>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1434,31 +1467,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>17.1</v>
+        <v>11.44</v>
       </c>
       <c r="G9" t="n">
-        <v>14.96</v>
+        <v>10.23</v>
       </c>
       <c r="H9" t="n">
-        <v>19.46</v>
+        <v>11.76</v>
       </c>
       <c r="I9" t="n">
-        <v>13.85</v>
+        <v>2.8</v>
       </c>
       <c r="J9" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="K9" t="n">
-        <v>14.96</v>
+        <v>10.01</v>
       </c>
       <c r="L9" t="n">
-        <v>15.28</v>
+        <v>11.2</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1471,70 +1504,64 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>2885185</v>
+        <v>3697242</v>
       </c>
       <c r="P9" t="n">
-        <v>13.79</v>
+        <v>10</v>
       </c>
       <c r="Q9" t="n">
-        <v>15.44</v>
+        <v>13.1</v>
       </c>
       <c r="R9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>15.5</v>
+        <v>13.42</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
       </c>
       <c r="U9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>-9.34</v>
+        <v>17.31</v>
       </c>
       <c r="W9" t="n">
-        <v>-9.69</v>
+        <v>14.51</v>
       </c>
       <c r="X9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="2" t="n">
-        <v>45503.41666666666</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB9" s="2" t="n">
-        <v>45503.41666666666</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
-        <v>14.96</v>
+        <v>10.23</v>
       </c>
       <c r="AE9" t="n">
-        <v>17.64</v>
+        <v>13.42</v>
       </c>
       <c r="AF9" t="n">
-        <v>12.49</v>
+        <v>10.56</v>
       </c>
       <c r="AG9" t="n">
-        <v>3.18</v>
+        <v>17.34</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.25</v>
-      </c>
+        <v>1.64</v>
+      </c>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1551,31 +1578,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>20.68</v>
+        <v>12.1</v>
       </c>
       <c r="G10" t="n">
-        <v>18.4</v>
+        <v>11.68</v>
       </c>
       <c r="H10" t="n">
-        <v>28.62</v>
+        <v>12.4</v>
       </c>
       <c r="I10" t="n">
-        <v>38.41</v>
+        <v>2.51</v>
       </c>
       <c r="J10" t="n">
-        <v>185</v>
+        <v>9</v>
       </c>
       <c r="K10" t="n">
-        <v>18.4</v>
+        <v>11.68</v>
       </c>
       <c r="L10" t="n">
-        <v>20.24</v>
+        <v>12.08</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1588,19 +1615,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>807277</v>
+        <v>719120</v>
       </c>
       <c r="P10" t="n">
-        <v>2.17</v>
+        <v>2.86</v>
       </c>
       <c r="Q10" t="n">
-        <v>20.54</v>
+        <v>11.92</v>
       </c>
       <c r="R10" t="b">
         <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>23.04</v>
+        <v>12.39</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1609,40 +1636,40 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>11.41</v>
+        <v>2.43</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.68</v>
+        <v>-1.46</v>
       </c>
       <c r="X10" t="b">
         <v>1</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>45572.41666666666</v>
+        <v>45426.41666666666</v>
       </c>
       <c r="Z10" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="AC10" t="n">
         <v>0</v>
       </c>
       <c r="AD10" t="n">
-        <v>18.4</v>
+        <v>11.68</v>
       </c>
       <c r="AE10" t="n">
-        <v>23.04</v>
+        <v>12.39</v>
       </c>
       <c r="AF10" t="n">
-        <v>11.03</v>
+        <v>3.44</v>
       </c>
       <c r="AG10" t="n">
-        <v>11.41</v>
+        <v>2.45</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -1650,8 +1677,10 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>1.03</v>
-      </c>
+        <v>0.71</v>
+      </c>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1668,31 +1697,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>28.64</v>
+        <v>13.23</v>
       </c>
       <c r="G11" t="n">
-        <v>28.08</v>
+        <v>12.37</v>
       </c>
       <c r="H11" t="n">
-        <v>27.22</v>
+        <v>15.11</v>
       </c>
       <c r="I11" t="n">
-        <v>-4.97</v>
+        <v>14.21</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="K11" t="n">
-        <v>28</v>
+        <v>12.37</v>
       </c>
       <c r="L11" t="n">
-        <v>28.48</v>
+        <v>12.68</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1705,70 +1734,72 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>1546271</v>
+        <v>2872871</v>
       </c>
       <c r="P11" t="n">
-        <v>1.79</v>
+        <v>4.75</v>
       </c>
       <c r="Q11" t="n">
-        <v>28.16</v>
+        <v>12.61</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>29</v>
+        <v>13.12</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
       </c>
       <c r="U11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>1.26</v>
+        <v>-0.85</v>
       </c>
       <c r="W11" t="n">
-        <v>-1.68</v>
+        <v>-4.7</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45454.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>28.08</v>
+        <v>12.37</v>
       </c>
       <c r="AE11" t="n">
-        <v>29</v>
+        <v>13.98</v>
       </c>
       <c r="AF11" t="n">
-        <v>1.96</v>
+        <v>6.53</v>
       </c>
       <c r="AG11" t="n">
-        <v>1.26</v>
+        <v>5.68</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.64</v>
-      </c>
+        <v>0.87</v>
+      </c>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1785,31 +1816,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45756.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>25.97</v>
+        <v>17.1</v>
       </c>
       <c r="G12" t="n">
-        <v>24.72</v>
+        <v>14.96</v>
       </c>
       <c r="H12" t="n">
-        <v>24.16</v>
+        <v>19.46</v>
       </c>
       <c r="I12" t="n">
-        <v>-6.96</v>
+        <v>13.85</v>
       </c>
       <c r="J12" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="K12" t="n">
-        <v>24.68</v>
+        <v>14.96</v>
       </c>
       <c r="L12" t="n">
-        <v>25.51</v>
+        <v>15.28</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1822,62 +1853,72 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>767605</v>
+        <v>2885185</v>
       </c>
       <c r="P12" t="n">
-        <v>4.04</v>
+        <v>13.79</v>
       </c>
       <c r="Q12" t="n">
-        <v>27.46</v>
+        <v>15.44</v>
       </c>
       <c r="R12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>29.03</v>
+        <v>15.5</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
       </c>
       <c r="U12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>11.79</v>
+        <v>-9.34</v>
       </c>
       <c r="W12" t="n">
-        <v>5.75</v>
+        <v>-9.69</v>
       </c>
       <c r="X12" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y12" s="2" t="n">
+        <v>45503.41666666666</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
       <c r="AA12" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB12" s="2" t="n">
+        <v>45503.41666666666</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0</v>
+      </c>
       <c r="AD12" t="n">
-        <v>24.72</v>
+        <v>14.96</v>
       </c>
       <c r="AE12" t="n">
-        <v>29.03</v>
+        <v>17.64</v>
       </c>
       <c r="AF12" t="n">
-        <v>4.81</v>
+        <v>12.49</v>
       </c>
       <c r="AG12" t="n">
-        <v>11.8</v>
+        <v>3.18</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>2.45</v>
-      </c>
+        <v>0.25</v>
+      </c>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1894,31 +1935,31 @@
         <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45783.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>25.32</v>
+        <v>20.68</v>
       </c>
       <c r="G13" t="n">
-        <v>24.12</v>
+        <v>18.4</v>
       </c>
       <c r="H13" t="n">
-        <v>23.99</v>
+        <v>28.62</v>
       </c>
       <c r="I13" t="n">
-        <v>-5.24</v>
+        <v>38.41</v>
       </c>
       <c r="J13" t="n">
-        <v>23</v>
+        <v>185</v>
       </c>
       <c r="K13" t="n">
-        <v>24.12</v>
+        <v>18.4</v>
       </c>
       <c r="L13" t="n">
-        <v>25.26</v>
+        <v>20.24</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1931,19 +1972,19 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>623052</v>
+        <v>807277</v>
       </c>
       <c r="P13" t="n">
-        <v>0.96</v>
+        <v>2.17</v>
       </c>
       <c r="Q13" t="n">
-        <v>26.96</v>
+        <v>20.54</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>26.96</v>
+        <v>23.04</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
@@ -1952,32 +1993,40 @@
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>6.48</v>
+        <v>11.41</v>
       </c>
       <c r="W13" t="n">
-        <v>6.48</v>
+        <v>-0.68</v>
       </c>
       <c r="X13" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y13" s="2" t="n">
+        <v>45572.41666666666</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>28</v>
+      </c>
       <c r="AA13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB13" s="2" t="n">
+        <v>45530.41666666666</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0</v>
+      </c>
       <c r="AD13" t="n">
-        <v>24.12</v>
+        <v>18.4</v>
       </c>
       <c r="AE13" t="n">
-        <v>26.96</v>
+        <v>23.04</v>
       </c>
       <c r="AF13" t="n">
-        <v>4.74</v>
+        <v>11.03</v>
       </c>
       <c r="AG13" t="n">
-        <v>6.48</v>
+        <v>11.41</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
@@ -1985,8 +2034,10 @@
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.37</v>
-      </c>
+        <v>1.03</v>
+      </c>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2003,31 +2054,31 @@
         <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>22.75</v>
+        <v>28.64</v>
       </c>
       <c r="G14" t="n">
-        <v>21.66</v>
+        <v>28.08</v>
       </c>
       <c r="H14" t="n">
-        <v>21.65</v>
+        <v>27.22</v>
       </c>
       <c r="I14" t="n">
-        <v>-4.85</v>
+        <v>-4.97</v>
       </c>
       <c r="J14" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>21.66</v>
+        <v>28</v>
       </c>
       <c r="L14" t="n">
-        <v>22.2</v>
+        <v>28.48</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2040,19 +2091,19 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>13689820</v>
+        <v>1546271</v>
       </c>
       <c r="P14" t="n">
-        <v>4.94</v>
+        <v>1.79</v>
       </c>
       <c r="Q14" t="n">
-        <v>23.7</v>
+        <v>28.16</v>
       </c>
       <c r="R14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>25.75</v>
+        <v>29</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
@@ -2061,32 +2112,40 @@
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>13.18</v>
+        <v>1.26</v>
       </c>
       <c r="W14" t="n">
-        <v>4.17</v>
+        <v>-1.68</v>
       </c>
       <c r="X14" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y14" s="2" t="n">
+        <v>45729.41666666666</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>1</v>
+      </c>
       <c r="AA14" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB14" s="2" t="n">
+        <v>45728.41666666666</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>0</v>
+      </c>
       <c r="AD14" t="n">
-        <v>21.66</v>
+        <v>28.08</v>
       </c>
       <c r="AE14" t="n">
-        <v>25.75</v>
+        <v>29</v>
       </c>
       <c r="AF14" t="n">
-        <v>4.78</v>
+        <v>1.96</v>
       </c>
       <c r="AG14" t="n">
-        <v>13.19</v>
+        <v>1.26</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
@@ -2094,8 +2153,10 @@
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>2.76</v>
-      </c>
+        <v>0.64</v>
+      </c>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2112,31 +2173,31 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>45756.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>21.88</v>
+        <v>25.97</v>
       </c>
       <c r="G15" t="n">
-        <v>21.35</v>
+        <v>24.72</v>
       </c>
       <c r="H15" t="n">
-        <v>20.53</v>
+        <v>24.16</v>
       </c>
       <c r="I15" t="n">
-        <v>-6.18</v>
+        <v>-6.96</v>
       </c>
       <c r="J15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K15" t="n">
-        <v>21.35</v>
+        <v>24.68</v>
       </c>
       <c r="L15" t="n">
-        <v>21.78</v>
+        <v>25.51</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2149,19 +2210,19 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>1476660</v>
+        <v>767605</v>
       </c>
       <c r="P15" t="n">
-        <v>1.3</v>
+        <v>4.04</v>
       </c>
       <c r="Q15" t="n">
-        <v>21.54</v>
+        <v>27.46</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>22.52</v>
+        <v>29.03</v>
       </c>
       <c r="T15" t="b">
         <v>0</v>
@@ -2170,40 +2231,32 @@
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>2.93</v>
+        <v>11.79</v>
       </c>
       <c r="W15" t="n">
-        <v>-1.55</v>
+        <v>5.75</v>
       </c>
       <c r="X15" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y15" s="2" t="n">
-        <v>45818.41666666666</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB15" s="2" t="n">
-        <v>45811.41666666666</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="n">
-        <v>21.35</v>
+        <v>24.72</v>
       </c>
       <c r="AE15" t="n">
-        <v>22.52</v>
+        <v>29.03</v>
       </c>
       <c r="AF15" t="n">
-        <v>2.41</v>
+        <v>4.81</v>
       </c>
       <c r="AG15" t="n">
-        <v>2.93</v>
+        <v>11.8</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2211,8 +2264,10 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>1.22</v>
-      </c>
+        <v>2.45</v>
+      </c>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2229,31 +2284,31 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>21.16</v>
+        <v>25.32</v>
       </c>
       <c r="G16" t="n">
-        <v>19.2</v>
+        <v>24.12</v>
       </c>
       <c r="H16" t="n">
-        <v>21.32</v>
+        <v>23.99</v>
       </c>
       <c r="I16" t="n">
-        <v>0.76</v>
+        <v>-5.24</v>
       </c>
       <c r="J16" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="K16" t="n">
-        <v>19.92</v>
+        <v>24.12</v>
       </c>
       <c r="L16" t="n">
-        <v>20.64</v>
+        <v>25.26</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2266,19 +2321,19 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>5666121</v>
+        <v>623052</v>
       </c>
       <c r="P16" t="n">
-        <v>4.75</v>
+        <v>0.96</v>
       </c>
       <c r="Q16" t="n">
-        <v>22.02</v>
+        <v>26.96</v>
       </c>
       <c r="R16" t="b">
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>22.52</v>
+        <v>26.96</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2287,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>6.43</v>
+        <v>6.48</v>
       </c>
       <c r="W16" t="n">
-        <v>4.06</v>
+        <v>6.48</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -2298,25 +2353,21 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB16" s="2" t="n">
-        <v>45833.41666666666</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="n">
-        <v>19.2</v>
+        <v>24.12</v>
       </c>
       <c r="AE16" t="n">
-        <v>22.52</v>
+        <v>26.96</v>
       </c>
       <c r="AF16" t="n">
-        <v>9.26</v>
+        <v>4.74</v>
       </c>
       <c r="AG16" t="n">
-        <v>6.43</v>
+        <v>6.48</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2324,8 +2375,10 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.6899999999999999</v>
-      </c>
+        <v>1.37</v>
+      </c>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2342,31 +2395,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45845.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>21.91</v>
+        <v>22.75</v>
       </c>
       <c r="G17" t="n">
-        <v>21.28</v>
+        <v>21.66</v>
       </c>
       <c r="H17" t="n">
-        <v>22.48</v>
+        <v>21.65</v>
       </c>
       <c r="I17" t="n">
-        <v>2.59</v>
+        <v>-4.85</v>
       </c>
       <c r="J17" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K17" t="n">
-        <v>21.29</v>
+        <v>21.66</v>
       </c>
       <c r="L17" t="n">
-        <v>21.84</v>
+        <v>22.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2379,19 +2432,19 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>1366828</v>
+        <v>13689820</v>
       </c>
       <c r="P17" t="n">
-        <v>1.44</v>
+        <v>4.94</v>
       </c>
       <c r="Q17" t="n">
-        <v>22.06</v>
+        <v>23.7</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>22.44</v>
+        <v>25.75</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -2400,40 +2453,32 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>2.41</v>
+        <v>13.18</v>
       </c>
       <c r="W17" t="n">
-        <v>0.68</v>
+        <v>4.17</v>
       </c>
       <c r="X17" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y17" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB17" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="AC17" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>21.28</v>
+        <v>21.66</v>
       </c>
       <c r="AE17" t="n">
-        <v>22.44</v>
+        <v>25.75</v>
       </c>
       <c r="AF17" t="n">
-        <v>2.88</v>
+        <v>4.78</v>
       </c>
       <c r="AG17" t="n">
-        <v>2.41</v>
+        <v>13.19</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2441,8 +2486,10 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.84</v>
-      </c>
+        <v>2.76</v>
+      </c>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2459,31 +2506,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45887.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>23.36</v>
+        <v>21.88</v>
       </c>
       <c r="G18" t="n">
-        <v>22.64</v>
+        <v>21.35</v>
       </c>
       <c r="H18" t="n">
-        <v>22.81</v>
+        <v>20.53</v>
       </c>
       <c r="I18" t="n">
-        <v>-2.36</v>
+        <v>-6.18</v>
       </c>
       <c r="J18" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K18" t="n">
-        <v>22.39</v>
+        <v>21.35</v>
       </c>
       <c r="L18" t="n">
-        <v>23.18</v>
+        <v>21.78</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2496,19 +2543,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>1011332</v>
+        <v>1476660</v>
       </c>
       <c r="P18" t="n">
-        <v>1.74</v>
+        <v>1.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>23.12</v>
+        <v>21.54</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>23.48</v>
+        <v>22.52</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2517,40 +2564,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>0.51</v>
+        <v>2.93</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.03</v>
+        <v>-1.55</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>45873.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>22.64</v>
+        <v>21.35</v>
       </c>
       <c r="AE18" t="n">
-        <v>23.48</v>
+        <v>22.52</v>
       </c>
       <c r="AF18" t="n">
-        <v>3.08</v>
+        <v>2.41</v>
       </c>
       <c r="AG18" t="n">
-        <v>0.51</v>
+        <v>2.93</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2558,8 +2605,10 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.17</v>
-      </c>
+        <v>1.22</v>
+      </c>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2576,31 +2625,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45900.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>21.7</v>
+        <v>21.16</v>
       </c>
       <c r="G19" t="n">
-        <v>21.06</v>
+        <v>19.2</v>
       </c>
       <c r="H19" t="n">
-        <v>21.02</v>
+        <v>21.32</v>
       </c>
       <c r="I19" t="n">
-        <v>-3.13</v>
+        <v>0.76</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K19" t="n">
-        <v>21.02</v>
+        <v>19.92</v>
       </c>
       <c r="L19" t="n">
-        <v>21.26</v>
+        <v>20.64</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2613,19 +2662,19 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>811883</v>
+        <v>5666121</v>
       </c>
       <c r="P19" t="n">
-        <v>2.81</v>
+        <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>21.61</v>
+        <v>22.02</v>
       </c>
       <c r="R19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>21.83</v>
+        <v>22.52</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
@@ -2634,40 +2683,36 @@
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>0.62</v>
+        <v>6.43</v>
       </c>
       <c r="W19" t="n">
-        <v>-0.4</v>
+        <v>4.06</v>
       </c>
       <c r="X19" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD19" t="n">
-        <v>21.06</v>
+        <v>19.2</v>
       </c>
       <c r="AE19" t="n">
-        <v>21.83</v>
+        <v>22.52</v>
       </c>
       <c r="AF19" t="n">
-        <v>2.95</v>
+        <v>9.26</v>
       </c>
       <c r="AG19" t="n">
-        <v>0.63</v>
+        <v>6.43</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
@@ -2675,8 +2720,10 @@
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.21</v>
-      </c>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2693,31 +2740,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45911.41666666666</v>
+        <v>45845.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45972.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>21.51</v>
+        <v>21.91</v>
       </c>
       <c r="G20" t="n">
-        <v>20.27</v>
+        <v>21.28</v>
       </c>
       <c r="H20" t="n">
-        <v>24.94</v>
+        <v>22.48</v>
       </c>
       <c r="I20" t="n">
-        <v>15.94</v>
+        <v>2.59</v>
       </c>
       <c r="J20" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="K20" t="n">
-        <v>20.28</v>
+        <v>21.29</v>
       </c>
       <c r="L20" t="n">
-        <v>20.96</v>
+        <v>21.84</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2730,70 +2777,72 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>2694406</v>
+        <v>1366828</v>
       </c>
       <c r="P20" t="n">
-        <v>3.42</v>
+        <v>1.44</v>
       </c>
       <c r="Q20" t="n">
-        <v>20.96</v>
+        <v>22.06</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>20.96</v>
+        <v>22.44</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20" t="n">
-        <v>-2.57</v>
+        <v>2.41</v>
       </c>
       <c r="W20" t="n">
-        <v>-2.57</v>
+        <v>0.68</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>45923.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="Z20" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>45911.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="AC20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD20" t="n">
-        <v>20.27</v>
+        <v>21.28</v>
       </c>
       <c r="AE20" t="n">
-        <v>22.19</v>
+        <v>22.44</v>
       </c>
       <c r="AF20" t="n">
-        <v>5.76</v>
+        <v>2.88</v>
       </c>
       <c r="AG20" t="n">
-        <v>3.16</v>
+        <v>2.41</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.55</v>
-      </c>
+        <v>0.84</v>
+      </c>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2810,94 +2859,98 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45994.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>46002.41666666666</v>
+        <v>45887.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>23.44</v>
+        <v>23.36</v>
       </c>
       <c r="G21" t="n">
-        <v>22.68</v>
+        <v>22.64</v>
       </c>
       <c r="H21" t="n">
-        <v>23.56</v>
+        <v>22.81</v>
       </c>
       <c r="I21" t="n">
+        <v>-2.36</v>
+      </c>
+      <c r="J21" t="n">
+        <v>15</v>
+      </c>
+      <c r="K21" t="n">
+        <v>22.39</v>
+      </c>
+      <c r="L21" t="n">
+        <v>23.18</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>1011332</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="R21" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="T21" t="b">
+        <v>0</v>
+      </c>
+      <c r="U21" t="b">
+        <v>0</v>
+      </c>
+      <c r="V21" t="n">
         <v>0.51</v>
       </c>
-      <c r="J21" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>22.51</v>
-      </c>
-      <c r="L21" t="n">
-        <v>23.43</v>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O21" t="n">
-        <v>2183354</v>
-      </c>
-      <c r="P21" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>23.05</v>
-      </c>
-      <c r="R21" t="b">
-        <v>1</v>
-      </c>
-      <c r="S21" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="T21" t="b">
-        <v>0</v>
-      </c>
-      <c r="U21" t="b">
-        <v>0</v>
-      </c>
-      <c r="V21" t="n">
-        <v>6.57</v>
-      </c>
       <c r="W21" t="n">
-        <v>-1.66</v>
+        <v>-1.03</v>
       </c>
       <c r="X21" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y21" s="2" t="n">
+        <v>45873.41666666666</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>1</v>
+      </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45994.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>22.68</v>
+        <v>22.64</v>
       </c>
       <c r="AE21" t="n">
-        <v>24.98</v>
+        <v>23.48</v>
       </c>
       <c r="AF21" t="n">
-        <v>3.24</v>
+        <v>3.08</v>
       </c>
       <c r="AG21" t="n">
-        <v>6.57</v>
+        <v>0.51</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2905,8 +2958,10 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>2.03</v>
-      </c>
+        <v>0.17</v>
+      </c>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2923,31 +2978,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>46016.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>46027.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>24.6</v>
+        <v>21.7</v>
       </c>
       <c r="G22" t="n">
-        <v>23.75</v>
+        <v>21.06</v>
       </c>
       <c r="H22" t="n">
-        <v>24.41</v>
+        <v>21.02</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.77</v>
+        <v>-3.13</v>
       </c>
       <c r="J22" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>23.41</v>
+        <v>21.02</v>
       </c>
       <c r="L22" t="n">
-        <v>24.09</v>
+        <v>21.26</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -2960,66 +3015,72 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>2756109</v>
+        <v>811883</v>
       </c>
       <c r="P22" t="n">
-        <v>3.54</v>
+        <v>2.81</v>
       </c>
       <c r="Q22" t="n">
-        <v>24.08</v>
+        <v>21.61</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>24.5</v>
+        <v>21.83</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
       </c>
       <c r="U22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>-0.41</v>
+        <v>0.62</v>
       </c>
       <c r="W22" t="n">
-        <v>-2.11</v>
+        <v>-0.4</v>
       </c>
       <c r="X22" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y22" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>1</v>
+      </c>
       <c r="AA22" t="b">
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>46016.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>23.75</v>
+        <v>21.06</v>
       </c>
       <c r="AE22" t="n">
-        <v>25.69</v>
+        <v>21.83</v>
       </c>
       <c r="AF22" t="n">
-        <v>3.46</v>
+        <v>2.95</v>
       </c>
       <c r="AG22" t="n">
-        <v>4.43</v>
+        <v>0.63</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>1.28</v>
-      </c>
+        <v>0.21</v>
+      </c>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3036,31 +3097,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>46069.41666666666</v>
+        <v>45972.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>26</v>
+        <v>21.51</v>
       </c>
       <c r="G23" t="n">
-        <v>24.3</v>
+        <v>20.27</v>
       </c>
       <c r="H23" t="n">
-        <v>28.5</v>
+        <v>24.94</v>
       </c>
       <c r="I23" t="n">
-        <v>9.619999999999999</v>
+        <v>15.94</v>
       </c>
       <c r="J23" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="K23" t="n">
-        <v>24.01</v>
+        <v>20.28</v>
       </c>
       <c r="L23" t="n">
-        <v>25.42</v>
+        <v>20.96</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3073,19 +3134,19 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>2965366</v>
+        <v>2694406</v>
       </c>
       <c r="P23" t="n">
-        <v>6.51</v>
+        <v>3.42</v>
       </c>
       <c r="Q23" t="n">
-        <v>25.42</v>
+        <v>20.96</v>
       </c>
       <c r="R23" t="b">
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>25.42</v>
+        <v>20.96</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
@@ -3094,40 +3155,40 @@
         <v>1</v>
       </c>
       <c r="V23" t="n">
-        <v>-2.23</v>
+        <v>-2.57</v>
       </c>
       <c r="W23" t="n">
-        <v>-2.23</v>
+        <v>-2.57</v>
       </c>
       <c r="X23" t="b">
         <v>1</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>46033.41666666666</v>
+        <v>45923.41666666666</v>
       </c>
       <c r="Z23" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AA23" t="b">
         <v>1</v>
       </c>
       <c r="AB23" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="AC23" t="n">
         <v>0</v>
       </c>
       <c r="AD23" t="n">
-        <v>24.3</v>
+        <v>20.27</v>
       </c>
       <c r="AE23" t="n">
-        <v>27.41</v>
+        <v>22.19</v>
       </c>
       <c r="AF23" t="n">
-        <v>6.54</v>
+        <v>5.76</v>
       </c>
       <c r="AG23" t="n">
-        <v>5.42</v>
+        <v>3.16</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
@@ -3135,8 +3196,10 @@
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.83</v>
-      </c>
+        <v>0.55</v>
+      </c>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3153,107 +3216,458 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>46002.41666666666</v>
+      </c>
+      <c r="F24" t="n">
+        <v>23.44</v>
+      </c>
+      <c r="G24" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="H24" t="n">
+        <v>23.56</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J24" t="n">
+        <v>8</v>
+      </c>
+      <c r="K24" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="L24" t="n">
+        <v>23.43</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>2183354</v>
+      </c>
+      <c r="P24" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>23.05</v>
+      </c>
+      <c r="R24" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="T24" t="b">
+        <v>0</v>
+      </c>
+      <c r="U24" t="b">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="W24" t="n">
+        <v>-1.66</v>
+      </c>
+      <c r="X24" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB24" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI24" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C25" t="b">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>46027.41666666666</v>
+      </c>
+      <c r="F25" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G25" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="H25" t="n">
+        <v>24.41</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="J25" t="n">
+        <v>11</v>
+      </c>
+      <c r="K25" t="n">
+        <v>23.41</v>
+      </c>
+      <c r="L25" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>2756109</v>
+      </c>
+      <c r="P25" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>24.08</v>
+      </c>
+      <c r="R25" t="b">
+        <v>1</v>
+      </c>
+      <c r="S25" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="T25" t="b">
+        <v>0</v>
+      </c>
+      <c r="U25" t="b">
+        <v>1</v>
+      </c>
+      <c r="V25" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="W25" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="X25" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB25" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C26" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>46069.41666666666</v>
+      </c>
+      <c r="F26" t="n">
+        <v>26</v>
+      </c>
+      <c r="G26" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="H26" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I26" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="J26" t="n">
+        <v>41</v>
+      </c>
+      <c r="K26" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="L26" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>2965366</v>
+      </c>
+      <c r="P26" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="R26" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="T26" t="b">
+        <v>0</v>
+      </c>
+      <c r="U26" t="b">
+        <v>1</v>
+      </c>
+      <c r="V26" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="W26" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="X26" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y26" s="2" t="n">
+        <v>46033.41666666666</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA26" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB26" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI26" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C27" t="b">
+        <v>0</v>
+      </c>
+      <c r="D27" s="2" t="n">
         <v>46120.41666666666</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E27" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F27" t="n">
         <v>26.61</v>
       </c>
-      <c r="G24" t="n">
+      <c r="G27" t="n">
         <v>25.21</v>
       </c>
-      <c r="H24" t="n">
+      <c r="H27" t="n">
         <v>28.7</v>
       </c>
-      <c r="I24" t="n">
+      <c r="I27" t="n">
         <v>7.85</v>
       </c>
-      <c r="J24" t="n">
+      <c r="J27" t="n">
         <v>19</v>
       </c>
-      <c r="K24" t="n">
+      <c r="K27" t="n">
         <v>23.8</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L27" t="n">
         <v>25.7</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>RANGE_BREAKDOWN</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="O24" t="n">
+      <c r="O27" t="n">
         <v>2499912</v>
       </c>
-      <c r="P24" t="n">
+      <c r="P27" t="n">
         <v>4.31</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="Q27" t="n">
         <v>26.8</v>
       </c>
-      <c r="R24" t="b">
-        <v>0</v>
-      </c>
-      <c r="S24" t="n">
+      <c r="R27" t="b">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
         <v>26.8</v>
       </c>
-      <c r="T24" t="b">
-        <v>1</v>
-      </c>
-      <c r="U24" t="b">
-        <v>0</v>
-      </c>
-      <c r="V24" t="n">
+      <c r="T27" t="b">
+        <v>1</v>
+      </c>
+      <c r="U27" t="b">
+        <v>0</v>
+      </c>
+      <c r="V27" t="n">
         <v>0.71</v>
       </c>
-      <c r="W24" t="n">
+      <c r="W27" t="n">
         <v>0.71</v>
       </c>
-      <c r="X24" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y24" s="2" t="n">
+      <c r="X27" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y27" s="2" t="n">
         <v>46120.41666666666</v>
       </c>
-      <c r="Z24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB24" s="2" t="n">
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB27" s="2" t="n">
         <v>46127.41666666666</v>
       </c>
-      <c r="AC24" t="n">
+      <c r="AC27" t="n">
         <v>3</v>
       </c>
-      <c r="AD24" t="n">
+      <c r="AD27" t="n">
         <v>25.21</v>
       </c>
-      <c r="AE24" t="n">
+      <c r="AE27" t="n">
         <v>26.8</v>
       </c>
-      <c r="AF24" t="n">
+      <c r="AF27" t="n">
         <v>5.26</v>
       </c>
-      <c r="AG24" t="n">
+      <c r="AG27" t="n">
         <v>0.71</v>
       </c>
-      <c r="AH24" t="inlineStr">
+      <c r="AH27" t="inlineStr">
         <is>
           <t>ANCHOR</t>
         </is>
       </c>
-      <c r="AI24" t="n">
+      <c r="AI27" t="n">
         <v>0.13</v>
       </c>
+      <c r="AJ27" t="inlineStr"/>
+      <c r="AK27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3266,7 +3680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:AK2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3282,104 +3696,184 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>total_trades</t>
+          <t>All_Time_High</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>winners</t>
+          <t>Entry_Date</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>losers</t>
+          <t>Exit_Date</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>win_rate</t>
+          <t>Entry_Price</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>median_pnl</t>
+          <t>Entry_Low</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>avg_pnl</t>
+          <t>Exit_Price</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>total_pnl</t>
+          <t>Trade_PnL_%</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>max_pnl</t>
+          <t>Days_Held</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>min_pnl</t>
+          <t>Entry_Support</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>std_pnl</t>
+          <t>Entry_Resistance</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>profit_factor</t>
+          <t>Exit_Reason</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>avg_win</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>avg_loss</t>
+          <t>Entry_Volume</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>expectancy</t>
+          <t>Today_%</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>risk_score</t>
+          <t>Trendline_Price</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>return_score</t>
+          <t>Breaks_Trendline</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>composite_score</t>
+          <t>Anchor_High</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Best_Strategy</t>
+          <t>Testing_Anchor</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>composite_score_best</t>
+          <t>Clears_Anchor</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Buffer_Gain</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Trand_line_Buffer_Gain</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Target_Hit</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Target_Hit_Date</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Bars_To_Target</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Trendline_Hit</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Trendline_Hit_Date</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Bars_To_Trendline</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Stop_Loss</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Target_Price</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Risk_%</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Reward_%</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Reward_Source</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>RR_Ratio</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Current_Price</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Current_Clears_Anchor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3387,64 +3881,116 @@
           <t>RANGE_BREAKOUT</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>23</v>
-      </c>
-      <c r="D2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E2" t="n">
-        <v>11</v>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>45546.41666666666</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>52.17</v>
+        <v>53.91</v>
       </c>
       <c r="G2" t="n">
-        <v>0.51</v>
+        <v>43.72</v>
       </c>
       <c r="H2" t="n">
-        <v>2.58</v>
+        <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>59.34</v>
+        <v>235.74</v>
       </c>
       <c r="J2" t="n">
-        <v>38.41</v>
+        <v>593</v>
       </c>
       <c r="K2" t="n">
-        <v>-11.36</v>
+        <v>43.03</v>
       </c>
       <c r="L2" t="n">
-        <v>10.64</v>
-      </c>
-      <c r="M2" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="N2" t="n">
-        <v>9.31</v>
+        <v>45.91</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
       </c>
       <c r="O2" t="n">
-        <v>4.76</v>
+        <v>128396</v>
       </c>
       <c r="P2" t="n">
-        <v>2.58</v>
+        <v>19.99</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.5084026632302405</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.49842</v>
+        <v>45.33</v>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>0.5024130652920962</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="U2" t="n">
-        <v>0.5024130652920962</v>
+        <v>48.75</v>
+      </c>
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="b">
+        <v>1</v>
+      </c>
+      <c r="V2" t="n">
+        <v>-9.57</v>
+      </c>
+      <c r="W2" t="n">
+        <v>-15.92</v>
+      </c>
+      <c r="X2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="2" t="n">
+        <v>45547.41666666666</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="2" t="n">
+        <v>45546.41666666666</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>43.72</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>59.63</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>181</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3458,7 +4004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3469,68 +4015,245 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>BUY_REASON</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>total_trades</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>winners</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>losers</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>win_rate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>median_pnl</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>avg_pnl</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>total_pnl</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>max_pnl</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>min_pnl</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>std_pnl</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>profit_factor</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>avg_win</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>avg_loss</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>expectancy</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>risk_score</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>return_score</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>composite_score</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>Best_Strategy</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>composite_score</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>total_trades</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>win_rate</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>profit_factor</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>median_pnl</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>expectancy</t>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>composite_score_best</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>AALR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.58</v>
+      </c>
+      <c r="J2" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-14.25</v>
+      </c>
+      <c r="L2" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="N2" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="O2" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="P2" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.2320120319001387</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.09086</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.1473208127600555</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>0.1473208127600555</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>JUFO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>RANGE_BREAKOUT</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="C3" t="n">
         <v>23</v>
       </c>
-      <c r="E2" t="n">
+      <c r="D3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F3" t="n">
         <v>52.17</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="I3" t="n">
+        <v>59.34</v>
+      </c>
+      <c r="J3" t="n">
+        <v>38.41</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-11.36</v>
+      </c>
+      <c r="L3" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="M3" t="n">
         <v>2.13</v>
       </c>
-      <c r="G2" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="H2" t="n">
+      <c r="N3" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="P3" t="n">
         <v>2.58</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.5084026632302405</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.49842</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.5024130652920962</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>0.5024130652920962</v>
       </c>
     </row>
   </sheetData>
@@ -3544,6 +4267,122 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Best_Strategy</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>composite_score</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>total_trades</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>win_rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>profit_factor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>median_pnl</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>expectancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AALR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-0.19</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>23</v>
+      </c>
+      <c r="E3" t="n">
+        <v>52.17</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2.58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:15:27.378806
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK44"/>
+  <dimension ref="A1:AK35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -766,7 +766,7 @@
         <v>50.52</v>
       </c>
       <c r="G3" t="n">
-        <v>46.76</v>
+        <v>45.03</v>
       </c>
       <c r="H3" t="n">
         <v>51.12</v>
@@ -839,13 +839,13 @@
         <v>0</v>
       </c>
       <c r="AD3" t="n">
-        <v>46.76</v>
+        <v>45.03</v>
       </c>
       <c r="AE3" t="n">
         <v>52.6</v>
       </c>
       <c r="AF3" t="n">
-        <v>7.44</v>
+        <v>10.87</v>
       </c>
       <c r="AG3" t="n">
         <v>4.12</v>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0.55</v>
+        <v>0.38</v>
       </c>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr"/>
@@ -919,7 +919,7 @@
         <v>12.94</v>
       </c>
       <c r="Q4" t="n">
-        <v>34.52</v>
+        <v>34.74</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
@@ -937,7 +937,7 @@
         <v>3.02</v>
       </c>
       <c r="W4" t="n">
-        <v>-11.74</v>
+        <v>-11.17</v>
       </c>
       <c r="X4" t="b">
         <v>1</v>
@@ -1123,7 +1123,7 @@
         <v>53.48</v>
       </c>
       <c r="G6" t="n">
-        <v>50.98</v>
+        <v>50.18</v>
       </c>
       <c r="H6" t="n">
         <v>49.83</v>
@@ -1192,13 +1192,13 @@
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>50.98</v>
+        <v>50.18</v>
       </c>
       <c r="AE6" t="n">
         <v>61.85</v>
       </c>
       <c r="AF6" t="n">
-        <v>4.67</v>
+        <v>6.17</v>
       </c>
       <c r="AG6" t="n">
         <v>15.65</v>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>3.35</v>
+        <v>2.54</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1229,31 +1229,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45592.41666666666</v>
+        <v>45594.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>45601.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>53.1</v>
+        <v>54</v>
       </c>
       <c r="G7" t="n">
-        <v>50.2</v>
+        <v>52.01</v>
       </c>
       <c r="H7" t="n">
         <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>-2.07</v>
+        <v>-3.7</v>
       </c>
       <c r="J7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
         <v>44</v>
       </c>
       <c r="L7" t="n">
-        <v>52.9</v>
+        <v>53.95</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>67103</v>
+        <v>36571</v>
       </c>
       <c r="P7" t="n">
-        <v>5.78</v>
+        <v>3.41</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.84</v>
+        <v>54.51</v>
       </c>
       <c r="R7" t="b">
         <v>0</v>
@@ -1287,10 +1287,10 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>9.210000000000001</v>
+        <v>7.39</v>
       </c>
       <c r="W7" t="n">
-        <v>3.28</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X7" t="b">
         <v>0</v>
@@ -1304,19 +1304,19 @@
         <v>45599.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AD7" t="n">
-        <v>50.2</v>
+        <v>52.01</v>
       </c>
       <c r="AE7" t="n">
         <v>57.99</v>
       </c>
       <c r="AF7" t="n">
-        <v>5.46</v>
+        <v>3.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>9.210000000000001</v>
+        <v>7.39</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>1.69</v>
+        <v>2</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1581,22 +1581,22 @@
         <v>45704.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45706.41666666666</v>
+        <v>45714.41666666666</v>
       </c>
       <c r="F10" t="n">
         <v>47.99</v>
       </c>
       <c r="G10" t="n">
-        <v>46.32</v>
+        <v>46</v>
       </c>
       <c r="H10" t="n">
-        <v>46.21</v>
+        <v>45.81</v>
       </c>
       <c r="I10" t="n">
-        <v>-3.71</v>
+        <v>-4.54</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K10" t="n">
         <v>46</v>
@@ -1652,13 +1652,13 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
-        <v>46.32</v>
+        <v>46</v>
       </c>
       <c r="AE10" t="n">
         <v>50.25</v>
       </c>
       <c r="AF10" t="n">
-        <v>3.48</v>
+        <v>4.15</v>
       </c>
       <c r="AG10" t="n">
         <v>4.71</v>
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>1.35</v>
+        <v>1.13</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1689,31 +1689,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45708.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45711.41666666666</v>
+        <v>45727.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>47.44</v>
+        <v>47.51</v>
       </c>
       <c r="G11" t="n">
-        <v>46.22</v>
+        <v>45.8</v>
       </c>
       <c r="H11" t="n">
-        <v>46</v>
+        <v>45.63</v>
       </c>
       <c r="I11" t="n">
-        <v>-3.04</v>
+        <v>-3.96</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K11" t="n">
-        <v>45.51</v>
+        <v>45.81</v>
       </c>
       <c r="L11" t="n">
-        <v>47.38</v>
+        <v>46.58</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1726,65 +1726,69 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>3312</v>
+        <v>31257</v>
       </c>
       <c r="P11" t="n">
-        <v>1.11</v>
+        <v>3.04</v>
       </c>
       <c r="Q11" t="n">
-        <v>46.66</v>
+        <v>46.46</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>48.88</v>
+        <v>46.7</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
       </c>
       <c r="U11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>3.04</v>
+        <v>-1.7</v>
       </c>
       <c r="W11" t="n">
-        <v>-1.64</v>
+        <v>-2.21</v>
       </c>
       <c r="X11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y11" s="2" t="n">
+        <v>45715.41666666666</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45708.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>46.22</v>
+        <v>45.8</v>
       </c>
       <c r="AE11" t="n">
-        <v>48.88</v>
+        <v>48.4</v>
       </c>
       <c r="AF11" t="n">
-        <v>2.57</v>
+        <v>3.6</v>
       </c>
       <c r="AG11" t="n">
-        <v>3.04</v>
+        <v>1.87</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>1.18</v>
+        <v>0.52</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1804,31 +1808,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45727.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>47.51</v>
+        <v>48.44</v>
       </c>
       <c r="G12" t="n">
-        <v>45.8</v>
+        <v>45.88</v>
       </c>
       <c r="H12" t="n">
-        <v>45.63</v>
+        <v>45.51</v>
       </c>
       <c r="I12" t="n">
-        <v>-3.96</v>
+        <v>-6.05</v>
       </c>
       <c r="J12" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="K12" t="n">
-        <v>45.81</v>
+        <v>45.6</v>
       </c>
       <c r="L12" t="n">
-        <v>46.58</v>
+        <v>46.75</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1841,19 +1845,19 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>31257</v>
+        <v>49292</v>
       </c>
       <c r="P12" t="n">
-        <v>3.04</v>
+        <v>5.14</v>
       </c>
       <c r="Q12" t="n">
-        <v>46.46</v>
+        <v>46.73</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>46.7</v>
+        <v>46.75</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1862,40 +1866,40 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-1.7</v>
+        <v>-3.49</v>
       </c>
       <c r="W12" t="n">
-        <v>-2.21</v>
+        <v>-3.53</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45734.41666666666</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>45.8</v>
+        <v>45.88</v>
       </c>
       <c r="AE12" t="n">
-        <v>48.4</v>
+        <v>49.59</v>
       </c>
       <c r="AF12" t="n">
-        <v>3.6</v>
+        <v>5.28</v>
       </c>
       <c r="AG12" t="n">
-        <v>1.87</v>
+        <v>2.37</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1903,7 +1907,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.52</v>
+        <v>0.45</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1911,7 +1915,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1920,34 +1924,34 @@
         </is>
       </c>
       <c r="C13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45736.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>48.44</v>
+        <v>13.43</v>
       </c>
       <c r="G13" t="n">
-        <v>46.07</v>
+        <v>12.66</v>
       </c>
       <c r="H13" t="n">
-        <v>46.04</v>
+        <v>13.26</v>
       </c>
       <c r="I13" t="n">
-        <v>-4.95</v>
+        <v>-1.25</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="K13" t="n">
-        <v>45.6</v>
+        <v>12.54</v>
       </c>
       <c r="L13" t="n">
-        <v>46.75</v>
+        <v>13.42</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1960,19 +1964,19 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>49292</v>
+        <v>3180532</v>
       </c>
       <c r="P13" t="n">
-        <v>5.14</v>
+        <v>3.32</v>
       </c>
       <c r="Q13" t="n">
-        <v>46.73</v>
+        <v>12.98</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>46.75</v>
+        <v>13.42</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
@@ -1981,40 +1985,40 @@
         <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>-3.49</v>
+        <v>-0.09</v>
       </c>
       <c r="W13" t="n">
-        <v>-3.53</v>
+        <v>-3.37</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45734.41666666666</v>
+        <v>45313.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>46.07</v>
+        <v>12.66</v>
       </c>
       <c r="AE13" t="n">
-        <v>49.59</v>
+        <v>14.32</v>
       </c>
       <c r="AF13" t="n">
-        <v>4.89</v>
+        <v>5.78</v>
       </c>
       <c r="AG13" t="n">
-        <v>2.37</v>
+        <v>6.61</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
@@ -2022,7 +2026,7 @@
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>0.48</v>
+        <v>1.14</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2030,7 +2034,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2039,34 +2043,34 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>47.87</v>
+        <v>15.59</v>
       </c>
       <c r="G14" t="n">
-        <v>46</v>
+        <v>13.66</v>
       </c>
       <c r="H14" t="n">
-        <v>58.81</v>
+        <v>16</v>
       </c>
       <c r="I14" t="n">
-        <v>22.85</v>
+        <v>2.62</v>
       </c>
       <c r="J14" t="n">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="K14" t="n">
-        <v>45</v>
+        <v>12.64</v>
       </c>
       <c r="L14" t="n">
-        <v>46.89</v>
+        <v>14.56</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2079,69 +2083,69 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>47815</v>
+        <v>708583</v>
       </c>
       <c r="P14" t="n">
-        <v>2.73</v>
+        <v>10.05</v>
       </c>
       <c r="Q14" t="n">
-        <v>46.62</v>
+        <v>13.78</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>51</v>
+        <v>15.04</v>
       </c>
       <c r="T14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>6.54</v>
+        <v>-3.54</v>
       </c>
       <c r="W14" t="n">
-        <v>-2.61</v>
+        <v>-11.62</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45336.41666666666</v>
       </c>
       <c r="Z14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>46</v>
+        <v>13.66</v>
       </c>
       <c r="AE14" t="n">
-        <v>51</v>
+        <v>17.99</v>
       </c>
       <c r="AF14" t="n">
-        <v>3.91</v>
+        <v>12.37</v>
       </c>
       <c r="AG14" t="n">
-        <v>6.54</v>
+        <v>15.39</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>1.67</v>
+        <v>1.24</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2158,34 +2162,34 @@
         </is>
       </c>
       <c r="C15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45322.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>13.43</v>
+        <v>15.92</v>
       </c>
       <c r="G15" t="n">
-        <v>13</v>
+        <v>14.54</v>
       </c>
       <c r="H15" t="n">
-        <v>13.26</v>
+        <v>14.11</v>
       </c>
       <c r="I15" t="n">
-        <v>-1.25</v>
+        <v>-11.36</v>
       </c>
       <c r="J15" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="K15" t="n">
-        <v>12.92</v>
+        <v>14.54</v>
       </c>
       <c r="L15" t="n">
-        <v>13.42</v>
+        <v>15.68</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2198,69 +2202,69 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>3180532</v>
+        <v>2359660</v>
       </c>
       <c r="P15" t="n">
-        <v>3.32</v>
+        <v>3.65</v>
       </c>
       <c r="Q15" t="n">
-        <v>12.98</v>
+        <v>15.3</v>
       </c>
       <c r="R15" t="b">
         <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>13.42</v>
+        <v>16.22</v>
       </c>
       <c r="T15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>-0.09</v>
+        <v>1.88</v>
       </c>
       <c r="W15" t="n">
-        <v>-3.37</v>
+        <v>-3.89</v>
       </c>
       <c r="X15" t="b">
         <v>1</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>45305.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="Z15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
       </c>
       <c r="AB15" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="AC15" t="n">
         <v>0</v>
       </c>
       <c r="AD15" t="n">
-        <v>13</v>
+        <v>14.54</v>
       </c>
       <c r="AE15" t="n">
-        <v>13.94</v>
+        <v>16.22</v>
       </c>
       <c r="AF15" t="n">
-        <v>3.22</v>
+        <v>8.69</v>
       </c>
       <c r="AG15" t="n">
-        <v>3.75</v>
+        <v>1.91</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>1.16</v>
+        <v>0.22</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2277,34 +2281,34 @@
         </is>
       </c>
       <c r="C16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>15.59</v>
+        <v>13.08</v>
       </c>
       <c r="G16" t="n">
-        <v>13.66</v>
+        <v>12.76</v>
       </c>
       <c r="H16" t="n">
-        <v>16</v>
+        <v>12.39</v>
       </c>
       <c r="I16" t="n">
-        <v>2.62</v>
+        <v>-5.26</v>
       </c>
       <c r="J16" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>12.64</v>
+        <v>12.22</v>
       </c>
       <c r="L16" t="n">
-        <v>14.56</v>
+        <v>13.04</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2317,69 +2321,65 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>708583</v>
+        <v>5618577</v>
       </c>
       <c r="P16" t="n">
-        <v>10.05</v>
+        <v>2.06</v>
       </c>
       <c r="Q16" t="n">
-        <v>13.78</v>
+        <v>12.72</v>
       </c>
       <c r="R16" t="b">
         <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>15.04</v>
+        <v>14.15</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
       </c>
       <c r="U16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>-3.54</v>
+        <v>8.18</v>
       </c>
       <c r="W16" t="n">
-        <v>-11.62</v>
+        <v>-2.75</v>
       </c>
       <c r="X16" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y16" s="2" t="n">
-        <v>45336.41666666666</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
         <v>1</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="AC16" t="n">
         <v>0</v>
       </c>
       <c r="AD16" t="n">
-        <v>13.66</v>
+        <v>12.76</v>
       </c>
       <c r="AE16" t="n">
-        <v>17.99</v>
+        <v>14.15</v>
       </c>
       <c r="AF16" t="n">
-        <v>12.37</v>
+        <v>2.45</v>
       </c>
       <c r="AG16" t="n">
-        <v>15.39</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>1.24</v>
+        <v>3.35</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2399,31 +2399,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45371.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>15.92</v>
+        <v>11.44</v>
       </c>
       <c r="G17" t="n">
-        <v>15.36</v>
+        <v>10.23</v>
       </c>
       <c r="H17" t="n">
-        <v>15.87</v>
+        <v>11.76</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.3</v>
+        <v>2.8</v>
       </c>
       <c r="J17" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
-        <v>14.54</v>
+        <v>10.01</v>
       </c>
       <c r="L17" t="n">
-        <v>15.68</v>
+        <v>11.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2436,61 +2436,53 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>2359660</v>
+        <v>3697242</v>
       </c>
       <c r="P17" t="n">
-        <v>3.65</v>
+        <v>10</v>
       </c>
       <c r="Q17" t="n">
-        <v>15.3</v>
+        <v>13.1</v>
       </c>
       <c r="R17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>16.22</v>
+        <v>13.42</v>
       </c>
       <c r="T17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U17" t="b">
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>1.88</v>
+        <v>17.31</v>
       </c>
       <c r="W17" t="n">
-        <v>-3.89</v>
+        <v>14.51</v>
       </c>
       <c r="X17" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y17" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB17" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="AC17" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>15.36</v>
+        <v>10.23</v>
       </c>
       <c r="AE17" t="n">
-        <v>16.22</v>
+        <v>13.42</v>
       </c>
       <c r="AF17" t="n">
-        <v>3.52</v>
+        <v>10.56</v>
       </c>
       <c r="AG17" t="n">
-        <v>1.91</v>
+        <v>17.34</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2498,7 +2490,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.54</v>
+        <v>1.64</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2518,31 +2510,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45376.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45377.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>16.38</v>
+        <v>12.1</v>
       </c>
       <c r="G18" t="n">
-        <v>15.92</v>
+        <v>11.68</v>
       </c>
       <c r="H18" t="n">
-        <v>15.86</v>
+        <v>12.4</v>
       </c>
       <c r="I18" t="n">
-        <v>-3.17</v>
+        <v>2.51</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K18" t="n">
-        <v>15.12</v>
+        <v>11.68</v>
       </c>
       <c r="L18" t="n">
-        <v>16</v>
+        <v>12.08</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2555,19 +2547,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>598633</v>
+        <v>719120</v>
       </c>
       <c r="P18" t="n">
-        <v>2.91</v>
+        <v>2.86</v>
       </c>
       <c r="Q18" t="n">
-        <v>15.85</v>
+        <v>11.92</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>19.6</v>
+        <v>12.39</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2576,36 +2568,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>19.63</v>
+        <v>2.43</v>
       </c>
       <c r="W18" t="n">
-        <v>-3.26</v>
+        <v>-1.46</v>
       </c>
       <c r="X18" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y18" s="2" t="n">
+        <v>45426.41666666666</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>1</v>
+      </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45376.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>15.92</v>
+        <v>11.68</v>
       </c>
       <c r="AE18" t="n">
-        <v>19.6</v>
+        <v>12.39</v>
       </c>
       <c r="AF18" t="n">
-        <v>2.83</v>
+        <v>3.44</v>
       </c>
       <c r="AG18" t="n">
-        <v>19.63</v>
+        <v>2.45</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2613,7 +2609,7 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>6.94</v>
+        <v>0.71</v>
       </c>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
@@ -2633,31 +2629,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>13.08</v>
+        <v>13.23</v>
       </c>
       <c r="G19" t="n">
-        <v>12.76</v>
+        <v>12.37</v>
       </c>
       <c r="H19" t="n">
-        <v>12.39</v>
+        <v>15.11</v>
       </c>
       <c r="I19" t="n">
-        <v>-5.26</v>
+        <v>14.21</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="K19" t="n">
-        <v>12.22</v>
+        <v>12.37</v>
       </c>
       <c r="L19" t="n">
-        <v>13.04</v>
+        <v>12.68</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2670,65 +2666,69 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>5618577</v>
+        <v>2872871</v>
       </c>
       <c r="P19" t="n">
-        <v>2.06</v>
+        <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>12.72</v>
+        <v>12.61</v>
       </c>
       <c r="R19" t="b">
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>14.15</v>
+        <v>13.12</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
       </c>
       <c r="U19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" t="n">
-        <v>8.18</v>
+        <v>-0.85</v>
       </c>
       <c r="W19" t="n">
-        <v>-2.75</v>
+        <v>-4.7</v>
       </c>
       <c r="X19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y19" s="2" t="n">
+        <v>45454.41666666666</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>11</v>
+      </c>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC19" t="n">
         <v>0</v>
       </c>
       <c r="AD19" t="n">
-        <v>12.76</v>
+        <v>12.37</v>
       </c>
       <c r="AE19" t="n">
-        <v>14.15</v>
+        <v>13.98</v>
       </c>
       <c r="AF19" t="n">
-        <v>2.45</v>
+        <v>6.53</v>
       </c>
       <c r="AG19" t="n">
-        <v>8.199999999999999</v>
+        <v>5.68</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>3.35</v>
+        <v>0.87</v>
       </c>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
@@ -2748,31 +2748,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>11.44</v>
+        <v>17.1</v>
       </c>
       <c r="G20" t="n">
-        <v>10.23</v>
+        <v>14.96</v>
       </c>
       <c r="H20" t="n">
-        <v>11.76</v>
+        <v>19.46</v>
       </c>
       <c r="I20" t="n">
-        <v>2.8</v>
+        <v>13.85</v>
       </c>
       <c r="J20" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="K20" t="n">
-        <v>10.01</v>
+        <v>14.96</v>
       </c>
       <c r="L20" t="n">
-        <v>11.2</v>
+        <v>15.28</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2785,61 +2785,69 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>3697242</v>
+        <v>2885185</v>
       </c>
       <c r="P20" t="n">
-        <v>10</v>
+        <v>13.79</v>
       </c>
       <c r="Q20" t="n">
-        <v>13.1</v>
+        <v>15.44</v>
       </c>
       <c r="R20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>13.42</v>
+        <v>15.5</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
-        <v>17.31</v>
+        <v>-9.34</v>
       </c>
       <c r="W20" t="n">
-        <v>14.51</v>
+        <v>-9.69</v>
       </c>
       <c r="X20" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y20" s="2" t="n">
+        <v>45503.41666666666</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
       <c r="AA20" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB20" s="2" t="n">
+        <v>45503.41666666666</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>0</v>
+      </c>
       <c r="AD20" t="n">
-        <v>10.23</v>
+        <v>14.96</v>
       </c>
       <c r="AE20" t="n">
-        <v>13.42</v>
+        <v>17.64</v>
       </c>
       <c r="AF20" t="n">
-        <v>10.56</v>
+        <v>12.49</v>
       </c>
       <c r="AG20" t="n">
-        <v>17.34</v>
+        <v>3.18</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>1.64</v>
+        <v>0.25</v>
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
@@ -2859,31 +2867,31 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45433.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>12.1</v>
+        <v>20.68</v>
       </c>
       <c r="G21" t="n">
-        <v>11.68</v>
+        <v>18.4</v>
       </c>
       <c r="H21" t="n">
-        <v>12.59</v>
+        <v>28.62</v>
       </c>
       <c r="I21" t="n">
-        <v>4.1</v>
+        <v>38.41</v>
       </c>
       <c r="J21" t="n">
-        <v>8</v>
+        <v>185</v>
       </c>
       <c r="K21" t="n">
-        <v>11.68</v>
+        <v>18.4</v>
       </c>
       <c r="L21" t="n">
-        <v>12.08</v>
+        <v>20.24</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2896,19 +2904,19 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>719120</v>
+        <v>807277</v>
       </c>
       <c r="P21" t="n">
-        <v>2.86</v>
+        <v>2.17</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.92</v>
+        <v>20.54</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>12.39</v>
+        <v>23.04</v>
       </c>
       <c r="T21" t="b">
         <v>0</v>
@@ -2917,40 +2925,40 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>2.43</v>
+        <v>11.41</v>
       </c>
       <c r="W21" t="n">
-        <v>-1.46</v>
+        <v>-0.68</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45426.41666666666</v>
+        <v>45572.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>11.68</v>
+        <v>18.4</v>
       </c>
       <c r="AE21" t="n">
-        <v>12.39</v>
+        <v>23.04</v>
       </c>
       <c r="AF21" t="n">
-        <v>3.44</v>
+        <v>11.03</v>
       </c>
       <c r="AG21" t="n">
-        <v>2.45</v>
+        <v>11.41</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2958,7 +2966,7 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.71</v>
+        <v>1.03</v>
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
@@ -2978,31 +2986,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>13.23</v>
+        <v>28.64</v>
       </c>
       <c r="G22" t="n">
-        <v>12.63</v>
+        <v>28.08</v>
       </c>
       <c r="H22" t="n">
-        <v>15.11</v>
+        <v>27.22</v>
       </c>
       <c r="I22" t="n">
-        <v>14.21</v>
+        <v>-4.97</v>
       </c>
       <c r="J22" t="n">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>12.37</v>
+        <v>28</v>
       </c>
       <c r="L22" t="n">
-        <v>12.68</v>
+        <v>28.48</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3015,69 +3023,69 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>2872871</v>
+        <v>1546271</v>
       </c>
       <c r="P22" t="n">
-        <v>4.75</v>
+        <v>1.79</v>
       </c>
       <c r="Q22" t="n">
-        <v>12.61</v>
+        <v>28.16</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>13.12</v>
+        <v>29</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
       </c>
       <c r="U22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>-0.85</v>
+        <v>1.26</v>
       </c>
       <c r="W22" t="n">
-        <v>-4.7</v>
+        <v>-1.68</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>45454.41666666666</v>
+        <v>45729.41666666666</v>
       </c>
       <c r="Z22" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>12.63</v>
+        <v>28.08</v>
       </c>
       <c r="AE22" t="n">
-        <v>13.98</v>
+        <v>29</v>
       </c>
       <c r="AF22" t="n">
-        <v>4.53</v>
+        <v>1.96</v>
       </c>
       <c r="AG22" t="n">
-        <v>5.68</v>
+        <v>1.26</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>1.25</v>
+        <v>0.64</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3097,31 +3105,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>17.1</v>
+        <v>25.97</v>
       </c>
       <c r="G23" t="n">
-        <v>15.02</v>
+        <v>24.72</v>
       </c>
       <c r="H23" t="n">
-        <v>19.46</v>
+        <v>25.2</v>
       </c>
       <c r="I23" t="n">
-        <v>13.85</v>
+        <v>-2.96</v>
       </c>
       <c r="J23" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="K23" t="n">
-        <v>14.96</v>
+        <v>24.68</v>
       </c>
       <c r="L23" t="n">
-        <v>15.28</v>
+        <v>25.51</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3134,69 +3142,61 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>2885185</v>
+        <v>767605</v>
       </c>
       <c r="P23" t="n">
-        <v>13.79</v>
+        <v>4.04</v>
       </c>
       <c r="Q23" t="n">
-        <v>15.44</v>
+        <v>27.46</v>
       </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>15.5</v>
+        <v>29.03</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
       </c>
       <c r="U23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>-9.34</v>
+        <v>11.79</v>
       </c>
       <c r="W23" t="n">
-        <v>-9.69</v>
+        <v>5.75</v>
       </c>
       <c r="X23" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y23" s="2" t="n">
-        <v>45503.41666666666</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB23" s="2" t="n">
-        <v>45503.41666666666</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="n">
-        <v>15.02</v>
+        <v>24.72</v>
       </c>
       <c r="AE23" t="n">
-        <v>17.64</v>
+        <v>29.03</v>
       </c>
       <c r="AF23" t="n">
-        <v>12.12</v>
+        <v>4.81</v>
       </c>
       <c r="AG23" t="n">
-        <v>3.18</v>
+        <v>11.8</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.26</v>
+        <v>2.45</v>
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
@@ -3216,31 +3216,31 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>45532.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F24" t="n">
-        <v>20.68</v>
+        <v>25.32</v>
       </c>
       <c r="G24" t="n">
-        <v>20.24</v>
+        <v>24.12</v>
       </c>
       <c r="H24" t="n">
-        <v>20</v>
+        <v>23.99</v>
       </c>
       <c r="I24" t="n">
-        <v>-3.29</v>
+        <v>-5.24</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K24" t="n">
-        <v>18.4</v>
+        <v>24.12</v>
       </c>
       <c r="L24" t="n">
-        <v>20.24</v>
+        <v>25.26</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>807277</v>
+        <v>623052</v>
       </c>
       <c r="P24" t="n">
-        <v>2.17</v>
+        <v>0.96</v>
       </c>
       <c r="Q24" t="n">
-        <v>20.54</v>
+        <v>26.96</v>
       </c>
       <c r="R24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>23.04</v>
+        <v>26.96</v>
       </c>
       <c r="T24" t="b">
         <v>0</v>
@@ -3274,10 +3274,10 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>11.41</v>
+        <v>6.48</v>
       </c>
       <c r="W24" t="n">
-        <v>-0.68</v>
+        <v>6.48</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3285,25 +3285,21 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB24" s="2" t="n">
-        <v>45530.41666666666</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="n">
-        <v>20.24</v>
+        <v>24.12</v>
       </c>
       <c r="AE24" t="n">
-        <v>23.04</v>
+        <v>26.96</v>
       </c>
       <c r="AF24" t="n">
-        <v>2.13</v>
+        <v>4.74</v>
       </c>
       <c r="AG24" t="n">
-        <v>11.41</v>
+        <v>6.48</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
@@ -3311,7 +3307,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>5.36</v>
+        <v>1.37</v>
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
@@ -3331,31 +3327,31 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>45538.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>45544.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F25" t="n">
-        <v>20.01</v>
+        <v>22.75</v>
       </c>
       <c r="G25" t="n">
-        <v>19.2</v>
+        <v>21.66</v>
       </c>
       <c r="H25" t="n">
-        <v>19.09</v>
+        <v>21.65</v>
       </c>
       <c r="I25" t="n">
-        <v>-4.6</v>
+        <v>-4.85</v>
       </c>
       <c r="J25" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="K25" t="n">
-        <v>19.18</v>
+        <v>21.66</v>
       </c>
       <c r="L25" t="n">
-        <v>19.92</v>
+        <v>22.2</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3368,19 +3364,19 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>604202</v>
+        <v>13689820</v>
       </c>
       <c r="P25" t="n">
-        <v>3.3</v>
+        <v>4.94</v>
       </c>
       <c r="Q25" t="n">
-        <v>20</v>
+        <v>23.7</v>
       </c>
       <c r="R25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>21.2</v>
+        <v>25.75</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
@@ -3389,10 +3385,10 @@
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>5.96</v>
+        <v>13.18</v>
       </c>
       <c r="W25" t="n">
-        <v>-0.04</v>
+        <v>4.17</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -3400,25 +3396,21 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB25" s="2" t="n">
-        <v>45538.41666666666</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="n">
-        <v>19.2</v>
+        <v>21.66</v>
       </c>
       <c r="AE25" t="n">
-        <v>21.2</v>
+        <v>25.75</v>
       </c>
       <c r="AF25" t="n">
-        <v>4.04</v>
+        <v>4.78</v>
       </c>
       <c r="AG25" t="n">
-        <v>5.96</v>
+        <v>13.19</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
@@ -3426,7 +3418,7 @@
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>1.48</v>
+        <v>2.76</v>
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
@@ -3446,31 +3438,31 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>45553.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F26" t="n">
-        <v>19.62</v>
+        <v>21.88</v>
       </c>
       <c r="G26" t="n">
-        <v>19.08</v>
+        <v>21.35</v>
       </c>
       <c r="H26" t="n">
-        <v>19.74</v>
+        <v>20.53</v>
       </c>
       <c r="I26" t="n">
-        <v>0.61</v>
+        <v>-6.18</v>
       </c>
       <c r="J26" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K26" t="n">
-        <v>18.93</v>
+        <v>21.35</v>
       </c>
       <c r="L26" t="n">
-        <v>19.52</v>
+        <v>21.78</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3483,19 +3475,19 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>340401</v>
+        <v>1476660</v>
       </c>
       <c r="P26" t="n">
-        <v>0.53</v>
+        <v>1.3</v>
       </c>
       <c r="Q26" t="n">
-        <v>19.64</v>
+        <v>21.54</v>
       </c>
       <c r="R26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>20.63</v>
+        <v>22.52</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
@@ -3504,16 +3496,16 @@
         <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>5.13</v>
+        <v>2.93</v>
       </c>
       <c r="W26" t="n">
-        <v>0.08</v>
+        <v>-1.55</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>45551.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z26" t="n">
         <v>2</v>
@@ -3522,22 +3514,22 @@
         <v>1</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>45547.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>19.08</v>
+        <v>21.35</v>
       </c>
       <c r="AE26" t="n">
-        <v>20.63</v>
+        <v>22.52</v>
       </c>
       <c r="AF26" t="n">
-        <v>2.77</v>
+        <v>2.41</v>
       </c>
       <c r="AG26" t="n">
-        <v>5.14</v>
+        <v>2.93</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
@@ -3545,7 +3537,7 @@
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>1.86</v>
+        <v>1.22</v>
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
@@ -3565,31 +3557,31 @@
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>45557.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>45692.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>20.2</v>
+        <v>21.16</v>
       </c>
       <c r="G27" t="n">
-        <v>20</v>
+        <v>19.2</v>
       </c>
       <c r="H27" t="n">
-        <v>27.62</v>
+        <v>21.32</v>
       </c>
       <c r="I27" t="n">
-        <v>36.71</v>
+        <v>0.76</v>
       </c>
       <c r="J27" t="n">
-        <v>135</v>
+        <v>8</v>
       </c>
       <c r="K27" t="n">
-        <v>19.62</v>
+        <v>19.92</v>
       </c>
       <c r="L27" t="n">
-        <v>20.1</v>
+        <v>20.64</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3602,19 +3594,19 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>244643</v>
+        <v>5666121</v>
       </c>
       <c r="P27" t="n">
-        <v>1</v>
+        <v>4.75</v>
       </c>
       <c r="Q27" t="n">
-        <v>19.52</v>
+        <v>22.02</v>
       </c>
       <c r="R27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>21.91</v>
+        <v>22.52</v>
       </c>
       <c r="T27" t="b">
         <v>0</v>
@@ -3623,40 +3615,36 @@
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>8.470000000000001</v>
+        <v>6.43</v>
       </c>
       <c r="W27" t="n">
-        <v>-3.37</v>
+        <v>4.06</v>
       </c>
       <c r="X27" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y27" s="2" t="n">
-        <v>45572.41666666666</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>10</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="b">
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>45557.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD27" t="n">
-        <v>20</v>
+        <v>19.2</v>
       </c>
       <c r="AE27" t="n">
-        <v>21.91</v>
+        <v>22.52</v>
       </c>
       <c r="AF27" t="n">
-        <v>0.99</v>
+        <v>9.26</v>
       </c>
       <c r="AG27" t="n">
-        <v>8.48</v>
+        <v>6.43</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -3664,7 +3652,7 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>8.57</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
@@ -3681,34 +3669,34 @@
         </is>
       </c>
       <c r="C28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>45697.41666666666</v>
+        <v>45845.41666666666</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="F28" t="n">
-        <v>30.02</v>
+        <v>21.91</v>
       </c>
       <c r="G28" t="n">
-        <v>28.39</v>
+        <v>21.28</v>
       </c>
       <c r="H28" t="n">
-        <v>28.62</v>
+        <v>22.48</v>
       </c>
       <c r="I28" t="n">
-        <v>-4.64</v>
+        <v>2.59</v>
       </c>
       <c r="J28" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="K28" t="n">
-        <v>27.62</v>
+        <v>21.29</v>
       </c>
       <c r="L28" t="n">
-        <v>28.46</v>
+        <v>21.84</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -3721,69 +3709,69 @@
         </is>
       </c>
       <c r="O28" t="n">
-        <v>884535</v>
+        <v>1366828</v>
       </c>
       <c r="P28" t="n">
-        <v>5.72</v>
+        <v>1.44</v>
       </c>
       <c r="Q28" t="n">
-        <v>28.44</v>
+        <v>22.06</v>
       </c>
       <c r="R28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>29.02</v>
+        <v>22.44</v>
       </c>
       <c r="T28" t="b">
         <v>0</v>
       </c>
       <c r="U28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V28" t="n">
-        <v>-3.32</v>
+        <v>2.41</v>
       </c>
       <c r="W28" t="n">
-        <v>-5.25</v>
+        <v>0.68</v>
       </c>
       <c r="X28" t="b">
         <v>1</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>45711.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="Z28" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AA28" t="b">
         <v>1</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>45697.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="AC28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD28" t="n">
-        <v>28.39</v>
+        <v>21.28</v>
       </c>
       <c r="AE28" t="n">
-        <v>31.42</v>
+        <v>22.44</v>
       </c>
       <c r="AF28" t="n">
-        <v>5.41</v>
+        <v>2.88</v>
       </c>
       <c r="AG28" t="n">
-        <v>4.69</v>
+        <v>2.41</v>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI28" t="n">
-        <v>0.87</v>
+        <v>0.84</v>
       </c>
       <c r="AJ28" t="inlineStr"/>
       <c r="AK28" t="inlineStr"/>
@@ -3803,31 +3791,31 @@
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45887.41666666666</v>
       </c>
       <c r="F29" t="n">
-        <v>28.64</v>
+        <v>23.36</v>
       </c>
       <c r="G29" t="n">
-        <v>28.08</v>
+        <v>22.64</v>
       </c>
       <c r="H29" t="n">
-        <v>27.22</v>
+        <v>22.81</v>
       </c>
       <c r="I29" t="n">
-        <v>-4.97</v>
+        <v>-2.36</v>
       </c>
       <c r="J29" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="K29" t="n">
-        <v>28</v>
+        <v>22.39</v>
       </c>
       <c r="L29" t="n">
-        <v>28.48</v>
+        <v>23.18</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3840,19 +3828,19 @@
         </is>
       </c>
       <c r="O29" t="n">
-        <v>1546271</v>
+        <v>1011332</v>
       </c>
       <c r="P29" t="n">
-        <v>1.79</v>
+        <v>1.74</v>
       </c>
       <c r="Q29" t="n">
-        <v>28.16</v>
+        <v>23.12</v>
       </c>
       <c r="R29" t="b">
         <v>1</v>
       </c>
       <c r="S29" t="n">
-        <v>29</v>
+        <v>23.48</v>
       </c>
       <c r="T29" t="b">
         <v>0</v>
@@ -3861,16 +3849,16 @@
         <v>0</v>
       </c>
       <c r="V29" t="n">
-        <v>1.26</v>
+        <v>0.51</v>
       </c>
       <c r="W29" t="n">
-        <v>-1.68</v>
+        <v>-1.03</v>
       </c>
       <c r="X29" t="b">
         <v>1</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45873.41666666666</v>
       </c>
       <c r="Z29" t="n">
         <v>1</v>
@@ -3879,22 +3867,22 @@
         <v>1</v>
       </c>
       <c r="AB29" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="AC29" t="n">
         <v>0</v>
       </c>
       <c r="AD29" t="n">
-        <v>28.08</v>
+        <v>22.64</v>
       </c>
       <c r="AE29" t="n">
-        <v>29</v>
+        <v>23.48</v>
       </c>
       <c r="AF29" t="n">
-        <v>1.96</v>
+        <v>3.08</v>
       </c>
       <c r="AG29" t="n">
-        <v>1.26</v>
+        <v>0.51</v>
       </c>
       <c r="AH29" t="inlineStr">
         <is>
@@ -3902,7 +3890,7 @@
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>0.64</v>
+        <v>0.17</v>
       </c>
       <c r="AJ29" t="inlineStr"/>
       <c r="AK29" t="inlineStr"/>
@@ -3922,31 +3910,31 @@
         <v>0</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>45754.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="F30" t="n">
-        <v>25.97</v>
+        <v>21.7</v>
       </c>
       <c r="G30" t="n">
-        <v>24.72</v>
+        <v>21.06</v>
       </c>
       <c r="H30" t="n">
-        <v>25.2</v>
+        <v>21.02</v>
       </c>
       <c r="I30" t="n">
-        <v>-2.96</v>
+        <v>-3.13</v>
       </c>
       <c r="J30" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="K30" t="n">
-        <v>24.68</v>
+        <v>21.02</v>
       </c>
       <c r="L30" t="n">
-        <v>25.51</v>
+        <v>21.26</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -3959,19 +3947,19 @@
         </is>
       </c>
       <c r="O30" t="n">
-        <v>767605</v>
+        <v>811883</v>
       </c>
       <c r="P30" t="n">
-        <v>4.04</v>
+        <v>2.81</v>
       </c>
       <c r="Q30" t="n">
-        <v>27.46</v>
+        <v>21.61</v>
       </c>
       <c r="R30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S30" t="n">
-        <v>29.03</v>
+        <v>21.83</v>
       </c>
       <c r="T30" t="b">
         <v>0</v>
@@ -3980,32 +3968,40 @@
         <v>0</v>
       </c>
       <c r="V30" t="n">
-        <v>11.79</v>
+        <v>0.62</v>
       </c>
       <c r="W30" t="n">
-        <v>5.75</v>
+        <v>-0.4</v>
       </c>
       <c r="X30" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y30" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>1</v>
+      </c>
       <c r="AA30" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB30" t="inlineStr"/>
-      <c r="AC30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB30" s="2" t="n">
+        <v>45897.41666666666</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
       <c r="AD30" t="n">
-        <v>24.72</v>
+        <v>21.06</v>
       </c>
       <c r="AE30" t="n">
-        <v>29.03</v>
+        <v>21.83</v>
       </c>
       <c r="AF30" t="n">
-        <v>4.81</v>
+        <v>2.95</v>
       </c>
       <c r="AG30" t="n">
-        <v>11.8</v>
+        <v>0.63</v>
       </c>
       <c r="AH30" t="inlineStr">
         <is>
@@ -4013,7 +4009,7 @@
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>2.45</v>
+        <v>0.21</v>
       </c>
       <c r="AJ30" t="inlineStr"/>
       <c r="AK30" t="inlineStr"/>
@@ -4033,31 +4029,31 @@
         <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>45763.41666666666</v>
+        <v>45972.41666666666</v>
       </c>
       <c r="F31" t="n">
-        <v>25.32</v>
+        <v>21.51</v>
       </c>
       <c r="G31" t="n">
-        <v>25.08</v>
+        <v>20.27</v>
       </c>
       <c r="H31" t="n">
-        <v>25.26</v>
+        <v>24.94</v>
       </c>
       <c r="I31" t="n">
-        <v>-0.25</v>
+        <v>15.94</v>
       </c>
       <c r="J31" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="K31" t="n">
-        <v>24.12</v>
+        <v>20.28</v>
       </c>
       <c r="L31" t="n">
-        <v>25.26</v>
+        <v>20.96</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -4070,65 +4066,69 @@
         </is>
       </c>
       <c r="O31" t="n">
-        <v>623052</v>
+        <v>2694406</v>
       </c>
       <c r="P31" t="n">
-        <v>0.96</v>
+        <v>3.42</v>
       </c>
       <c r="Q31" t="n">
-        <v>25.52</v>
+        <v>20.96</v>
       </c>
       <c r="R31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S31" t="n">
-        <v>26.96</v>
+        <v>20.96</v>
       </c>
       <c r="T31" t="b">
         <v>0</v>
       </c>
       <c r="U31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V31" t="n">
-        <v>6.48</v>
+        <v>-2.57</v>
       </c>
       <c r="W31" t="n">
-        <v>0.79</v>
+        <v>-2.57</v>
       </c>
       <c r="X31" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y31" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>8</v>
+      </c>
       <c r="AA31" t="b">
         <v>1</v>
       </c>
       <c r="AB31" s="2" t="n">
-        <v>45761.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="AC31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD31" t="n">
-        <v>25.08</v>
+        <v>20.27</v>
       </c>
       <c r="AE31" t="n">
-        <v>26.96</v>
+        <v>22.19</v>
       </c>
       <c r="AF31" t="n">
-        <v>0.95</v>
+        <v>5.76</v>
       </c>
       <c r="AG31" t="n">
-        <v>6.48</v>
+        <v>3.16</v>
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI31" t="n">
-        <v>6.82</v>
+        <v>0.55</v>
       </c>
       <c r="AJ31" t="inlineStr"/>
       <c r="AK31" t="inlineStr"/>
@@ -4148,31 +4148,31 @@
         <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>45775.41666666666</v>
+        <v>45994.41666666666</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>45781.41666666666</v>
+        <v>46002.41666666666</v>
       </c>
       <c r="F32" t="n">
-        <v>25.33</v>
+        <v>23.44</v>
       </c>
       <c r="G32" t="n">
-        <v>25.12</v>
+        <v>22.68</v>
       </c>
       <c r="H32" t="n">
-        <v>25.04</v>
+        <v>23.56</v>
       </c>
       <c r="I32" t="n">
-        <v>-1.14</v>
+        <v>0.51</v>
       </c>
       <c r="J32" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K32" t="n">
-        <v>24.55</v>
+        <v>22.51</v>
       </c>
       <c r="L32" t="n">
-        <v>25.28</v>
+        <v>23.2</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -4185,31 +4185,31 @@
         </is>
       </c>
       <c r="O32" t="n">
-        <v>5196323</v>
+        <v>2183354</v>
       </c>
       <c r="P32" t="n">
-        <v>0.83</v>
+        <v>1.78</v>
       </c>
       <c r="Q32" t="n">
-        <v>25.92</v>
+        <v>22.87</v>
       </c>
       <c r="R32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S32" t="n">
-        <v>25.28</v>
+        <v>24.98</v>
       </c>
       <c r="T32" t="b">
         <v>0</v>
       </c>
       <c r="U32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V32" t="n">
-        <v>-0.19</v>
+        <v>6.57</v>
       </c>
       <c r="W32" t="n">
-        <v>2.34</v>
+        <v>-2.43</v>
       </c>
       <c r="X32" t="b">
         <v>0</v>
@@ -4217,29 +4217,33 @@
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB32" t="inlineStr"/>
-      <c r="AC32" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB32" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>0</v>
+      </c>
       <c r="AD32" t="n">
-        <v>25.12</v>
+        <v>22.68</v>
       </c>
       <c r="AE32" t="n">
-        <v>26.05</v>
+        <v>24.98</v>
       </c>
       <c r="AF32" t="n">
-        <v>0.82</v>
+        <v>3.24</v>
       </c>
       <c r="AG32" t="n">
-        <v>2.87</v>
+        <v>6.57</v>
       </c>
       <c r="AH32" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI32" t="n">
-        <v>3.5</v>
+        <v>2.03</v>
       </c>
       <c r="AJ32" t="inlineStr"/>
       <c r="AK32" t="inlineStr"/>
@@ -4259,31 +4263,31 @@
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>46016.41666666666</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>46027.41666666666</v>
       </c>
       <c r="F33" t="n">
-        <v>22.75</v>
+        <v>24.6</v>
       </c>
       <c r="G33" t="n">
-        <v>21.68</v>
+        <v>23.75</v>
       </c>
       <c r="H33" t="n">
-        <v>21.65</v>
+        <v>24.41</v>
       </c>
       <c r="I33" t="n">
-        <v>-4.85</v>
+        <v>-0.77</v>
       </c>
       <c r="J33" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K33" t="n">
-        <v>21.66</v>
+        <v>23.41</v>
       </c>
       <c r="L33" t="n">
-        <v>22.2</v>
+        <v>24.09</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -4296,31 +4300,31 @@
         </is>
       </c>
       <c r="O33" t="n">
-        <v>13689820</v>
+        <v>2756109</v>
       </c>
       <c r="P33" t="n">
-        <v>4.94</v>
+        <v>3.54</v>
       </c>
       <c r="Q33" t="n">
-        <v>23.7</v>
+        <v>24.08</v>
       </c>
       <c r="R33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S33" t="n">
-        <v>25.75</v>
+        <v>24.5</v>
       </c>
       <c r="T33" t="b">
         <v>0</v>
       </c>
       <c r="U33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V33" t="n">
-        <v>13.18</v>
+        <v>-0.41</v>
       </c>
       <c r="W33" t="n">
-        <v>4.17</v>
+        <v>-2.11</v>
       </c>
       <c r="X33" t="b">
         <v>0</v>
@@ -4328,29 +4332,33 @@
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
       <c r="AA33" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB33" t="inlineStr"/>
-      <c r="AC33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB33" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
       <c r="AD33" t="n">
-        <v>21.68</v>
+        <v>23.75</v>
       </c>
       <c r="AE33" t="n">
-        <v>25.75</v>
+        <v>25.69</v>
       </c>
       <c r="AF33" t="n">
-        <v>4.71</v>
+        <v>3.46</v>
       </c>
       <c r="AG33" t="n">
-        <v>13.19</v>
+        <v>4.43</v>
       </c>
       <c r="AH33" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI33" t="n">
-        <v>2.8</v>
+        <v>1.28</v>
       </c>
       <c r="AJ33" t="inlineStr"/>
       <c r="AK33" t="inlineStr"/>
@@ -4370,31 +4378,31 @@
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>45820.41666666666</v>
+        <v>46069.41666666666</v>
       </c>
       <c r="F34" t="n">
-        <v>21.88</v>
+        <v>26</v>
       </c>
       <c r="G34" t="n">
-        <v>21.6</v>
+        <v>24.3</v>
       </c>
       <c r="H34" t="n">
-        <v>21.78</v>
+        <v>28.5</v>
       </c>
       <c r="I34" t="n">
-        <v>-0.48</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J34" t="n">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="K34" t="n">
-        <v>21.35</v>
+        <v>24.01</v>
       </c>
       <c r="L34" t="n">
-        <v>21.78</v>
+        <v>25.42</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -4407,37 +4415,37 @@
         </is>
       </c>
       <c r="O34" t="n">
-        <v>1476660</v>
+        <v>2965366</v>
       </c>
       <c r="P34" t="n">
-        <v>1.3</v>
+        <v>6.51</v>
       </c>
       <c r="Q34" t="n">
-        <v>21.54</v>
+        <v>25.42</v>
       </c>
       <c r="R34" t="b">
         <v>1</v>
       </c>
       <c r="S34" t="n">
-        <v>22.52</v>
+        <v>25.42</v>
       </c>
       <c r="T34" t="b">
         <v>0</v>
       </c>
       <c r="U34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V34" t="n">
-        <v>2.93</v>
+        <v>-2.23</v>
       </c>
       <c r="W34" t="n">
-        <v>-1.55</v>
+        <v>-2.23</v>
       </c>
       <c r="X34" t="b">
         <v>1</v>
       </c>
       <c r="Y34" s="2" t="n">
-        <v>45818.41666666666</v>
+        <v>46033.41666666666</v>
       </c>
       <c r="Z34" t="n">
         <v>2</v>
@@ -4446,30 +4454,30 @@
         <v>1</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="AC34" t="n">
         <v>0</v>
       </c>
       <c r="AD34" t="n">
-        <v>21.6</v>
+        <v>24.3</v>
       </c>
       <c r="AE34" t="n">
-        <v>22.52</v>
+        <v>27.41</v>
       </c>
       <c r="AF34" t="n">
-        <v>1.28</v>
+        <v>6.54</v>
       </c>
       <c r="AG34" t="n">
-        <v>2.93</v>
+        <v>5.42</v>
       </c>
       <c r="AH34" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI34" t="n">
-        <v>2.29</v>
+        <v>0.83</v>
       </c>
       <c r="AJ34" t="inlineStr"/>
       <c r="AK34" t="inlineStr"/>
@@ -4489,31 +4497,31 @@
         <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>46120.41666666666</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>46139.41666666666</v>
       </c>
       <c r="F35" t="n">
-        <v>21.16</v>
+        <v>26.61</v>
       </c>
       <c r="G35" t="n">
-        <v>20.2</v>
+        <v>25.4</v>
       </c>
       <c r="H35" t="n">
-        <v>21.32</v>
+        <v>28.7</v>
       </c>
       <c r="I35" t="n">
-        <v>0.76</v>
+        <v>7.85</v>
       </c>
       <c r="J35" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="K35" t="n">
-        <v>19.92</v>
+        <v>23.8</v>
       </c>
       <c r="L35" t="n">
-        <v>20.64</v>
+        <v>25.7</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -4526,57 +4534,61 @@
         </is>
       </c>
       <c r="O35" t="n">
-        <v>5666121</v>
+        <v>2499912</v>
       </c>
       <c r="P35" t="n">
-        <v>4.75</v>
+        <v>4.31</v>
       </c>
       <c r="Q35" t="n">
-        <v>22.02</v>
+        <v>25.73</v>
       </c>
       <c r="R35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S35" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="T35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U35" t="b">
         <v>0</v>
       </c>
       <c r="V35" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="W35" t="n">
-        <v>4.06</v>
+        <v>-3.31</v>
       </c>
       <c r="X35" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y35" t="inlineStr"/>
-      <c r="Z35" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
       <c r="AA35" t="b">
         <v>1</v>
       </c>
       <c r="AB35" s="2" t="n">
-        <v>45833.41666666666</v>
+        <v>46120.41666666666</v>
       </c>
       <c r="AC35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD35" t="n">
-        <v>20.2</v>
+        <v>25.4</v>
       </c>
       <c r="AE35" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="AF35" t="n">
-        <v>4.54</v>
+        <v>4.55</v>
       </c>
       <c r="AG35" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="AH35" t="inlineStr">
         <is>
@@ -4584,1073 +4596,10 @@
         </is>
       </c>
       <c r="AI35" t="n">
-        <v>1.42</v>
+        <v>0.16</v>
       </c>
       <c r="AJ35" t="inlineStr"/>
       <c r="AK35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C36" t="b">
-        <v>0</v>
-      </c>
-      <c r="D36" s="2" t="n">
-        <v>45845.41666666666</v>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>45860.41666666666</v>
-      </c>
-      <c r="F36" t="n">
-        <v>21.91</v>
-      </c>
-      <c r="G36" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="H36" t="n">
-        <v>22.48</v>
-      </c>
-      <c r="I36" t="n">
-        <v>2.59</v>
-      </c>
-      <c r="J36" t="n">
-        <v>15</v>
-      </c>
-      <c r="K36" t="n">
-        <v>21.29</v>
-      </c>
-      <c r="L36" t="n">
-        <v>21.84</v>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O36" t="n">
-        <v>1366828</v>
-      </c>
-      <c r="P36" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>22.06</v>
-      </c>
-      <c r="R36" t="b">
-        <v>0</v>
-      </c>
-      <c r="S36" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="T36" t="b">
-        <v>0</v>
-      </c>
-      <c r="U36" t="b">
-        <v>0</v>
-      </c>
-      <c r="V36" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="W36" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="X36" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y36" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="Z36" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA36" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB36" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="AC36" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD36" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="AE36" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="AF36" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="AG36" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="AH36" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI36" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="AJ36" t="inlineStr"/>
-      <c r="AK36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C37" t="b">
-        <v>0</v>
-      </c>
-      <c r="D37" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="E37" s="2" t="n">
-        <v>45887.41666666666</v>
-      </c>
-      <c r="F37" t="n">
-        <v>23.36</v>
-      </c>
-      <c r="G37" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="H37" t="n">
-        <v>22.81</v>
-      </c>
-      <c r="I37" t="n">
-        <v>-2.36</v>
-      </c>
-      <c r="J37" t="n">
-        <v>15</v>
-      </c>
-      <c r="K37" t="n">
-        <v>22.39</v>
-      </c>
-      <c r="L37" t="n">
-        <v>23.18</v>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O37" t="n">
-        <v>1011332</v>
-      </c>
-      <c r="P37" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>23.12</v>
-      </c>
-      <c r="R37" t="b">
-        <v>1</v>
-      </c>
-      <c r="S37" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="T37" t="b">
-        <v>0</v>
-      </c>
-      <c r="U37" t="b">
-        <v>0</v>
-      </c>
-      <c r="V37" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="W37" t="n">
-        <v>-1.03</v>
-      </c>
-      <c r="X37" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y37" s="2" t="n">
-        <v>45873.41666666666</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA37" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB37" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="AC37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD37" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="AE37" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="AF37" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="AG37" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="AH37" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI37" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="AJ37" t="inlineStr"/>
-      <c r="AK37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C38" t="b">
-        <v>0</v>
-      </c>
-      <c r="D38" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="F38" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="G38" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="H38" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="I38" t="n">
-        <v>-3.13</v>
-      </c>
-      <c r="J38" t="n">
-        <v>3</v>
-      </c>
-      <c r="K38" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="L38" t="n">
-        <v>21.26</v>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O38" t="n">
-        <v>811883</v>
-      </c>
-      <c r="P38" t="n">
-        <v>2.81</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>21.61</v>
-      </c>
-      <c r="R38" t="b">
-        <v>1</v>
-      </c>
-      <c r="S38" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="T38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U38" t="b">
-        <v>0</v>
-      </c>
-      <c r="V38" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="W38" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="X38" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y38" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="Z38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA38" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB38" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="AC38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD38" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="AE38" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="AF38" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="AG38" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="AH38" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI38" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="AJ38" t="inlineStr"/>
-      <c r="AK38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C39" t="b">
-        <v>0</v>
-      </c>
-      <c r="D39" s="2" t="n">
-        <v>45910.41666666666</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>45972.41666666666</v>
-      </c>
-      <c r="F39" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="G39" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="H39" t="n">
-        <v>24.94</v>
-      </c>
-      <c r="I39" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="J39" t="n">
-        <v>62</v>
-      </c>
-      <c r="K39" t="n">
-        <v>20.28</v>
-      </c>
-      <c r="L39" t="n">
-        <v>20.64</v>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O39" t="n">
-        <v>1216645</v>
-      </c>
-      <c r="P39" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>20.32</v>
-      </c>
-      <c r="R39" t="b">
-        <v>1</v>
-      </c>
-      <c r="S39" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="T39" t="b">
-        <v>0</v>
-      </c>
-      <c r="U39" t="b">
-        <v>0</v>
-      </c>
-      <c r="V39" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="W39" t="n">
-        <v>-2.31</v>
-      </c>
-      <c r="X39" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y39" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="Z39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA39" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB39" s="2" t="n">
-        <v>45910.41666666666</v>
-      </c>
-      <c r="AC39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD39" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="AE39" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="AF39" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="AG39" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="AH39" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI39" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AJ39" t="inlineStr"/>
-      <c r="AK39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C40" t="b">
-        <v>0</v>
-      </c>
-      <c r="D40" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="E40" s="2" t="n">
-        <v>46002.41666666666</v>
-      </c>
-      <c r="F40" t="n">
-        <v>23.44</v>
-      </c>
-      <c r="G40" t="n">
-        <v>23.03</v>
-      </c>
-      <c r="H40" t="n">
-        <v>23.56</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="J40" t="n">
-        <v>8</v>
-      </c>
-      <c r="K40" t="n">
-        <v>22.51</v>
-      </c>
-      <c r="L40" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O40" t="n">
-        <v>2183354</v>
-      </c>
-      <c r="P40" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>22.87</v>
-      </c>
-      <c r="R40" t="b">
-        <v>1</v>
-      </c>
-      <c r="S40" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="T40" t="b">
-        <v>0</v>
-      </c>
-      <c r="U40" t="b">
-        <v>0</v>
-      </c>
-      <c r="V40" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="W40" t="n">
-        <v>-2.43</v>
-      </c>
-      <c r="X40" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
-      <c r="AA40" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB40" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="AC40" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD40" t="n">
-        <v>23.03</v>
-      </c>
-      <c r="AE40" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="AF40" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="AG40" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="AH40" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI40" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="AJ40" t="inlineStr"/>
-      <c r="AK40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C41" t="b">
-        <v>0</v>
-      </c>
-      <c r="D41" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>46027.41666666666</v>
-      </c>
-      <c r="F41" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G41" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="H41" t="n">
-        <v>24.41</v>
-      </c>
-      <c r="I41" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="J41" t="n">
-        <v>11</v>
-      </c>
-      <c r="K41" t="n">
-        <v>23.41</v>
-      </c>
-      <c r="L41" t="n">
-        <v>24.09</v>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O41" t="n">
-        <v>2756109</v>
-      </c>
-      <c r="P41" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>24.08</v>
-      </c>
-      <c r="R41" t="b">
-        <v>1</v>
-      </c>
-      <c r="S41" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="T41" t="b">
-        <v>0</v>
-      </c>
-      <c r="U41" t="b">
-        <v>1</v>
-      </c>
-      <c r="V41" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="W41" t="n">
-        <v>-2.11</v>
-      </c>
-      <c r="X41" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr"/>
-      <c r="AA41" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB41" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="AC41" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD41" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="AE41" t="n">
-        <v>25.69</v>
-      </c>
-      <c r="AF41" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="AG41" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="AH41" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI41" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="AJ41" t="inlineStr"/>
-      <c r="AK41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C42" t="b">
-        <v>0</v>
-      </c>
-      <c r="D42" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="E42" s="2" t="n">
-        <v>46036.41666666666</v>
-      </c>
-      <c r="F42" t="n">
-        <v>26</v>
-      </c>
-      <c r="G42" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="H42" t="n">
-        <v>25.99</v>
-      </c>
-      <c r="I42" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="J42" t="n">
-        <v>8</v>
-      </c>
-      <c r="K42" t="n">
-        <v>24.01</v>
-      </c>
-      <c r="L42" t="n">
-        <v>25.17</v>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O42" t="n">
-        <v>2965366</v>
-      </c>
-      <c r="P42" t="n">
-        <v>6.51</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>24.92</v>
-      </c>
-      <c r="R42" t="b">
-        <v>1</v>
-      </c>
-      <c r="S42" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="T42" t="b">
-        <v>0</v>
-      </c>
-      <c r="U42" t="b">
-        <v>1</v>
-      </c>
-      <c r="V42" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="W42" t="n">
-        <v>-4.15</v>
-      </c>
-      <c r="X42" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y42" s="2" t="n">
-        <v>46033.41666666666</v>
-      </c>
-      <c r="Z42" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA42" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB42" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="AC42" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD42" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="AE42" t="n">
-        <v>27.41</v>
-      </c>
-      <c r="AF42" t="n">
-        <v>6.54</v>
-      </c>
-      <c r="AG42" t="n">
-        <v>5.42</v>
-      </c>
-      <c r="AH42" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI42" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="AJ42" t="inlineStr"/>
-      <c r="AK42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C43" t="b">
-        <v>0</v>
-      </c>
-      <c r="D43" s="2" t="n">
-        <v>46044.41666666666</v>
-      </c>
-      <c r="E43" s="2" t="n">
-        <v>46069.41666666666</v>
-      </c>
-      <c r="F43" t="n">
-        <v>27.31</v>
-      </c>
-      <c r="G43" t="n">
-        <v>26.63</v>
-      </c>
-      <c r="H43" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="I43" t="n">
-        <v>4.36</v>
-      </c>
-      <c r="J43" t="n">
-        <v>25</v>
-      </c>
-      <c r="K43" t="n">
-        <v>25.81</v>
-      </c>
-      <c r="L43" t="n">
-        <v>27.29</v>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O43" t="n">
-        <v>1547845</v>
-      </c>
-      <c r="P43" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="R43" t="b">
-        <v>1</v>
-      </c>
-      <c r="S43" t="n">
-        <v>27.99</v>
-      </c>
-      <c r="T43" t="b">
-        <v>0</v>
-      </c>
-      <c r="U43" t="b">
-        <v>0</v>
-      </c>
-      <c r="V43" t="n">
-        <v>2.49</v>
-      </c>
-      <c r="W43" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="X43" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y43" s="2" t="n">
-        <v>46047.41666666666</v>
-      </c>
-      <c r="Z43" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA43" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB43" s="2" t="n">
-        <v>46044.41666666666</v>
-      </c>
-      <c r="AC43" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD43" t="n">
-        <v>26.63</v>
-      </c>
-      <c r="AE43" t="n">
-        <v>27.99</v>
-      </c>
-      <c r="AF43" t="n">
-        <v>2.49</v>
-      </c>
-      <c r="AG43" t="n">
-        <v>2.49</v>
-      </c>
-      <c r="AH43" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI43" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ43" t="inlineStr"/>
-      <c r="AK43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C44" t="b">
-        <v>0</v>
-      </c>
-      <c r="D44" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="E44" s="2" t="n">
-        <v>46139.41666666666</v>
-      </c>
-      <c r="F44" t="n">
-        <v>26.61</v>
-      </c>
-      <c r="G44" t="n">
-        <v>25.51</v>
-      </c>
-      <c r="H44" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="I44" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="J44" t="n">
-        <v>19</v>
-      </c>
-      <c r="K44" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="L44" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O44" t="n">
-        <v>2499912</v>
-      </c>
-      <c r="P44" t="n">
-        <v>4.31</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>25.73</v>
-      </c>
-      <c r="R44" t="b">
-        <v>1</v>
-      </c>
-      <c r="S44" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="T44" t="b">
-        <v>1</v>
-      </c>
-      <c r="U44" t="b">
-        <v>0</v>
-      </c>
-      <c r="V44" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="W44" t="n">
-        <v>-3.31</v>
-      </c>
-      <c r="X44" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y44" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="Z44" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA44" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB44" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="AC44" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD44" t="n">
-        <v>25.51</v>
-      </c>
-      <c r="AE44" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="AF44" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="AG44" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="AH44" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI44" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="AJ44" t="inlineStr"/>
-      <c r="AK44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5868,31 +4817,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45826.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>66</v>
+        <v>47.87</v>
       </c>
       <c r="G2" t="n">
-        <v>57.6</v>
+        <v>46</v>
       </c>
       <c r="H2" t="n">
         <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>174.24</v>
+        <v>278.11</v>
       </c>
       <c r="J2" t="n">
-        <v>313</v>
+        <v>384</v>
       </c>
       <c r="K2" t="n">
-        <v>53.01</v>
+        <v>45</v>
       </c>
       <c r="L2" t="n">
-        <v>61.79</v>
+        <v>46.89</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -5905,19 +4854,19 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>63278</v>
+        <v>47815</v>
       </c>
       <c r="P2" t="n">
-        <v>10.61</v>
+        <v>2.73</v>
       </c>
       <c r="Q2" t="n">
-        <v>64.90000000000001</v>
+        <v>46.62</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>66.55</v>
+        <v>51</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -5926,16 +4875,16 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>0.83</v>
+        <v>6.54</v>
       </c>
       <c r="W2" t="n">
-        <v>-1.67</v>
+        <v>-2.61</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45826.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="Z2" t="n">
         <v>0</v>
@@ -5944,22 +4893,22 @@
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45826.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>57.6</v>
+        <v>46</v>
       </c>
       <c r="AE2" t="n">
-        <v>66.55</v>
+        <v>51</v>
       </c>
       <c r="AF2" t="n">
-        <v>12.73</v>
+        <v>3.91</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.83</v>
+        <v>6.54</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
@@ -5967,7 +4916,7 @@
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.67</v>
       </c>
       <c r="AJ2" t="n">
         <v>181</v>
@@ -6109,55 +5058,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>30.77</v>
+        <v>27.27</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.71</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.16</v>
+        <v>-2.31</v>
       </c>
       <c r="I2" t="n">
-        <v>-2.07</v>
+        <v>-25.44</v>
       </c>
       <c r="J2" t="n">
-        <v>22.85</v>
+        <v>12.48</v>
       </c>
       <c r="K2" t="n">
         <v>-14.25</v>
       </c>
       <c r="L2" t="n">
-        <v>9.800000000000001</v>
+        <v>7.68</v>
       </c>
       <c r="M2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="N2" t="n">
-        <v>11.7</v>
+        <v>7.98</v>
       </c>
       <c r="O2" t="n">
-        <v>5.43</v>
+        <v>6.17</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.16</v>
+        <v>-2.31</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1480731481481481</v>
+        <v>0.1209768433179723</v>
       </c>
       <c r="R2" t="n">
-        <v>0.04039000000000001</v>
+        <v>-0.09292000000000003</v>
       </c>
       <c r="S2" t="n">
-        <v>0.08346325925925926</v>
+        <v>-0.007361262672811078</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -6165,7 +5114,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.08346325925925926</v>
+        <v>-0.007361262672811078</v>
       </c>
     </row>
     <row r="3">
@@ -6180,55 +5129,55 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
-        <v>43.33</v>
+        <v>52.17</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.28</v>
+        <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.25</v>
+        <v>2.75</v>
       </c>
       <c r="I3" t="n">
-        <v>67.41</v>
+        <v>63.34</v>
       </c>
       <c r="J3" t="n">
-        <v>36.71</v>
+        <v>38.41</v>
       </c>
       <c r="K3" t="n">
-        <v>-5.26</v>
+        <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>8.85</v>
+        <v>10.51</v>
       </c>
       <c r="M3" t="n">
-        <v>2.55</v>
+        <v>2.31</v>
       </c>
       <c r="N3" t="n">
-        <v>8.529999999999999</v>
+        <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>2.56</v>
+        <v>4.39</v>
       </c>
       <c r="P3" t="n">
-        <v>2.25</v>
+        <v>2.75</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5112057106598985</v>
+        <v>0.5176452432667247</v>
       </c>
       <c r="R3" t="n">
-        <v>0.49103</v>
+        <v>0.51042</v>
       </c>
       <c r="S3" t="n">
-        <v>0.4991002842639594</v>
+        <v>0.5133100973066899</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -6236,7 +5185,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.4991002842639594</v>
+        <v>0.5133100973066899</v>
       </c>
     </row>
   </sheetData>
@@ -6307,22 +5256,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.08</v>
+        <v>-0.01</v>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>30.77</v>
+        <v>27.27</v>
       </c>
       <c r="F2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.71</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.16</v>
+        <v>-2.31</v>
       </c>
     </row>
     <row r="3">
@@ -6337,22 +5286,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="D3" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E3" t="n">
-        <v>43.33</v>
+        <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>2.55</v>
+        <v>2.31</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.28</v>
+        <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.25</v>
+        <v>2.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:19:56.405651
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK35"/>
+  <dimension ref="A1:AK27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,7 +983,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -992,101 +992,101 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45554.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>53.91</v>
+        <v>13.43</v>
       </c>
       <c r="G5" t="n">
-        <v>43.72</v>
+        <v>12.66</v>
       </c>
       <c r="H5" t="n">
-        <v>51.11</v>
+        <v>13.26</v>
       </c>
       <c r="I5" t="n">
-        <v>-5.19</v>
+        <v>-1.25</v>
       </c>
       <c r="J5" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="L5" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>3180532</v>
+      </c>
+      <c r="P5" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>12.98</v>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+      <c r="V5" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="W5" t="n">
+        <v>-3.37</v>
+      </c>
+      <c r="X5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>45313.41666666666</v>
+      </c>
+      <c r="Z5" t="n">
         <v>8</v>
       </c>
-      <c r="K5" t="n">
-        <v>43.03</v>
-      </c>
-      <c r="L5" t="n">
-        <v>45.91</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>128396</v>
-      </c>
-      <c r="P5" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>45.33</v>
-      </c>
-      <c r="R5" t="b">
-        <v>1</v>
-      </c>
-      <c r="S5" t="n">
-        <v>48.75</v>
-      </c>
-      <c r="T5" t="b">
-        <v>0</v>
-      </c>
-      <c r="U5" t="b">
-        <v>1</v>
-      </c>
-      <c r="V5" t="n">
-        <v>-9.57</v>
-      </c>
-      <c r="W5" t="n">
-        <v>-15.92</v>
-      </c>
-      <c r="X5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y5" s="2" t="n">
-        <v>45547.41666666666</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1</v>
-      </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>43.72</v>
+        <v>12.66</v>
       </c>
       <c r="AE5" t="n">
-        <v>59.63</v>
+        <v>14.32</v>
       </c>
       <c r="AF5" t="n">
-        <v>18.9</v>
+        <v>5.78</v>
       </c>
       <c r="AG5" t="n">
-        <v>10.61</v>
+        <v>6.61</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.14</v>
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1111,34 +1111,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45558.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45567.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>53.48</v>
+        <v>15.59</v>
       </c>
       <c r="G6" t="n">
-        <v>50.18</v>
+        <v>13.66</v>
       </c>
       <c r="H6" t="n">
-        <v>49.83</v>
+        <v>16</v>
       </c>
       <c r="I6" t="n">
-        <v>-6.82</v>
+        <v>2.62</v>
       </c>
       <c r="J6" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="K6" t="n">
-        <v>50.18</v>
+        <v>12.64</v>
       </c>
       <c r="L6" t="n">
-        <v>52.39</v>
+        <v>14.56</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1151,65 +1151,69 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>188748</v>
+        <v>708583</v>
       </c>
       <c r="P6" t="n">
-        <v>4.9</v>
+        <v>10.05</v>
       </c>
       <c r="Q6" t="n">
-        <v>50.5</v>
+        <v>13.78</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>61.85</v>
+        <v>15.04</v>
       </c>
       <c r="T6" t="b">
         <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>15.65</v>
+        <v>-3.54</v>
       </c>
       <c r="W6" t="n">
-        <v>-5.57</v>
+        <v>-11.62</v>
       </c>
       <c r="X6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>45336.41666666666</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>8</v>
+      </c>
       <c r="AA6" t="b">
         <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>45558.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>50.18</v>
+        <v>13.66</v>
       </c>
       <c r="AE6" t="n">
-        <v>61.85</v>
+        <v>17.99</v>
       </c>
       <c r="AF6" t="n">
-        <v>6.17</v>
+        <v>12.37</v>
       </c>
       <c r="AG6" t="n">
-        <v>15.65</v>
+        <v>15.39</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>2.54</v>
+        <v>1.24</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1217,7 +1221,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1229,31 +1233,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45594.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45601.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>54</v>
+        <v>15.92</v>
       </c>
       <c r="G7" t="n">
-        <v>52.01</v>
+        <v>14.54</v>
       </c>
       <c r="H7" t="n">
-        <v>52</v>
+        <v>14.11</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.7</v>
+        <v>-11.36</v>
       </c>
       <c r="J7" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>44</v>
+        <v>14.54</v>
       </c>
       <c r="L7" t="n">
-        <v>53.95</v>
+        <v>15.68</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1266,57 +1270,61 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>36571</v>
+        <v>2359660</v>
       </c>
       <c r="P7" t="n">
-        <v>3.41</v>
+        <v>3.65</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.51</v>
+        <v>15.3</v>
       </c>
       <c r="R7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>57.99</v>
+        <v>16.22</v>
       </c>
       <c r="T7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>7.39</v>
+        <v>1.88</v>
       </c>
       <c r="W7" t="n">
-        <v>0.9399999999999999</v>
+        <v>-3.89</v>
       </c>
       <c r="X7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45599.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD7" t="n">
-        <v>52.01</v>
+        <v>14.54</v>
       </c>
       <c r="AE7" t="n">
-        <v>57.99</v>
+        <v>16.22</v>
       </c>
       <c r="AF7" t="n">
-        <v>3.69</v>
+        <v>8.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>7.39</v>
+        <v>1.91</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1324,7 +1332,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>2</v>
+        <v>0.22</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1332,7 +1340,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1344,31 +1352,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45603.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45608.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>54.34</v>
+        <v>13.08</v>
       </c>
       <c r="G8" t="n">
-        <v>52.65</v>
+        <v>12.76</v>
       </c>
       <c r="H8" t="n">
-        <v>51.7</v>
+        <v>12.39</v>
       </c>
       <c r="I8" t="n">
-        <v>-4.86</v>
+        <v>-5.26</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>51.6</v>
+        <v>12.22</v>
       </c>
       <c r="L8" t="n">
-        <v>54.24</v>
+        <v>13.04</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1381,19 +1389,19 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>18287</v>
+        <v>5618577</v>
       </c>
       <c r="P8" t="n">
-        <v>0.6899999999999999</v>
+        <v>2.06</v>
       </c>
       <c r="Q8" t="n">
-        <v>53.58</v>
+        <v>12.72</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>57.84</v>
+        <v>14.15</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
@@ -1402,10 +1410,10 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>6.44</v>
+        <v>8.18</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.4</v>
+        <v>-2.75</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1416,22 +1424,22 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45603.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>52.65</v>
+        <v>12.76</v>
       </c>
       <c r="AE8" t="n">
-        <v>57.84</v>
+        <v>14.15</v>
       </c>
       <c r="AF8" t="n">
-        <v>3.11</v>
+        <v>2.45</v>
       </c>
       <c r="AG8" t="n">
-        <v>6.44</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1439,7 +1447,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>2.07</v>
+        <v>3.35</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
@@ -1447,7 +1455,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1459,31 +1467,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45624.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45669.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>49.88</v>
+        <v>11.44</v>
       </c>
       <c r="G9" t="n">
-        <v>47.93</v>
+        <v>10.23</v>
       </c>
       <c r="H9" t="n">
-        <v>55</v>
+        <v>11.76</v>
       </c>
       <c r="I9" t="n">
-        <v>10.26</v>
+        <v>2.8</v>
       </c>
       <c r="J9" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="K9" t="n">
-        <v>48</v>
+        <v>10.01</v>
       </c>
       <c r="L9" t="n">
-        <v>49.58</v>
+        <v>11.2</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1496,19 +1504,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>431</v>
+        <v>3697242</v>
       </c>
       <c r="P9" t="n">
-        <v>1.14</v>
+        <v>10</v>
       </c>
       <c r="Q9" t="n">
-        <v>51.55</v>
+        <v>13.1</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>51.55</v>
+        <v>13.42</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1517,40 +1525,32 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>3.35</v>
+        <v>17.31</v>
       </c>
       <c r="W9" t="n">
-        <v>3.35</v>
+        <v>14.51</v>
       </c>
       <c r="X9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="2" t="n">
-        <v>45631.41666666666</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB9" s="2" t="n">
-        <v>45631.41666666666</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
-        <v>47.93</v>
+        <v>10.23</v>
       </c>
       <c r="AE9" t="n">
-        <v>51.55</v>
+        <v>13.42</v>
       </c>
       <c r="AF9" t="n">
-        <v>3.91</v>
+        <v>10.56</v>
       </c>
       <c r="AG9" t="n">
-        <v>3.35</v>
+        <v>17.34</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.86</v>
+        <v>1.64</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1566,7 +1566,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1578,31 +1578,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45704.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45714.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>47.99</v>
+        <v>12.1</v>
       </c>
       <c r="G10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="H10" t="n">
-        <v>45.81</v>
+        <v>12.4</v>
       </c>
       <c r="I10" t="n">
-        <v>-4.54</v>
+        <v>2.51</v>
       </c>
       <c r="J10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="L10" t="n">
-        <v>47.97</v>
+        <v>12.08</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1615,19 +1615,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>6897</v>
+        <v>719120</v>
       </c>
       <c r="P10" t="n">
-        <v>3.61</v>
+        <v>2.86</v>
       </c>
       <c r="Q10" t="n">
-        <v>48.54</v>
+        <v>11.92</v>
       </c>
       <c r="R10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>50.25</v>
+        <v>12.39</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1636,32 +1636,40 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>4.71</v>
+        <v>2.43</v>
       </c>
       <c r="W10" t="n">
-        <v>1.15</v>
+        <v>-1.46</v>
       </c>
       <c r="X10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y10" s="2" t="n">
+        <v>45426.41666666666</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1</v>
+      </c>
       <c r="AA10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB10" s="2" t="n">
+        <v>45425.41666666666</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
       <c r="AD10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="AE10" t="n">
-        <v>50.25</v>
+        <v>12.39</v>
       </c>
       <c r="AF10" t="n">
-        <v>4.15</v>
+        <v>3.44</v>
       </c>
       <c r="AG10" t="n">
-        <v>4.71</v>
+        <v>2.45</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -1669,7 +1677,7 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>1.13</v>
+        <v>0.71</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1677,7 +1685,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1689,31 +1697,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45727.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>47.51</v>
+        <v>13.23</v>
       </c>
       <c r="G11" t="n">
-        <v>45.8</v>
+        <v>12.37</v>
       </c>
       <c r="H11" t="n">
-        <v>45.63</v>
+        <v>15.11</v>
       </c>
       <c r="I11" t="n">
-        <v>-3.96</v>
+        <v>14.21</v>
       </c>
       <c r="J11" t="n">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="K11" t="n">
-        <v>45.81</v>
+        <v>12.37</v>
       </c>
       <c r="L11" t="n">
-        <v>46.58</v>
+        <v>12.68</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1726,19 +1734,19 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>31257</v>
+        <v>2872871</v>
       </c>
       <c r="P11" t="n">
-        <v>3.04</v>
+        <v>4.75</v>
       </c>
       <c r="Q11" t="n">
-        <v>46.46</v>
+        <v>12.61</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>46.7</v>
+        <v>13.12</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -1747,40 +1755,40 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.7</v>
+        <v>-0.85</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.21</v>
+        <v>-4.7</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45454.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>45.8</v>
+        <v>12.37</v>
       </c>
       <c r="AE11" t="n">
-        <v>48.4</v>
+        <v>13.98</v>
       </c>
       <c r="AF11" t="n">
-        <v>3.6</v>
+        <v>6.53</v>
       </c>
       <c r="AG11" t="n">
-        <v>1.87</v>
+        <v>5.68</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -1788,7 +1796,7 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.52</v>
+        <v>0.87</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1796,7 +1804,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1808,31 +1816,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45754.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>48.44</v>
+        <v>17.1</v>
       </c>
       <c r="G12" t="n">
-        <v>45.88</v>
+        <v>14.96</v>
       </c>
       <c r="H12" t="n">
-        <v>45.51</v>
+        <v>19.46</v>
       </c>
       <c r="I12" t="n">
-        <v>-6.05</v>
+        <v>13.85</v>
       </c>
       <c r="J12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K12" t="n">
-        <v>45.6</v>
+        <v>14.96</v>
       </c>
       <c r="L12" t="n">
-        <v>46.75</v>
+        <v>15.28</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1845,19 +1853,19 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>49292</v>
+        <v>2885185</v>
       </c>
       <c r="P12" t="n">
-        <v>5.14</v>
+        <v>13.79</v>
       </c>
       <c r="Q12" t="n">
-        <v>46.73</v>
+        <v>15.44</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>46.75</v>
+        <v>15.5</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1866,40 +1874,40 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.49</v>
+        <v>-9.34</v>
       </c>
       <c r="W12" t="n">
-        <v>-3.53</v>
+        <v>-9.69</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>45734.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="Z12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>45.88</v>
+        <v>14.96</v>
       </c>
       <c r="AE12" t="n">
-        <v>49.59</v>
+        <v>17.64</v>
       </c>
       <c r="AF12" t="n">
-        <v>5.28</v>
+        <v>12.49</v>
       </c>
       <c r="AG12" t="n">
-        <v>2.37</v>
+        <v>3.18</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1907,7 +1915,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1924,34 +1932,34 @@
         </is>
       </c>
       <c r="C13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45322.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>13.43</v>
+        <v>20.68</v>
       </c>
       <c r="G13" t="n">
-        <v>12.66</v>
+        <v>18.4</v>
       </c>
       <c r="H13" t="n">
-        <v>13.26</v>
+        <v>28.62</v>
       </c>
       <c r="I13" t="n">
-        <v>-1.25</v>
+        <v>38.41</v>
       </c>
       <c r="J13" t="n">
-        <v>21</v>
+        <v>185</v>
       </c>
       <c r="K13" t="n">
-        <v>12.54</v>
+        <v>18.4</v>
       </c>
       <c r="L13" t="n">
-        <v>13.42</v>
+        <v>20.24</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1964,69 +1972,69 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>3180532</v>
+        <v>807277</v>
       </c>
       <c r="P13" t="n">
-        <v>3.32</v>
+        <v>2.17</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.98</v>
+        <v>20.54</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>13.42</v>
+        <v>23.04</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.09</v>
+        <v>11.41</v>
       </c>
       <c r="W13" t="n">
-        <v>-3.37</v>
+        <v>-0.68</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45313.41666666666</v>
+        <v>45572.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>12.66</v>
+        <v>18.4</v>
       </c>
       <c r="AE13" t="n">
-        <v>14.32</v>
+        <v>23.04</v>
       </c>
       <c r="AF13" t="n">
-        <v>5.78</v>
+        <v>11.03</v>
       </c>
       <c r="AG13" t="n">
-        <v>6.61</v>
+        <v>11.41</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.14</v>
+        <v>1.03</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2043,34 +2051,34 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>15.59</v>
+        <v>28.64</v>
       </c>
       <c r="G14" t="n">
-        <v>13.66</v>
+        <v>28.08</v>
       </c>
       <c r="H14" t="n">
-        <v>16</v>
+        <v>27.22</v>
       </c>
       <c r="I14" t="n">
-        <v>2.62</v>
+        <v>-4.97</v>
       </c>
       <c r="J14" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>12.64</v>
+        <v>28</v>
       </c>
       <c r="L14" t="n">
-        <v>14.56</v>
+        <v>28.48</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2083,69 +2091,69 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>708583</v>
+        <v>1546271</v>
       </c>
       <c r="P14" t="n">
-        <v>10.05</v>
+        <v>1.79</v>
       </c>
       <c r="Q14" t="n">
-        <v>13.78</v>
+        <v>28.16</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>15.04</v>
+        <v>29</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.54</v>
+        <v>1.26</v>
       </c>
       <c r="W14" t="n">
-        <v>-11.62</v>
+        <v>-1.68</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>45336.41666666666</v>
+        <v>45729.41666666666</v>
       </c>
       <c r="Z14" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>13.66</v>
+        <v>28.08</v>
       </c>
       <c r="AE14" t="n">
-        <v>17.99</v>
+        <v>29</v>
       </c>
       <c r="AF14" t="n">
-        <v>12.37</v>
+        <v>1.96</v>
       </c>
       <c r="AG14" t="n">
-        <v>15.39</v>
+        <v>1.26</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>1.24</v>
+        <v>0.64</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2165,31 +2173,31 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45379.41666666666</v>
+        <v>45756.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>15.92</v>
+        <v>25.97</v>
       </c>
       <c r="G15" t="n">
-        <v>14.54</v>
+        <v>24.72</v>
       </c>
       <c r="H15" t="n">
-        <v>14.11</v>
+        <v>24.16</v>
       </c>
       <c r="I15" t="n">
-        <v>-11.36</v>
+        <v>-6.96</v>
       </c>
       <c r="J15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K15" t="n">
-        <v>14.54</v>
+        <v>24.68</v>
       </c>
       <c r="L15" t="n">
-        <v>15.68</v>
+        <v>25.51</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2202,61 +2210,53 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>2359660</v>
+        <v>767605</v>
       </c>
       <c r="P15" t="n">
-        <v>3.65</v>
+        <v>4.04</v>
       </c>
       <c r="Q15" t="n">
-        <v>15.3</v>
+        <v>27.46</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>16.22</v>
+        <v>29.03</v>
       </c>
       <c r="T15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15" t="b">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>1.88</v>
+        <v>11.79</v>
       </c>
       <c r="W15" t="n">
-        <v>-3.89</v>
+        <v>5.75</v>
       </c>
       <c r="X15" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y15" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB15" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="n">
-        <v>14.54</v>
+        <v>24.72</v>
       </c>
       <c r="AE15" t="n">
-        <v>16.22</v>
+        <v>29.03</v>
       </c>
       <c r="AF15" t="n">
-        <v>8.69</v>
+        <v>4.81</v>
       </c>
       <c r="AG15" t="n">
-        <v>1.91</v>
+        <v>11.8</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.22</v>
+        <v>2.45</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2284,31 +2284,31 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>13.08</v>
+        <v>25.32</v>
       </c>
       <c r="G16" t="n">
-        <v>12.76</v>
+        <v>24.12</v>
       </c>
       <c r="H16" t="n">
-        <v>12.39</v>
+        <v>23.99</v>
       </c>
       <c r="I16" t="n">
-        <v>-5.26</v>
+        <v>-5.24</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K16" t="n">
-        <v>12.22</v>
+        <v>24.12</v>
       </c>
       <c r="L16" t="n">
-        <v>13.04</v>
+        <v>25.26</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>5618577</v>
+        <v>623052</v>
       </c>
       <c r="P16" t="n">
-        <v>2.06</v>
+        <v>0.96</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.72</v>
+        <v>26.96</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>14.15</v>
+        <v>26.96</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2342,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>8.18</v>
+        <v>6.48</v>
       </c>
       <c r="W16" t="n">
-        <v>-2.75</v>
+        <v>6.48</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -2353,25 +2353,21 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB16" s="2" t="n">
-        <v>45398.41666666666</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="n">
-        <v>12.76</v>
+        <v>24.12</v>
       </c>
       <c r="AE16" t="n">
-        <v>14.15</v>
+        <v>26.96</v>
       </c>
       <c r="AF16" t="n">
-        <v>2.45</v>
+        <v>4.74</v>
       </c>
       <c r="AG16" t="n">
-        <v>8.199999999999999</v>
+        <v>6.48</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2379,7 +2375,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>3.35</v>
+        <v>1.37</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2399,31 +2395,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>11.44</v>
+        <v>22.75</v>
       </c>
       <c r="G17" t="n">
-        <v>10.23</v>
+        <v>21.66</v>
       </c>
       <c r="H17" t="n">
-        <v>11.76</v>
+        <v>21.65</v>
       </c>
       <c r="I17" t="n">
-        <v>2.8</v>
+        <v>-4.85</v>
       </c>
       <c r="J17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K17" t="n">
-        <v>10.01</v>
+        <v>21.66</v>
       </c>
       <c r="L17" t="n">
-        <v>11.2</v>
+        <v>22.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2436,19 +2432,19 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>3697242</v>
+        <v>13689820</v>
       </c>
       <c r="P17" t="n">
-        <v>10</v>
+        <v>4.94</v>
       </c>
       <c r="Q17" t="n">
-        <v>13.1</v>
+        <v>23.7</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>13.42</v>
+        <v>25.75</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -2457,10 +2453,10 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>17.31</v>
+        <v>13.18</v>
       </c>
       <c r="W17" t="n">
-        <v>14.51</v>
+        <v>4.17</v>
       </c>
       <c r="X17" t="b">
         <v>0</v>
@@ -2473,16 +2469,16 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>10.23</v>
+        <v>21.66</v>
       </c>
       <c r="AE17" t="n">
-        <v>13.42</v>
+        <v>25.75</v>
       </c>
       <c r="AF17" t="n">
-        <v>10.56</v>
+        <v>4.78</v>
       </c>
       <c r="AG17" t="n">
-        <v>17.34</v>
+        <v>13.19</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2490,7 +2486,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>1.64</v>
+        <v>2.76</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2510,31 +2506,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45434.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>12.1</v>
+        <v>21.88</v>
       </c>
       <c r="G18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="H18" t="n">
-        <v>12.4</v>
+        <v>20.53</v>
       </c>
       <c r="I18" t="n">
-        <v>2.51</v>
+        <v>-6.18</v>
       </c>
       <c r="J18" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="L18" t="n">
-        <v>12.08</v>
+        <v>21.78</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2547,19 +2543,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>719120</v>
+        <v>1476660</v>
       </c>
       <c r="P18" t="n">
-        <v>2.86</v>
+        <v>1.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.92</v>
+        <v>21.54</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>12.39</v>
+        <v>22.52</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2568,40 +2564,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>2.43</v>
+        <v>2.93</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.46</v>
+        <v>-1.55</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>45426.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="AE18" t="n">
-        <v>12.39</v>
+        <v>22.52</v>
       </c>
       <c r="AF18" t="n">
-        <v>3.44</v>
+        <v>2.41</v>
       </c>
       <c r="AG18" t="n">
-        <v>2.45</v>
+        <v>2.93</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2609,7 +2605,7 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.71</v>
+        <v>1.22</v>
       </c>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
@@ -2629,31 +2625,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>13.23</v>
+        <v>21.16</v>
       </c>
       <c r="G19" t="n">
-        <v>12.37</v>
+        <v>19.2</v>
       </c>
       <c r="H19" t="n">
-        <v>15.11</v>
+        <v>21.32</v>
       </c>
       <c r="I19" t="n">
-        <v>14.21</v>
+        <v>0.76</v>
       </c>
       <c r="J19" t="n">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="K19" t="n">
-        <v>12.37</v>
+        <v>19.92</v>
       </c>
       <c r="L19" t="n">
-        <v>12.68</v>
+        <v>20.64</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2666,69 +2662,65 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>2872871</v>
+        <v>5666121</v>
       </c>
       <c r="P19" t="n">
         <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>12.61</v>
+        <v>22.02</v>
       </c>
       <c r="R19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>13.12</v>
+        <v>22.52</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
       </c>
       <c r="U19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.85</v>
+        <v>6.43</v>
       </c>
       <c r="W19" t="n">
-        <v>-4.7</v>
+        <v>4.06</v>
       </c>
       <c r="X19" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="2" t="n">
-        <v>45454.41666666666</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD19" t="n">
-        <v>12.37</v>
+        <v>19.2</v>
       </c>
       <c r="AE19" t="n">
-        <v>13.98</v>
+        <v>22.52</v>
       </c>
       <c r="AF19" t="n">
-        <v>6.53</v>
+        <v>9.26</v>
       </c>
       <c r="AG19" t="n">
-        <v>5.68</v>
+        <v>6.43</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.87</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
@@ -2748,31 +2740,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45845.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>17.1</v>
+        <v>21.91</v>
       </c>
       <c r="G20" t="n">
-        <v>14.96</v>
+        <v>21.28</v>
       </c>
       <c r="H20" t="n">
-        <v>19.46</v>
+        <v>22.48</v>
       </c>
       <c r="I20" t="n">
-        <v>13.85</v>
+        <v>2.59</v>
       </c>
       <c r="J20" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="K20" t="n">
-        <v>14.96</v>
+        <v>21.29</v>
       </c>
       <c r="L20" t="n">
-        <v>15.28</v>
+        <v>21.84</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2785,69 +2777,69 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>2885185</v>
+        <v>1366828</v>
       </c>
       <c r="P20" t="n">
-        <v>13.79</v>
+        <v>1.44</v>
       </c>
       <c r="Q20" t="n">
-        <v>15.44</v>
+        <v>22.06</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>15.5</v>
+        <v>22.44</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20" t="n">
-        <v>-9.34</v>
+        <v>2.41</v>
       </c>
       <c r="W20" t="n">
-        <v>-9.69</v>
+        <v>0.68</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="Z20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="AC20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD20" t="n">
-        <v>14.96</v>
+        <v>21.28</v>
       </c>
       <c r="AE20" t="n">
-        <v>17.64</v>
+        <v>22.44</v>
       </c>
       <c r="AF20" t="n">
-        <v>12.49</v>
+        <v>2.88</v>
       </c>
       <c r="AG20" t="n">
-        <v>3.18</v>
+        <v>2.41</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.25</v>
+        <v>0.84</v>
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
@@ -2867,31 +2859,31 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45889.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>20.68</v>
+        <v>23.36</v>
       </c>
       <c r="G21" t="n">
-        <v>18.4</v>
+        <v>22.64</v>
       </c>
       <c r="H21" t="n">
-        <v>28.62</v>
+        <v>21.62</v>
       </c>
       <c r="I21" t="n">
-        <v>38.41</v>
+        <v>-7.43</v>
       </c>
       <c r="J21" t="n">
-        <v>185</v>
+        <v>17</v>
       </c>
       <c r="K21" t="n">
-        <v>18.4</v>
+        <v>22.39</v>
       </c>
       <c r="L21" t="n">
-        <v>20.24</v>
+        <v>23.18</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2904,61 +2896,61 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>807277</v>
+        <v>1011332</v>
       </c>
       <c r="P21" t="n">
-        <v>2.17</v>
+        <v>1.74</v>
       </c>
       <c r="Q21" t="n">
-        <v>20.54</v>
+        <v>23.34</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>23.04</v>
+        <v>23.48</v>
       </c>
       <c r="T21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U21" t="b">
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>11.41</v>
+        <v>0.51</v>
       </c>
       <c r="W21" t="n">
-        <v>-0.68</v>
+        <v>-0.09</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45572.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>18.4</v>
+        <v>22.64</v>
       </c>
       <c r="AE21" t="n">
-        <v>23.04</v>
+        <v>23.48</v>
       </c>
       <c r="AF21" t="n">
-        <v>11.03</v>
+        <v>3.08</v>
       </c>
       <c r="AG21" t="n">
-        <v>11.41</v>
+        <v>0.51</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2966,7 +2958,7 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>1.03</v>
+        <v>0.17</v>
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
@@ -2986,31 +2978,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45902.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>28.64</v>
+        <v>21.7</v>
       </c>
       <c r="G22" t="n">
-        <v>28.08</v>
+        <v>21.02</v>
       </c>
       <c r="H22" t="n">
-        <v>27.22</v>
+        <v>20.82</v>
       </c>
       <c r="I22" t="n">
-        <v>-4.97</v>
+        <v>-4.02</v>
       </c>
       <c r="J22" t="n">
         <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>28</v>
+        <v>21.02</v>
       </c>
       <c r="L22" t="n">
-        <v>28.48</v>
+        <v>21.26</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3023,19 +3015,19 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>1546271</v>
+        <v>811883</v>
       </c>
       <c r="P22" t="n">
-        <v>1.79</v>
+        <v>2.81</v>
       </c>
       <c r="Q22" t="n">
-        <v>28.16</v>
+        <v>21.61</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>29</v>
+        <v>21.83</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
@@ -3044,16 +3036,16 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>1.26</v>
+        <v>0.62</v>
       </c>
       <c r="W22" t="n">
-        <v>-1.68</v>
+        <v>-0.4</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -3062,22 +3054,22 @@
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>28.08</v>
+        <v>21.02</v>
       </c>
       <c r="AE22" t="n">
-        <v>29</v>
+        <v>21.83</v>
       </c>
       <c r="AF22" t="n">
-        <v>1.96</v>
+        <v>3.13</v>
       </c>
       <c r="AG22" t="n">
-        <v>1.26</v>
+        <v>0.63</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
@@ -3085,7 +3077,7 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.64</v>
+        <v>0.2</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3105,31 +3097,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45754.41666666666</v>
+        <v>45972.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>25.97</v>
+        <v>21.51</v>
       </c>
       <c r="G23" t="n">
-        <v>24.72</v>
+        <v>20.27</v>
       </c>
       <c r="H23" t="n">
-        <v>25.2</v>
+        <v>24.94</v>
       </c>
       <c r="I23" t="n">
-        <v>-2.96</v>
+        <v>15.94</v>
       </c>
       <c r="J23" t="n">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="K23" t="n">
-        <v>24.68</v>
+        <v>20.28</v>
       </c>
       <c r="L23" t="n">
-        <v>25.51</v>
+        <v>20.96</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3142,61 +3134,69 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>767605</v>
+        <v>2694406</v>
       </c>
       <c r="P23" t="n">
-        <v>4.04</v>
+        <v>3.42</v>
       </c>
       <c r="Q23" t="n">
-        <v>27.46</v>
+        <v>21.93</v>
       </c>
       <c r="R23" t="b">
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>29.03</v>
+        <v>20.96</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
       </c>
       <c r="U23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V23" t="n">
-        <v>11.79</v>
+        <v>-2.57</v>
       </c>
       <c r="W23" t="n">
-        <v>5.75</v>
+        <v>1.94</v>
       </c>
       <c r="X23" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y23" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>8</v>
+      </c>
       <c r="AA23" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB23" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>8</v>
+      </c>
       <c r="AD23" t="n">
-        <v>24.72</v>
+        <v>20.27</v>
       </c>
       <c r="AE23" t="n">
-        <v>29.03</v>
+        <v>22.19</v>
       </c>
       <c r="AF23" t="n">
-        <v>4.81</v>
+        <v>5.76</v>
       </c>
       <c r="AG23" t="n">
-        <v>11.8</v>
+        <v>3.16</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>2.45</v>
+        <v>0.55</v>
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
@@ -3216,31 +3216,31 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45994.41666666666</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>45783.41666666666</v>
+        <v>46002.41666666666</v>
       </c>
       <c r="F24" t="n">
-        <v>25.32</v>
+        <v>23.44</v>
       </c>
       <c r="G24" t="n">
-        <v>24.12</v>
+        <v>22.68</v>
       </c>
       <c r="H24" t="n">
-        <v>23.99</v>
+        <v>23.56</v>
       </c>
       <c r="I24" t="n">
-        <v>-5.24</v>
+        <v>0.51</v>
       </c>
       <c r="J24" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="K24" t="n">
-        <v>24.12</v>
+        <v>22.51</v>
       </c>
       <c r="L24" t="n">
-        <v>25.26</v>
+        <v>23.2</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>623052</v>
+        <v>2183354</v>
       </c>
       <c r="P24" t="n">
-        <v>0.96</v>
+        <v>1.78</v>
       </c>
       <c r="Q24" t="n">
-        <v>26.96</v>
+        <v>22.87</v>
       </c>
       <c r="R24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>26.96</v>
+        <v>24.98</v>
       </c>
       <c r="T24" t="b">
         <v>0</v>
@@ -3274,10 +3274,10 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>6.48</v>
+        <v>6.57</v>
       </c>
       <c r="W24" t="n">
-        <v>6.48</v>
+        <v>-2.43</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3285,21 +3285,25 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB24" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0</v>
+      </c>
       <c r="AD24" t="n">
-        <v>24.12</v>
+        <v>22.68</v>
       </c>
       <c r="AE24" t="n">
-        <v>26.96</v>
+        <v>24.98</v>
       </c>
       <c r="AF24" t="n">
-        <v>4.74</v>
+        <v>3.24</v>
       </c>
       <c r="AG24" t="n">
-        <v>6.48</v>
+        <v>6.57</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
@@ -3307,7 +3311,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>1.37</v>
+        <v>2.03</v>
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
@@ -3327,31 +3331,31 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>46016.41666666666</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>46027.41666666666</v>
       </c>
       <c r="F25" t="n">
-        <v>22.75</v>
+        <v>24.6</v>
       </c>
       <c r="G25" t="n">
-        <v>21.66</v>
+        <v>23.75</v>
       </c>
       <c r="H25" t="n">
-        <v>21.65</v>
+        <v>24.41</v>
       </c>
       <c r="I25" t="n">
-        <v>-4.85</v>
+        <v>-0.77</v>
       </c>
       <c r="J25" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K25" t="n">
-        <v>21.66</v>
+        <v>23.41</v>
       </c>
       <c r="L25" t="n">
-        <v>22.2</v>
+        <v>24.09</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3364,31 +3368,31 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>13689820</v>
+        <v>2756109</v>
       </c>
       <c r="P25" t="n">
-        <v>4.94</v>
+        <v>3.54</v>
       </c>
       <c r="Q25" t="n">
-        <v>23.7</v>
+        <v>24.08</v>
       </c>
       <c r="R25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>25.75</v>
+        <v>24.5</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
       </c>
       <c r="U25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V25" t="n">
-        <v>13.18</v>
+        <v>-0.41</v>
       </c>
       <c r="W25" t="n">
-        <v>4.17</v>
+        <v>-2.11</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -3396,29 +3400,33 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB25" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0</v>
+      </c>
       <c r="AD25" t="n">
-        <v>21.66</v>
+        <v>23.75</v>
       </c>
       <c r="AE25" t="n">
-        <v>25.75</v>
+        <v>25.69</v>
       </c>
       <c r="AF25" t="n">
-        <v>4.78</v>
+        <v>3.46</v>
       </c>
       <c r="AG25" t="n">
-        <v>13.19</v>
+        <v>4.43</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>2.76</v>
+        <v>1.28</v>
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
@@ -3438,31 +3446,31 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>46069.41666666666</v>
       </c>
       <c r="F26" t="n">
-        <v>21.88</v>
+        <v>26</v>
       </c>
       <c r="G26" t="n">
-        <v>21.35</v>
+        <v>24.3</v>
       </c>
       <c r="H26" t="n">
-        <v>20.53</v>
+        <v>28.5</v>
       </c>
       <c r="I26" t="n">
-        <v>-6.18</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="K26" t="n">
-        <v>21.35</v>
+        <v>24.01</v>
       </c>
       <c r="L26" t="n">
-        <v>21.78</v>
+        <v>25.42</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3475,37 +3483,37 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>1476660</v>
+        <v>2965366</v>
       </c>
       <c r="P26" t="n">
-        <v>1.3</v>
+        <v>6.51</v>
       </c>
       <c r="Q26" t="n">
-        <v>21.54</v>
+        <v>25.42</v>
       </c>
       <c r="R26" t="b">
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>22.52</v>
+        <v>25.42</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
       </c>
       <c r="U26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V26" t="n">
-        <v>2.93</v>
+        <v>-2.23</v>
       </c>
       <c r="W26" t="n">
-        <v>-1.55</v>
+        <v>-2.23</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>45818.41666666666</v>
+        <v>46033.41666666666</v>
       </c>
       <c r="Z26" t="n">
         <v>2</v>
@@ -3514,30 +3522,30 @@
         <v>1</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>21.35</v>
+        <v>24.3</v>
       </c>
       <c r="AE26" t="n">
-        <v>22.52</v>
+        <v>27.41</v>
       </c>
       <c r="AF26" t="n">
-        <v>2.41</v>
+        <v>6.54</v>
       </c>
       <c r="AG26" t="n">
-        <v>2.93</v>
+        <v>5.42</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>1.22</v>
+        <v>0.83</v>
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
@@ -3557,31 +3565,31 @@
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>46120.41666666666</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>46139.41666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>21.16</v>
+        <v>26.61</v>
       </c>
       <c r="G27" t="n">
-        <v>19.2</v>
+        <v>25.4</v>
       </c>
       <c r="H27" t="n">
-        <v>21.32</v>
+        <v>28.7</v>
       </c>
       <c r="I27" t="n">
-        <v>0.76</v>
+        <v>7.85</v>
       </c>
       <c r="J27" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="K27" t="n">
-        <v>19.92</v>
+        <v>23.8</v>
       </c>
       <c r="L27" t="n">
-        <v>20.64</v>
+        <v>25.7</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3594,57 +3602,61 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>5666121</v>
+        <v>2499912</v>
       </c>
       <c r="P27" t="n">
-        <v>4.75</v>
+        <v>4.31</v>
       </c>
       <c r="Q27" t="n">
-        <v>22.02</v>
+        <v>25.73</v>
       </c>
       <c r="R27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S27" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="T27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U27" t="b">
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="W27" t="n">
-        <v>4.06</v>
+        <v>-3.31</v>
       </c>
       <c r="X27" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y27" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
       <c r="AA27" t="b">
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>45833.41666666666</v>
+        <v>46120.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>19.2</v>
+        <v>25.4</v>
       </c>
       <c r="AE27" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="AF27" t="n">
-        <v>9.26</v>
+        <v>4.55</v>
       </c>
       <c r="AG27" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -3652,954 +3664,10 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.16</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C28" t="b">
-        <v>0</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>45845.41666666666</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>45860.41666666666</v>
-      </c>
-      <c r="F28" t="n">
-        <v>21.91</v>
-      </c>
-      <c r="G28" t="n">
-        <v>21.28</v>
-      </c>
-      <c r="H28" t="n">
-        <v>22.48</v>
-      </c>
-      <c r="I28" t="n">
-        <v>2.59</v>
-      </c>
-      <c r="J28" t="n">
-        <v>15</v>
-      </c>
-      <c r="K28" t="n">
-        <v>21.29</v>
-      </c>
-      <c r="L28" t="n">
-        <v>21.84</v>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O28" t="n">
-        <v>1366828</v>
-      </c>
-      <c r="P28" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>22.06</v>
-      </c>
-      <c r="R28" t="b">
-        <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="T28" t="b">
-        <v>0</v>
-      </c>
-      <c r="U28" t="b">
-        <v>0</v>
-      </c>
-      <c r="V28" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="W28" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="X28" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y28" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA28" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB28" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="AC28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD28" t="n">
-        <v>21.28</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="AH28" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI28" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AJ28" t="inlineStr"/>
-      <c r="AK28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C29" t="b">
-        <v>0</v>
-      </c>
-      <c r="D29" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>45887.41666666666</v>
-      </c>
-      <c r="F29" t="n">
-        <v>23.36</v>
-      </c>
-      <c r="G29" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="H29" t="n">
-        <v>22.81</v>
-      </c>
-      <c r="I29" t="n">
-        <v>-2.36</v>
-      </c>
-      <c r="J29" t="n">
-        <v>15</v>
-      </c>
-      <c r="K29" t="n">
-        <v>22.39</v>
-      </c>
-      <c r="L29" t="n">
-        <v>23.18</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O29" t="n">
-        <v>1011332</v>
-      </c>
-      <c r="P29" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>23.12</v>
-      </c>
-      <c r="R29" t="b">
-        <v>1</v>
-      </c>
-      <c r="S29" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="T29" t="b">
-        <v>0</v>
-      </c>
-      <c r="U29" t="b">
-        <v>0</v>
-      </c>
-      <c r="V29" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="W29" t="n">
-        <v>-1.03</v>
-      </c>
-      <c r="X29" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y29" s="2" t="n">
-        <v>45873.41666666666</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA29" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB29" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="AC29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="AE29" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="AF29" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="AG29" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="AH29" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI29" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="AJ29" t="inlineStr"/>
-      <c r="AK29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C30" t="b">
-        <v>0</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="F30" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="G30" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="H30" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="I30" t="n">
-        <v>-3.13</v>
-      </c>
-      <c r="J30" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="L30" t="n">
-        <v>21.26</v>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O30" t="n">
-        <v>811883</v>
-      </c>
-      <c r="P30" t="n">
-        <v>2.81</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>21.61</v>
-      </c>
-      <c r="R30" t="b">
-        <v>1</v>
-      </c>
-      <c r="S30" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="T30" t="b">
-        <v>0</v>
-      </c>
-      <c r="U30" t="b">
-        <v>0</v>
-      </c>
-      <c r="V30" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="W30" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="X30" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y30" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA30" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB30" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="AC30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="AE30" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="AF30" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="AG30" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="AH30" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI30" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="AJ30" t="inlineStr"/>
-      <c r="AK30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C31" t="b">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>45972.41666666666</v>
-      </c>
-      <c r="F31" t="n">
-        <v>21.51</v>
-      </c>
-      <c r="G31" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="H31" t="n">
-        <v>24.94</v>
-      </c>
-      <c r="I31" t="n">
-        <v>15.94</v>
-      </c>
-      <c r="J31" t="n">
-        <v>61</v>
-      </c>
-      <c r="K31" t="n">
-        <v>20.28</v>
-      </c>
-      <c r="L31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O31" t="n">
-        <v>2694406</v>
-      </c>
-      <c r="P31" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="R31" t="b">
-        <v>1</v>
-      </c>
-      <c r="S31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="T31" t="b">
-        <v>0</v>
-      </c>
-      <c r="U31" t="b">
-        <v>1</v>
-      </c>
-      <c r="V31" t="n">
-        <v>-2.57</v>
-      </c>
-      <c r="W31" t="n">
-        <v>-2.57</v>
-      </c>
-      <c r="X31" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y31" s="2" t="n">
-        <v>45923.41666666666</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA31" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB31" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="AE31" t="n">
-        <v>22.19</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>5.76</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="AH31" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI31" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AJ31" t="inlineStr"/>
-      <c r="AK31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C32" t="b">
-        <v>0</v>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>46002.41666666666</v>
-      </c>
-      <c r="F32" t="n">
-        <v>23.44</v>
-      </c>
-      <c r="G32" t="n">
-        <v>22.68</v>
-      </c>
-      <c r="H32" t="n">
-        <v>23.56</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="J32" t="n">
-        <v>8</v>
-      </c>
-      <c r="K32" t="n">
-        <v>22.51</v>
-      </c>
-      <c r="L32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O32" t="n">
-        <v>2183354</v>
-      </c>
-      <c r="P32" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>22.87</v>
-      </c>
-      <c r="R32" t="b">
-        <v>1</v>
-      </c>
-      <c r="S32" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="T32" t="b">
-        <v>0</v>
-      </c>
-      <c r="U32" t="b">
-        <v>0</v>
-      </c>
-      <c r="V32" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="W32" t="n">
-        <v>-2.43</v>
-      </c>
-      <c r="X32" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB32" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="AC32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>22.68</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="AG32" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="AH32" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI32" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AJ32" t="inlineStr"/>
-      <c r="AK32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C33" t="b">
-        <v>0</v>
-      </c>
-      <c r="D33" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>46027.41666666666</v>
-      </c>
-      <c r="F33" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G33" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="H33" t="n">
-        <v>24.41</v>
-      </c>
-      <c r="I33" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="J33" t="n">
-        <v>11</v>
-      </c>
-      <c r="K33" t="n">
-        <v>23.41</v>
-      </c>
-      <c r="L33" t="n">
-        <v>24.09</v>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O33" t="n">
-        <v>2756109</v>
-      </c>
-      <c r="P33" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>24.08</v>
-      </c>
-      <c r="R33" t="b">
-        <v>1</v>
-      </c>
-      <c r="S33" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="T33" t="b">
-        <v>0</v>
-      </c>
-      <c r="U33" t="b">
-        <v>1</v>
-      </c>
-      <c r="V33" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="W33" t="n">
-        <v>-2.11</v>
-      </c>
-      <c r="X33" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB33" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="AC33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD33" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="AE33" t="n">
-        <v>25.69</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="AH33" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI33" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="AJ33" t="inlineStr"/>
-      <c r="AK33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C34" t="b">
-        <v>0</v>
-      </c>
-      <c r="D34" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>46069.41666666666</v>
-      </c>
-      <c r="F34" t="n">
-        <v>26</v>
-      </c>
-      <c r="G34" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="H34" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="I34" t="n">
-        <v>9.619999999999999</v>
-      </c>
-      <c r="J34" t="n">
-        <v>41</v>
-      </c>
-      <c r="K34" t="n">
-        <v>24.01</v>
-      </c>
-      <c r="L34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O34" t="n">
-        <v>2965366</v>
-      </c>
-      <c r="P34" t="n">
-        <v>6.51</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="R34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="T34" t="b">
-        <v>0</v>
-      </c>
-      <c r="U34" t="b">
-        <v>1</v>
-      </c>
-      <c r="V34" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="W34" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="X34" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y34" s="2" t="n">
-        <v>46033.41666666666</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA34" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB34" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="AC34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="AE34" t="n">
-        <v>27.41</v>
-      </c>
-      <c r="AF34" t="n">
-        <v>6.54</v>
-      </c>
-      <c r="AG34" t="n">
-        <v>5.42</v>
-      </c>
-      <c r="AH34" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI34" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="AJ34" t="inlineStr"/>
-      <c r="AK34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C35" t="b">
-        <v>0</v>
-      </c>
-      <c r="D35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>46139.41666666666</v>
-      </c>
-      <c r="F35" t="n">
-        <v>26.61</v>
-      </c>
-      <c r="G35" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="H35" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="I35" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="J35" t="n">
-        <v>19</v>
-      </c>
-      <c r="K35" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="L35" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O35" t="n">
-        <v>2499912</v>
-      </c>
-      <c r="P35" t="n">
-        <v>4.31</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>25.73</v>
-      </c>
-      <c r="R35" t="b">
-        <v>1</v>
-      </c>
-      <c r="S35" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="T35" t="b">
-        <v>1</v>
-      </c>
-      <c r="U35" t="b">
-        <v>0</v>
-      </c>
-      <c r="V35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="W35" t="n">
-        <v>-3.31</v>
-      </c>
-      <c r="X35" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA35" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="AC35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="AE35" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="AG35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="AH35" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI35" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AJ35" t="inlineStr"/>
-      <c r="AK35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4817,31 +3885,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>47.87</v>
+        <v>53.91</v>
       </c>
       <c r="G2" t="n">
-        <v>46</v>
+        <v>43.72</v>
       </c>
       <c r="H2" t="n">
         <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>278.11</v>
+        <v>235.74</v>
       </c>
       <c r="J2" t="n">
-        <v>384</v>
+        <v>593</v>
       </c>
       <c r="K2" t="n">
-        <v>45</v>
+        <v>43.03</v>
       </c>
       <c r="L2" t="n">
-        <v>46.89</v>
+        <v>45.91</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -4854,37 +3922,37 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>47815</v>
+        <v>128396</v>
       </c>
       <c r="P2" t="n">
-        <v>2.73</v>
+        <v>19.99</v>
       </c>
       <c r="Q2" t="n">
-        <v>46.62</v>
+        <v>54.94</v>
       </c>
       <c r="R2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>51</v>
+        <v>48.75</v>
       </c>
       <c r="T2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>6.54</v>
+        <v>-9.57</v>
       </c>
       <c r="W2" t="n">
-        <v>-2.61</v>
+        <v>1.91</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="Z2" t="n">
         <v>0</v>
@@ -4893,30 +3961,30 @@
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45547.41666666666</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD2" t="n">
-        <v>46</v>
+        <v>43.72</v>
       </c>
       <c r="AE2" t="n">
-        <v>51</v>
+        <v>59.63</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.91</v>
+        <v>18.9</v>
       </c>
       <c r="AG2" t="n">
-        <v>6.54</v>
+        <v>10.61</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>1.67</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ2" t="n">
         <v>181</v>
@@ -5058,25 +4126,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>27.27</v>
+        <v>66.67</v>
       </c>
       <c r="G2" t="n">
-        <v>-4.54</v>
+        <v>1.19</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
       <c r="I2" t="n">
-        <v>-25.44</v>
+        <v>-0.58</v>
       </c>
       <c r="J2" t="n">
         <v>12.48</v>
@@ -5085,28 +4153,28 @@
         <v>-14.25</v>
       </c>
       <c r="L2" t="n">
-        <v>7.68</v>
+        <v>13.42</v>
       </c>
       <c r="M2" t="n">
-        <v>0.48</v>
+        <v>0.96</v>
       </c>
       <c r="N2" t="n">
-        <v>7.98</v>
+        <v>6.84</v>
       </c>
       <c r="O2" t="n">
-        <v>6.17</v>
+        <v>14.25</v>
       </c>
       <c r="P2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1209768433179723</v>
+        <v>0.2320120319001387</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.09292000000000003</v>
+        <v>0.09086</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.007361262672811078</v>
+        <v>0.1473208127600555</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -5114,7 +4182,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>-0.007361262672811078</v>
+        <v>0.1473208127600555</v>
       </c>
     </row>
     <row r="3">
@@ -5144,10 +4212,10 @@
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.75</v>
+        <v>2.32</v>
       </c>
       <c r="I3" t="n">
-        <v>63.34</v>
+        <v>53.38</v>
       </c>
       <c r="J3" t="n">
         <v>38.41</v>
@@ -5156,28 +4224,28 @@
         <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>10.51</v>
+        <v>10.82</v>
       </c>
       <c r="M3" t="n">
-        <v>2.31</v>
+        <v>1.92</v>
       </c>
       <c r="N3" t="n">
         <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>4.39</v>
+        <v>5.3</v>
       </c>
       <c r="P3" t="n">
-        <v>2.75</v>
+        <v>2.32</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5176452432667247</v>
+        <v>0.4975755922165821</v>
       </c>
       <c r="R3" t="n">
-        <v>0.51042</v>
+        <v>0.48054</v>
       </c>
       <c r="S3" t="n">
-        <v>0.5133100973066899</v>
+        <v>0.4873542368866328</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -5185,7 +4253,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.5133100973066899</v>
+        <v>0.4873542368866328</v>
       </c>
     </row>
   </sheetData>
@@ -5256,22 +4324,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.01</v>
+        <v>0.15</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>27.27</v>
+        <v>66.67</v>
       </c>
       <c r="F2" t="n">
-        <v>0.48</v>
+        <v>0.96</v>
       </c>
       <c r="G2" t="n">
-        <v>-4.54</v>
+        <v>1.19</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
     </row>
     <row r="3">
@@ -5286,7 +4354,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.51</v>
+        <v>0.49</v>
       </c>
       <c r="D3" t="n">
         <v>23</v>
@@ -5295,13 +4363,13 @@
         <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>2.31</v>
+        <v>1.92</v>
       </c>
       <c r="G3" t="n">
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.75</v>
+        <v>2.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:20:44.656412
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -2862,7 +2862,7 @@
         <v>45872.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45889.41666666666</v>
+        <v>45887.41666666666</v>
       </c>
       <c r="F21" t="n">
         <v>23.36</v>
@@ -2871,13 +2871,13 @@
         <v>22.64</v>
       </c>
       <c r="H21" t="n">
-        <v>21.62</v>
+        <v>22.81</v>
       </c>
       <c r="I21" t="n">
-        <v>-7.43</v>
+        <v>-2.36</v>
       </c>
       <c r="J21" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K21" t="n">
         <v>22.39</v>
@@ -2902,7 +2902,7 @@
         <v>1.74</v>
       </c>
       <c r="Q21" t="n">
-        <v>23.34</v>
+        <v>23.12</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
@@ -2911,7 +2911,7 @@
         <v>23.48</v>
       </c>
       <c r="T21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U21" t="b">
         <v>0</v>
@@ -2920,16 +2920,16 @@
         <v>0.51</v>
       </c>
       <c r="W21" t="n">
-        <v>-0.09</v>
+        <v>-1.03</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45873.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2981,22 +2981,22 @@
         <v>45897.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45902.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="F22" t="n">
         <v>21.7</v>
       </c>
       <c r="G22" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="H22" t="n">
         <v>21.02</v>
       </c>
-      <c r="H22" t="n">
-        <v>20.82</v>
-      </c>
       <c r="I22" t="n">
-        <v>-4.02</v>
+        <v>-3.13</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
         <v>21.02</v>
@@ -3060,13 +3060,13 @@
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>21.02</v>
+        <v>21.06</v>
       </c>
       <c r="AE22" t="n">
         <v>21.83</v>
       </c>
       <c r="AF22" t="n">
-        <v>3.13</v>
+        <v>2.95</v>
       </c>
       <c r="AG22" t="n">
         <v>0.63</v>
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3140,10 +3140,10 @@
         <v>3.42</v>
       </c>
       <c r="Q23" t="n">
-        <v>21.93</v>
+        <v>20.96</v>
       </c>
       <c r="R23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="n">
         <v>20.96</v>
@@ -3158,7 +3158,7 @@
         <v>-2.57</v>
       </c>
       <c r="W23" t="n">
-        <v>1.94</v>
+        <v>-2.57</v>
       </c>
       <c r="X23" t="b">
         <v>1</v>
@@ -3173,10 +3173,10 @@
         <v>1</v>
       </c>
       <c r="AB23" s="2" t="n">
-        <v>45923.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="AC23" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AD23" t="n">
         <v>20.27</v>
@@ -3240,7 +3240,7 @@
         <v>22.51</v>
       </c>
       <c r="L24" t="n">
-        <v>23.2</v>
+        <v>23.43</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3259,7 +3259,7 @@
         <v>1.78</v>
       </c>
       <c r="Q24" t="n">
-        <v>22.87</v>
+        <v>23.05</v>
       </c>
       <c r="R24" t="b">
         <v>1</v>
@@ -3277,7 +3277,7 @@
         <v>6.57</v>
       </c>
       <c r="W24" t="n">
-        <v>-2.43</v>
+        <v>-1.66</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3574,7 +3574,7 @@
         <v>26.61</v>
       </c>
       <c r="G27" t="n">
-        <v>25.4</v>
+        <v>25.21</v>
       </c>
       <c r="H27" t="n">
         <v>28.7</v>
@@ -3608,10 +3608,10 @@
         <v>4.31</v>
       </c>
       <c r="Q27" t="n">
-        <v>25.73</v>
+        <v>26.8</v>
       </c>
       <c r="R27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
         <v>26.8</v>
@@ -3626,7 +3626,7 @@
         <v>0.71</v>
       </c>
       <c r="W27" t="n">
-        <v>-3.31</v>
+        <v>0.71</v>
       </c>
       <c r="X27" t="b">
         <v>1</v>
@@ -3641,19 +3641,19 @@
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>46120.41666666666</v>
+        <v>46127.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD27" t="n">
-        <v>25.4</v>
+        <v>25.21</v>
       </c>
       <c r="AE27" t="n">
         <v>26.8</v>
       </c>
       <c r="AF27" t="n">
-        <v>4.55</v>
+        <v>5.26</v>
       </c>
       <c r="AG27" t="n">
         <v>0.71</v>
@@ -3664,7 +3664,7 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
@@ -3928,10 +3928,10 @@
         <v>19.99</v>
       </c>
       <c r="Q2" t="n">
-        <v>54.94</v>
+        <v>45.33</v>
       </c>
       <c r="R2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2" t="n">
         <v>48.75</v>
@@ -3946,25 +3946,25 @@
         <v>-9.57</v>
       </c>
       <c r="W2" t="n">
-        <v>1.91</v>
+        <v>-15.92</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
+        <v>45547.41666666666</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="2" t="n">
         <v>45546.41666666666</v>
       </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB2" s="2" t="n">
-        <v>45547.41666666666</v>
-      </c>
       <c r="AC2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD2" t="n">
         <v>43.72</v>
@@ -4212,10 +4212,10 @@
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.32</v>
+        <v>2.58</v>
       </c>
       <c r="I3" t="n">
-        <v>53.38</v>
+        <v>59.34</v>
       </c>
       <c r="J3" t="n">
         <v>38.41</v>
@@ -4224,28 +4224,28 @@
         <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>10.82</v>
+        <v>10.64</v>
       </c>
       <c r="M3" t="n">
-        <v>1.92</v>
+        <v>2.13</v>
       </c>
       <c r="N3" t="n">
         <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>5.3</v>
+        <v>4.76</v>
       </c>
       <c r="P3" t="n">
-        <v>2.32</v>
+        <v>2.58</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4975755922165821</v>
+        <v>0.5084026632302405</v>
       </c>
       <c r="R3" t="n">
-        <v>0.48054</v>
+        <v>0.49842</v>
       </c>
       <c r="S3" t="n">
-        <v>0.4873542368866328</v>
+        <v>0.5024130652920962</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -4253,7 +4253,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.4873542368866328</v>
+        <v>0.5024130652920962</v>
       </c>
     </row>
   </sheetData>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="D3" t="n">
         <v>23</v>
@@ -4363,13 +4363,13 @@
         <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>1.92</v>
+        <v>2.13</v>
       </c>
       <c r="G3" t="n">
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.32</v>
+        <v>2.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:30:53.106848
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK27"/>
+  <dimension ref="A1:AK35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,7 +983,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -992,34 +992,34 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45322.41666666666</v>
+        <v>45554.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>13.43</v>
+        <v>53.91</v>
       </c>
       <c r="G5" t="n">
-        <v>12.66</v>
+        <v>43.72</v>
       </c>
       <c r="H5" t="n">
-        <v>13.26</v>
+        <v>51.11</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.25</v>
+        <v>-5.19</v>
       </c>
       <c r="J5" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>12.54</v>
+        <v>43.03</v>
       </c>
       <c r="L5" t="n">
-        <v>13.42</v>
+        <v>45.91</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1032,19 +1032,19 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>3180532</v>
+        <v>128396</v>
       </c>
       <c r="P5" t="n">
-        <v>3.32</v>
+        <v>19.99</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.98</v>
+        <v>45.33</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>13.42</v>
+        <v>48.75</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
@@ -1053,40 +1053,40 @@
         <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.09</v>
+        <v>-9.57</v>
       </c>
       <c r="W5" t="n">
-        <v>-3.37</v>
+        <v>-15.92</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>45313.41666666666</v>
+        <v>45547.41666666666</v>
       </c>
       <c r="Z5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>12.66</v>
+        <v>43.72</v>
       </c>
       <c r="AE5" t="n">
-        <v>14.32</v>
+        <v>59.63</v>
       </c>
       <c r="AF5" t="n">
-        <v>5.78</v>
+        <v>18.9</v>
       </c>
       <c r="AG5" t="n">
-        <v>6.61</v>
+        <v>10.61</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>1.14</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1111,34 +1111,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45558.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45567.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>15.59</v>
+        <v>53.48</v>
       </c>
       <c r="G6" t="n">
-        <v>13.66</v>
+        <v>50.18</v>
       </c>
       <c r="H6" t="n">
-        <v>16</v>
+        <v>49.83</v>
       </c>
       <c r="I6" t="n">
-        <v>2.62</v>
+        <v>-6.82</v>
       </c>
       <c r="J6" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="K6" t="n">
-        <v>12.64</v>
+        <v>50.18</v>
       </c>
       <c r="L6" t="n">
-        <v>14.56</v>
+        <v>52.39</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1151,69 +1151,65 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>708583</v>
+        <v>188748</v>
       </c>
       <c r="P6" t="n">
-        <v>10.05</v>
+        <v>4.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>13.78</v>
+        <v>50.5</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>15.04</v>
+        <v>61.85</v>
       </c>
       <c r="T6" t="b">
         <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.54</v>
+        <v>15.65</v>
       </c>
       <c r="W6" t="n">
-        <v>-11.62</v>
+        <v>-5.57</v>
       </c>
       <c r="X6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="2" t="n">
-        <v>45336.41666666666</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="b">
         <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45558.41666666666</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>13.66</v>
+        <v>50.18</v>
       </c>
       <c r="AE6" t="n">
-        <v>17.99</v>
+        <v>61.85</v>
       </c>
       <c r="AF6" t="n">
-        <v>12.37</v>
+        <v>6.17</v>
       </c>
       <c r="AG6" t="n">
-        <v>15.39</v>
+        <v>15.65</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>1.24</v>
+        <v>2.54</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1221,7 +1217,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1233,31 +1229,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45594.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45379.41666666666</v>
+        <v>45601.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>15.92</v>
+        <v>54</v>
       </c>
       <c r="G7" t="n">
-        <v>14.54</v>
+        <v>52.01</v>
       </c>
       <c r="H7" t="n">
-        <v>14.11</v>
+        <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>-11.36</v>
+        <v>-3.7</v>
       </c>
       <c r="J7" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>14.54</v>
+        <v>44</v>
       </c>
       <c r="L7" t="n">
-        <v>15.68</v>
+        <v>53.95</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1270,61 +1266,57 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>2359660</v>
+        <v>36571</v>
       </c>
       <c r="P7" t="n">
-        <v>3.65</v>
+        <v>3.41</v>
       </c>
       <c r="Q7" t="n">
-        <v>15.3</v>
+        <v>54.51</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>16.22</v>
+        <v>57.99</v>
       </c>
       <c r="T7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>1.88</v>
+        <v>7.39</v>
       </c>
       <c r="W7" t="n">
-        <v>-3.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45599.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD7" t="n">
-        <v>14.54</v>
+        <v>52.01</v>
       </c>
       <c r="AE7" t="n">
-        <v>16.22</v>
+        <v>57.99</v>
       </c>
       <c r="AF7" t="n">
-        <v>8.69</v>
+        <v>3.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>1.91</v>
+        <v>7.39</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1332,7 +1324,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.22</v>
+        <v>2</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1340,7 +1332,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1352,31 +1344,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45603.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45608.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>13.08</v>
+        <v>54.34</v>
       </c>
       <c r="G8" t="n">
-        <v>12.76</v>
+        <v>52.65</v>
       </c>
       <c r="H8" t="n">
-        <v>12.39</v>
+        <v>51.7</v>
       </c>
       <c r="I8" t="n">
-        <v>-5.26</v>
+        <v>-4.86</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>12.22</v>
+        <v>51.6</v>
       </c>
       <c r="L8" t="n">
-        <v>13.04</v>
+        <v>54.24</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1389,19 +1381,19 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>5618577</v>
+        <v>18287</v>
       </c>
       <c r="P8" t="n">
-        <v>2.06</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.72</v>
+        <v>53.58</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>14.15</v>
+        <v>57.84</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
@@ -1410,10 +1402,10 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>8.18</v>
+        <v>6.44</v>
       </c>
       <c r="W8" t="n">
-        <v>-2.75</v>
+        <v>-1.4</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1424,22 +1416,22 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45603.41666666666</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>12.76</v>
+        <v>52.65</v>
       </c>
       <c r="AE8" t="n">
-        <v>14.15</v>
+        <v>57.84</v>
       </c>
       <c r="AF8" t="n">
-        <v>2.45</v>
+        <v>3.11</v>
       </c>
       <c r="AG8" t="n">
-        <v>8.199999999999999</v>
+        <v>6.44</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1447,7 +1439,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>3.35</v>
+        <v>2.07</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
@@ -1455,7 +1447,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1467,31 +1459,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45624.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45669.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>11.44</v>
+        <v>49.88</v>
       </c>
       <c r="G9" t="n">
-        <v>10.23</v>
+        <v>47.93</v>
       </c>
       <c r="H9" t="n">
-        <v>11.76</v>
+        <v>55</v>
       </c>
       <c r="I9" t="n">
-        <v>2.8</v>
+        <v>10.26</v>
       </c>
       <c r="J9" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>10.01</v>
+        <v>48</v>
       </c>
       <c r="L9" t="n">
-        <v>11.2</v>
+        <v>49.58</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1504,19 +1496,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>3697242</v>
+        <v>431</v>
       </c>
       <c r="P9" t="n">
-        <v>10</v>
+        <v>1.14</v>
       </c>
       <c r="Q9" t="n">
-        <v>13.1</v>
+        <v>51.55</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>13.42</v>
+        <v>51.55</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1525,32 +1517,40 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>17.31</v>
+        <v>3.35</v>
       </c>
       <c r="W9" t="n">
-        <v>14.51</v>
+        <v>3.35</v>
       </c>
       <c r="X9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>45631.41666666666</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>5</v>
+      </c>
       <c r="AA9" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2" t="n">
+        <v>45631.41666666666</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>5</v>
+      </c>
       <c r="AD9" t="n">
-        <v>10.23</v>
+        <v>47.93</v>
       </c>
       <c r="AE9" t="n">
-        <v>13.42</v>
+        <v>51.55</v>
       </c>
       <c r="AF9" t="n">
-        <v>10.56</v>
+        <v>3.91</v>
       </c>
       <c r="AG9" t="n">
-        <v>17.34</v>
+        <v>3.35</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>1.64</v>
+        <v>0.86</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1566,7 +1566,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1578,31 +1578,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45704.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45434.41666666666</v>
+        <v>45714.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>12.1</v>
+        <v>47.99</v>
       </c>
       <c r="G10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="H10" t="n">
-        <v>12.4</v>
+        <v>45.81</v>
       </c>
       <c r="I10" t="n">
-        <v>2.51</v>
+        <v>-4.54</v>
       </c>
       <c r="J10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="L10" t="n">
-        <v>12.08</v>
+        <v>47.97</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1615,19 +1615,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>719120</v>
+        <v>6897</v>
       </c>
       <c r="P10" t="n">
-        <v>2.86</v>
+        <v>3.61</v>
       </c>
       <c r="Q10" t="n">
-        <v>11.92</v>
+        <v>48.54</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>12.39</v>
+        <v>50.25</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1636,40 +1636,32 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>2.43</v>
+        <v>4.71</v>
       </c>
       <c r="W10" t="n">
-        <v>-1.46</v>
+        <v>1.15</v>
       </c>
       <c r="X10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="2" t="n">
-        <v>45426.41666666666</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB10" s="2" t="n">
-        <v>45425.41666666666</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="AE10" t="n">
-        <v>12.39</v>
+        <v>50.25</v>
       </c>
       <c r="AF10" t="n">
-        <v>3.44</v>
+        <v>4.15</v>
       </c>
       <c r="AG10" t="n">
-        <v>2.45</v>
+        <v>4.71</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -1677,7 +1669,7 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.71</v>
+        <v>1.13</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1685,7 +1677,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1697,31 +1689,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45727.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>13.23</v>
+        <v>47.51</v>
       </c>
       <c r="G11" t="n">
-        <v>12.37</v>
+        <v>45.8</v>
       </c>
       <c r="H11" t="n">
-        <v>15.11</v>
+        <v>45.63</v>
       </c>
       <c r="I11" t="n">
-        <v>14.21</v>
+        <v>-3.96</v>
       </c>
       <c r="J11" t="n">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="K11" t="n">
-        <v>12.37</v>
+        <v>45.81</v>
       </c>
       <c r="L11" t="n">
-        <v>12.68</v>
+        <v>46.58</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1734,19 +1726,19 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>2872871</v>
+        <v>31257</v>
       </c>
       <c r="P11" t="n">
-        <v>4.75</v>
+        <v>3.04</v>
       </c>
       <c r="Q11" t="n">
-        <v>12.61</v>
+        <v>46.46</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>13.12</v>
+        <v>46.7</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -1755,40 +1747,40 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>-0.85</v>
+        <v>-1.7</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.7</v>
+        <v>-2.21</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45454.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>12.37</v>
+        <v>45.8</v>
       </c>
       <c r="AE11" t="n">
-        <v>13.98</v>
+        <v>48.4</v>
       </c>
       <c r="AF11" t="n">
-        <v>6.53</v>
+        <v>3.6</v>
       </c>
       <c r="AG11" t="n">
-        <v>5.68</v>
+        <v>1.87</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -1796,7 +1788,7 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.87</v>
+        <v>0.52</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1804,7 +1796,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1816,31 +1808,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>17.1</v>
+        <v>48.44</v>
       </c>
       <c r="G12" t="n">
-        <v>14.96</v>
+        <v>45.88</v>
       </c>
       <c r="H12" t="n">
-        <v>19.46</v>
+        <v>45.51</v>
       </c>
       <c r="I12" t="n">
-        <v>13.85</v>
+        <v>-6.05</v>
       </c>
       <c r="J12" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K12" t="n">
-        <v>14.96</v>
+        <v>45.6</v>
       </c>
       <c r="L12" t="n">
-        <v>15.28</v>
+        <v>46.75</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1853,19 +1845,19 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>2885185</v>
+        <v>49292</v>
       </c>
       <c r="P12" t="n">
-        <v>13.79</v>
+        <v>5.14</v>
       </c>
       <c r="Q12" t="n">
-        <v>15.44</v>
+        <v>46.73</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>15.5</v>
+        <v>46.75</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1874,40 +1866,40 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-9.34</v>
+        <v>-3.49</v>
       </c>
       <c r="W12" t="n">
-        <v>-9.69</v>
+        <v>-3.53</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45734.41666666666</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>14.96</v>
+        <v>45.88</v>
       </c>
       <c r="AE12" t="n">
-        <v>17.64</v>
+        <v>49.59</v>
       </c>
       <c r="AF12" t="n">
-        <v>12.49</v>
+        <v>5.28</v>
       </c>
       <c r="AG12" t="n">
-        <v>3.18</v>
+        <v>2.37</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1915,7 +1907,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.25</v>
+        <v>0.45</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1932,34 +1924,34 @@
         </is>
       </c>
       <c r="C13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>20.68</v>
+        <v>13.43</v>
       </c>
       <c r="G13" t="n">
-        <v>18.4</v>
+        <v>12.66</v>
       </c>
       <c r="H13" t="n">
-        <v>28.62</v>
+        <v>13.26</v>
       </c>
       <c r="I13" t="n">
-        <v>38.41</v>
+        <v>-1.25</v>
       </c>
       <c r="J13" t="n">
-        <v>185</v>
+        <v>21</v>
       </c>
       <c r="K13" t="n">
-        <v>18.4</v>
+        <v>12.54</v>
       </c>
       <c r="L13" t="n">
-        <v>20.24</v>
+        <v>13.42</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1972,69 +1964,69 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>807277</v>
+        <v>3180532</v>
       </c>
       <c r="P13" t="n">
-        <v>2.17</v>
+        <v>3.32</v>
       </c>
       <c r="Q13" t="n">
-        <v>20.54</v>
+        <v>12.98</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>23.04</v>
+        <v>13.42</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>11.41</v>
+        <v>-0.09</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.68</v>
+        <v>-3.37</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45572.41666666666</v>
+        <v>45313.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>18.4</v>
+        <v>12.66</v>
       </c>
       <c r="AE13" t="n">
-        <v>23.04</v>
+        <v>14.32</v>
       </c>
       <c r="AF13" t="n">
-        <v>11.03</v>
+        <v>5.78</v>
       </c>
       <c r="AG13" t="n">
-        <v>11.41</v>
+        <v>6.61</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.03</v>
+        <v>1.14</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2051,34 +2043,34 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>28.64</v>
+        <v>15.59</v>
       </c>
       <c r="G14" t="n">
-        <v>28.08</v>
+        <v>13.66</v>
       </c>
       <c r="H14" t="n">
-        <v>27.22</v>
+        <v>16</v>
       </c>
       <c r="I14" t="n">
-        <v>-4.97</v>
+        <v>2.62</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="K14" t="n">
-        <v>28</v>
+        <v>12.64</v>
       </c>
       <c r="L14" t="n">
-        <v>28.48</v>
+        <v>14.56</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2091,69 +2083,69 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>1546271</v>
+        <v>708583</v>
       </c>
       <c r="P14" t="n">
-        <v>1.79</v>
+        <v>10.05</v>
       </c>
       <c r="Q14" t="n">
-        <v>28.16</v>
+        <v>13.78</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>29</v>
+        <v>15.04</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>1.26</v>
+        <v>-3.54</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.68</v>
+        <v>-11.62</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45336.41666666666</v>
       </c>
       <c r="Z14" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>28.08</v>
+        <v>13.66</v>
       </c>
       <c r="AE14" t="n">
-        <v>29</v>
+        <v>17.99</v>
       </c>
       <c r="AF14" t="n">
-        <v>1.96</v>
+        <v>12.37</v>
       </c>
       <c r="AG14" t="n">
-        <v>1.26</v>
+        <v>15.39</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.64</v>
+        <v>1.24</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2173,31 +2165,31 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45756.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>25.97</v>
+        <v>15.92</v>
       </c>
       <c r="G15" t="n">
-        <v>24.72</v>
+        <v>14.54</v>
       </c>
       <c r="H15" t="n">
-        <v>24.16</v>
+        <v>14.11</v>
       </c>
       <c r="I15" t="n">
-        <v>-6.96</v>
+        <v>-11.36</v>
       </c>
       <c r="J15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K15" t="n">
-        <v>24.68</v>
+        <v>14.54</v>
       </c>
       <c r="L15" t="n">
-        <v>25.51</v>
+        <v>15.68</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2210,53 +2202,61 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>767605</v>
+        <v>2359660</v>
       </c>
       <c r="P15" t="n">
-        <v>4.04</v>
+        <v>3.65</v>
       </c>
       <c r="Q15" t="n">
-        <v>27.46</v>
+        <v>15.3</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>29.03</v>
+        <v>16.22</v>
       </c>
       <c r="T15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U15" t="b">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>11.79</v>
+        <v>1.88</v>
       </c>
       <c r="W15" t="n">
-        <v>5.75</v>
+        <v>-3.89</v>
       </c>
       <c r="X15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y15" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
       <c r="AA15" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB15" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0</v>
+      </c>
       <c r="AD15" t="n">
-        <v>24.72</v>
+        <v>14.54</v>
       </c>
       <c r="AE15" t="n">
-        <v>29.03</v>
+        <v>16.22</v>
       </c>
       <c r="AF15" t="n">
-        <v>4.81</v>
+        <v>8.69</v>
       </c>
       <c r="AG15" t="n">
-        <v>11.8</v>
+        <v>1.91</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>2.45</v>
+        <v>0.22</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2284,31 +2284,31 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45783.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>25.32</v>
+        <v>13.08</v>
       </c>
       <c r="G16" t="n">
-        <v>24.12</v>
+        <v>12.76</v>
       </c>
       <c r="H16" t="n">
-        <v>23.99</v>
+        <v>12.39</v>
       </c>
       <c r="I16" t="n">
-        <v>-5.24</v>
+        <v>-5.26</v>
       </c>
       <c r="J16" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>24.12</v>
+        <v>12.22</v>
       </c>
       <c r="L16" t="n">
-        <v>25.26</v>
+        <v>13.04</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>623052</v>
+        <v>5618577</v>
       </c>
       <c r="P16" t="n">
-        <v>0.96</v>
+        <v>2.06</v>
       </c>
       <c r="Q16" t="n">
-        <v>26.96</v>
+        <v>12.72</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>26.96</v>
+        <v>14.15</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2342,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>6.48</v>
+        <v>8.18</v>
       </c>
       <c r="W16" t="n">
-        <v>6.48</v>
+        <v>-2.75</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -2353,21 +2353,25 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB16" s="2" t="n">
+        <v>45398.41666666666</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
       <c r="AD16" t="n">
-        <v>24.12</v>
+        <v>12.76</v>
       </c>
       <c r="AE16" t="n">
-        <v>26.96</v>
+        <v>14.15</v>
       </c>
       <c r="AF16" t="n">
-        <v>4.74</v>
+        <v>2.45</v>
       </c>
       <c r="AG16" t="n">
-        <v>6.48</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2375,7 +2379,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>1.37</v>
+        <v>3.35</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2395,31 +2399,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>22.75</v>
+        <v>11.44</v>
       </c>
       <c r="G17" t="n">
-        <v>21.66</v>
+        <v>10.23</v>
       </c>
       <c r="H17" t="n">
-        <v>21.65</v>
+        <v>11.76</v>
       </c>
       <c r="I17" t="n">
-        <v>-4.85</v>
+        <v>2.8</v>
       </c>
       <c r="J17" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
-        <v>21.66</v>
+        <v>10.01</v>
       </c>
       <c r="L17" t="n">
-        <v>22.2</v>
+        <v>11.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2432,19 +2436,19 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>13689820</v>
+        <v>3697242</v>
       </c>
       <c r="P17" t="n">
-        <v>4.94</v>
+        <v>10</v>
       </c>
       <c r="Q17" t="n">
-        <v>23.7</v>
+        <v>13.1</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>25.75</v>
+        <v>13.42</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -2453,10 +2457,10 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>13.18</v>
+        <v>17.31</v>
       </c>
       <c r="W17" t="n">
-        <v>4.17</v>
+        <v>14.51</v>
       </c>
       <c r="X17" t="b">
         <v>0</v>
@@ -2469,16 +2473,16 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>21.66</v>
+        <v>10.23</v>
       </c>
       <c r="AE17" t="n">
-        <v>25.75</v>
+        <v>13.42</v>
       </c>
       <c r="AF17" t="n">
-        <v>4.78</v>
+        <v>10.56</v>
       </c>
       <c r="AG17" t="n">
-        <v>13.19</v>
+        <v>17.34</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2486,7 +2490,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>2.76</v>
+        <v>1.64</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2506,31 +2510,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>21.88</v>
+        <v>12.1</v>
       </c>
       <c r="G18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="H18" t="n">
-        <v>20.53</v>
+        <v>12.4</v>
       </c>
       <c r="I18" t="n">
-        <v>-6.18</v>
+        <v>2.51</v>
       </c>
       <c r="J18" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="L18" t="n">
-        <v>21.78</v>
+        <v>12.08</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2543,19 +2547,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>1476660</v>
+        <v>719120</v>
       </c>
       <c r="P18" t="n">
-        <v>1.3</v>
+        <v>2.86</v>
       </c>
       <c r="Q18" t="n">
-        <v>21.54</v>
+        <v>11.92</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>22.52</v>
+        <v>12.39</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2564,40 +2568,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>2.93</v>
+        <v>2.43</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.55</v>
+        <v>-1.46</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>45818.41666666666</v>
+        <v>45426.41666666666</v>
       </c>
       <c r="Z18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="AE18" t="n">
-        <v>22.52</v>
+        <v>12.39</v>
       </c>
       <c r="AF18" t="n">
-        <v>2.41</v>
+        <v>3.44</v>
       </c>
       <c r="AG18" t="n">
-        <v>2.93</v>
+        <v>2.45</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2605,7 +2609,7 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>1.22</v>
+        <v>0.71</v>
       </c>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
@@ -2625,31 +2629,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>21.16</v>
+        <v>13.23</v>
       </c>
       <c r="G19" t="n">
-        <v>19.2</v>
+        <v>12.37</v>
       </c>
       <c r="H19" t="n">
-        <v>21.32</v>
+        <v>15.11</v>
       </c>
       <c r="I19" t="n">
-        <v>0.76</v>
+        <v>14.21</v>
       </c>
       <c r="J19" t="n">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="K19" t="n">
-        <v>19.92</v>
+        <v>12.37</v>
       </c>
       <c r="L19" t="n">
-        <v>20.64</v>
+        <v>12.68</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2662,65 +2666,69 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>5666121</v>
+        <v>2872871</v>
       </c>
       <c r="P19" t="n">
         <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>22.02</v>
+        <v>12.61</v>
       </c>
       <c r="R19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>22.52</v>
+        <v>13.12</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
       </c>
       <c r="U19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" t="n">
-        <v>6.43</v>
+        <v>-0.85</v>
       </c>
       <c r="W19" t="n">
-        <v>4.06</v>
+        <v>-4.7</v>
       </c>
       <c r="X19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y19" s="2" t="n">
+        <v>45454.41666666666</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>11</v>
+      </c>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45833.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD19" t="n">
-        <v>19.2</v>
+        <v>12.37</v>
       </c>
       <c r="AE19" t="n">
-        <v>22.52</v>
+        <v>13.98</v>
       </c>
       <c r="AF19" t="n">
-        <v>9.26</v>
+        <v>6.53</v>
       </c>
       <c r="AG19" t="n">
-        <v>6.43</v>
+        <v>5.68</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.87</v>
       </c>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
@@ -2740,31 +2748,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45845.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>21.91</v>
+        <v>17.1</v>
       </c>
       <c r="G20" t="n">
-        <v>21.28</v>
+        <v>14.96</v>
       </c>
       <c r="H20" t="n">
-        <v>22.48</v>
+        <v>19.46</v>
       </c>
       <c r="I20" t="n">
-        <v>2.59</v>
+        <v>13.85</v>
       </c>
       <c r="J20" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="K20" t="n">
-        <v>21.29</v>
+        <v>14.96</v>
       </c>
       <c r="L20" t="n">
-        <v>21.84</v>
+        <v>15.28</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2777,69 +2785,69 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>1366828</v>
+        <v>2885185</v>
       </c>
       <c r="P20" t="n">
-        <v>1.44</v>
+        <v>13.79</v>
       </c>
       <c r="Q20" t="n">
-        <v>22.06</v>
+        <v>15.44</v>
       </c>
       <c r="R20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>22.44</v>
+        <v>15.5</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
-        <v>2.41</v>
+        <v>-9.34</v>
       </c>
       <c r="W20" t="n">
-        <v>0.68</v>
+        <v>-9.69</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>45847.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="Z20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>45847.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="AC20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD20" t="n">
-        <v>21.28</v>
+        <v>14.96</v>
       </c>
       <c r="AE20" t="n">
-        <v>22.44</v>
+        <v>17.64</v>
       </c>
       <c r="AF20" t="n">
-        <v>2.88</v>
+        <v>12.49</v>
       </c>
       <c r="AG20" t="n">
-        <v>2.41</v>
+        <v>3.18</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.84</v>
+        <v>0.25</v>
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
@@ -2859,31 +2867,31 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45887.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>23.36</v>
+        <v>20.68</v>
       </c>
       <c r="G21" t="n">
-        <v>22.64</v>
+        <v>18.4</v>
       </c>
       <c r="H21" t="n">
-        <v>22.81</v>
+        <v>28.62</v>
       </c>
       <c r="I21" t="n">
-        <v>-2.36</v>
+        <v>38.41</v>
       </c>
       <c r="J21" t="n">
-        <v>15</v>
+        <v>185</v>
       </c>
       <c r="K21" t="n">
-        <v>22.39</v>
+        <v>18.4</v>
       </c>
       <c r="L21" t="n">
-        <v>23.18</v>
+        <v>20.24</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2896,19 +2904,19 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>1011332</v>
+        <v>807277</v>
       </c>
       <c r="P21" t="n">
-        <v>1.74</v>
+        <v>2.17</v>
       </c>
       <c r="Q21" t="n">
-        <v>23.12</v>
+        <v>20.54</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>23.48</v>
+        <v>23.04</v>
       </c>
       <c r="T21" t="b">
         <v>0</v>
@@ -2917,40 +2925,40 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>0.51</v>
+        <v>11.41</v>
       </c>
       <c r="W21" t="n">
-        <v>-1.03</v>
+        <v>-0.68</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45873.41666666666</v>
+        <v>45572.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>22.64</v>
+        <v>18.4</v>
       </c>
       <c r="AE21" t="n">
-        <v>23.48</v>
+        <v>23.04</v>
       </c>
       <c r="AF21" t="n">
-        <v>3.08</v>
+        <v>11.03</v>
       </c>
       <c r="AG21" t="n">
-        <v>0.51</v>
+        <v>11.41</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2958,7 +2966,7 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.17</v>
+        <v>1.03</v>
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
@@ -2978,31 +2986,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45900.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>21.7</v>
+        <v>28.64</v>
       </c>
       <c r="G22" t="n">
-        <v>21.06</v>
+        <v>28.08</v>
       </c>
       <c r="H22" t="n">
-        <v>21.02</v>
+        <v>27.22</v>
       </c>
       <c r="I22" t="n">
-        <v>-3.13</v>
+        <v>-4.97</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>21.02</v>
+        <v>28</v>
       </c>
       <c r="L22" t="n">
-        <v>21.26</v>
+        <v>28.48</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3015,19 +3023,19 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>811883</v>
+        <v>1546271</v>
       </c>
       <c r="P22" t="n">
-        <v>2.81</v>
+        <v>1.79</v>
       </c>
       <c r="Q22" t="n">
-        <v>21.61</v>
+        <v>28.16</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>21.83</v>
+        <v>29</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
@@ -3036,16 +3044,16 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>0.62</v>
+        <v>1.26</v>
       </c>
       <c r="W22" t="n">
-        <v>-0.4</v>
+        <v>-1.68</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>45900.41666666666</v>
+        <v>45729.41666666666</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -3054,22 +3062,22 @@
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>21.06</v>
+        <v>28.08</v>
       </c>
       <c r="AE22" t="n">
-        <v>21.83</v>
+        <v>29</v>
       </c>
       <c r="AF22" t="n">
-        <v>2.95</v>
+        <v>1.96</v>
       </c>
       <c r="AG22" t="n">
-        <v>0.63</v>
+        <v>1.26</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
@@ -3077,7 +3085,7 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.21</v>
+        <v>0.64</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3097,31 +3105,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>45911.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45972.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>21.51</v>
+        <v>25.97</v>
       </c>
       <c r="G23" t="n">
-        <v>20.27</v>
+        <v>24.72</v>
       </c>
       <c r="H23" t="n">
-        <v>24.94</v>
+        <v>25.2</v>
       </c>
       <c r="I23" t="n">
-        <v>15.94</v>
+        <v>-2.96</v>
       </c>
       <c r="J23" t="n">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="K23" t="n">
-        <v>20.28</v>
+        <v>24.68</v>
       </c>
       <c r="L23" t="n">
-        <v>20.96</v>
+        <v>25.51</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3134,69 +3142,61 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>2694406</v>
+        <v>767605</v>
       </c>
       <c r="P23" t="n">
-        <v>3.42</v>
+        <v>4.04</v>
       </c>
       <c r="Q23" t="n">
-        <v>20.96</v>
+        <v>27.46</v>
       </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>20.96</v>
+        <v>29.03</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
       </c>
       <c r="U23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>-2.57</v>
+        <v>11.79</v>
       </c>
       <c r="W23" t="n">
-        <v>-2.57</v>
+        <v>5.75</v>
       </c>
       <c r="X23" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y23" s="2" t="n">
-        <v>45923.41666666666</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB23" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="n">
-        <v>20.27</v>
+        <v>24.72</v>
       </c>
       <c r="AE23" t="n">
-        <v>22.19</v>
+        <v>29.03</v>
       </c>
       <c r="AF23" t="n">
-        <v>5.76</v>
+        <v>4.81</v>
       </c>
       <c r="AG23" t="n">
-        <v>3.16</v>
+        <v>11.8</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.55</v>
+        <v>2.45</v>
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
@@ -3216,31 +3216,31 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>45994.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>46002.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F24" t="n">
-        <v>23.44</v>
+        <v>25.32</v>
       </c>
       <c r="G24" t="n">
-        <v>22.68</v>
+        <v>24.12</v>
       </c>
       <c r="H24" t="n">
-        <v>23.56</v>
+        <v>23.99</v>
       </c>
       <c r="I24" t="n">
-        <v>0.51</v>
+        <v>-5.24</v>
       </c>
       <c r="J24" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="K24" t="n">
-        <v>22.51</v>
+        <v>24.12</v>
       </c>
       <c r="L24" t="n">
-        <v>23.43</v>
+        <v>25.26</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>2183354</v>
+        <v>623052</v>
       </c>
       <c r="P24" t="n">
-        <v>1.78</v>
+        <v>0.96</v>
       </c>
       <c r="Q24" t="n">
-        <v>23.05</v>
+        <v>26.96</v>
       </c>
       <c r="R24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>24.98</v>
+        <v>26.96</v>
       </c>
       <c r="T24" t="b">
         <v>0</v>
@@ -3274,10 +3274,10 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>6.57</v>
+        <v>6.48</v>
       </c>
       <c r="W24" t="n">
-        <v>-1.66</v>
+        <v>6.48</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3285,25 +3285,21 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB24" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="n">
-        <v>22.68</v>
+        <v>24.12</v>
       </c>
       <c r="AE24" t="n">
-        <v>24.98</v>
+        <v>26.96</v>
       </c>
       <c r="AF24" t="n">
-        <v>3.24</v>
+        <v>4.74</v>
       </c>
       <c r="AG24" t="n">
-        <v>6.57</v>
+        <v>6.48</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
@@ -3311,7 +3307,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>2.03</v>
+        <v>1.37</v>
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
@@ -3331,31 +3327,31 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>46016.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>46027.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F25" t="n">
-        <v>24.6</v>
+        <v>22.75</v>
       </c>
       <c r="G25" t="n">
-        <v>23.75</v>
+        <v>21.66</v>
       </c>
       <c r="H25" t="n">
-        <v>24.41</v>
+        <v>21.65</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.77</v>
+        <v>-4.85</v>
       </c>
       <c r="J25" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="K25" t="n">
-        <v>23.41</v>
+        <v>21.66</v>
       </c>
       <c r="L25" t="n">
-        <v>24.09</v>
+        <v>22.2</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3368,31 +3364,31 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>2756109</v>
+        <v>13689820</v>
       </c>
       <c r="P25" t="n">
-        <v>3.54</v>
+        <v>4.94</v>
       </c>
       <c r="Q25" t="n">
-        <v>24.08</v>
+        <v>23.7</v>
       </c>
       <c r="R25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>24.5</v>
+        <v>25.75</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
       </c>
       <c r="U25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>-0.41</v>
+        <v>13.18</v>
       </c>
       <c r="W25" t="n">
-        <v>-2.11</v>
+        <v>4.17</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -3400,33 +3396,29 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB25" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="n">
-        <v>23.75</v>
+        <v>21.66</v>
       </c>
       <c r="AE25" t="n">
-        <v>25.69</v>
+        <v>25.75</v>
       </c>
       <c r="AF25" t="n">
-        <v>3.46</v>
+        <v>4.78</v>
       </c>
       <c r="AG25" t="n">
-        <v>4.43</v>
+        <v>13.19</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>1.28</v>
+        <v>2.76</v>
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
@@ -3446,31 +3438,31 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>46069.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F26" t="n">
-        <v>26</v>
+        <v>21.88</v>
       </c>
       <c r="G26" t="n">
-        <v>24.3</v>
+        <v>21.35</v>
       </c>
       <c r="H26" t="n">
-        <v>28.5</v>
+        <v>20.53</v>
       </c>
       <c r="I26" t="n">
-        <v>9.619999999999999</v>
+        <v>-6.18</v>
       </c>
       <c r="J26" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="K26" t="n">
-        <v>24.01</v>
+        <v>21.35</v>
       </c>
       <c r="L26" t="n">
-        <v>25.42</v>
+        <v>21.78</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3483,37 +3475,37 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>2965366</v>
+        <v>1476660</v>
       </c>
       <c r="P26" t="n">
-        <v>6.51</v>
+        <v>1.3</v>
       </c>
       <c r="Q26" t="n">
-        <v>25.42</v>
+        <v>21.54</v>
       </c>
       <c r="R26" t="b">
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>25.42</v>
+        <v>22.52</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
       </c>
       <c r="U26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>-2.23</v>
+        <v>2.93</v>
       </c>
       <c r="W26" t="n">
-        <v>-2.23</v>
+        <v>-1.55</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>46033.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z26" t="n">
         <v>2</v>
@@ -3522,30 +3514,30 @@
         <v>1</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>24.3</v>
+        <v>21.35</v>
       </c>
       <c r="AE26" t="n">
-        <v>27.41</v>
+        <v>22.52</v>
       </c>
       <c r="AF26" t="n">
-        <v>6.54</v>
+        <v>2.41</v>
       </c>
       <c r="AG26" t="n">
-        <v>5.42</v>
+        <v>2.93</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>0.83</v>
+        <v>1.22</v>
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
@@ -3565,31 +3557,31 @@
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>46120.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>46139.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>26.61</v>
+        <v>21.16</v>
       </c>
       <c r="G27" t="n">
-        <v>25.21</v>
+        <v>19.2</v>
       </c>
       <c r="H27" t="n">
-        <v>28.7</v>
+        <v>21.32</v>
       </c>
       <c r="I27" t="n">
-        <v>7.85</v>
+        <v>0.76</v>
       </c>
       <c r="J27" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="K27" t="n">
-        <v>23.8</v>
+        <v>19.92</v>
       </c>
       <c r="L27" t="n">
-        <v>25.7</v>
+        <v>20.64</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3602,61 +3594,57 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>2499912</v>
+        <v>5666121</v>
       </c>
       <c r="P27" t="n">
-        <v>4.31</v>
+        <v>4.75</v>
       </c>
       <c r="Q27" t="n">
-        <v>26.8</v>
+        <v>22.02</v>
       </c>
       <c r="R27" t="b">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>26.8</v>
+        <v>22.52</v>
       </c>
       <c r="T27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U27" t="b">
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>0.71</v>
+        <v>6.43</v>
       </c>
       <c r="W27" t="n">
-        <v>0.71</v>
+        <v>4.06</v>
       </c>
       <c r="X27" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y27" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="b">
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>46127.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD27" t="n">
-        <v>25.21</v>
+        <v>19.2</v>
       </c>
       <c r="AE27" t="n">
-        <v>26.8</v>
+        <v>22.52</v>
       </c>
       <c r="AF27" t="n">
-        <v>5.26</v>
+        <v>9.26</v>
       </c>
       <c r="AG27" t="n">
-        <v>0.71</v>
+        <v>6.43</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -3664,10 +3652,954 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.13</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C28" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>45845.41666666666</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>45860.41666666666</v>
+      </c>
+      <c r="F28" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="G28" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="H28" t="n">
+        <v>22.48</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="J28" t="n">
+        <v>15</v>
+      </c>
+      <c r="K28" t="n">
+        <v>21.29</v>
+      </c>
+      <c r="L28" t="n">
+        <v>21.84</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>1366828</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>22.06</v>
+      </c>
+      <c r="R28" t="b">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="T28" t="b">
+        <v>0</v>
+      </c>
+      <c r="U28" t="b">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="X28" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y28" s="2" t="n">
+        <v>45847.41666666666</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB28" s="2" t="n">
+        <v>45847.41666666666</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C29" t="b">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>45872.41666666666</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>45887.41666666666</v>
+      </c>
+      <c r="F29" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="G29" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="H29" t="n">
+        <v>22.81</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-2.36</v>
+      </c>
+      <c r="J29" t="n">
+        <v>15</v>
+      </c>
+      <c r="K29" t="n">
+        <v>22.39</v>
+      </c>
+      <c r="L29" t="n">
+        <v>23.18</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>1011332</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="T29" t="b">
+        <v>0</v>
+      </c>
+      <c r="U29" t="b">
+        <v>0</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="W29" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="X29" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y29" s="2" t="n">
+        <v>45873.41666666666</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA29" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB29" s="2" t="n">
+        <v>45872.41666666666</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AJ29" t="inlineStr"/>
+      <c r="AK29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C30" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>45897.41666666666</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="F30" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="G30" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="H30" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-3.13</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="L30" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>811883</v>
+      </c>
+      <c r="P30" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="T30" t="b">
+        <v>0</v>
+      </c>
+      <c r="U30" t="b">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="W30" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="X30" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y30" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA30" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB30" s="2" t="n">
+        <v>45897.41666666666</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C31" t="b">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>45972.41666666666</v>
+      </c>
+      <c r="F31" t="n">
+        <v>21.51</v>
+      </c>
+      <c r="G31" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="H31" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="I31" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="J31" t="n">
+        <v>61</v>
+      </c>
+      <c r="K31" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="L31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>2694406</v>
+      </c>
+      <c r="P31" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="T31" t="b">
+        <v>0</v>
+      </c>
+      <c r="U31" t="b">
+        <v>1</v>
+      </c>
+      <c r="V31" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="W31" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="X31" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA31" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB31" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ31" t="inlineStr"/>
+      <c r="AK31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>46002.41666666666</v>
+      </c>
+      <c r="F32" t="n">
+        <v>23.44</v>
+      </c>
+      <c r="G32" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="H32" t="n">
+        <v>23.56</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J32" t="n">
+        <v>8</v>
+      </c>
+      <c r="K32" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="L32" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>2183354</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>22.87</v>
+      </c>
+      <c r="R32" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="T32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V32" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="W32" t="n">
+        <v>-2.43</v>
+      </c>
+      <c r="X32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB32" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AJ32" t="inlineStr"/>
+      <c r="AK32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C33" t="b">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>46027.41666666666</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G33" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="H33" t="n">
+        <v>24.41</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="J33" t="n">
+        <v>11</v>
+      </c>
+      <c r="K33" t="n">
+        <v>23.41</v>
+      </c>
+      <c r="L33" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O33" t="n">
+        <v>2756109</v>
+      </c>
+      <c r="P33" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>24.08</v>
+      </c>
+      <c r="R33" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="T33" t="b">
+        <v>0</v>
+      </c>
+      <c r="U33" t="b">
+        <v>1</v>
+      </c>
+      <c r="V33" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="W33" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="X33" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB33" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="AJ33" t="inlineStr"/>
+      <c r="AK33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>46069.41666666666</v>
+      </c>
+      <c r="F34" t="n">
+        <v>26</v>
+      </c>
+      <c r="G34" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I34" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="J34" t="n">
+        <v>41</v>
+      </c>
+      <c r="K34" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="L34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>2965366</v>
+      </c>
+      <c r="P34" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="R34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="T34" t="b">
+        <v>0</v>
+      </c>
+      <c r="U34" t="b">
+        <v>1</v>
+      </c>
+      <c r="V34" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="W34" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="X34" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="2" t="n">
+        <v>46033.41666666666</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA34" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI34" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AJ34" t="inlineStr"/>
+      <c r="AK34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C35" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>46139.41666666666</v>
+      </c>
+      <c r="F35" t="n">
+        <v>26.61</v>
+      </c>
+      <c r="G35" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="I35" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="J35" t="n">
+        <v>19</v>
+      </c>
+      <c r="K35" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="L35" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>2499912</v>
+      </c>
+      <c r="P35" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>25.73</v>
+      </c>
+      <c r="R35" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="T35" t="b">
+        <v>1</v>
+      </c>
+      <c r="U35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="W35" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="X35" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI35" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3885,31 +4817,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>53.91</v>
+        <v>47.87</v>
       </c>
       <c r="G2" t="n">
-        <v>43.72</v>
+        <v>46</v>
       </c>
       <c r="H2" t="n">
         <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>235.74</v>
+        <v>278.11</v>
       </c>
       <c r="J2" t="n">
-        <v>593</v>
+        <v>384</v>
       </c>
       <c r="K2" t="n">
-        <v>43.03</v>
+        <v>45</v>
       </c>
       <c r="L2" t="n">
-        <v>45.91</v>
+        <v>46.89</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -3922,69 +4854,69 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>128396</v>
+        <v>47815</v>
       </c>
       <c r="P2" t="n">
-        <v>19.99</v>
+        <v>2.73</v>
       </c>
       <c r="Q2" t="n">
-        <v>45.33</v>
+        <v>46.62</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>48.75</v>
+        <v>51</v>
       </c>
       <c r="T2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>-9.57</v>
+        <v>6.54</v>
       </c>
       <c r="W2" t="n">
-        <v>-15.92</v>
+        <v>-2.61</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45547.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="Z2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>43.72</v>
+        <v>46</v>
       </c>
       <c r="AE2" t="n">
-        <v>59.63</v>
+        <v>51</v>
       </c>
       <c r="AF2" t="n">
-        <v>18.9</v>
+        <v>3.91</v>
       </c>
       <c r="AG2" t="n">
-        <v>10.61</v>
+        <v>6.54</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.67</v>
       </c>
       <c r="AJ2" t="n">
         <v>181</v>
@@ -4126,25 +5058,25 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>66.67</v>
+        <v>27.27</v>
       </c>
       <c r="G2" t="n">
-        <v>1.19</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.58</v>
+        <v>-25.44</v>
       </c>
       <c r="J2" t="n">
         <v>12.48</v>
@@ -4153,28 +5085,28 @@
         <v>-14.25</v>
       </c>
       <c r="L2" t="n">
-        <v>13.42</v>
+        <v>7.68</v>
       </c>
       <c r="M2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="N2" t="n">
-        <v>6.84</v>
+        <v>7.98</v>
       </c>
       <c r="O2" t="n">
-        <v>14.25</v>
+        <v>6.17</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.2320120319001387</v>
+        <v>0.1209768433179723</v>
       </c>
       <c r="R2" t="n">
-        <v>0.09086</v>
+        <v>-0.09292000000000003</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1473208127600555</v>
+        <v>-0.007361262672811078</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -4182,7 +5114,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.1473208127600555</v>
+        <v>-0.007361262672811078</v>
       </c>
     </row>
     <row r="3">
@@ -4212,10 +5144,10 @@
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
       <c r="I3" t="n">
-        <v>59.34</v>
+        <v>63.34</v>
       </c>
       <c r="J3" t="n">
         <v>38.41</v>
@@ -4224,28 +5156,28 @@
         <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>10.64</v>
+        <v>10.51</v>
       </c>
       <c r="M3" t="n">
-        <v>2.13</v>
+        <v>2.31</v>
       </c>
       <c r="N3" t="n">
         <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>4.76</v>
+        <v>4.39</v>
       </c>
       <c r="P3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5084026632302405</v>
+        <v>0.5176452432667247</v>
       </c>
       <c r="R3" t="n">
-        <v>0.49842</v>
+        <v>0.51042</v>
       </c>
       <c r="S3" t="n">
-        <v>0.5024130652920962</v>
+        <v>0.5133100973066899</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -4253,7 +5185,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.5024130652920962</v>
+        <v>0.5133100973066899</v>
       </c>
     </row>
   </sheetData>
@@ -4324,22 +5256,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.15</v>
+        <v>-0.01</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>66.67</v>
+        <v>27.27</v>
       </c>
       <c r="F2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="G2" t="n">
-        <v>1.19</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
     </row>
     <row r="3">
@@ -4354,7 +5286,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="D3" t="n">
         <v>23</v>
@@ -4363,13 +5295,13 @@
         <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>2.13</v>
+        <v>2.31</v>
       </c>
       <c r="G3" t="n">
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:35:19.862143
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK35"/>
+  <dimension ref="A1:AK27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,7 +983,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -992,101 +992,101 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45554.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>53.91</v>
+        <v>13.43</v>
       </c>
       <c r="G5" t="n">
-        <v>43.72</v>
+        <v>12.66</v>
       </c>
       <c r="H5" t="n">
-        <v>51.11</v>
+        <v>13.26</v>
       </c>
       <c r="I5" t="n">
-        <v>-5.19</v>
+        <v>-1.25</v>
       </c>
       <c r="J5" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="L5" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>3180532</v>
+      </c>
+      <c r="P5" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>12.98</v>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+      <c r="V5" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="W5" t="n">
+        <v>-3.37</v>
+      </c>
+      <c r="X5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>45313.41666666666</v>
+      </c>
+      <c r="Z5" t="n">
         <v>8</v>
       </c>
-      <c r="K5" t="n">
-        <v>43.03</v>
-      </c>
-      <c r="L5" t="n">
-        <v>45.91</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>128396</v>
-      </c>
-      <c r="P5" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>45.33</v>
-      </c>
-      <c r="R5" t="b">
-        <v>1</v>
-      </c>
-      <c r="S5" t="n">
-        <v>48.75</v>
-      </c>
-      <c r="T5" t="b">
-        <v>0</v>
-      </c>
-      <c r="U5" t="b">
-        <v>1</v>
-      </c>
-      <c r="V5" t="n">
-        <v>-9.57</v>
-      </c>
-      <c r="W5" t="n">
-        <v>-15.92</v>
-      </c>
-      <c r="X5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y5" s="2" t="n">
-        <v>45547.41666666666</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1</v>
-      </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>43.72</v>
+        <v>12.66</v>
       </c>
       <c r="AE5" t="n">
-        <v>59.63</v>
+        <v>14.32</v>
       </c>
       <c r="AF5" t="n">
-        <v>18.9</v>
+        <v>5.78</v>
       </c>
       <c r="AG5" t="n">
-        <v>10.61</v>
+        <v>6.61</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.14</v>
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1111,34 +1111,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45558.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45567.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>53.48</v>
+        <v>15.59</v>
       </c>
       <c r="G6" t="n">
-        <v>50.18</v>
+        <v>13.66</v>
       </c>
       <c r="H6" t="n">
-        <v>49.83</v>
+        <v>16</v>
       </c>
       <c r="I6" t="n">
-        <v>-6.82</v>
+        <v>2.62</v>
       </c>
       <c r="J6" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="K6" t="n">
-        <v>50.18</v>
+        <v>12.64</v>
       </c>
       <c r="L6" t="n">
-        <v>52.39</v>
+        <v>14.56</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1151,65 +1151,69 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>188748</v>
+        <v>708583</v>
       </c>
       <c r="P6" t="n">
-        <v>4.9</v>
+        <v>10.05</v>
       </c>
       <c r="Q6" t="n">
-        <v>50.5</v>
+        <v>13.78</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>61.85</v>
+        <v>15.04</v>
       </c>
       <c r="T6" t="b">
         <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>15.65</v>
+        <v>-3.54</v>
       </c>
       <c r="W6" t="n">
-        <v>-5.57</v>
+        <v>-11.62</v>
       </c>
       <c r="X6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>45336.41666666666</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>8</v>
+      </c>
       <c r="AA6" t="b">
         <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>45558.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>50.18</v>
+        <v>13.66</v>
       </c>
       <c r="AE6" t="n">
-        <v>61.85</v>
+        <v>17.99</v>
       </c>
       <c r="AF6" t="n">
-        <v>6.17</v>
+        <v>12.37</v>
       </c>
       <c r="AG6" t="n">
-        <v>15.65</v>
+        <v>15.39</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>2.54</v>
+        <v>1.24</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1217,7 +1221,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1229,31 +1233,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45594.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45601.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>54</v>
+        <v>15.92</v>
       </c>
       <c r="G7" t="n">
-        <v>52.01</v>
+        <v>14.54</v>
       </c>
       <c r="H7" t="n">
-        <v>52</v>
+        <v>14.11</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.7</v>
+        <v>-11.36</v>
       </c>
       <c r="J7" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>44</v>
+        <v>14.54</v>
       </c>
       <c r="L7" t="n">
-        <v>53.95</v>
+        <v>15.68</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1266,57 +1270,61 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>36571</v>
+        <v>2359660</v>
       </c>
       <c r="P7" t="n">
-        <v>3.41</v>
+        <v>3.65</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.51</v>
+        <v>15.3</v>
       </c>
       <c r="R7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>57.99</v>
+        <v>16.22</v>
       </c>
       <c r="T7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>7.39</v>
+        <v>1.88</v>
       </c>
       <c r="W7" t="n">
-        <v>0.9399999999999999</v>
+        <v>-3.89</v>
       </c>
       <c r="X7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45599.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD7" t="n">
-        <v>52.01</v>
+        <v>14.54</v>
       </c>
       <c r="AE7" t="n">
-        <v>57.99</v>
+        <v>16.22</v>
       </c>
       <c r="AF7" t="n">
-        <v>3.69</v>
+        <v>8.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>7.39</v>
+        <v>1.91</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1324,7 +1332,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>2</v>
+        <v>0.22</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1332,7 +1340,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1344,31 +1352,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45603.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45608.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>54.34</v>
+        <v>13.08</v>
       </c>
       <c r="G8" t="n">
-        <v>52.65</v>
+        <v>12.76</v>
       </c>
       <c r="H8" t="n">
-        <v>51.7</v>
+        <v>12.39</v>
       </c>
       <c r="I8" t="n">
-        <v>-4.86</v>
+        <v>-5.26</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>51.6</v>
+        <v>12.22</v>
       </c>
       <c r="L8" t="n">
-        <v>54.24</v>
+        <v>13.04</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1381,19 +1389,19 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>18287</v>
+        <v>5618577</v>
       </c>
       <c r="P8" t="n">
-        <v>0.6899999999999999</v>
+        <v>2.06</v>
       </c>
       <c r="Q8" t="n">
-        <v>53.58</v>
+        <v>12.72</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>57.84</v>
+        <v>14.15</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
@@ -1402,10 +1410,10 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>6.44</v>
+        <v>8.18</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.4</v>
+        <v>-2.75</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1416,22 +1424,22 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45603.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>52.65</v>
+        <v>12.76</v>
       </c>
       <c r="AE8" t="n">
-        <v>57.84</v>
+        <v>14.15</v>
       </c>
       <c r="AF8" t="n">
-        <v>3.11</v>
+        <v>2.45</v>
       </c>
       <c r="AG8" t="n">
-        <v>6.44</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1439,7 +1447,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>2.07</v>
+        <v>3.35</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
@@ -1447,7 +1455,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1459,31 +1467,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45624.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45669.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>49.88</v>
+        <v>11.44</v>
       </c>
       <c r="G9" t="n">
-        <v>47.93</v>
+        <v>10.23</v>
       </c>
       <c r="H9" t="n">
-        <v>55</v>
+        <v>11.76</v>
       </c>
       <c r="I9" t="n">
-        <v>10.26</v>
+        <v>2.8</v>
       </c>
       <c r="J9" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="K9" t="n">
-        <v>48</v>
+        <v>10.01</v>
       </c>
       <c r="L9" t="n">
-        <v>49.58</v>
+        <v>11.2</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1496,19 +1504,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>431</v>
+        <v>3697242</v>
       </c>
       <c r="P9" t="n">
-        <v>1.14</v>
+        <v>10</v>
       </c>
       <c r="Q9" t="n">
-        <v>51.55</v>
+        <v>13.1</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>51.55</v>
+        <v>13.42</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1517,40 +1525,32 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>3.35</v>
+        <v>17.31</v>
       </c>
       <c r="W9" t="n">
-        <v>3.35</v>
+        <v>14.51</v>
       </c>
       <c r="X9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="2" t="n">
-        <v>45631.41666666666</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB9" s="2" t="n">
-        <v>45631.41666666666</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
-        <v>47.93</v>
+        <v>10.23</v>
       </c>
       <c r="AE9" t="n">
-        <v>51.55</v>
+        <v>13.42</v>
       </c>
       <c r="AF9" t="n">
-        <v>3.91</v>
+        <v>10.56</v>
       </c>
       <c r="AG9" t="n">
-        <v>3.35</v>
+        <v>17.34</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.86</v>
+        <v>1.64</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1566,7 +1566,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1578,31 +1578,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45704.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45714.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>47.99</v>
+        <v>12.1</v>
       </c>
       <c r="G10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="H10" t="n">
-        <v>45.81</v>
+        <v>12.4</v>
       </c>
       <c r="I10" t="n">
-        <v>-4.54</v>
+        <v>2.51</v>
       </c>
       <c r="J10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="L10" t="n">
-        <v>47.97</v>
+        <v>12.08</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1615,19 +1615,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>6897</v>
+        <v>719120</v>
       </c>
       <c r="P10" t="n">
-        <v>3.61</v>
+        <v>2.86</v>
       </c>
       <c r="Q10" t="n">
-        <v>48.54</v>
+        <v>11.92</v>
       </c>
       <c r="R10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>50.25</v>
+        <v>12.39</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1636,32 +1636,40 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>4.71</v>
+        <v>2.43</v>
       </c>
       <c r="W10" t="n">
-        <v>1.15</v>
+        <v>-1.46</v>
       </c>
       <c r="X10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y10" s="2" t="n">
+        <v>45426.41666666666</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1</v>
+      </c>
       <c r="AA10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB10" s="2" t="n">
+        <v>45425.41666666666</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
       <c r="AD10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="AE10" t="n">
-        <v>50.25</v>
+        <v>12.39</v>
       </c>
       <c r="AF10" t="n">
-        <v>4.15</v>
+        <v>3.44</v>
       </c>
       <c r="AG10" t="n">
-        <v>4.71</v>
+        <v>2.45</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -1669,7 +1677,7 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>1.13</v>
+        <v>0.71</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1677,7 +1685,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1689,31 +1697,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45727.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>47.51</v>
+        <v>13.23</v>
       </c>
       <c r="G11" t="n">
-        <v>45.8</v>
+        <v>12.37</v>
       </c>
       <c r="H11" t="n">
-        <v>45.63</v>
+        <v>15.11</v>
       </c>
       <c r="I11" t="n">
-        <v>-3.96</v>
+        <v>14.21</v>
       </c>
       <c r="J11" t="n">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="K11" t="n">
-        <v>45.81</v>
+        <v>12.37</v>
       </c>
       <c r="L11" t="n">
-        <v>46.58</v>
+        <v>12.68</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1726,19 +1734,19 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>31257</v>
+        <v>2872871</v>
       </c>
       <c r="P11" t="n">
-        <v>3.04</v>
+        <v>4.75</v>
       </c>
       <c r="Q11" t="n">
-        <v>46.46</v>
+        <v>12.61</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>46.7</v>
+        <v>13.12</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -1747,40 +1755,40 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.7</v>
+        <v>-0.85</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.21</v>
+        <v>-4.7</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45454.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>45.8</v>
+        <v>12.37</v>
       </c>
       <c r="AE11" t="n">
-        <v>48.4</v>
+        <v>13.98</v>
       </c>
       <c r="AF11" t="n">
-        <v>3.6</v>
+        <v>6.53</v>
       </c>
       <c r="AG11" t="n">
-        <v>1.87</v>
+        <v>5.68</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -1788,7 +1796,7 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.52</v>
+        <v>0.87</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1796,7 +1804,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1808,31 +1816,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45754.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>48.44</v>
+        <v>17.1</v>
       </c>
       <c r="G12" t="n">
-        <v>45.88</v>
+        <v>14.96</v>
       </c>
       <c r="H12" t="n">
-        <v>45.51</v>
+        <v>19.46</v>
       </c>
       <c r="I12" t="n">
-        <v>-6.05</v>
+        <v>13.85</v>
       </c>
       <c r="J12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K12" t="n">
-        <v>45.6</v>
+        <v>14.96</v>
       </c>
       <c r="L12" t="n">
-        <v>46.75</v>
+        <v>15.28</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1845,19 +1853,19 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>49292</v>
+        <v>2885185</v>
       </c>
       <c r="P12" t="n">
-        <v>5.14</v>
+        <v>13.79</v>
       </c>
       <c r="Q12" t="n">
-        <v>46.73</v>
+        <v>15.44</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>46.75</v>
+        <v>15.5</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1866,40 +1874,40 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.49</v>
+        <v>-9.34</v>
       </c>
       <c r="W12" t="n">
-        <v>-3.53</v>
+        <v>-9.69</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>45734.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="Z12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>45.88</v>
+        <v>14.96</v>
       </c>
       <c r="AE12" t="n">
-        <v>49.59</v>
+        <v>17.64</v>
       </c>
       <c r="AF12" t="n">
-        <v>5.28</v>
+        <v>12.49</v>
       </c>
       <c r="AG12" t="n">
-        <v>2.37</v>
+        <v>3.18</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1907,7 +1915,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1924,34 +1932,34 @@
         </is>
       </c>
       <c r="C13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45322.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>13.43</v>
+        <v>20.68</v>
       </c>
       <c r="G13" t="n">
-        <v>12.66</v>
+        <v>18.4</v>
       </c>
       <c r="H13" t="n">
-        <v>13.26</v>
+        <v>28.62</v>
       </c>
       <c r="I13" t="n">
-        <v>-1.25</v>
+        <v>38.41</v>
       </c>
       <c r="J13" t="n">
-        <v>21</v>
+        <v>185</v>
       </c>
       <c r="K13" t="n">
-        <v>12.54</v>
+        <v>18.4</v>
       </c>
       <c r="L13" t="n">
-        <v>13.42</v>
+        <v>20.24</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1964,69 +1972,69 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>3180532</v>
+        <v>807277</v>
       </c>
       <c r="P13" t="n">
-        <v>3.32</v>
+        <v>2.17</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.98</v>
+        <v>20.54</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>13.42</v>
+        <v>23.04</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.09</v>
+        <v>11.41</v>
       </c>
       <c r="W13" t="n">
-        <v>-3.37</v>
+        <v>-0.68</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45313.41666666666</v>
+        <v>45572.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>12.66</v>
+        <v>18.4</v>
       </c>
       <c r="AE13" t="n">
-        <v>14.32</v>
+        <v>23.04</v>
       </c>
       <c r="AF13" t="n">
-        <v>5.78</v>
+        <v>11.03</v>
       </c>
       <c r="AG13" t="n">
-        <v>6.61</v>
+        <v>11.41</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.14</v>
+        <v>1.03</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2043,34 +2051,34 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>15.59</v>
+        <v>28.64</v>
       </c>
       <c r="G14" t="n">
-        <v>13.66</v>
+        <v>28.08</v>
       </c>
       <c r="H14" t="n">
-        <v>16</v>
+        <v>27.22</v>
       </c>
       <c r="I14" t="n">
-        <v>2.62</v>
+        <v>-4.97</v>
       </c>
       <c r="J14" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>12.64</v>
+        <v>28</v>
       </c>
       <c r="L14" t="n">
-        <v>14.56</v>
+        <v>28.48</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2083,69 +2091,69 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>708583</v>
+        <v>1546271</v>
       </c>
       <c r="P14" t="n">
-        <v>10.05</v>
+        <v>1.79</v>
       </c>
       <c r="Q14" t="n">
-        <v>13.78</v>
+        <v>28.16</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>15.04</v>
+        <v>29</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.54</v>
+        <v>1.26</v>
       </c>
       <c r="W14" t="n">
-        <v>-11.62</v>
+        <v>-1.68</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>45336.41666666666</v>
+        <v>45729.41666666666</v>
       </c>
       <c r="Z14" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>13.66</v>
+        <v>28.08</v>
       </c>
       <c r="AE14" t="n">
-        <v>17.99</v>
+        <v>29</v>
       </c>
       <c r="AF14" t="n">
-        <v>12.37</v>
+        <v>1.96</v>
       </c>
       <c r="AG14" t="n">
-        <v>15.39</v>
+        <v>1.26</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>1.24</v>
+        <v>0.64</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2165,31 +2173,31 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45379.41666666666</v>
+        <v>45756.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>15.92</v>
+        <v>25.97</v>
       </c>
       <c r="G15" t="n">
-        <v>14.54</v>
+        <v>24.72</v>
       </c>
       <c r="H15" t="n">
-        <v>14.11</v>
+        <v>24.16</v>
       </c>
       <c r="I15" t="n">
-        <v>-11.36</v>
+        <v>-6.96</v>
       </c>
       <c r="J15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K15" t="n">
-        <v>14.54</v>
+        <v>24.68</v>
       </c>
       <c r="L15" t="n">
-        <v>15.68</v>
+        <v>25.51</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2202,61 +2210,53 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>2359660</v>
+        <v>767605</v>
       </c>
       <c r="P15" t="n">
-        <v>3.65</v>
+        <v>4.04</v>
       </c>
       <c r="Q15" t="n">
-        <v>15.3</v>
+        <v>27.46</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>16.22</v>
+        <v>29.03</v>
       </c>
       <c r="T15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15" t="b">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>1.88</v>
+        <v>11.79</v>
       </c>
       <c r="W15" t="n">
-        <v>-3.89</v>
+        <v>5.75</v>
       </c>
       <c r="X15" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y15" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB15" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="n">
-        <v>14.54</v>
+        <v>24.72</v>
       </c>
       <c r="AE15" t="n">
-        <v>16.22</v>
+        <v>29.03</v>
       </c>
       <c r="AF15" t="n">
-        <v>8.69</v>
+        <v>4.81</v>
       </c>
       <c r="AG15" t="n">
-        <v>1.91</v>
+        <v>11.8</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.22</v>
+        <v>2.45</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2284,31 +2284,31 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>13.08</v>
+        <v>25.32</v>
       </c>
       <c r="G16" t="n">
-        <v>12.76</v>
+        <v>24.12</v>
       </c>
       <c r="H16" t="n">
-        <v>12.39</v>
+        <v>23.99</v>
       </c>
       <c r="I16" t="n">
-        <v>-5.26</v>
+        <v>-5.24</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K16" t="n">
-        <v>12.22</v>
+        <v>24.12</v>
       </c>
       <c r="L16" t="n">
-        <v>13.04</v>
+        <v>25.26</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>5618577</v>
+        <v>623052</v>
       </c>
       <c r="P16" t="n">
-        <v>2.06</v>
+        <v>0.96</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.72</v>
+        <v>26.96</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>14.15</v>
+        <v>26.96</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2342,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>8.18</v>
+        <v>6.48</v>
       </c>
       <c r="W16" t="n">
-        <v>-2.75</v>
+        <v>6.48</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -2353,25 +2353,21 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB16" s="2" t="n">
-        <v>45398.41666666666</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="n">
-        <v>12.76</v>
+        <v>24.12</v>
       </c>
       <c r="AE16" t="n">
-        <v>14.15</v>
+        <v>26.96</v>
       </c>
       <c r="AF16" t="n">
-        <v>2.45</v>
+        <v>4.74</v>
       </c>
       <c r="AG16" t="n">
-        <v>8.199999999999999</v>
+        <v>6.48</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2379,7 +2375,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>3.35</v>
+        <v>1.37</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2399,31 +2395,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>11.44</v>
+        <v>22.75</v>
       </c>
       <c r="G17" t="n">
-        <v>10.23</v>
+        <v>21.66</v>
       </c>
       <c r="H17" t="n">
-        <v>11.76</v>
+        <v>21.65</v>
       </c>
       <c r="I17" t="n">
-        <v>2.8</v>
+        <v>-4.85</v>
       </c>
       <c r="J17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K17" t="n">
-        <v>10.01</v>
+        <v>21.66</v>
       </c>
       <c r="L17" t="n">
-        <v>11.2</v>
+        <v>22.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2436,19 +2432,19 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>3697242</v>
+        <v>13689820</v>
       </c>
       <c r="P17" t="n">
-        <v>10</v>
+        <v>4.94</v>
       </c>
       <c r="Q17" t="n">
-        <v>13.1</v>
+        <v>23.7</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>13.42</v>
+        <v>25.75</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -2457,10 +2453,10 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>17.31</v>
+        <v>13.18</v>
       </c>
       <c r="W17" t="n">
-        <v>14.51</v>
+        <v>4.17</v>
       </c>
       <c r="X17" t="b">
         <v>0</v>
@@ -2473,16 +2469,16 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>10.23</v>
+        <v>21.66</v>
       </c>
       <c r="AE17" t="n">
-        <v>13.42</v>
+        <v>25.75</v>
       </c>
       <c r="AF17" t="n">
-        <v>10.56</v>
+        <v>4.78</v>
       </c>
       <c r="AG17" t="n">
-        <v>17.34</v>
+        <v>13.19</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2490,7 +2486,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>1.64</v>
+        <v>2.76</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2510,31 +2506,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45434.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>12.1</v>
+        <v>21.88</v>
       </c>
       <c r="G18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="H18" t="n">
-        <v>12.4</v>
+        <v>20.53</v>
       </c>
       <c r="I18" t="n">
-        <v>2.51</v>
+        <v>-6.18</v>
       </c>
       <c r="J18" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="L18" t="n">
-        <v>12.08</v>
+        <v>21.78</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2547,19 +2543,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>719120</v>
+        <v>1476660</v>
       </c>
       <c r="P18" t="n">
-        <v>2.86</v>
+        <v>1.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.92</v>
+        <v>21.54</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>12.39</v>
+        <v>22.52</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2568,40 +2564,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>2.43</v>
+        <v>2.93</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.46</v>
+        <v>-1.55</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>45426.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="AE18" t="n">
-        <v>12.39</v>
+        <v>22.52</v>
       </c>
       <c r="AF18" t="n">
-        <v>3.44</v>
+        <v>2.41</v>
       </c>
       <c r="AG18" t="n">
-        <v>2.45</v>
+        <v>2.93</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2609,7 +2605,7 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.71</v>
+        <v>1.22</v>
       </c>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
@@ -2629,31 +2625,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>13.23</v>
+        <v>21.16</v>
       </c>
       <c r="G19" t="n">
-        <v>12.37</v>
+        <v>19.2</v>
       </c>
       <c r="H19" t="n">
-        <v>15.11</v>
+        <v>21.32</v>
       </c>
       <c r="I19" t="n">
-        <v>14.21</v>
+        <v>0.76</v>
       </c>
       <c r="J19" t="n">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="K19" t="n">
-        <v>12.37</v>
+        <v>19.92</v>
       </c>
       <c r="L19" t="n">
-        <v>12.68</v>
+        <v>20.64</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2666,69 +2662,65 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>2872871</v>
+        <v>5666121</v>
       </c>
       <c r="P19" t="n">
         <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>12.61</v>
+        <v>22.02</v>
       </c>
       <c r="R19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>13.12</v>
+        <v>22.52</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
       </c>
       <c r="U19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.85</v>
+        <v>6.43</v>
       </c>
       <c r="W19" t="n">
-        <v>-4.7</v>
+        <v>4.06</v>
       </c>
       <c r="X19" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="2" t="n">
-        <v>45454.41666666666</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD19" t="n">
-        <v>12.37</v>
+        <v>19.2</v>
       </c>
       <c r="AE19" t="n">
-        <v>13.98</v>
+        <v>22.52</v>
       </c>
       <c r="AF19" t="n">
-        <v>6.53</v>
+        <v>9.26</v>
       </c>
       <c r="AG19" t="n">
-        <v>5.68</v>
+        <v>6.43</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.87</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
@@ -2748,31 +2740,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45845.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>17.1</v>
+        <v>21.91</v>
       </c>
       <c r="G20" t="n">
-        <v>14.96</v>
+        <v>21.28</v>
       </c>
       <c r="H20" t="n">
-        <v>19.46</v>
+        <v>22.48</v>
       </c>
       <c r="I20" t="n">
-        <v>13.85</v>
+        <v>2.59</v>
       </c>
       <c r="J20" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="K20" t="n">
-        <v>14.96</v>
+        <v>21.29</v>
       </c>
       <c r="L20" t="n">
-        <v>15.28</v>
+        <v>21.84</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2785,69 +2777,69 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>2885185</v>
+        <v>1366828</v>
       </c>
       <c r="P20" t="n">
-        <v>13.79</v>
+        <v>1.44</v>
       </c>
       <c r="Q20" t="n">
-        <v>15.44</v>
+        <v>22.06</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>15.5</v>
+        <v>22.44</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20" t="n">
-        <v>-9.34</v>
+        <v>2.41</v>
       </c>
       <c r="W20" t="n">
-        <v>-9.69</v>
+        <v>0.68</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="Z20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="AC20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD20" t="n">
-        <v>14.96</v>
+        <v>21.28</v>
       </c>
       <c r="AE20" t="n">
-        <v>17.64</v>
+        <v>22.44</v>
       </c>
       <c r="AF20" t="n">
-        <v>12.49</v>
+        <v>2.88</v>
       </c>
       <c r="AG20" t="n">
-        <v>3.18</v>
+        <v>2.41</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.25</v>
+        <v>0.84</v>
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
@@ -2867,31 +2859,31 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45887.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>20.68</v>
+        <v>23.36</v>
       </c>
       <c r="G21" t="n">
-        <v>18.4</v>
+        <v>22.64</v>
       </c>
       <c r="H21" t="n">
-        <v>28.62</v>
+        <v>22.81</v>
       </c>
       <c r="I21" t="n">
-        <v>38.41</v>
+        <v>-2.36</v>
       </c>
       <c r="J21" t="n">
-        <v>185</v>
+        <v>15</v>
       </c>
       <c r="K21" t="n">
-        <v>18.4</v>
+        <v>22.39</v>
       </c>
       <c r="L21" t="n">
-        <v>20.24</v>
+        <v>23.18</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2904,19 +2896,19 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>807277</v>
+        <v>1011332</v>
       </c>
       <c r="P21" t="n">
-        <v>2.17</v>
+        <v>1.74</v>
       </c>
       <c r="Q21" t="n">
-        <v>20.54</v>
+        <v>23.12</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>23.04</v>
+        <v>23.48</v>
       </c>
       <c r="T21" t="b">
         <v>0</v>
@@ -2925,40 +2917,40 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>11.41</v>
+        <v>0.51</v>
       </c>
       <c r="W21" t="n">
-        <v>-0.68</v>
+        <v>-1.03</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45572.41666666666</v>
+        <v>45873.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>18.4</v>
+        <v>22.64</v>
       </c>
       <c r="AE21" t="n">
-        <v>23.04</v>
+        <v>23.48</v>
       </c>
       <c r="AF21" t="n">
-        <v>11.03</v>
+        <v>3.08</v>
       </c>
       <c r="AG21" t="n">
-        <v>11.41</v>
+        <v>0.51</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2966,7 +2958,7 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>1.03</v>
+        <v>0.17</v>
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
@@ -2986,31 +2978,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>28.64</v>
+        <v>21.7</v>
       </c>
       <c r="G22" t="n">
-        <v>28.08</v>
+        <v>21.06</v>
       </c>
       <c r="H22" t="n">
-        <v>27.22</v>
+        <v>21.02</v>
       </c>
       <c r="I22" t="n">
-        <v>-4.97</v>
+        <v>-3.13</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>28</v>
+        <v>21.02</v>
       </c>
       <c r="L22" t="n">
-        <v>28.48</v>
+        <v>21.26</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3023,19 +3015,19 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>1546271</v>
+        <v>811883</v>
       </c>
       <c r="P22" t="n">
-        <v>1.79</v>
+        <v>2.81</v>
       </c>
       <c r="Q22" t="n">
-        <v>28.16</v>
+        <v>21.61</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>29</v>
+        <v>21.83</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
@@ -3044,16 +3036,16 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>1.26</v>
+        <v>0.62</v>
       </c>
       <c r="W22" t="n">
-        <v>-1.68</v>
+        <v>-0.4</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -3062,22 +3054,22 @@
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>28.08</v>
+        <v>21.06</v>
       </c>
       <c r="AE22" t="n">
-        <v>29</v>
+        <v>21.83</v>
       </c>
       <c r="AF22" t="n">
-        <v>1.96</v>
+        <v>2.95</v>
       </c>
       <c r="AG22" t="n">
-        <v>1.26</v>
+        <v>0.63</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
@@ -3085,7 +3077,7 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.64</v>
+        <v>0.21</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3105,31 +3097,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45754.41666666666</v>
+        <v>45972.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>25.97</v>
+        <v>21.51</v>
       </c>
       <c r="G23" t="n">
-        <v>24.72</v>
+        <v>20.27</v>
       </c>
       <c r="H23" t="n">
-        <v>25.2</v>
+        <v>24.94</v>
       </c>
       <c r="I23" t="n">
-        <v>-2.96</v>
+        <v>15.94</v>
       </c>
       <c r="J23" t="n">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="K23" t="n">
-        <v>24.68</v>
+        <v>20.28</v>
       </c>
       <c r="L23" t="n">
-        <v>25.51</v>
+        <v>20.96</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3142,61 +3134,69 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>767605</v>
+        <v>2694406</v>
       </c>
       <c r="P23" t="n">
-        <v>4.04</v>
+        <v>3.42</v>
       </c>
       <c r="Q23" t="n">
-        <v>27.46</v>
+        <v>20.96</v>
       </c>
       <c r="R23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>29.03</v>
+        <v>20.96</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
       </c>
       <c r="U23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V23" t="n">
-        <v>11.79</v>
+        <v>-2.57</v>
       </c>
       <c r="W23" t="n">
-        <v>5.75</v>
+        <v>-2.57</v>
       </c>
       <c r="X23" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y23" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>8</v>
+      </c>
       <c r="AA23" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB23" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>0</v>
+      </c>
       <c r="AD23" t="n">
-        <v>24.72</v>
+        <v>20.27</v>
       </c>
       <c r="AE23" t="n">
-        <v>29.03</v>
+        <v>22.19</v>
       </c>
       <c r="AF23" t="n">
-        <v>4.81</v>
+        <v>5.76</v>
       </c>
       <c r="AG23" t="n">
-        <v>11.8</v>
+        <v>3.16</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>2.45</v>
+        <v>0.55</v>
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
@@ -3216,31 +3216,31 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45994.41666666666</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>45783.41666666666</v>
+        <v>46002.41666666666</v>
       </c>
       <c r="F24" t="n">
-        <v>25.32</v>
+        <v>23.44</v>
       </c>
       <c r="G24" t="n">
-        <v>24.12</v>
+        <v>22.68</v>
       </c>
       <c r="H24" t="n">
-        <v>23.99</v>
+        <v>23.56</v>
       </c>
       <c r="I24" t="n">
-        <v>-5.24</v>
+        <v>0.51</v>
       </c>
       <c r="J24" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="K24" t="n">
-        <v>24.12</v>
+        <v>22.51</v>
       </c>
       <c r="L24" t="n">
-        <v>25.26</v>
+        <v>23.43</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>623052</v>
+        <v>2183354</v>
       </c>
       <c r="P24" t="n">
-        <v>0.96</v>
+        <v>1.78</v>
       </c>
       <c r="Q24" t="n">
-        <v>26.96</v>
+        <v>23.05</v>
       </c>
       <c r="R24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>26.96</v>
+        <v>24.98</v>
       </c>
       <c r="T24" t="b">
         <v>0</v>
@@ -3274,10 +3274,10 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>6.48</v>
+        <v>6.57</v>
       </c>
       <c r="W24" t="n">
-        <v>6.48</v>
+        <v>-1.66</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3285,21 +3285,25 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB24" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0</v>
+      </c>
       <c r="AD24" t="n">
-        <v>24.12</v>
+        <v>22.68</v>
       </c>
       <c r="AE24" t="n">
-        <v>26.96</v>
+        <v>24.98</v>
       </c>
       <c r="AF24" t="n">
-        <v>4.74</v>
+        <v>3.24</v>
       </c>
       <c r="AG24" t="n">
-        <v>6.48</v>
+        <v>6.57</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
@@ -3307,7 +3311,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>1.37</v>
+        <v>2.03</v>
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
@@ -3327,31 +3331,31 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>46016.41666666666</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>46027.41666666666</v>
       </c>
       <c r="F25" t="n">
-        <v>22.75</v>
+        <v>24.6</v>
       </c>
       <c r="G25" t="n">
-        <v>21.66</v>
+        <v>23.75</v>
       </c>
       <c r="H25" t="n">
-        <v>21.65</v>
+        <v>24.41</v>
       </c>
       <c r="I25" t="n">
-        <v>-4.85</v>
+        <v>-0.77</v>
       </c>
       <c r="J25" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K25" t="n">
-        <v>21.66</v>
+        <v>23.41</v>
       </c>
       <c r="L25" t="n">
-        <v>22.2</v>
+        <v>24.09</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3364,31 +3368,31 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>13689820</v>
+        <v>2756109</v>
       </c>
       <c r="P25" t="n">
-        <v>4.94</v>
+        <v>3.54</v>
       </c>
       <c r="Q25" t="n">
-        <v>23.7</v>
+        <v>24.08</v>
       </c>
       <c r="R25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>25.75</v>
+        <v>24.5</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
       </c>
       <c r="U25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V25" t="n">
-        <v>13.18</v>
+        <v>-0.41</v>
       </c>
       <c r="W25" t="n">
-        <v>4.17</v>
+        <v>-2.11</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -3396,29 +3400,33 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB25" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0</v>
+      </c>
       <c r="AD25" t="n">
-        <v>21.66</v>
+        <v>23.75</v>
       </c>
       <c r="AE25" t="n">
-        <v>25.75</v>
+        <v>25.69</v>
       </c>
       <c r="AF25" t="n">
-        <v>4.78</v>
+        <v>3.46</v>
       </c>
       <c r="AG25" t="n">
-        <v>13.19</v>
+        <v>4.43</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>2.76</v>
+        <v>1.28</v>
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
@@ -3438,31 +3446,31 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>46069.41666666666</v>
       </c>
       <c r="F26" t="n">
-        <v>21.88</v>
+        <v>26</v>
       </c>
       <c r="G26" t="n">
-        <v>21.35</v>
+        <v>24.3</v>
       </c>
       <c r="H26" t="n">
-        <v>20.53</v>
+        <v>28.5</v>
       </c>
       <c r="I26" t="n">
-        <v>-6.18</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="K26" t="n">
-        <v>21.35</v>
+        <v>24.01</v>
       </c>
       <c r="L26" t="n">
-        <v>21.78</v>
+        <v>25.42</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3475,37 +3483,37 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>1476660</v>
+        <v>2965366</v>
       </c>
       <c r="P26" t="n">
-        <v>1.3</v>
+        <v>6.51</v>
       </c>
       <c r="Q26" t="n">
-        <v>21.54</v>
+        <v>25.42</v>
       </c>
       <c r="R26" t="b">
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>22.52</v>
+        <v>25.42</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
       </c>
       <c r="U26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V26" t="n">
-        <v>2.93</v>
+        <v>-2.23</v>
       </c>
       <c r="W26" t="n">
-        <v>-1.55</v>
+        <v>-2.23</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>45818.41666666666</v>
+        <v>46033.41666666666</v>
       </c>
       <c r="Z26" t="n">
         <v>2</v>
@@ -3514,30 +3522,30 @@
         <v>1</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>21.35</v>
+        <v>24.3</v>
       </c>
       <c r="AE26" t="n">
-        <v>22.52</v>
+        <v>27.41</v>
       </c>
       <c r="AF26" t="n">
-        <v>2.41</v>
+        <v>6.54</v>
       </c>
       <c r="AG26" t="n">
-        <v>2.93</v>
+        <v>5.42</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>1.22</v>
+        <v>0.83</v>
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
@@ -3557,31 +3565,31 @@
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>46120.41666666666</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>46139.41666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>21.16</v>
+        <v>26.61</v>
       </c>
       <c r="G27" t="n">
-        <v>19.2</v>
+        <v>25.21</v>
       </c>
       <c r="H27" t="n">
-        <v>21.32</v>
+        <v>28.7</v>
       </c>
       <c r="I27" t="n">
-        <v>0.76</v>
+        <v>7.85</v>
       </c>
       <c r="J27" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="K27" t="n">
-        <v>19.92</v>
+        <v>23.8</v>
       </c>
       <c r="L27" t="n">
-        <v>20.64</v>
+        <v>25.7</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3594,57 +3602,61 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>5666121</v>
+        <v>2499912</v>
       </c>
       <c r="P27" t="n">
-        <v>4.75</v>
+        <v>4.31</v>
       </c>
       <c r="Q27" t="n">
-        <v>22.02</v>
+        <v>26.8</v>
       </c>
       <c r="R27" t="b">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="T27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U27" t="b">
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="W27" t="n">
-        <v>4.06</v>
+        <v>0.71</v>
       </c>
       <c r="X27" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y27" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
       <c r="AA27" t="b">
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>45833.41666666666</v>
+        <v>46127.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD27" t="n">
-        <v>19.2</v>
+        <v>25.21</v>
       </c>
       <c r="AE27" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="AF27" t="n">
-        <v>9.26</v>
+        <v>5.26</v>
       </c>
       <c r="AG27" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -3652,954 +3664,10 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.13</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C28" t="b">
-        <v>0</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>45845.41666666666</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>45860.41666666666</v>
-      </c>
-      <c r="F28" t="n">
-        <v>21.91</v>
-      </c>
-      <c r="G28" t="n">
-        <v>21.28</v>
-      </c>
-      <c r="H28" t="n">
-        <v>22.48</v>
-      </c>
-      <c r="I28" t="n">
-        <v>2.59</v>
-      </c>
-      <c r="J28" t="n">
-        <v>15</v>
-      </c>
-      <c r="K28" t="n">
-        <v>21.29</v>
-      </c>
-      <c r="L28" t="n">
-        <v>21.84</v>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O28" t="n">
-        <v>1366828</v>
-      </c>
-      <c r="P28" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>22.06</v>
-      </c>
-      <c r="R28" t="b">
-        <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="T28" t="b">
-        <v>0</v>
-      </c>
-      <c r="U28" t="b">
-        <v>0</v>
-      </c>
-      <c r="V28" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="W28" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="X28" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y28" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA28" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB28" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="AC28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD28" t="n">
-        <v>21.28</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="AH28" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI28" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AJ28" t="inlineStr"/>
-      <c r="AK28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C29" t="b">
-        <v>0</v>
-      </c>
-      <c r="D29" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>45887.41666666666</v>
-      </c>
-      <c r="F29" t="n">
-        <v>23.36</v>
-      </c>
-      <c r="G29" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="H29" t="n">
-        <v>22.81</v>
-      </c>
-      <c r="I29" t="n">
-        <v>-2.36</v>
-      </c>
-      <c r="J29" t="n">
-        <v>15</v>
-      </c>
-      <c r="K29" t="n">
-        <v>22.39</v>
-      </c>
-      <c r="L29" t="n">
-        <v>23.18</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O29" t="n">
-        <v>1011332</v>
-      </c>
-      <c r="P29" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>23.12</v>
-      </c>
-      <c r="R29" t="b">
-        <v>1</v>
-      </c>
-      <c r="S29" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="T29" t="b">
-        <v>0</v>
-      </c>
-      <c r="U29" t="b">
-        <v>0</v>
-      </c>
-      <c r="V29" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="W29" t="n">
-        <v>-1.03</v>
-      </c>
-      <c r="X29" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y29" s="2" t="n">
-        <v>45873.41666666666</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA29" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB29" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="AC29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="AE29" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="AF29" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="AG29" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="AH29" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI29" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="AJ29" t="inlineStr"/>
-      <c r="AK29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C30" t="b">
-        <v>0</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="F30" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="G30" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="H30" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="I30" t="n">
-        <v>-3.13</v>
-      </c>
-      <c r="J30" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="L30" t="n">
-        <v>21.26</v>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O30" t="n">
-        <v>811883</v>
-      </c>
-      <c r="P30" t="n">
-        <v>2.81</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>21.61</v>
-      </c>
-      <c r="R30" t="b">
-        <v>1</v>
-      </c>
-      <c r="S30" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="T30" t="b">
-        <v>0</v>
-      </c>
-      <c r="U30" t="b">
-        <v>0</v>
-      </c>
-      <c r="V30" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="W30" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="X30" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y30" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA30" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB30" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="AC30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="AE30" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="AF30" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="AG30" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="AH30" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI30" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="AJ30" t="inlineStr"/>
-      <c r="AK30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C31" t="b">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>45972.41666666666</v>
-      </c>
-      <c r="F31" t="n">
-        <v>21.51</v>
-      </c>
-      <c r="G31" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="H31" t="n">
-        <v>24.94</v>
-      </c>
-      <c r="I31" t="n">
-        <v>15.94</v>
-      </c>
-      <c r="J31" t="n">
-        <v>61</v>
-      </c>
-      <c r="K31" t="n">
-        <v>20.28</v>
-      </c>
-      <c r="L31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O31" t="n">
-        <v>2694406</v>
-      </c>
-      <c r="P31" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="R31" t="b">
-        <v>1</v>
-      </c>
-      <c r="S31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="T31" t="b">
-        <v>0</v>
-      </c>
-      <c r="U31" t="b">
-        <v>1</v>
-      </c>
-      <c r="V31" t="n">
-        <v>-2.57</v>
-      </c>
-      <c r="W31" t="n">
-        <v>-2.57</v>
-      </c>
-      <c r="X31" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y31" s="2" t="n">
-        <v>45923.41666666666</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA31" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB31" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="AE31" t="n">
-        <v>22.19</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>5.76</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="AH31" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI31" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AJ31" t="inlineStr"/>
-      <c r="AK31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C32" t="b">
-        <v>0</v>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>46002.41666666666</v>
-      </c>
-      <c r="F32" t="n">
-        <v>23.44</v>
-      </c>
-      <c r="G32" t="n">
-        <v>22.68</v>
-      </c>
-      <c r="H32" t="n">
-        <v>23.56</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="J32" t="n">
-        <v>8</v>
-      </c>
-      <c r="K32" t="n">
-        <v>22.51</v>
-      </c>
-      <c r="L32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O32" t="n">
-        <v>2183354</v>
-      </c>
-      <c r="P32" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>22.87</v>
-      </c>
-      <c r="R32" t="b">
-        <v>1</v>
-      </c>
-      <c r="S32" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="T32" t="b">
-        <v>0</v>
-      </c>
-      <c r="U32" t="b">
-        <v>0</v>
-      </c>
-      <c r="V32" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="W32" t="n">
-        <v>-2.43</v>
-      </c>
-      <c r="X32" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB32" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="AC32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>22.68</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="AG32" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="AH32" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI32" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AJ32" t="inlineStr"/>
-      <c r="AK32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C33" t="b">
-        <v>0</v>
-      </c>
-      <c r="D33" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>46027.41666666666</v>
-      </c>
-      <c r="F33" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G33" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="H33" t="n">
-        <v>24.41</v>
-      </c>
-      <c r="I33" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="J33" t="n">
-        <v>11</v>
-      </c>
-      <c r="K33" t="n">
-        <v>23.41</v>
-      </c>
-      <c r="L33" t="n">
-        <v>24.09</v>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O33" t="n">
-        <v>2756109</v>
-      </c>
-      <c r="P33" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>24.08</v>
-      </c>
-      <c r="R33" t="b">
-        <v>1</v>
-      </c>
-      <c r="S33" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="T33" t="b">
-        <v>0</v>
-      </c>
-      <c r="U33" t="b">
-        <v>1</v>
-      </c>
-      <c r="V33" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="W33" t="n">
-        <v>-2.11</v>
-      </c>
-      <c r="X33" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB33" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="AC33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD33" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="AE33" t="n">
-        <v>25.69</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="AH33" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI33" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="AJ33" t="inlineStr"/>
-      <c r="AK33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C34" t="b">
-        <v>0</v>
-      </c>
-      <c r="D34" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>46069.41666666666</v>
-      </c>
-      <c r="F34" t="n">
-        <v>26</v>
-      </c>
-      <c r="G34" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="H34" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="I34" t="n">
-        <v>9.619999999999999</v>
-      </c>
-      <c r="J34" t="n">
-        <v>41</v>
-      </c>
-      <c r="K34" t="n">
-        <v>24.01</v>
-      </c>
-      <c r="L34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O34" t="n">
-        <v>2965366</v>
-      </c>
-      <c r="P34" t="n">
-        <v>6.51</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="R34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="T34" t="b">
-        <v>0</v>
-      </c>
-      <c r="U34" t="b">
-        <v>1</v>
-      </c>
-      <c r="V34" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="W34" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="X34" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y34" s="2" t="n">
-        <v>46033.41666666666</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA34" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB34" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="AC34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="AE34" t="n">
-        <v>27.41</v>
-      </c>
-      <c r="AF34" t="n">
-        <v>6.54</v>
-      </c>
-      <c r="AG34" t="n">
-        <v>5.42</v>
-      </c>
-      <c r="AH34" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI34" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="AJ34" t="inlineStr"/>
-      <c r="AK34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C35" t="b">
-        <v>0</v>
-      </c>
-      <c r="D35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>46139.41666666666</v>
-      </c>
-      <c r="F35" t="n">
-        <v>26.61</v>
-      </c>
-      <c r="G35" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="H35" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="I35" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="J35" t="n">
-        <v>19</v>
-      </c>
-      <c r="K35" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="L35" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O35" t="n">
-        <v>2499912</v>
-      </c>
-      <c r="P35" t="n">
-        <v>4.31</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>25.73</v>
-      </c>
-      <c r="R35" t="b">
-        <v>1</v>
-      </c>
-      <c r="S35" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="T35" t="b">
-        <v>1</v>
-      </c>
-      <c r="U35" t="b">
-        <v>0</v>
-      </c>
-      <c r="V35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="W35" t="n">
-        <v>-3.31</v>
-      </c>
-      <c r="X35" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA35" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="AC35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="AE35" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="AG35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="AH35" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI35" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AJ35" t="inlineStr"/>
-      <c r="AK35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4817,31 +3885,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>47.87</v>
+        <v>53.91</v>
       </c>
       <c r="G2" t="n">
-        <v>46</v>
+        <v>43.72</v>
       </c>
       <c r="H2" t="n">
         <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>278.11</v>
+        <v>235.74</v>
       </c>
       <c r="J2" t="n">
-        <v>384</v>
+        <v>593</v>
       </c>
       <c r="K2" t="n">
-        <v>45</v>
+        <v>43.03</v>
       </c>
       <c r="L2" t="n">
-        <v>46.89</v>
+        <v>45.91</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -4854,69 +3922,69 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>47815</v>
+        <v>128396</v>
       </c>
       <c r="P2" t="n">
-        <v>2.73</v>
+        <v>19.99</v>
       </c>
       <c r="Q2" t="n">
-        <v>46.62</v>
+        <v>45.33</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>51</v>
+        <v>48.75</v>
       </c>
       <c r="T2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>6.54</v>
+        <v>-9.57</v>
       </c>
       <c r="W2" t="n">
-        <v>-2.61</v>
+        <v>-15.92</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45547.41666666666</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>46</v>
+        <v>43.72</v>
       </c>
       <c r="AE2" t="n">
-        <v>51</v>
+        <v>59.63</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.91</v>
+        <v>18.9</v>
       </c>
       <c r="AG2" t="n">
-        <v>6.54</v>
+        <v>10.61</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>1.67</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ2" t="n">
         <v>181</v>
@@ -5058,25 +4126,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>27.27</v>
+        <v>66.67</v>
       </c>
       <c r="G2" t="n">
-        <v>-4.54</v>
+        <v>1.19</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
       <c r="I2" t="n">
-        <v>-25.44</v>
+        <v>-0.58</v>
       </c>
       <c r="J2" t="n">
         <v>12.48</v>
@@ -5085,28 +4153,28 @@
         <v>-14.25</v>
       </c>
       <c r="L2" t="n">
-        <v>7.68</v>
+        <v>13.42</v>
       </c>
       <c r="M2" t="n">
-        <v>0.48</v>
+        <v>0.96</v>
       </c>
       <c r="N2" t="n">
-        <v>7.98</v>
+        <v>6.84</v>
       </c>
       <c r="O2" t="n">
-        <v>6.17</v>
+        <v>14.25</v>
       </c>
       <c r="P2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1209768433179723</v>
+        <v>0.2320120319001387</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.09292000000000003</v>
+        <v>0.09086</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.007361262672811078</v>
+        <v>0.1473208127600555</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -5114,7 +4182,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>-0.007361262672811078</v>
+        <v>0.1473208127600555</v>
       </c>
     </row>
     <row r="3">
@@ -5144,10 +4212,10 @@
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
       <c r="I3" t="n">
-        <v>63.34</v>
+        <v>59.34</v>
       </c>
       <c r="J3" t="n">
         <v>38.41</v>
@@ -5156,28 +4224,28 @@
         <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>10.51</v>
+        <v>10.64</v>
       </c>
       <c r="M3" t="n">
-        <v>2.31</v>
+        <v>2.13</v>
       </c>
       <c r="N3" t="n">
         <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>4.39</v>
+        <v>4.76</v>
       </c>
       <c r="P3" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5176452432667247</v>
+        <v>0.5084026632302405</v>
       </c>
       <c r="R3" t="n">
-        <v>0.51042</v>
+        <v>0.49842</v>
       </c>
       <c r="S3" t="n">
-        <v>0.5133100973066899</v>
+        <v>0.5024130652920962</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -5185,7 +4253,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.5133100973066899</v>
+        <v>0.5024130652920962</v>
       </c>
     </row>
   </sheetData>
@@ -5256,22 +4324,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.01</v>
+        <v>0.15</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>27.27</v>
+        <v>66.67</v>
       </c>
       <c r="F2" t="n">
-        <v>0.48</v>
+        <v>0.96</v>
       </c>
       <c r="G2" t="n">
-        <v>-4.54</v>
+        <v>1.19</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
     </row>
     <row r="3">
@@ -5286,7 +4354,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.51</v>
+        <v>0.5</v>
       </c>
       <c r="D3" t="n">
         <v>23</v>
@@ -5295,13 +4363,13 @@
         <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>2.31</v>
+        <v>2.13</v>
       </c>
       <c r="G3" t="n">
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:35:31.546715
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK27"/>
+  <dimension ref="A1:AK35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,7 +983,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -992,34 +992,34 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45322.41666666666</v>
+        <v>45554.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>13.43</v>
+        <v>53.91</v>
       </c>
       <c r="G5" t="n">
-        <v>12.66</v>
+        <v>43.72</v>
       </c>
       <c r="H5" t="n">
-        <v>13.26</v>
+        <v>51.11</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.25</v>
+        <v>-5.19</v>
       </c>
       <c r="J5" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>12.54</v>
+        <v>43.03</v>
       </c>
       <c r="L5" t="n">
-        <v>13.42</v>
+        <v>45.91</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1032,19 +1032,19 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>3180532</v>
+        <v>128396</v>
       </c>
       <c r="P5" t="n">
-        <v>3.32</v>
+        <v>19.99</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.98</v>
+        <v>45.33</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>13.42</v>
+        <v>48.75</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
@@ -1053,40 +1053,40 @@
         <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.09</v>
+        <v>-9.57</v>
       </c>
       <c r="W5" t="n">
-        <v>-3.37</v>
+        <v>-15.92</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>45313.41666666666</v>
+        <v>45547.41666666666</v>
       </c>
       <c r="Z5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>12.66</v>
+        <v>43.72</v>
       </c>
       <c r="AE5" t="n">
-        <v>14.32</v>
+        <v>59.63</v>
       </c>
       <c r="AF5" t="n">
-        <v>5.78</v>
+        <v>18.9</v>
       </c>
       <c r="AG5" t="n">
-        <v>6.61</v>
+        <v>10.61</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>1.14</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1111,34 +1111,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45558.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45567.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>15.59</v>
+        <v>53.48</v>
       </c>
       <c r="G6" t="n">
-        <v>13.66</v>
+        <v>50.18</v>
       </c>
       <c r="H6" t="n">
-        <v>16</v>
+        <v>49.83</v>
       </c>
       <c r="I6" t="n">
-        <v>2.62</v>
+        <v>-6.82</v>
       </c>
       <c r="J6" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="K6" t="n">
-        <v>12.64</v>
+        <v>50.18</v>
       </c>
       <c r="L6" t="n">
-        <v>14.56</v>
+        <v>52.39</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1151,69 +1151,65 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>708583</v>
+        <v>188748</v>
       </c>
       <c r="P6" t="n">
-        <v>10.05</v>
+        <v>4.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>13.78</v>
+        <v>50.5</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>15.04</v>
+        <v>61.85</v>
       </c>
       <c r="T6" t="b">
         <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.54</v>
+        <v>15.65</v>
       </c>
       <c r="W6" t="n">
-        <v>-11.62</v>
+        <v>-5.57</v>
       </c>
       <c r="X6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="2" t="n">
-        <v>45336.41666666666</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="b">
         <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45558.41666666666</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>13.66</v>
+        <v>50.18</v>
       </c>
       <c r="AE6" t="n">
-        <v>17.99</v>
+        <v>61.85</v>
       </c>
       <c r="AF6" t="n">
-        <v>12.37</v>
+        <v>6.17</v>
       </c>
       <c r="AG6" t="n">
-        <v>15.39</v>
+        <v>15.65</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>1.24</v>
+        <v>2.54</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1221,7 +1217,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1233,31 +1229,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45594.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45379.41666666666</v>
+        <v>45601.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>15.92</v>
+        <v>54</v>
       </c>
       <c r="G7" t="n">
-        <v>14.54</v>
+        <v>52.01</v>
       </c>
       <c r="H7" t="n">
-        <v>14.11</v>
+        <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>-11.36</v>
+        <v>-3.7</v>
       </c>
       <c r="J7" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>14.54</v>
+        <v>44</v>
       </c>
       <c r="L7" t="n">
-        <v>15.68</v>
+        <v>53.95</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1270,61 +1266,57 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>2359660</v>
+        <v>36571</v>
       </c>
       <c r="P7" t="n">
-        <v>3.65</v>
+        <v>3.41</v>
       </c>
       <c r="Q7" t="n">
-        <v>15.3</v>
+        <v>54.51</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>16.22</v>
+        <v>57.99</v>
       </c>
       <c r="T7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>1.88</v>
+        <v>7.39</v>
       </c>
       <c r="W7" t="n">
-        <v>-3.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45599.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD7" t="n">
-        <v>14.54</v>
+        <v>52.01</v>
       </c>
       <c r="AE7" t="n">
-        <v>16.22</v>
+        <v>57.99</v>
       </c>
       <c r="AF7" t="n">
-        <v>8.69</v>
+        <v>3.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>1.91</v>
+        <v>7.39</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1332,7 +1324,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.22</v>
+        <v>2</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1340,7 +1332,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1352,31 +1344,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45603.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45608.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>13.08</v>
+        <v>54.34</v>
       </c>
       <c r="G8" t="n">
-        <v>12.76</v>
+        <v>52.65</v>
       </c>
       <c r="H8" t="n">
-        <v>12.39</v>
+        <v>51.7</v>
       </c>
       <c r="I8" t="n">
-        <v>-5.26</v>
+        <v>-4.86</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>12.22</v>
+        <v>51.6</v>
       </c>
       <c r="L8" t="n">
-        <v>13.04</v>
+        <v>54.24</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1389,19 +1381,19 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>5618577</v>
+        <v>18287</v>
       </c>
       <c r="P8" t="n">
-        <v>2.06</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.72</v>
+        <v>53.58</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>14.15</v>
+        <v>57.84</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
@@ -1410,10 +1402,10 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>8.18</v>
+        <v>6.44</v>
       </c>
       <c r="W8" t="n">
-        <v>-2.75</v>
+        <v>-1.4</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1424,22 +1416,22 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45603.41666666666</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>12.76</v>
+        <v>52.65</v>
       </c>
       <c r="AE8" t="n">
-        <v>14.15</v>
+        <v>57.84</v>
       </c>
       <c r="AF8" t="n">
-        <v>2.45</v>
+        <v>3.11</v>
       </c>
       <c r="AG8" t="n">
-        <v>8.199999999999999</v>
+        <v>6.44</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1447,7 +1439,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>3.35</v>
+        <v>2.07</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
@@ -1455,7 +1447,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1467,31 +1459,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45624.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45669.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>11.44</v>
+        <v>49.88</v>
       </c>
       <c r="G9" t="n">
-        <v>10.23</v>
+        <v>47.93</v>
       </c>
       <c r="H9" t="n">
-        <v>11.76</v>
+        <v>55</v>
       </c>
       <c r="I9" t="n">
-        <v>2.8</v>
+        <v>10.26</v>
       </c>
       <c r="J9" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>10.01</v>
+        <v>48</v>
       </c>
       <c r="L9" t="n">
-        <v>11.2</v>
+        <v>49.58</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1504,19 +1496,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>3697242</v>
+        <v>431</v>
       </c>
       <c r="P9" t="n">
-        <v>10</v>
+        <v>1.14</v>
       </c>
       <c r="Q9" t="n">
-        <v>13.1</v>
+        <v>51.55</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>13.42</v>
+        <v>51.55</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1525,32 +1517,40 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>17.31</v>
+        <v>3.35</v>
       </c>
       <c r="W9" t="n">
-        <v>14.51</v>
+        <v>3.35</v>
       </c>
       <c r="X9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>45631.41666666666</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>5</v>
+      </c>
       <c r="AA9" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2" t="n">
+        <v>45631.41666666666</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>5</v>
+      </c>
       <c r="AD9" t="n">
-        <v>10.23</v>
+        <v>47.93</v>
       </c>
       <c r="AE9" t="n">
-        <v>13.42</v>
+        <v>51.55</v>
       </c>
       <c r="AF9" t="n">
-        <v>10.56</v>
+        <v>3.91</v>
       </c>
       <c r="AG9" t="n">
-        <v>17.34</v>
+        <v>3.35</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>1.64</v>
+        <v>0.86</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1566,7 +1566,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1578,31 +1578,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45704.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45434.41666666666</v>
+        <v>45714.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>12.1</v>
+        <v>47.99</v>
       </c>
       <c r="G10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="H10" t="n">
-        <v>12.4</v>
+        <v>45.81</v>
       </c>
       <c r="I10" t="n">
-        <v>2.51</v>
+        <v>-4.54</v>
       </c>
       <c r="J10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="L10" t="n">
-        <v>12.08</v>
+        <v>47.97</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1615,19 +1615,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>719120</v>
+        <v>6897</v>
       </c>
       <c r="P10" t="n">
-        <v>2.86</v>
+        <v>3.61</v>
       </c>
       <c r="Q10" t="n">
-        <v>11.92</v>
+        <v>48.54</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>12.39</v>
+        <v>50.25</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1636,40 +1636,32 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>2.43</v>
+        <v>4.71</v>
       </c>
       <c r="W10" t="n">
-        <v>-1.46</v>
+        <v>1.15</v>
       </c>
       <c r="X10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="2" t="n">
-        <v>45426.41666666666</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB10" s="2" t="n">
-        <v>45425.41666666666</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="AE10" t="n">
-        <v>12.39</v>
+        <v>50.25</v>
       </c>
       <c r="AF10" t="n">
-        <v>3.44</v>
+        <v>4.15</v>
       </c>
       <c r="AG10" t="n">
-        <v>2.45</v>
+        <v>4.71</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -1677,7 +1669,7 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.71</v>
+        <v>1.13</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1685,7 +1677,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1697,31 +1689,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45727.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>13.23</v>
+        <v>47.51</v>
       </c>
       <c r="G11" t="n">
-        <v>12.37</v>
+        <v>45.8</v>
       </c>
       <c r="H11" t="n">
-        <v>15.11</v>
+        <v>45.63</v>
       </c>
       <c r="I11" t="n">
-        <v>14.21</v>
+        <v>-3.96</v>
       </c>
       <c r="J11" t="n">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="K11" t="n">
-        <v>12.37</v>
+        <v>45.81</v>
       </c>
       <c r="L11" t="n">
-        <v>12.68</v>
+        <v>46.58</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1734,19 +1726,19 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>2872871</v>
+        <v>31257</v>
       </c>
       <c r="P11" t="n">
-        <v>4.75</v>
+        <v>3.04</v>
       </c>
       <c r="Q11" t="n">
-        <v>12.61</v>
+        <v>46.46</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>13.12</v>
+        <v>46.7</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -1755,40 +1747,40 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>-0.85</v>
+        <v>-1.7</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.7</v>
+        <v>-2.21</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45454.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>12.37</v>
+        <v>45.8</v>
       </c>
       <c r="AE11" t="n">
-        <v>13.98</v>
+        <v>48.4</v>
       </c>
       <c r="AF11" t="n">
-        <v>6.53</v>
+        <v>3.6</v>
       </c>
       <c r="AG11" t="n">
-        <v>5.68</v>
+        <v>1.87</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -1796,7 +1788,7 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.87</v>
+        <v>0.52</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1804,7 +1796,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1816,31 +1808,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>17.1</v>
+        <v>48.44</v>
       </c>
       <c r="G12" t="n">
-        <v>14.96</v>
+        <v>45.88</v>
       </c>
       <c r="H12" t="n">
-        <v>19.46</v>
+        <v>45.51</v>
       </c>
       <c r="I12" t="n">
-        <v>13.85</v>
+        <v>-6.05</v>
       </c>
       <c r="J12" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K12" t="n">
-        <v>14.96</v>
+        <v>45.6</v>
       </c>
       <c r="L12" t="n">
-        <v>15.28</v>
+        <v>46.75</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1853,19 +1845,19 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>2885185</v>
+        <v>49292</v>
       </c>
       <c r="P12" t="n">
-        <v>13.79</v>
+        <v>5.14</v>
       </c>
       <c r="Q12" t="n">
-        <v>15.44</v>
+        <v>46.73</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>15.5</v>
+        <v>46.75</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1874,40 +1866,40 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-9.34</v>
+        <v>-3.49</v>
       </c>
       <c r="W12" t="n">
-        <v>-9.69</v>
+        <v>-3.53</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45734.41666666666</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>14.96</v>
+        <v>45.88</v>
       </c>
       <c r="AE12" t="n">
-        <v>17.64</v>
+        <v>49.59</v>
       </c>
       <c r="AF12" t="n">
-        <v>12.49</v>
+        <v>5.28</v>
       </c>
       <c r="AG12" t="n">
-        <v>3.18</v>
+        <v>2.37</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1915,7 +1907,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.25</v>
+        <v>0.45</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1932,34 +1924,34 @@
         </is>
       </c>
       <c r="C13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>20.68</v>
+        <v>13.43</v>
       </c>
       <c r="G13" t="n">
-        <v>18.4</v>
+        <v>12.66</v>
       </c>
       <c r="H13" t="n">
-        <v>28.62</v>
+        <v>13.26</v>
       </c>
       <c r="I13" t="n">
-        <v>38.41</v>
+        <v>-1.25</v>
       </c>
       <c r="J13" t="n">
-        <v>185</v>
+        <v>21</v>
       </c>
       <c r="K13" t="n">
-        <v>18.4</v>
+        <v>12.54</v>
       </c>
       <c r="L13" t="n">
-        <v>20.24</v>
+        <v>13.42</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1972,69 +1964,69 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>807277</v>
+        <v>3180532</v>
       </c>
       <c r="P13" t="n">
-        <v>2.17</v>
+        <v>3.32</v>
       </c>
       <c r="Q13" t="n">
-        <v>20.54</v>
+        <v>12.98</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>23.04</v>
+        <v>13.42</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>11.41</v>
+        <v>-0.09</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.68</v>
+        <v>-3.37</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45572.41666666666</v>
+        <v>45313.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>18.4</v>
+        <v>12.66</v>
       </c>
       <c r="AE13" t="n">
-        <v>23.04</v>
+        <v>14.32</v>
       </c>
       <c r="AF13" t="n">
-        <v>11.03</v>
+        <v>5.78</v>
       </c>
       <c r="AG13" t="n">
-        <v>11.41</v>
+        <v>6.61</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.03</v>
+        <v>1.14</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2051,34 +2043,34 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>28.64</v>
+        <v>15.59</v>
       </c>
       <c r="G14" t="n">
-        <v>28.08</v>
+        <v>13.66</v>
       </c>
       <c r="H14" t="n">
-        <v>27.22</v>
+        <v>16</v>
       </c>
       <c r="I14" t="n">
-        <v>-4.97</v>
+        <v>2.62</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="K14" t="n">
-        <v>28</v>
+        <v>12.64</v>
       </c>
       <c r="L14" t="n">
-        <v>28.48</v>
+        <v>14.56</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2091,69 +2083,69 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>1546271</v>
+        <v>708583</v>
       </c>
       <c r="P14" t="n">
-        <v>1.79</v>
+        <v>10.05</v>
       </c>
       <c r="Q14" t="n">
-        <v>28.16</v>
+        <v>13.78</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>29</v>
+        <v>15.04</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>1.26</v>
+        <v>-3.54</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.68</v>
+        <v>-11.62</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45336.41666666666</v>
       </c>
       <c r="Z14" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>28.08</v>
+        <v>13.66</v>
       </c>
       <c r="AE14" t="n">
-        <v>29</v>
+        <v>17.99</v>
       </c>
       <c r="AF14" t="n">
-        <v>1.96</v>
+        <v>12.37</v>
       </c>
       <c r="AG14" t="n">
-        <v>1.26</v>
+        <v>15.39</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.64</v>
+        <v>1.24</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2173,31 +2165,31 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45756.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>25.97</v>
+        <v>15.92</v>
       </c>
       <c r="G15" t="n">
-        <v>24.72</v>
+        <v>14.54</v>
       </c>
       <c r="H15" t="n">
-        <v>24.16</v>
+        <v>14.11</v>
       </c>
       <c r="I15" t="n">
-        <v>-6.96</v>
+        <v>-11.36</v>
       </c>
       <c r="J15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K15" t="n">
-        <v>24.68</v>
+        <v>14.54</v>
       </c>
       <c r="L15" t="n">
-        <v>25.51</v>
+        <v>15.68</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2210,53 +2202,61 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>767605</v>
+        <v>2359660</v>
       </c>
       <c r="P15" t="n">
-        <v>4.04</v>
+        <v>3.65</v>
       </c>
       <c r="Q15" t="n">
-        <v>27.46</v>
+        <v>15.3</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>29.03</v>
+        <v>16.22</v>
       </c>
       <c r="T15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U15" t="b">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>11.79</v>
+        <v>1.88</v>
       </c>
       <c r="W15" t="n">
-        <v>5.75</v>
+        <v>-3.89</v>
       </c>
       <c r="X15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y15" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
       <c r="AA15" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB15" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0</v>
+      </c>
       <c r="AD15" t="n">
-        <v>24.72</v>
+        <v>14.54</v>
       </c>
       <c r="AE15" t="n">
-        <v>29.03</v>
+        <v>16.22</v>
       </c>
       <c r="AF15" t="n">
-        <v>4.81</v>
+        <v>8.69</v>
       </c>
       <c r="AG15" t="n">
-        <v>11.8</v>
+        <v>1.91</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>2.45</v>
+        <v>0.22</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2284,31 +2284,31 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45783.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>25.32</v>
+        <v>13.08</v>
       </c>
       <c r="G16" t="n">
-        <v>24.12</v>
+        <v>12.76</v>
       </c>
       <c r="H16" t="n">
-        <v>23.99</v>
+        <v>12.39</v>
       </c>
       <c r="I16" t="n">
-        <v>-5.24</v>
+        <v>-5.26</v>
       </c>
       <c r="J16" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>24.12</v>
+        <v>12.22</v>
       </c>
       <c r="L16" t="n">
-        <v>25.26</v>
+        <v>13.04</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>623052</v>
+        <v>5618577</v>
       </c>
       <c r="P16" t="n">
-        <v>0.96</v>
+        <v>2.06</v>
       </c>
       <c r="Q16" t="n">
-        <v>26.96</v>
+        <v>12.72</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>26.96</v>
+        <v>14.15</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2342,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>6.48</v>
+        <v>8.18</v>
       </c>
       <c r="W16" t="n">
-        <v>6.48</v>
+        <v>-2.75</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -2353,21 +2353,25 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB16" s="2" t="n">
+        <v>45398.41666666666</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
       <c r="AD16" t="n">
-        <v>24.12</v>
+        <v>12.76</v>
       </c>
       <c r="AE16" t="n">
-        <v>26.96</v>
+        <v>14.15</v>
       </c>
       <c r="AF16" t="n">
-        <v>4.74</v>
+        <v>2.45</v>
       </c>
       <c r="AG16" t="n">
-        <v>6.48</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2375,7 +2379,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>1.37</v>
+        <v>3.35</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2395,31 +2399,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>22.75</v>
+        <v>11.44</v>
       </c>
       <c r="G17" t="n">
-        <v>21.66</v>
+        <v>10.23</v>
       </c>
       <c r="H17" t="n">
-        <v>21.65</v>
+        <v>11.76</v>
       </c>
       <c r="I17" t="n">
-        <v>-4.85</v>
+        <v>2.8</v>
       </c>
       <c r="J17" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
-        <v>21.66</v>
+        <v>10.01</v>
       </c>
       <c r="L17" t="n">
-        <v>22.2</v>
+        <v>11.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2432,19 +2436,19 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>13689820</v>
+        <v>3697242</v>
       </c>
       <c r="P17" t="n">
-        <v>4.94</v>
+        <v>10</v>
       </c>
       <c r="Q17" t="n">
-        <v>23.7</v>
+        <v>13.1</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>25.75</v>
+        <v>13.42</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -2453,10 +2457,10 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>13.18</v>
+        <v>17.31</v>
       </c>
       <c r="W17" t="n">
-        <v>4.17</v>
+        <v>14.51</v>
       </c>
       <c r="X17" t="b">
         <v>0</v>
@@ -2469,16 +2473,16 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>21.66</v>
+        <v>10.23</v>
       </c>
       <c r="AE17" t="n">
-        <v>25.75</v>
+        <v>13.42</v>
       </c>
       <c r="AF17" t="n">
-        <v>4.78</v>
+        <v>10.56</v>
       </c>
       <c r="AG17" t="n">
-        <v>13.19</v>
+        <v>17.34</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2486,7 +2490,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>2.76</v>
+        <v>1.64</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2506,31 +2510,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>21.88</v>
+        <v>12.1</v>
       </c>
       <c r="G18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="H18" t="n">
-        <v>20.53</v>
+        <v>12.4</v>
       </c>
       <c r="I18" t="n">
-        <v>-6.18</v>
+        <v>2.51</v>
       </c>
       <c r="J18" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="L18" t="n">
-        <v>21.78</v>
+        <v>12.08</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2543,19 +2547,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>1476660</v>
+        <v>719120</v>
       </c>
       <c r="P18" t="n">
-        <v>1.3</v>
+        <v>2.86</v>
       </c>
       <c r="Q18" t="n">
-        <v>21.54</v>
+        <v>11.92</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>22.52</v>
+        <v>12.39</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2564,40 +2568,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>2.93</v>
+        <v>2.43</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.55</v>
+        <v>-1.46</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>45818.41666666666</v>
+        <v>45426.41666666666</v>
       </c>
       <c r="Z18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="AE18" t="n">
-        <v>22.52</v>
+        <v>12.39</v>
       </c>
       <c r="AF18" t="n">
-        <v>2.41</v>
+        <v>3.44</v>
       </c>
       <c r="AG18" t="n">
-        <v>2.93</v>
+        <v>2.45</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2605,7 +2609,7 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>1.22</v>
+        <v>0.71</v>
       </c>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
@@ -2625,31 +2629,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>21.16</v>
+        <v>13.23</v>
       </c>
       <c r="G19" t="n">
-        <v>19.2</v>
+        <v>12.37</v>
       </c>
       <c r="H19" t="n">
-        <v>21.32</v>
+        <v>15.11</v>
       </c>
       <c r="I19" t="n">
-        <v>0.76</v>
+        <v>14.21</v>
       </c>
       <c r="J19" t="n">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="K19" t="n">
-        <v>19.92</v>
+        <v>12.37</v>
       </c>
       <c r="L19" t="n">
-        <v>20.64</v>
+        <v>12.68</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2662,65 +2666,69 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>5666121</v>
+        <v>2872871</v>
       </c>
       <c r="P19" t="n">
         <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>22.02</v>
+        <v>12.61</v>
       </c>
       <c r="R19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>22.52</v>
+        <v>13.12</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
       </c>
       <c r="U19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" t="n">
-        <v>6.43</v>
+        <v>-0.85</v>
       </c>
       <c r="W19" t="n">
-        <v>4.06</v>
+        <v>-4.7</v>
       </c>
       <c r="X19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y19" s="2" t="n">
+        <v>45454.41666666666</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>11</v>
+      </c>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45833.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD19" t="n">
-        <v>19.2</v>
+        <v>12.37</v>
       </c>
       <c r="AE19" t="n">
-        <v>22.52</v>
+        <v>13.98</v>
       </c>
       <c r="AF19" t="n">
-        <v>9.26</v>
+        <v>6.53</v>
       </c>
       <c r="AG19" t="n">
-        <v>6.43</v>
+        <v>5.68</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.87</v>
       </c>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
@@ -2740,31 +2748,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45845.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>21.91</v>
+        <v>17.1</v>
       </c>
       <c r="G20" t="n">
-        <v>21.28</v>
+        <v>14.96</v>
       </c>
       <c r="H20" t="n">
-        <v>22.48</v>
+        <v>19.46</v>
       </c>
       <c r="I20" t="n">
-        <v>2.59</v>
+        <v>13.85</v>
       </c>
       <c r="J20" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="K20" t="n">
-        <v>21.29</v>
+        <v>14.96</v>
       </c>
       <c r="L20" t="n">
-        <v>21.84</v>
+        <v>15.28</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2777,69 +2785,69 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>1366828</v>
+        <v>2885185</v>
       </c>
       <c r="P20" t="n">
-        <v>1.44</v>
+        <v>13.79</v>
       </c>
       <c r="Q20" t="n">
-        <v>22.06</v>
+        <v>15.44</v>
       </c>
       <c r="R20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>22.44</v>
+        <v>15.5</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
-        <v>2.41</v>
+        <v>-9.34</v>
       </c>
       <c r="W20" t="n">
-        <v>0.68</v>
+        <v>-9.69</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>45847.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="Z20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>45847.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="AC20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD20" t="n">
-        <v>21.28</v>
+        <v>14.96</v>
       </c>
       <c r="AE20" t="n">
-        <v>22.44</v>
+        <v>17.64</v>
       </c>
       <c r="AF20" t="n">
-        <v>2.88</v>
+        <v>12.49</v>
       </c>
       <c r="AG20" t="n">
-        <v>2.41</v>
+        <v>3.18</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.84</v>
+        <v>0.25</v>
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
@@ -2859,31 +2867,31 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45887.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>23.36</v>
+        <v>20.68</v>
       </c>
       <c r="G21" t="n">
-        <v>22.64</v>
+        <v>18.4</v>
       </c>
       <c r="H21" t="n">
-        <v>22.81</v>
+        <v>28.62</v>
       </c>
       <c r="I21" t="n">
-        <v>-2.36</v>
+        <v>38.41</v>
       </c>
       <c r="J21" t="n">
-        <v>15</v>
+        <v>185</v>
       </c>
       <c r="K21" t="n">
-        <v>22.39</v>
+        <v>18.4</v>
       </c>
       <c r="L21" t="n">
-        <v>23.18</v>
+        <v>20.24</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2896,19 +2904,19 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>1011332</v>
+        <v>807277</v>
       </c>
       <c r="P21" t="n">
-        <v>1.74</v>
+        <v>2.17</v>
       </c>
       <c r="Q21" t="n">
-        <v>23.12</v>
+        <v>20.54</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>23.48</v>
+        <v>23.04</v>
       </c>
       <c r="T21" t="b">
         <v>0</v>
@@ -2917,40 +2925,40 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>0.51</v>
+        <v>11.41</v>
       </c>
       <c r="W21" t="n">
-        <v>-1.03</v>
+        <v>-0.68</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45873.41666666666</v>
+        <v>45572.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>22.64</v>
+        <v>18.4</v>
       </c>
       <c r="AE21" t="n">
-        <v>23.48</v>
+        <v>23.04</v>
       </c>
       <c r="AF21" t="n">
-        <v>3.08</v>
+        <v>11.03</v>
       </c>
       <c r="AG21" t="n">
-        <v>0.51</v>
+        <v>11.41</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2958,7 +2966,7 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.17</v>
+        <v>1.03</v>
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
@@ -2978,31 +2986,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45900.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>21.7</v>
+        <v>28.64</v>
       </c>
       <c r="G22" t="n">
-        <v>21.06</v>
+        <v>28.08</v>
       </c>
       <c r="H22" t="n">
-        <v>21.02</v>
+        <v>27.22</v>
       </c>
       <c r="I22" t="n">
-        <v>-3.13</v>
+        <v>-4.97</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>21.02</v>
+        <v>28</v>
       </c>
       <c r="L22" t="n">
-        <v>21.26</v>
+        <v>28.48</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3015,19 +3023,19 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>811883</v>
+        <v>1546271</v>
       </c>
       <c r="P22" t="n">
-        <v>2.81</v>
+        <v>1.79</v>
       </c>
       <c r="Q22" t="n">
-        <v>21.61</v>
+        <v>28.16</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>21.83</v>
+        <v>29</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
@@ -3036,16 +3044,16 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>0.62</v>
+        <v>1.26</v>
       </c>
       <c r="W22" t="n">
-        <v>-0.4</v>
+        <v>-1.68</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>45900.41666666666</v>
+        <v>45729.41666666666</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -3054,22 +3062,22 @@
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>21.06</v>
+        <v>28.08</v>
       </c>
       <c r="AE22" t="n">
-        <v>21.83</v>
+        <v>29</v>
       </c>
       <c r="AF22" t="n">
-        <v>2.95</v>
+        <v>1.96</v>
       </c>
       <c r="AG22" t="n">
-        <v>0.63</v>
+        <v>1.26</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
@@ -3077,7 +3085,7 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.21</v>
+        <v>0.64</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3097,31 +3105,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>45911.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45972.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>21.51</v>
+        <v>25.97</v>
       </c>
       <c r="G23" t="n">
-        <v>20.27</v>
+        <v>24.72</v>
       </c>
       <c r="H23" t="n">
-        <v>24.94</v>
+        <v>25.2</v>
       </c>
       <c r="I23" t="n">
-        <v>15.94</v>
+        <v>-2.96</v>
       </c>
       <c r="J23" t="n">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="K23" t="n">
-        <v>20.28</v>
+        <v>24.68</v>
       </c>
       <c r="L23" t="n">
-        <v>20.96</v>
+        <v>25.51</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3134,69 +3142,61 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>2694406</v>
+        <v>767605</v>
       </c>
       <c r="P23" t="n">
-        <v>3.42</v>
+        <v>4.04</v>
       </c>
       <c r="Q23" t="n">
-        <v>20.96</v>
+        <v>27.46</v>
       </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>20.96</v>
+        <v>29.03</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
       </c>
       <c r="U23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>-2.57</v>
+        <v>11.79</v>
       </c>
       <c r="W23" t="n">
-        <v>-2.57</v>
+        <v>5.75</v>
       </c>
       <c r="X23" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y23" s="2" t="n">
-        <v>45923.41666666666</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB23" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="n">
-        <v>20.27</v>
+        <v>24.72</v>
       </c>
       <c r="AE23" t="n">
-        <v>22.19</v>
+        <v>29.03</v>
       </c>
       <c r="AF23" t="n">
-        <v>5.76</v>
+        <v>4.81</v>
       </c>
       <c r="AG23" t="n">
-        <v>3.16</v>
+        <v>11.8</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.55</v>
+        <v>2.45</v>
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
@@ -3216,31 +3216,31 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>45994.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>46002.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F24" t="n">
-        <v>23.44</v>
+        <v>25.32</v>
       </c>
       <c r="G24" t="n">
-        <v>22.68</v>
+        <v>24.12</v>
       </c>
       <c r="H24" t="n">
-        <v>23.56</v>
+        <v>23.99</v>
       </c>
       <c r="I24" t="n">
-        <v>0.51</v>
+        <v>-5.24</v>
       </c>
       <c r="J24" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="K24" t="n">
-        <v>22.51</v>
+        <v>24.12</v>
       </c>
       <c r="L24" t="n">
-        <v>23.43</v>
+        <v>25.26</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>2183354</v>
+        <v>623052</v>
       </c>
       <c r="P24" t="n">
-        <v>1.78</v>
+        <v>0.96</v>
       </c>
       <c r="Q24" t="n">
-        <v>23.05</v>
+        <v>26.96</v>
       </c>
       <c r="R24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>24.98</v>
+        <v>26.96</v>
       </c>
       <c r="T24" t="b">
         <v>0</v>
@@ -3274,10 +3274,10 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>6.57</v>
+        <v>6.48</v>
       </c>
       <c r="W24" t="n">
-        <v>-1.66</v>
+        <v>6.48</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3285,25 +3285,21 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB24" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="n">
-        <v>22.68</v>
+        <v>24.12</v>
       </c>
       <c r="AE24" t="n">
-        <v>24.98</v>
+        <v>26.96</v>
       </c>
       <c r="AF24" t="n">
-        <v>3.24</v>
+        <v>4.74</v>
       </c>
       <c r="AG24" t="n">
-        <v>6.57</v>
+        <v>6.48</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
@@ -3311,7 +3307,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>2.03</v>
+        <v>1.37</v>
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
@@ -3331,31 +3327,31 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>46016.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>46027.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F25" t="n">
-        <v>24.6</v>
+        <v>22.75</v>
       </c>
       <c r="G25" t="n">
-        <v>23.75</v>
+        <v>21.66</v>
       </c>
       <c r="H25" t="n">
-        <v>24.41</v>
+        <v>21.65</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.77</v>
+        <v>-4.85</v>
       </c>
       <c r="J25" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="K25" t="n">
-        <v>23.41</v>
+        <v>21.66</v>
       </c>
       <c r="L25" t="n">
-        <v>24.09</v>
+        <v>22.2</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3368,31 +3364,31 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>2756109</v>
+        <v>13689820</v>
       </c>
       <c r="P25" t="n">
-        <v>3.54</v>
+        <v>4.94</v>
       </c>
       <c r="Q25" t="n">
-        <v>24.08</v>
+        <v>23.7</v>
       </c>
       <c r="R25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>24.5</v>
+        <v>25.75</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
       </c>
       <c r="U25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>-0.41</v>
+        <v>13.18</v>
       </c>
       <c r="W25" t="n">
-        <v>-2.11</v>
+        <v>4.17</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -3400,33 +3396,29 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB25" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="n">
-        <v>23.75</v>
+        <v>21.66</v>
       </c>
       <c r="AE25" t="n">
-        <v>25.69</v>
+        <v>25.75</v>
       </c>
       <c r="AF25" t="n">
-        <v>3.46</v>
+        <v>4.78</v>
       </c>
       <c r="AG25" t="n">
-        <v>4.43</v>
+        <v>13.19</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>1.28</v>
+        <v>2.76</v>
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
@@ -3446,31 +3438,31 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>46069.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F26" t="n">
-        <v>26</v>
+        <v>21.88</v>
       </c>
       <c r="G26" t="n">
-        <v>24.3</v>
+        <v>21.35</v>
       </c>
       <c r="H26" t="n">
-        <v>28.5</v>
+        <v>20.53</v>
       </c>
       <c r="I26" t="n">
-        <v>9.619999999999999</v>
+        <v>-6.18</v>
       </c>
       <c r="J26" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="K26" t="n">
-        <v>24.01</v>
+        <v>21.35</v>
       </c>
       <c r="L26" t="n">
-        <v>25.42</v>
+        <v>21.78</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3483,37 +3475,37 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>2965366</v>
+        <v>1476660</v>
       </c>
       <c r="P26" t="n">
-        <v>6.51</v>
+        <v>1.3</v>
       </c>
       <c r="Q26" t="n">
-        <v>25.42</v>
+        <v>21.54</v>
       </c>
       <c r="R26" t="b">
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>25.42</v>
+        <v>22.52</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
       </c>
       <c r="U26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>-2.23</v>
+        <v>2.93</v>
       </c>
       <c r="W26" t="n">
-        <v>-2.23</v>
+        <v>-1.55</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>46033.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z26" t="n">
         <v>2</v>
@@ -3522,30 +3514,30 @@
         <v>1</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>24.3</v>
+        <v>21.35</v>
       </c>
       <c r="AE26" t="n">
-        <v>27.41</v>
+        <v>22.52</v>
       </c>
       <c r="AF26" t="n">
-        <v>6.54</v>
+        <v>2.41</v>
       </c>
       <c r="AG26" t="n">
-        <v>5.42</v>
+        <v>2.93</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>0.83</v>
+        <v>1.22</v>
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
@@ -3565,31 +3557,31 @@
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>46120.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>46139.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>26.61</v>
+        <v>21.16</v>
       </c>
       <c r="G27" t="n">
-        <v>25.21</v>
+        <v>19.2</v>
       </c>
       <c r="H27" t="n">
-        <v>28.7</v>
+        <v>21.32</v>
       </c>
       <c r="I27" t="n">
-        <v>7.85</v>
+        <v>0.76</v>
       </c>
       <c r="J27" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="K27" t="n">
-        <v>23.8</v>
+        <v>19.92</v>
       </c>
       <c r="L27" t="n">
-        <v>25.7</v>
+        <v>20.64</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3602,61 +3594,57 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>2499912</v>
+        <v>5666121</v>
       </c>
       <c r="P27" t="n">
-        <v>4.31</v>
+        <v>4.75</v>
       </c>
       <c r="Q27" t="n">
-        <v>26.8</v>
+        <v>22.02</v>
       </c>
       <c r="R27" t="b">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>26.8</v>
+        <v>22.52</v>
       </c>
       <c r="T27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U27" t="b">
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>0.71</v>
+        <v>6.43</v>
       </c>
       <c r="W27" t="n">
-        <v>0.71</v>
+        <v>4.06</v>
       </c>
       <c r="X27" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y27" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="b">
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>46127.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD27" t="n">
-        <v>25.21</v>
+        <v>19.2</v>
       </c>
       <c r="AE27" t="n">
-        <v>26.8</v>
+        <v>22.52</v>
       </c>
       <c r="AF27" t="n">
-        <v>5.26</v>
+        <v>9.26</v>
       </c>
       <c r="AG27" t="n">
-        <v>0.71</v>
+        <v>6.43</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -3664,10 +3652,954 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.13</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C28" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>45845.41666666666</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>45860.41666666666</v>
+      </c>
+      <c r="F28" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="G28" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="H28" t="n">
+        <v>22.48</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="J28" t="n">
+        <v>15</v>
+      </c>
+      <c r="K28" t="n">
+        <v>21.29</v>
+      </c>
+      <c r="L28" t="n">
+        <v>21.84</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>1366828</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>22.06</v>
+      </c>
+      <c r="R28" t="b">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="T28" t="b">
+        <v>0</v>
+      </c>
+      <c r="U28" t="b">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="X28" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y28" s="2" t="n">
+        <v>45847.41666666666</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB28" s="2" t="n">
+        <v>45847.41666666666</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C29" t="b">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>45872.41666666666</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>45887.41666666666</v>
+      </c>
+      <c r="F29" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="G29" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="H29" t="n">
+        <v>22.81</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-2.36</v>
+      </c>
+      <c r="J29" t="n">
+        <v>15</v>
+      </c>
+      <c r="K29" t="n">
+        <v>22.39</v>
+      </c>
+      <c r="L29" t="n">
+        <v>23.18</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>1011332</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="T29" t="b">
+        <v>0</v>
+      </c>
+      <c r="U29" t="b">
+        <v>0</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="W29" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="X29" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y29" s="2" t="n">
+        <v>45873.41666666666</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA29" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB29" s="2" t="n">
+        <v>45872.41666666666</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AJ29" t="inlineStr"/>
+      <c r="AK29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C30" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>45897.41666666666</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="F30" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="G30" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="H30" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-3.13</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="L30" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>811883</v>
+      </c>
+      <c r="P30" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="T30" t="b">
+        <v>0</v>
+      </c>
+      <c r="U30" t="b">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="W30" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="X30" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y30" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA30" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB30" s="2" t="n">
+        <v>45897.41666666666</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C31" t="b">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>45972.41666666666</v>
+      </c>
+      <c r="F31" t="n">
+        <v>21.51</v>
+      </c>
+      <c r="G31" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="H31" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="I31" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="J31" t="n">
+        <v>61</v>
+      </c>
+      <c r="K31" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="L31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>2694406</v>
+      </c>
+      <c r="P31" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="T31" t="b">
+        <v>0</v>
+      </c>
+      <c r="U31" t="b">
+        <v>1</v>
+      </c>
+      <c r="V31" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="W31" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="X31" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA31" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB31" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ31" t="inlineStr"/>
+      <c r="AK31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>46002.41666666666</v>
+      </c>
+      <c r="F32" t="n">
+        <v>23.44</v>
+      </c>
+      <c r="G32" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="H32" t="n">
+        <v>23.56</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J32" t="n">
+        <v>8</v>
+      </c>
+      <c r="K32" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="L32" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>2183354</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>22.87</v>
+      </c>
+      <c r="R32" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="T32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V32" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="W32" t="n">
+        <v>-2.43</v>
+      </c>
+      <c r="X32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB32" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AJ32" t="inlineStr"/>
+      <c r="AK32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C33" t="b">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>46027.41666666666</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G33" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="H33" t="n">
+        <v>24.41</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="J33" t="n">
+        <v>11</v>
+      </c>
+      <c r="K33" t="n">
+        <v>23.41</v>
+      </c>
+      <c r="L33" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O33" t="n">
+        <v>2756109</v>
+      </c>
+      <c r="P33" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>24.08</v>
+      </c>
+      <c r="R33" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="T33" t="b">
+        <v>0</v>
+      </c>
+      <c r="U33" t="b">
+        <v>1</v>
+      </c>
+      <c r="V33" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="W33" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="X33" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB33" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="AJ33" t="inlineStr"/>
+      <c r="AK33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>46069.41666666666</v>
+      </c>
+      <c r="F34" t="n">
+        <v>26</v>
+      </c>
+      <c r="G34" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I34" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="J34" t="n">
+        <v>41</v>
+      </c>
+      <c r="K34" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="L34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>2965366</v>
+      </c>
+      <c r="P34" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="R34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="T34" t="b">
+        <v>0</v>
+      </c>
+      <c r="U34" t="b">
+        <v>1</v>
+      </c>
+      <c r="V34" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="W34" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="X34" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="2" t="n">
+        <v>46033.41666666666</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA34" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI34" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AJ34" t="inlineStr"/>
+      <c r="AK34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C35" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>46139.41666666666</v>
+      </c>
+      <c r="F35" t="n">
+        <v>26.61</v>
+      </c>
+      <c r="G35" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="I35" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="J35" t="n">
+        <v>19</v>
+      </c>
+      <c r="K35" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="L35" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>2499912</v>
+      </c>
+      <c r="P35" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>25.73</v>
+      </c>
+      <c r="R35" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="T35" t="b">
+        <v>1</v>
+      </c>
+      <c r="U35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="W35" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="X35" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI35" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3885,31 +4817,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>53.91</v>
+        <v>47.87</v>
       </c>
       <c r="G2" t="n">
-        <v>43.72</v>
+        <v>46</v>
       </c>
       <c r="H2" t="n">
         <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>235.74</v>
+        <v>278.11</v>
       </c>
       <c r="J2" t="n">
-        <v>593</v>
+        <v>384</v>
       </c>
       <c r="K2" t="n">
-        <v>43.03</v>
+        <v>45</v>
       </c>
       <c r="L2" t="n">
-        <v>45.91</v>
+        <v>46.89</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -3922,69 +4854,69 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>128396</v>
+        <v>47815</v>
       </c>
       <c r="P2" t="n">
-        <v>19.99</v>
+        <v>2.73</v>
       </c>
       <c r="Q2" t="n">
-        <v>45.33</v>
+        <v>46.62</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>48.75</v>
+        <v>51</v>
       </c>
       <c r="T2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>-9.57</v>
+        <v>6.54</v>
       </c>
       <c r="W2" t="n">
-        <v>-15.92</v>
+        <v>-2.61</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45547.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="Z2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>43.72</v>
+        <v>46</v>
       </c>
       <c r="AE2" t="n">
-        <v>59.63</v>
+        <v>51</v>
       </c>
       <c r="AF2" t="n">
-        <v>18.9</v>
+        <v>3.91</v>
       </c>
       <c r="AG2" t="n">
-        <v>10.61</v>
+        <v>6.54</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.67</v>
       </c>
       <c r="AJ2" t="n">
         <v>181</v>
@@ -4126,25 +5058,25 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>66.67</v>
+        <v>27.27</v>
       </c>
       <c r="G2" t="n">
-        <v>1.19</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.58</v>
+        <v>-25.44</v>
       </c>
       <c r="J2" t="n">
         <v>12.48</v>
@@ -4153,28 +5085,28 @@
         <v>-14.25</v>
       </c>
       <c r="L2" t="n">
-        <v>13.42</v>
+        <v>7.68</v>
       </c>
       <c r="M2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="N2" t="n">
-        <v>6.84</v>
+        <v>7.98</v>
       </c>
       <c r="O2" t="n">
-        <v>14.25</v>
+        <v>6.17</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.2320120319001387</v>
+        <v>0.1209768433179723</v>
       </c>
       <c r="R2" t="n">
-        <v>0.09086</v>
+        <v>-0.09292000000000003</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1473208127600555</v>
+        <v>-0.007361262672811078</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -4182,7 +5114,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.1473208127600555</v>
+        <v>-0.007361262672811078</v>
       </c>
     </row>
     <row r="3">
@@ -4212,10 +5144,10 @@
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
       <c r="I3" t="n">
-        <v>59.34</v>
+        <v>63.34</v>
       </c>
       <c r="J3" t="n">
         <v>38.41</v>
@@ -4224,28 +5156,28 @@
         <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>10.64</v>
+        <v>10.51</v>
       </c>
       <c r="M3" t="n">
-        <v>2.13</v>
+        <v>2.31</v>
       </c>
       <c r="N3" t="n">
         <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>4.76</v>
+        <v>4.39</v>
       </c>
       <c r="P3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5084026632302405</v>
+        <v>0.5176452432667247</v>
       </c>
       <c r="R3" t="n">
-        <v>0.49842</v>
+        <v>0.51042</v>
       </c>
       <c r="S3" t="n">
-        <v>0.5024130652920962</v>
+        <v>0.5133100973066899</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -4253,7 +5185,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.5024130652920962</v>
+        <v>0.5133100973066899</v>
       </c>
     </row>
   </sheetData>
@@ -4324,22 +5256,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.15</v>
+        <v>-0.01</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>66.67</v>
+        <v>27.27</v>
       </c>
       <c r="F2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="G2" t="n">
-        <v>1.19</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
     </row>
     <row r="3">
@@ -4354,7 +5286,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="D3" t="n">
         <v>23</v>
@@ -4363,13 +5295,13 @@
         <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>2.13</v>
+        <v>2.31</v>
       </c>
       <c r="G3" t="n">
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:41:02.741810
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK35"/>
+  <dimension ref="A1:AK27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,7 +983,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -992,101 +992,101 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45554.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>53.91</v>
+        <v>13.43</v>
       </c>
       <c r="G5" t="n">
-        <v>43.72</v>
+        <v>12.66</v>
       </c>
       <c r="H5" t="n">
-        <v>51.11</v>
+        <v>13.26</v>
       </c>
       <c r="I5" t="n">
-        <v>-5.19</v>
+        <v>-1.25</v>
       </c>
       <c r="J5" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="L5" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>3180532</v>
+      </c>
+      <c r="P5" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>12.98</v>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+      <c r="V5" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="W5" t="n">
+        <v>-3.37</v>
+      </c>
+      <c r="X5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>45313.41666666666</v>
+      </c>
+      <c r="Z5" t="n">
         <v>8</v>
       </c>
-      <c r="K5" t="n">
-        <v>43.03</v>
-      </c>
-      <c r="L5" t="n">
-        <v>45.91</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>128396</v>
-      </c>
-      <c r="P5" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>45.33</v>
-      </c>
-      <c r="R5" t="b">
-        <v>1</v>
-      </c>
-      <c r="S5" t="n">
-        <v>48.75</v>
-      </c>
-      <c r="T5" t="b">
-        <v>0</v>
-      </c>
-      <c r="U5" t="b">
-        <v>1</v>
-      </c>
-      <c r="V5" t="n">
-        <v>-9.57</v>
-      </c>
-      <c r="W5" t="n">
-        <v>-15.92</v>
-      </c>
-      <c r="X5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y5" s="2" t="n">
-        <v>45547.41666666666</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1</v>
-      </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>43.72</v>
+        <v>12.66</v>
       </c>
       <c r="AE5" t="n">
-        <v>59.63</v>
+        <v>14.32</v>
       </c>
       <c r="AF5" t="n">
-        <v>18.9</v>
+        <v>5.78</v>
       </c>
       <c r="AG5" t="n">
-        <v>10.61</v>
+        <v>6.61</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.14</v>
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1111,34 +1111,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45558.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45567.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>53.48</v>
+        <v>15.59</v>
       </c>
       <c r="G6" t="n">
-        <v>50.18</v>
+        <v>13.66</v>
       </c>
       <c r="H6" t="n">
-        <v>49.83</v>
+        <v>16</v>
       </c>
       <c r="I6" t="n">
-        <v>-6.82</v>
+        <v>2.62</v>
       </c>
       <c r="J6" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="K6" t="n">
-        <v>50.18</v>
+        <v>12.64</v>
       </c>
       <c r="L6" t="n">
-        <v>52.39</v>
+        <v>14.56</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1151,65 +1151,69 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>188748</v>
+        <v>708583</v>
       </c>
       <c r="P6" t="n">
-        <v>4.9</v>
+        <v>10.05</v>
       </c>
       <c r="Q6" t="n">
-        <v>50.5</v>
+        <v>13.78</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>61.85</v>
+        <v>15.04</v>
       </c>
       <c r="T6" t="b">
         <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>15.65</v>
+        <v>-3.54</v>
       </c>
       <c r="W6" t="n">
-        <v>-5.57</v>
+        <v>-11.62</v>
       </c>
       <c r="X6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>45336.41666666666</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>8</v>
+      </c>
       <c r="AA6" t="b">
         <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>45558.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>50.18</v>
+        <v>13.66</v>
       </c>
       <c r="AE6" t="n">
-        <v>61.85</v>
+        <v>17.99</v>
       </c>
       <c r="AF6" t="n">
-        <v>6.17</v>
+        <v>12.37</v>
       </c>
       <c r="AG6" t="n">
-        <v>15.65</v>
+        <v>15.39</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>2.54</v>
+        <v>1.24</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1217,7 +1221,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1229,31 +1233,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45594.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45601.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>54</v>
+        <v>15.92</v>
       </c>
       <c r="G7" t="n">
-        <v>52.01</v>
+        <v>14.54</v>
       </c>
       <c r="H7" t="n">
-        <v>52</v>
+        <v>14.11</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.7</v>
+        <v>-11.36</v>
       </c>
       <c r="J7" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>44</v>
+        <v>14.54</v>
       </c>
       <c r="L7" t="n">
-        <v>53.95</v>
+        <v>15.68</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1266,57 +1270,61 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>36571</v>
+        <v>2359660</v>
       </c>
       <c r="P7" t="n">
-        <v>3.41</v>
+        <v>3.65</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.51</v>
+        <v>15.3</v>
       </c>
       <c r="R7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>57.99</v>
+        <v>16.22</v>
       </c>
       <c r="T7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>7.39</v>
+        <v>1.88</v>
       </c>
       <c r="W7" t="n">
-        <v>0.9399999999999999</v>
+        <v>-3.89</v>
       </c>
       <c r="X7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45599.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD7" t="n">
-        <v>52.01</v>
+        <v>14.54</v>
       </c>
       <c r="AE7" t="n">
-        <v>57.99</v>
+        <v>16.22</v>
       </c>
       <c r="AF7" t="n">
-        <v>3.69</v>
+        <v>8.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>7.39</v>
+        <v>1.91</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1324,7 +1332,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>2</v>
+        <v>0.22</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1332,7 +1340,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1344,31 +1352,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45603.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45608.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>54.34</v>
+        <v>13.08</v>
       </c>
       <c r="G8" t="n">
-        <v>52.65</v>
+        <v>12.76</v>
       </c>
       <c r="H8" t="n">
-        <v>51.7</v>
+        <v>12.39</v>
       </c>
       <c r="I8" t="n">
-        <v>-4.86</v>
+        <v>-5.26</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>51.6</v>
+        <v>12.22</v>
       </c>
       <c r="L8" t="n">
-        <v>54.24</v>
+        <v>13.04</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1381,19 +1389,19 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>18287</v>
+        <v>5618577</v>
       </c>
       <c r="P8" t="n">
-        <v>0.6899999999999999</v>
+        <v>2.06</v>
       </c>
       <c r="Q8" t="n">
-        <v>53.58</v>
+        <v>12.72</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>57.84</v>
+        <v>14.15</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
@@ -1402,10 +1410,10 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>6.44</v>
+        <v>8.18</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.4</v>
+        <v>-2.75</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1416,22 +1424,22 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45603.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>52.65</v>
+        <v>12.76</v>
       </c>
       <c r="AE8" t="n">
-        <v>57.84</v>
+        <v>14.15</v>
       </c>
       <c r="AF8" t="n">
-        <v>3.11</v>
+        <v>2.45</v>
       </c>
       <c r="AG8" t="n">
-        <v>6.44</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1439,7 +1447,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>2.07</v>
+        <v>3.35</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
@@ -1447,7 +1455,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1459,31 +1467,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45624.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45669.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>49.88</v>
+        <v>11.44</v>
       </c>
       <c r="G9" t="n">
-        <v>47.93</v>
+        <v>10.23</v>
       </c>
       <c r="H9" t="n">
-        <v>55</v>
+        <v>11.76</v>
       </c>
       <c r="I9" t="n">
-        <v>10.26</v>
+        <v>2.8</v>
       </c>
       <c r="J9" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="K9" t="n">
-        <v>48</v>
+        <v>10.01</v>
       </c>
       <c r="L9" t="n">
-        <v>49.58</v>
+        <v>11.2</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1496,19 +1504,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>431</v>
+        <v>3697242</v>
       </c>
       <c r="P9" t="n">
-        <v>1.14</v>
+        <v>10</v>
       </c>
       <c r="Q9" t="n">
-        <v>51.55</v>
+        <v>13.1</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>51.55</v>
+        <v>13.42</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1517,40 +1525,32 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>3.35</v>
+        <v>17.31</v>
       </c>
       <c r="W9" t="n">
-        <v>3.35</v>
+        <v>14.51</v>
       </c>
       <c r="X9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="2" t="n">
-        <v>45631.41666666666</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB9" s="2" t="n">
-        <v>45631.41666666666</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
-        <v>47.93</v>
+        <v>10.23</v>
       </c>
       <c r="AE9" t="n">
-        <v>51.55</v>
+        <v>13.42</v>
       </c>
       <c r="AF9" t="n">
-        <v>3.91</v>
+        <v>10.56</v>
       </c>
       <c r="AG9" t="n">
-        <v>3.35</v>
+        <v>17.34</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.86</v>
+        <v>1.64</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1566,7 +1566,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1578,31 +1578,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45704.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45714.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>47.99</v>
+        <v>12.1</v>
       </c>
       <c r="G10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="H10" t="n">
-        <v>45.81</v>
+        <v>12.4</v>
       </c>
       <c r="I10" t="n">
-        <v>-4.54</v>
+        <v>2.51</v>
       </c>
       <c r="J10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="L10" t="n">
-        <v>47.97</v>
+        <v>12.08</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1615,19 +1615,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>6897</v>
+        <v>719120</v>
       </c>
       <c r="P10" t="n">
-        <v>3.61</v>
+        <v>2.86</v>
       </c>
       <c r="Q10" t="n">
-        <v>48.54</v>
+        <v>11.92</v>
       </c>
       <c r="R10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>50.25</v>
+        <v>12.39</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1636,32 +1636,40 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>4.71</v>
+        <v>2.43</v>
       </c>
       <c r="W10" t="n">
-        <v>1.15</v>
+        <v>-1.46</v>
       </c>
       <c r="X10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y10" s="2" t="n">
+        <v>45426.41666666666</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1</v>
+      </c>
       <c r="AA10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB10" s="2" t="n">
+        <v>45425.41666666666</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
       <c r="AD10" t="n">
-        <v>46</v>
+        <v>11.68</v>
       </c>
       <c r="AE10" t="n">
-        <v>50.25</v>
+        <v>12.39</v>
       </c>
       <c r="AF10" t="n">
-        <v>4.15</v>
+        <v>3.44</v>
       </c>
       <c r="AG10" t="n">
-        <v>4.71</v>
+        <v>2.45</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -1669,7 +1677,7 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>1.13</v>
+        <v>0.71</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1677,7 +1685,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1689,31 +1697,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45727.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>47.51</v>
+        <v>13.23</v>
       </c>
       <c r="G11" t="n">
-        <v>45.8</v>
+        <v>12.37</v>
       </c>
       <c r="H11" t="n">
-        <v>45.63</v>
+        <v>15.11</v>
       </c>
       <c r="I11" t="n">
-        <v>-3.96</v>
+        <v>14.21</v>
       </c>
       <c r="J11" t="n">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="K11" t="n">
-        <v>45.81</v>
+        <v>12.37</v>
       </c>
       <c r="L11" t="n">
-        <v>46.58</v>
+        <v>12.68</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1726,19 +1734,19 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>31257</v>
+        <v>2872871</v>
       </c>
       <c r="P11" t="n">
-        <v>3.04</v>
+        <v>4.75</v>
       </c>
       <c r="Q11" t="n">
-        <v>46.46</v>
+        <v>12.61</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>46.7</v>
+        <v>13.12</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -1747,40 +1755,40 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.7</v>
+        <v>-0.85</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.21</v>
+        <v>-4.7</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45454.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>45.8</v>
+        <v>12.37</v>
       </c>
       <c r="AE11" t="n">
-        <v>48.4</v>
+        <v>13.98</v>
       </c>
       <c r="AF11" t="n">
-        <v>3.6</v>
+        <v>6.53</v>
       </c>
       <c r="AG11" t="n">
-        <v>1.87</v>
+        <v>5.68</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -1788,7 +1796,7 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.52</v>
+        <v>0.87</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1796,7 +1804,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AALR</t>
+          <t>JUFO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1808,31 +1816,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45754.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>48.44</v>
+        <v>17.1</v>
       </c>
       <c r="G12" t="n">
-        <v>45.88</v>
+        <v>14.96</v>
       </c>
       <c r="H12" t="n">
-        <v>45.51</v>
+        <v>19.46</v>
       </c>
       <c r="I12" t="n">
-        <v>-6.05</v>
+        <v>13.85</v>
       </c>
       <c r="J12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K12" t="n">
-        <v>45.6</v>
+        <v>14.96</v>
       </c>
       <c r="L12" t="n">
-        <v>46.75</v>
+        <v>15.28</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1845,19 +1853,19 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>49292</v>
+        <v>2885185</v>
       </c>
       <c r="P12" t="n">
-        <v>5.14</v>
+        <v>13.79</v>
       </c>
       <c r="Q12" t="n">
-        <v>46.73</v>
+        <v>15.44</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>46.75</v>
+        <v>15.5</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1866,40 +1874,40 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.49</v>
+        <v>-9.34</v>
       </c>
       <c r="W12" t="n">
-        <v>-3.53</v>
+        <v>-9.69</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>45734.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="Z12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>45.88</v>
+        <v>14.96</v>
       </c>
       <c r="AE12" t="n">
-        <v>49.59</v>
+        <v>17.64</v>
       </c>
       <c r="AF12" t="n">
-        <v>5.28</v>
+        <v>12.49</v>
       </c>
       <c r="AG12" t="n">
-        <v>2.37</v>
+        <v>3.18</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1907,7 +1915,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1924,34 +1932,34 @@
         </is>
       </c>
       <c r="C13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45322.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>13.43</v>
+        <v>20.68</v>
       </c>
       <c r="G13" t="n">
-        <v>12.66</v>
+        <v>18.4</v>
       </c>
       <c r="H13" t="n">
-        <v>13.26</v>
+        <v>28.62</v>
       </c>
       <c r="I13" t="n">
-        <v>-1.25</v>
+        <v>38.41</v>
       </c>
       <c r="J13" t="n">
-        <v>21</v>
+        <v>185</v>
       </c>
       <c r="K13" t="n">
-        <v>12.54</v>
+        <v>18.4</v>
       </c>
       <c r="L13" t="n">
-        <v>13.42</v>
+        <v>20.24</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1964,69 +1972,69 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>3180532</v>
+        <v>807277</v>
       </c>
       <c r="P13" t="n">
-        <v>3.32</v>
+        <v>2.17</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.98</v>
+        <v>20.54</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>13.42</v>
+        <v>23.04</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.09</v>
+        <v>11.41</v>
       </c>
       <c r="W13" t="n">
-        <v>-3.37</v>
+        <v>-0.68</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45313.41666666666</v>
+        <v>45572.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>12.66</v>
+        <v>18.4</v>
       </c>
       <c r="AE13" t="n">
-        <v>14.32</v>
+        <v>23.04</v>
       </c>
       <c r="AF13" t="n">
-        <v>5.78</v>
+        <v>11.03</v>
       </c>
       <c r="AG13" t="n">
-        <v>6.61</v>
+        <v>11.41</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.14</v>
+        <v>1.03</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2043,34 +2051,34 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>15.59</v>
+        <v>28.64</v>
       </c>
       <c r="G14" t="n">
-        <v>13.66</v>
+        <v>28.08</v>
       </c>
       <c r="H14" t="n">
-        <v>16</v>
+        <v>27.22</v>
       </c>
       <c r="I14" t="n">
-        <v>2.62</v>
+        <v>-4.97</v>
       </c>
       <c r="J14" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>12.64</v>
+        <v>28</v>
       </c>
       <c r="L14" t="n">
-        <v>14.56</v>
+        <v>28.48</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2083,69 +2091,69 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>708583</v>
+        <v>1546271</v>
       </c>
       <c r="P14" t="n">
-        <v>10.05</v>
+        <v>1.79</v>
       </c>
       <c r="Q14" t="n">
-        <v>13.78</v>
+        <v>28.16</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>15.04</v>
+        <v>29</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.54</v>
+        <v>1.26</v>
       </c>
       <c r="W14" t="n">
-        <v>-11.62</v>
+        <v>-1.68</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>45336.41666666666</v>
+        <v>45729.41666666666</v>
       </c>
       <c r="Z14" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>13.66</v>
+        <v>28.08</v>
       </c>
       <c r="AE14" t="n">
-        <v>17.99</v>
+        <v>29</v>
       </c>
       <c r="AF14" t="n">
-        <v>12.37</v>
+        <v>1.96</v>
       </c>
       <c r="AG14" t="n">
-        <v>15.39</v>
+        <v>1.26</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>1.24</v>
+        <v>0.64</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2165,31 +2173,31 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45379.41666666666</v>
+        <v>45756.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>15.92</v>
+        <v>25.97</v>
       </c>
       <c r="G15" t="n">
-        <v>14.54</v>
+        <v>24.72</v>
       </c>
       <c r="H15" t="n">
-        <v>14.11</v>
+        <v>24.16</v>
       </c>
       <c r="I15" t="n">
-        <v>-11.36</v>
+        <v>-6.96</v>
       </c>
       <c r="J15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K15" t="n">
-        <v>14.54</v>
+        <v>24.68</v>
       </c>
       <c r="L15" t="n">
-        <v>15.68</v>
+        <v>25.51</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2202,61 +2210,53 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>2359660</v>
+        <v>767605</v>
       </c>
       <c r="P15" t="n">
-        <v>3.65</v>
+        <v>4.04</v>
       </c>
       <c r="Q15" t="n">
-        <v>15.3</v>
+        <v>27.46</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>16.22</v>
+        <v>29.03</v>
       </c>
       <c r="T15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15" t="b">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>1.88</v>
+        <v>11.79</v>
       </c>
       <c r="W15" t="n">
-        <v>-3.89</v>
+        <v>5.75</v>
       </c>
       <c r="X15" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y15" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB15" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="n">
-        <v>14.54</v>
+        <v>24.72</v>
       </c>
       <c r="AE15" t="n">
-        <v>16.22</v>
+        <v>29.03</v>
       </c>
       <c r="AF15" t="n">
-        <v>8.69</v>
+        <v>4.81</v>
       </c>
       <c r="AG15" t="n">
-        <v>1.91</v>
+        <v>11.8</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.22</v>
+        <v>2.45</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2284,31 +2284,31 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>13.08</v>
+        <v>25.32</v>
       </c>
       <c r="G16" t="n">
-        <v>12.76</v>
+        <v>24.12</v>
       </c>
       <c r="H16" t="n">
-        <v>12.39</v>
+        <v>23.99</v>
       </c>
       <c r="I16" t="n">
-        <v>-5.26</v>
+        <v>-5.24</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K16" t="n">
-        <v>12.22</v>
+        <v>24.12</v>
       </c>
       <c r="L16" t="n">
-        <v>13.04</v>
+        <v>25.26</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>5618577</v>
+        <v>623052</v>
       </c>
       <c r="P16" t="n">
-        <v>2.06</v>
+        <v>0.96</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.72</v>
+        <v>26.96</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>14.15</v>
+        <v>26.96</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2342,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>8.18</v>
+        <v>6.48</v>
       </c>
       <c r="W16" t="n">
-        <v>-2.75</v>
+        <v>6.48</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -2353,25 +2353,21 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB16" s="2" t="n">
-        <v>45398.41666666666</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="n">
-        <v>12.76</v>
+        <v>24.12</v>
       </c>
       <c r="AE16" t="n">
-        <v>14.15</v>
+        <v>26.96</v>
       </c>
       <c r="AF16" t="n">
-        <v>2.45</v>
+        <v>4.74</v>
       </c>
       <c r="AG16" t="n">
-        <v>8.199999999999999</v>
+        <v>6.48</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2379,7 +2375,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>3.35</v>
+        <v>1.37</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2399,31 +2395,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>11.44</v>
+        <v>22.75</v>
       </c>
       <c r="G17" t="n">
-        <v>10.23</v>
+        <v>21.66</v>
       </c>
       <c r="H17" t="n">
-        <v>11.76</v>
+        <v>21.65</v>
       </c>
       <c r="I17" t="n">
-        <v>2.8</v>
+        <v>-4.85</v>
       </c>
       <c r="J17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K17" t="n">
-        <v>10.01</v>
+        <v>21.66</v>
       </c>
       <c r="L17" t="n">
-        <v>11.2</v>
+        <v>22.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2436,19 +2432,19 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>3697242</v>
+        <v>13689820</v>
       </c>
       <c r="P17" t="n">
-        <v>10</v>
+        <v>4.94</v>
       </c>
       <c r="Q17" t="n">
-        <v>13.1</v>
+        <v>23.7</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>13.42</v>
+        <v>25.75</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -2457,10 +2453,10 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>17.31</v>
+        <v>13.18</v>
       </c>
       <c r="W17" t="n">
-        <v>14.51</v>
+        <v>4.17</v>
       </c>
       <c r="X17" t="b">
         <v>0</v>
@@ -2473,16 +2469,16 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>10.23</v>
+        <v>21.66</v>
       </c>
       <c r="AE17" t="n">
-        <v>13.42</v>
+        <v>25.75</v>
       </c>
       <c r="AF17" t="n">
-        <v>10.56</v>
+        <v>4.78</v>
       </c>
       <c r="AG17" t="n">
-        <v>17.34</v>
+        <v>13.19</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2490,7 +2486,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>1.64</v>
+        <v>2.76</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2510,31 +2506,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45434.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>12.1</v>
+        <v>21.88</v>
       </c>
       <c r="G18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="H18" t="n">
-        <v>12.4</v>
+        <v>20.53</v>
       </c>
       <c r="I18" t="n">
-        <v>2.51</v>
+        <v>-6.18</v>
       </c>
       <c r="J18" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="L18" t="n">
-        <v>12.08</v>
+        <v>21.78</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2547,19 +2543,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>719120</v>
+        <v>1476660</v>
       </c>
       <c r="P18" t="n">
-        <v>2.86</v>
+        <v>1.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.92</v>
+        <v>21.54</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>12.39</v>
+        <v>22.52</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2568,40 +2564,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>2.43</v>
+        <v>2.93</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.46</v>
+        <v>-1.55</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>45426.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>11.68</v>
+        <v>21.35</v>
       </c>
       <c r="AE18" t="n">
-        <v>12.39</v>
+        <v>22.52</v>
       </c>
       <c r="AF18" t="n">
-        <v>3.44</v>
+        <v>2.41</v>
       </c>
       <c r="AG18" t="n">
-        <v>2.45</v>
+        <v>2.93</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2609,7 +2605,7 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.71</v>
+        <v>1.22</v>
       </c>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
@@ -2629,31 +2625,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>13.23</v>
+        <v>21.16</v>
       </c>
       <c r="G19" t="n">
-        <v>12.37</v>
+        <v>19.2</v>
       </c>
       <c r="H19" t="n">
-        <v>15.11</v>
+        <v>21.32</v>
       </c>
       <c r="I19" t="n">
-        <v>14.21</v>
+        <v>0.76</v>
       </c>
       <c r="J19" t="n">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="K19" t="n">
-        <v>12.37</v>
+        <v>19.92</v>
       </c>
       <c r="L19" t="n">
-        <v>12.68</v>
+        <v>20.64</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2666,69 +2662,65 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>2872871</v>
+        <v>5666121</v>
       </c>
       <c r="P19" t="n">
         <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>12.61</v>
+        <v>22.02</v>
       </c>
       <c r="R19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>13.12</v>
+        <v>22.52</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
       </c>
       <c r="U19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.85</v>
+        <v>6.43</v>
       </c>
       <c r="W19" t="n">
-        <v>-4.7</v>
+        <v>4.06</v>
       </c>
       <c r="X19" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="2" t="n">
-        <v>45454.41666666666</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD19" t="n">
-        <v>12.37</v>
+        <v>19.2</v>
       </c>
       <c r="AE19" t="n">
-        <v>13.98</v>
+        <v>22.52</v>
       </c>
       <c r="AF19" t="n">
-        <v>6.53</v>
+        <v>9.26</v>
       </c>
       <c r="AG19" t="n">
-        <v>5.68</v>
+        <v>6.43</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.87</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
@@ -2748,31 +2740,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45845.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45860.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>17.1</v>
+        <v>21.91</v>
       </c>
       <c r="G20" t="n">
-        <v>14.96</v>
+        <v>21.28</v>
       </c>
       <c r="H20" t="n">
-        <v>19.46</v>
+        <v>22.48</v>
       </c>
       <c r="I20" t="n">
-        <v>13.85</v>
+        <v>2.59</v>
       </c>
       <c r="J20" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="K20" t="n">
-        <v>14.96</v>
+        <v>21.29</v>
       </c>
       <c r="L20" t="n">
-        <v>15.28</v>
+        <v>21.84</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2785,69 +2777,69 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>2885185</v>
+        <v>1366828</v>
       </c>
       <c r="P20" t="n">
-        <v>13.79</v>
+        <v>1.44</v>
       </c>
       <c r="Q20" t="n">
-        <v>15.44</v>
+        <v>22.06</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>15.5</v>
+        <v>22.44</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20" t="n">
-        <v>-9.34</v>
+        <v>2.41</v>
       </c>
       <c r="W20" t="n">
-        <v>-9.69</v>
+        <v>0.68</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="Z20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45847.41666666666</v>
       </c>
       <c r="AC20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD20" t="n">
-        <v>14.96</v>
+        <v>21.28</v>
       </c>
       <c r="AE20" t="n">
-        <v>17.64</v>
+        <v>22.44</v>
       </c>
       <c r="AF20" t="n">
-        <v>12.49</v>
+        <v>2.88</v>
       </c>
       <c r="AG20" t="n">
-        <v>3.18</v>
+        <v>2.41</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.25</v>
+        <v>0.84</v>
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
@@ -2867,31 +2859,31 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45887.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>20.68</v>
+        <v>23.36</v>
       </c>
       <c r="G21" t="n">
-        <v>18.4</v>
+        <v>22.64</v>
       </c>
       <c r="H21" t="n">
-        <v>28.62</v>
+        <v>22.81</v>
       </c>
       <c r="I21" t="n">
-        <v>38.41</v>
+        <v>-2.36</v>
       </c>
       <c r="J21" t="n">
-        <v>185</v>
+        <v>15</v>
       </c>
       <c r="K21" t="n">
-        <v>18.4</v>
+        <v>22.39</v>
       </c>
       <c r="L21" t="n">
-        <v>20.24</v>
+        <v>23.18</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2904,19 +2896,19 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>807277</v>
+        <v>1011332</v>
       </c>
       <c r="P21" t="n">
-        <v>2.17</v>
+        <v>1.74</v>
       </c>
       <c r="Q21" t="n">
-        <v>20.54</v>
+        <v>23.12</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>23.04</v>
+        <v>23.48</v>
       </c>
       <c r="T21" t="b">
         <v>0</v>
@@ -2925,40 +2917,40 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>11.41</v>
+        <v>0.51</v>
       </c>
       <c r="W21" t="n">
-        <v>-0.68</v>
+        <v>-1.03</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45572.41666666666</v>
+        <v>45873.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45872.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>18.4</v>
+        <v>22.64</v>
       </c>
       <c r="AE21" t="n">
-        <v>23.04</v>
+        <v>23.48</v>
       </c>
       <c r="AF21" t="n">
-        <v>11.03</v>
+        <v>3.08</v>
       </c>
       <c r="AG21" t="n">
-        <v>11.41</v>
+        <v>0.51</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2966,7 +2958,7 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>1.03</v>
+        <v>0.17</v>
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
@@ -2986,31 +2978,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>28.64</v>
+        <v>21.7</v>
       </c>
       <c r="G22" t="n">
-        <v>28.08</v>
+        <v>21.06</v>
       </c>
       <c r="H22" t="n">
-        <v>27.22</v>
+        <v>21.02</v>
       </c>
       <c r="I22" t="n">
-        <v>-4.97</v>
+        <v>-3.13</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>28</v>
+        <v>21.02</v>
       </c>
       <c r="L22" t="n">
-        <v>28.48</v>
+        <v>21.26</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3023,19 +3015,19 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>1546271</v>
+        <v>811883</v>
       </c>
       <c r="P22" t="n">
-        <v>1.79</v>
+        <v>2.81</v>
       </c>
       <c r="Q22" t="n">
-        <v>28.16</v>
+        <v>21.61</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>29</v>
+        <v>21.83</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
@@ -3044,16 +3036,16 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>1.26</v>
+        <v>0.62</v>
       </c>
       <c r="W22" t="n">
-        <v>-1.68</v>
+        <v>-0.4</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45900.41666666666</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -3062,22 +3054,22 @@
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45897.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>28.08</v>
+        <v>21.06</v>
       </c>
       <c r="AE22" t="n">
-        <v>29</v>
+        <v>21.83</v>
       </c>
       <c r="AF22" t="n">
-        <v>1.96</v>
+        <v>2.95</v>
       </c>
       <c r="AG22" t="n">
-        <v>1.26</v>
+        <v>0.63</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
@@ -3085,7 +3077,7 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.64</v>
+        <v>0.21</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3105,31 +3097,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45911.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45754.41666666666</v>
+        <v>45972.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>25.97</v>
+        <v>21.51</v>
       </c>
       <c r="G23" t="n">
-        <v>24.72</v>
+        <v>20.27</v>
       </c>
       <c r="H23" t="n">
-        <v>25.2</v>
+        <v>24.94</v>
       </c>
       <c r="I23" t="n">
-        <v>-2.96</v>
+        <v>15.94</v>
       </c>
       <c r="J23" t="n">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="K23" t="n">
-        <v>24.68</v>
+        <v>20.28</v>
       </c>
       <c r="L23" t="n">
-        <v>25.51</v>
+        <v>20.96</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3142,61 +3134,69 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>767605</v>
+        <v>2694406</v>
       </c>
       <c r="P23" t="n">
-        <v>4.04</v>
+        <v>3.42</v>
       </c>
       <c r="Q23" t="n">
-        <v>27.46</v>
+        <v>20.96</v>
       </c>
       <c r="R23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>29.03</v>
+        <v>20.96</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
       </c>
       <c r="U23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V23" t="n">
-        <v>11.79</v>
+        <v>-2.57</v>
       </c>
       <c r="W23" t="n">
-        <v>5.75</v>
+        <v>-2.57</v>
       </c>
       <c r="X23" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y23" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>8</v>
+      </c>
       <c r="AA23" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB23" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>0</v>
+      </c>
       <c r="AD23" t="n">
-        <v>24.72</v>
+        <v>20.27</v>
       </c>
       <c r="AE23" t="n">
-        <v>29.03</v>
+        <v>22.19</v>
       </c>
       <c r="AF23" t="n">
-        <v>4.81</v>
+        <v>5.76</v>
       </c>
       <c r="AG23" t="n">
-        <v>11.8</v>
+        <v>3.16</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>2.45</v>
+        <v>0.55</v>
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
@@ -3216,31 +3216,31 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45994.41666666666</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>45783.41666666666</v>
+        <v>46002.41666666666</v>
       </c>
       <c r="F24" t="n">
-        <v>25.32</v>
+        <v>23.44</v>
       </c>
       <c r="G24" t="n">
-        <v>24.12</v>
+        <v>22.68</v>
       </c>
       <c r="H24" t="n">
-        <v>23.99</v>
+        <v>23.56</v>
       </c>
       <c r="I24" t="n">
-        <v>-5.24</v>
+        <v>0.51</v>
       </c>
       <c r="J24" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="K24" t="n">
-        <v>24.12</v>
+        <v>22.51</v>
       </c>
       <c r="L24" t="n">
-        <v>25.26</v>
+        <v>23.43</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>623052</v>
+        <v>2183354</v>
       </c>
       <c r="P24" t="n">
-        <v>0.96</v>
+        <v>1.78</v>
       </c>
       <c r="Q24" t="n">
-        <v>26.96</v>
+        <v>23.05</v>
       </c>
       <c r="R24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>26.96</v>
+        <v>24.98</v>
       </c>
       <c r="T24" t="b">
         <v>0</v>
@@ -3274,10 +3274,10 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>6.48</v>
+        <v>6.57</v>
       </c>
       <c r="W24" t="n">
-        <v>6.48</v>
+        <v>-1.66</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3285,21 +3285,25 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB24" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0</v>
+      </c>
       <c r="AD24" t="n">
-        <v>24.12</v>
+        <v>22.68</v>
       </c>
       <c r="AE24" t="n">
-        <v>26.96</v>
+        <v>24.98</v>
       </c>
       <c r="AF24" t="n">
-        <v>4.74</v>
+        <v>3.24</v>
       </c>
       <c r="AG24" t="n">
-        <v>6.48</v>
+        <v>6.57</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
@@ -3307,7 +3311,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>1.37</v>
+        <v>2.03</v>
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
@@ -3327,31 +3331,31 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>46016.41666666666</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>46027.41666666666</v>
       </c>
       <c r="F25" t="n">
-        <v>22.75</v>
+        <v>24.6</v>
       </c>
       <c r="G25" t="n">
-        <v>21.66</v>
+        <v>23.75</v>
       </c>
       <c r="H25" t="n">
-        <v>21.65</v>
+        <v>24.41</v>
       </c>
       <c r="I25" t="n">
-        <v>-4.85</v>
+        <v>-0.77</v>
       </c>
       <c r="J25" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K25" t="n">
-        <v>21.66</v>
+        <v>23.41</v>
       </c>
       <c r="L25" t="n">
-        <v>22.2</v>
+        <v>24.09</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3364,31 +3368,31 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>13689820</v>
+        <v>2756109</v>
       </c>
       <c r="P25" t="n">
-        <v>4.94</v>
+        <v>3.54</v>
       </c>
       <c r="Q25" t="n">
-        <v>23.7</v>
+        <v>24.08</v>
       </c>
       <c r="R25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>25.75</v>
+        <v>24.5</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
       </c>
       <c r="U25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V25" t="n">
-        <v>13.18</v>
+        <v>-0.41</v>
       </c>
       <c r="W25" t="n">
-        <v>4.17</v>
+        <v>-2.11</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -3396,29 +3400,33 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB25" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0</v>
+      </c>
       <c r="AD25" t="n">
-        <v>21.66</v>
+        <v>23.75</v>
       </c>
       <c r="AE25" t="n">
-        <v>25.75</v>
+        <v>25.69</v>
       </c>
       <c r="AF25" t="n">
-        <v>4.78</v>
+        <v>3.46</v>
       </c>
       <c r="AG25" t="n">
-        <v>13.19</v>
+        <v>4.43</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>2.76</v>
+        <v>1.28</v>
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
@@ -3438,31 +3446,31 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>46069.41666666666</v>
       </c>
       <c r="F26" t="n">
-        <v>21.88</v>
+        <v>26</v>
       </c>
       <c r="G26" t="n">
-        <v>21.35</v>
+        <v>24.3</v>
       </c>
       <c r="H26" t="n">
-        <v>20.53</v>
+        <v>28.5</v>
       </c>
       <c r="I26" t="n">
-        <v>-6.18</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="K26" t="n">
-        <v>21.35</v>
+        <v>24.01</v>
       </c>
       <c r="L26" t="n">
-        <v>21.78</v>
+        <v>25.42</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3475,37 +3483,37 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>1476660</v>
+        <v>2965366</v>
       </c>
       <c r="P26" t="n">
-        <v>1.3</v>
+        <v>6.51</v>
       </c>
       <c r="Q26" t="n">
-        <v>21.54</v>
+        <v>25.42</v>
       </c>
       <c r="R26" t="b">
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>22.52</v>
+        <v>25.42</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
       </c>
       <c r="U26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V26" t="n">
-        <v>2.93</v>
+        <v>-2.23</v>
       </c>
       <c r="W26" t="n">
-        <v>-1.55</v>
+        <v>-2.23</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>45818.41666666666</v>
+        <v>46033.41666666666</v>
       </c>
       <c r="Z26" t="n">
         <v>2</v>
@@ -3514,30 +3522,30 @@
         <v>1</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>46028.41666666666</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>21.35</v>
+        <v>24.3</v>
       </c>
       <c r="AE26" t="n">
-        <v>22.52</v>
+        <v>27.41</v>
       </c>
       <c r="AF26" t="n">
-        <v>2.41</v>
+        <v>6.54</v>
       </c>
       <c r="AG26" t="n">
-        <v>2.93</v>
+        <v>5.42</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>1.22</v>
+        <v>0.83</v>
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
@@ -3557,31 +3565,31 @@
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>46120.41666666666</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>46139.41666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>21.16</v>
+        <v>26.61</v>
       </c>
       <c r="G27" t="n">
-        <v>19.2</v>
+        <v>25.21</v>
       </c>
       <c r="H27" t="n">
-        <v>21.32</v>
+        <v>28.7</v>
       </c>
       <c r="I27" t="n">
-        <v>0.76</v>
+        <v>7.85</v>
       </c>
       <c r="J27" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="K27" t="n">
-        <v>19.92</v>
+        <v>23.8</v>
       </c>
       <c r="L27" t="n">
-        <v>20.64</v>
+        <v>25.7</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3594,57 +3602,61 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>5666121</v>
+        <v>2499912</v>
       </c>
       <c r="P27" t="n">
-        <v>4.75</v>
+        <v>4.31</v>
       </c>
       <c r="Q27" t="n">
-        <v>22.02</v>
+        <v>26.8</v>
       </c>
       <c r="R27" t="b">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="T27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U27" t="b">
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="W27" t="n">
-        <v>4.06</v>
+        <v>0.71</v>
       </c>
       <c r="X27" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y27" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
       <c r="AA27" t="b">
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>45833.41666666666</v>
+        <v>46127.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD27" t="n">
-        <v>19.2</v>
+        <v>25.21</v>
       </c>
       <c r="AE27" t="n">
-        <v>22.52</v>
+        <v>26.8</v>
       </c>
       <c r="AF27" t="n">
-        <v>9.26</v>
+        <v>5.26</v>
       </c>
       <c r="AG27" t="n">
-        <v>6.43</v>
+        <v>0.71</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -3652,954 +3664,10 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.13</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C28" t="b">
-        <v>0</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>45845.41666666666</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>45860.41666666666</v>
-      </c>
-      <c r="F28" t="n">
-        <v>21.91</v>
-      </c>
-      <c r="G28" t="n">
-        <v>21.28</v>
-      </c>
-      <c r="H28" t="n">
-        <v>22.48</v>
-      </c>
-      <c r="I28" t="n">
-        <v>2.59</v>
-      </c>
-      <c r="J28" t="n">
-        <v>15</v>
-      </c>
-      <c r="K28" t="n">
-        <v>21.29</v>
-      </c>
-      <c r="L28" t="n">
-        <v>21.84</v>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O28" t="n">
-        <v>1366828</v>
-      </c>
-      <c r="P28" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>22.06</v>
-      </c>
-      <c r="R28" t="b">
-        <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="T28" t="b">
-        <v>0</v>
-      </c>
-      <c r="U28" t="b">
-        <v>0</v>
-      </c>
-      <c r="V28" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="W28" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="X28" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y28" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA28" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB28" s="2" t="n">
-        <v>45847.41666666666</v>
-      </c>
-      <c r="AC28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD28" t="n">
-        <v>21.28</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>22.44</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="AH28" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI28" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AJ28" t="inlineStr"/>
-      <c r="AK28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C29" t="b">
-        <v>0</v>
-      </c>
-      <c r="D29" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>45887.41666666666</v>
-      </c>
-      <c r="F29" t="n">
-        <v>23.36</v>
-      </c>
-      <c r="G29" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="H29" t="n">
-        <v>22.81</v>
-      </c>
-      <c r="I29" t="n">
-        <v>-2.36</v>
-      </c>
-      <c r="J29" t="n">
-        <v>15</v>
-      </c>
-      <c r="K29" t="n">
-        <v>22.39</v>
-      </c>
-      <c r="L29" t="n">
-        <v>23.18</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O29" t="n">
-        <v>1011332</v>
-      </c>
-      <c r="P29" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>23.12</v>
-      </c>
-      <c r="R29" t="b">
-        <v>1</v>
-      </c>
-      <c r="S29" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="T29" t="b">
-        <v>0</v>
-      </c>
-      <c r="U29" t="b">
-        <v>0</v>
-      </c>
-      <c r="V29" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="W29" t="n">
-        <v>-1.03</v>
-      </c>
-      <c r="X29" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y29" s="2" t="n">
-        <v>45873.41666666666</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA29" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB29" s="2" t="n">
-        <v>45872.41666666666</v>
-      </c>
-      <c r="AC29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="AE29" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="AF29" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="AG29" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="AH29" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI29" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="AJ29" t="inlineStr"/>
-      <c r="AK29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C30" t="b">
-        <v>0</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="F30" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="G30" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="H30" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="I30" t="n">
-        <v>-3.13</v>
-      </c>
-      <c r="J30" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" t="n">
-        <v>21.02</v>
-      </c>
-      <c r="L30" t="n">
-        <v>21.26</v>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O30" t="n">
-        <v>811883</v>
-      </c>
-      <c r="P30" t="n">
-        <v>2.81</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>21.61</v>
-      </c>
-      <c r="R30" t="b">
-        <v>1</v>
-      </c>
-      <c r="S30" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="T30" t="b">
-        <v>0</v>
-      </c>
-      <c r="U30" t="b">
-        <v>0</v>
-      </c>
-      <c r="V30" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="W30" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="X30" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y30" s="2" t="n">
-        <v>45900.41666666666</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA30" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB30" s="2" t="n">
-        <v>45897.41666666666</v>
-      </c>
-      <c r="AC30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>21.06</v>
-      </c>
-      <c r="AE30" t="n">
-        <v>21.83</v>
-      </c>
-      <c r="AF30" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="AG30" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="AH30" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI30" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="AJ30" t="inlineStr"/>
-      <c r="AK30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C31" t="b">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>45972.41666666666</v>
-      </c>
-      <c r="F31" t="n">
-        <v>21.51</v>
-      </c>
-      <c r="G31" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="H31" t="n">
-        <v>24.94</v>
-      </c>
-      <c r="I31" t="n">
-        <v>15.94</v>
-      </c>
-      <c r="J31" t="n">
-        <v>61</v>
-      </c>
-      <c r="K31" t="n">
-        <v>20.28</v>
-      </c>
-      <c r="L31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O31" t="n">
-        <v>2694406</v>
-      </c>
-      <c r="P31" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="R31" t="b">
-        <v>1</v>
-      </c>
-      <c r="S31" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="T31" t="b">
-        <v>0</v>
-      </c>
-      <c r="U31" t="b">
-        <v>1</v>
-      </c>
-      <c r="V31" t="n">
-        <v>-2.57</v>
-      </c>
-      <c r="W31" t="n">
-        <v>-2.57</v>
-      </c>
-      <c r="X31" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y31" s="2" t="n">
-        <v>45923.41666666666</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA31" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB31" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>20.27</v>
-      </c>
-      <c r="AE31" t="n">
-        <v>22.19</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>5.76</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="AH31" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI31" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AJ31" t="inlineStr"/>
-      <c r="AK31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C32" t="b">
-        <v>0</v>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>46002.41666666666</v>
-      </c>
-      <c r="F32" t="n">
-        <v>23.44</v>
-      </c>
-      <c r="G32" t="n">
-        <v>22.68</v>
-      </c>
-      <c r="H32" t="n">
-        <v>23.56</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="J32" t="n">
-        <v>8</v>
-      </c>
-      <c r="K32" t="n">
-        <v>22.51</v>
-      </c>
-      <c r="L32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O32" t="n">
-        <v>2183354</v>
-      </c>
-      <c r="P32" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>22.87</v>
-      </c>
-      <c r="R32" t="b">
-        <v>1</v>
-      </c>
-      <c r="S32" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="T32" t="b">
-        <v>0</v>
-      </c>
-      <c r="U32" t="b">
-        <v>0</v>
-      </c>
-      <c r="V32" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="W32" t="n">
-        <v>-2.43</v>
-      </c>
-      <c r="X32" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB32" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="AC32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>22.68</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>24.98</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="AG32" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="AH32" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI32" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AJ32" t="inlineStr"/>
-      <c r="AK32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C33" t="b">
-        <v>0</v>
-      </c>
-      <c r="D33" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>46027.41666666666</v>
-      </c>
-      <c r="F33" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G33" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="H33" t="n">
-        <v>24.41</v>
-      </c>
-      <c r="I33" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="J33" t="n">
-        <v>11</v>
-      </c>
-      <c r="K33" t="n">
-        <v>23.41</v>
-      </c>
-      <c r="L33" t="n">
-        <v>24.09</v>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O33" t="n">
-        <v>2756109</v>
-      </c>
-      <c r="P33" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>24.08</v>
-      </c>
-      <c r="R33" t="b">
-        <v>1</v>
-      </c>
-      <c r="S33" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="T33" t="b">
-        <v>0</v>
-      </c>
-      <c r="U33" t="b">
-        <v>1</v>
-      </c>
-      <c r="V33" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="W33" t="n">
-        <v>-2.11</v>
-      </c>
-      <c r="X33" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB33" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="AC33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD33" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="AE33" t="n">
-        <v>25.69</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="AH33" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI33" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="AJ33" t="inlineStr"/>
-      <c r="AK33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C34" t="b">
-        <v>0</v>
-      </c>
-      <c r="D34" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>46069.41666666666</v>
-      </c>
-      <c r="F34" t="n">
-        <v>26</v>
-      </c>
-      <c r="G34" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="H34" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="I34" t="n">
-        <v>9.619999999999999</v>
-      </c>
-      <c r="J34" t="n">
-        <v>41</v>
-      </c>
-      <c r="K34" t="n">
-        <v>24.01</v>
-      </c>
-      <c r="L34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O34" t="n">
-        <v>2965366</v>
-      </c>
-      <c r="P34" t="n">
-        <v>6.51</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="R34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S34" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="T34" t="b">
-        <v>0</v>
-      </c>
-      <c r="U34" t="b">
-        <v>1</v>
-      </c>
-      <c r="V34" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="W34" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="X34" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y34" s="2" t="n">
-        <v>46033.41666666666</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA34" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB34" s="2" t="n">
-        <v>46028.41666666666</v>
-      </c>
-      <c r="AC34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="AE34" t="n">
-        <v>27.41</v>
-      </c>
-      <c r="AF34" t="n">
-        <v>6.54</v>
-      </c>
-      <c r="AG34" t="n">
-        <v>5.42</v>
-      </c>
-      <c r="AH34" t="inlineStr">
-        <is>
-          <t>RANGE</t>
-        </is>
-      </c>
-      <c r="AI34" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="AJ34" t="inlineStr"/>
-      <c r="AK34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>JUFO</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKOUT</t>
-        </is>
-      </c>
-      <c r="C35" t="b">
-        <v>0</v>
-      </c>
-      <c r="D35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>46139.41666666666</v>
-      </c>
-      <c r="F35" t="n">
-        <v>26.61</v>
-      </c>
-      <c r="G35" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="H35" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="I35" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="J35" t="n">
-        <v>19</v>
-      </c>
-      <c r="K35" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="L35" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>RANGE_BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="O35" t="n">
-        <v>2499912</v>
-      </c>
-      <c r="P35" t="n">
-        <v>4.31</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>25.73</v>
-      </c>
-      <c r="R35" t="b">
-        <v>1</v>
-      </c>
-      <c r="S35" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="T35" t="b">
-        <v>1</v>
-      </c>
-      <c r="U35" t="b">
-        <v>0</v>
-      </c>
-      <c r="V35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="W35" t="n">
-        <v>-3.31</v>
-      </c>
-      <c r="X35" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA35" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB35" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="AC35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="AE35" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="AG35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="AH35" t="inlineStr">
-        <is>
-          <t>ANCHOR</t>
-        </is>
-      </c>
-      <c r="AI35" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AJ35" t="inlineStr"/>
-      <c r="AK35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4817,31 +3885,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>47.87</v>
+        <v>53.91</v>
       </c>
       <c r="G2" t="n">
-        <v>46</v>
+        <v>43.72</v>
       </c>
       <c r="H2" t="n">
         <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>278.11</v>
+        <v>235.74</v>
       </c>
       <c r="J2" t="n">
-        <v>384</v>
+        <v>593</v>
       </c>
       <c r="K2" t="n">
-        <v>45</v>
+        <v>43.03</v>
       </c>
       <c r="L2" t="n">
-        <v>46.89</v>
+        <v>45.91</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -4854,69 +3922,69 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>47815</v>
+        <v>128396</v>
       </c>
       <c r="P2" t="n">
-        <v>2.73</v>
+        <v>19.99</v>
       </c>
       <c r="Q2" t="n">
-        <v>46.62</v>
+        <v>45.33</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>51</v>
+        <v>48.75</v>
       </c>
       <c r="T2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>6.54</v>
+        <v>-9.57</v>
       </c>
       <c r="W2" t="n">
-        <v>-2.61</v>
+        <v>-15.92</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45547.41666666666</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45755.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>46</v>
+        <v>43.72</v>
       </c>
       <c r="AE2" t="n">
-        <v>51</v>
+        <v>59.63</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.91</v>
+        <v>18.9</v>
       </c>
       <c r="AG2" t="n">
-        <v>6.54</v>
+        <v>10.61</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>1.67</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ2" t="n">
         <v>181</v>
@@ -5058,25 +4126,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>27.27</v>
+        <v>66.67</v>
       </c>
       <c r="G2" t="n">
-        <v>-4.54</v>
+        <v>1.19</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
       <c r="I2" t="n">
-        <v>-25.44</v>
+        <v>-0.58</v>
       </c>
       <c r="J2" t="n">
         <v>12.48</v>
@@ -5085,28 +4153,28 @@
         <v>-14.25</v>
       </c>
       <c r="L2" t="n">
-        <v>7.68</v>
+        <v>13.42</v>
       </c>
       <c r="M2" t="n">
-        <v>0.48</v>
+        <v>0.96</v>
       </c>
       <c r="N2" t="n">
-        <v>7.98</v>
+        <v>6.84</v>
       </c>
       <c r="O2" t="n">
-        <v>6.17</v>
+        <v>14.25</v>
       </c>
       <c r="P2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1209768433179723</v>
+        <v>0.2320120319001387</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.09292000000000003</v>
+        <v>0.09086</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.007361262672811078</v>
+        <v>0.1473208127600555</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -5114,7 +4182,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>-0.007361262672811078</v>
+        <v>0.1473208127600555</v>
       </c>
     </row>
     <row r="3">
@@ -5144,10 +4212,10 @@
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
       <c r="I3" t="n">
-        <v>63.34</v>
+        <v>59.34</v>
       </c>
       <c r="J3" t="n">
         <v>38.41</v>
@@ -5156,28 +4224,28 @@
         <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>10.51</v>
+        <v>10.64</v>
       </c>
       <c r="M3" t="n">
-        <v>2.31</v>
+        <v>2.13</v>
       </c>
       <c r="N3" t="n">
         <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>4.39</v>
+        <v>4.76</v>
       </c>
       <c r="P3" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5176452432667247</v>
+        <v>0.5084026632302405</v>
       </c>
       <c r="R3" t="n">
-        <v>0.51042</v>
+        <v>0.49842</v>
       </c>
       <c r="S3" t="n">
-        <v>0.5133100973066899</v>
+        <v>0.5024130652920962</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -5185,7 +4253,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.5133100973066899</v>
+        <v>0.5024130652920962</v>
       </c>
     </row>
   </sheetData>
@@ -5256,22 +4324,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.01</v>
+        <v>0.15</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>27.27</v>
+        <v>66.67</v>
       </c>
       <c r="F2" t="n">
-        <v>0.48</v>
+        <v>0.96</v>
       </c>
       <c r="G2" t="n">
-        <v>-4.54</v>
+        <v>1.19</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.31</v>
+        <v>-0.19</v>
       </c>
     </row>
     <row r="3">
@@ -5286,7 +4354,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.51</v>
+        <v>0.5</v>
       </c>
       <c r="D3" t="n">
         <v>23</v>
@@ -5295,13 +4363,13 @@
         <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>2.31</v>
+        <v>2.13</v>
       </c>
       <c r="G3" t="n">
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-27 18:44:24.294661
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK27"/>
+  <dimension ref="A1:AK35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,7 +983,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -992,34 +992,34 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45322.41666666666</v>
+        <v>45554.41666666666</v>
       </c>
       <c r="F5" t="n">
-        <v>13.43</v>
+        <v>53.91</v>
       </c>
       <c r="G5" t="n">
-        <v>12.66</v>
+        <v>43.72</v>
       </c>
       <c r="H5" t="n">
-        <v>13.26</v>
+        <v>51.11</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.25</v>
+        <v>-5.19</v>
       </c>
       <c r="J5" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>12.54</v>
+        <v>43.03</v>
       </c>
       <c r="L5" t="n">
-        <v>13.42</v>
+        <v>45.91</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1032,19 +1032,19 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>3180532</v>
+        <v>128396</v>
       </c>
       <c r="P5" t="n">
-        <v>3.32</v>
+        <v>19.99</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.98</v>
+        <v>45.33</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>13.42</v>
+        <v>48.75</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
@@ -1053,40 +1053,40 @@
         <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.09</v>
+        <v>-9.57</v>
       </c>
       <c r="W5" t="n">
-        <v>-3.37</v>
+        <v>-15.92</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>45313.41666666666</v>
+        <v>45547.41666666666</v>
       </c>
       <c r="Z5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>45301.41666666666</v>
+        <v>45546.41666666666</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>12.66</v>
+        <v>43.72</v>
       </c>
       <c r="AE5" t="n">
-        <v>14.32</v>
+        <v>59.63</v>
       </c>
       <c r="AF5" t="n">
-        <v>5.78</v>
+        <v>18.9</v>
       </c>
       <c r="AG5" t="n">
-        <v>6.61</v>
+        <v>10.61</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>1.14</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1111,34 +1111,34 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45558.41666666666</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45351.41666666666</v>
+        <v>45567.41666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>15.59</v>
+        <v>53.48</v>
       </c>
       <c r="G6" t="n">
-        <v>13.66</v>
+        <v>50.18</v>
       </c>
       <c r="H6" t="n">
-        <v>16</v>
+        <v>49.83</v>
       </c>
       <c r="I6" t="n">
-        <v>2.62</v>
+        <v>-6.82</v>
       </c>
       <c r="J6" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="K6" t="n">
-        <v>12.64</v>
+        <v>50.18</v>
       </c>
       <c r="L6" t="n">
-        <v>14.56</v>
+        <v>52.39</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1151,69 +1151,65 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>708583</v>
+        <v>188748</v>
       </c>
       <c r="P6" t="n">
-        <v>10.05</v>
+        <v>4.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>13.78</v>
+        <v>50.5</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>15.04</v>
+        <v>61.85</v>
       </c>
       <c r="T6" t="b">
         <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.54</v>
+        <v>15.65</v>
       </c>
       <c r="W6" t="n">
-        <v>-11.62</v>
+        <v>-5.57</v>
       </c>
       <c r="X6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="2" t="n">
-        <v>45336.41666666666</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="b">
         <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>45326.41666666666</v>
+        <v>45558.41666666666</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>13.66</v>
+        <v>50.18</v>
       </c>
       <c r="AE6" t="n">
-        <v>17.99</v>
+        <v>61.85</v>
       </c>
       <c r="AF6" t="n">
-        <v>12.37</v>
+        <v>6.17</v>
       </c>
       <c r="AG6" t="n">
-        <v>15.39</v>
+        <v>15.65</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>1.24</v>
+        <v>2.54</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1221,7 +1217,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1233,31 +1229,31 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45594.41666666666</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45379.41666666666</v>
+        <v>45601.41666666666</v>
       </c>
       <c r="F7" t="n">
-        <v>15.92</v>
+        <v>54</v>
       </c>
       <c r="G7" t="n">
-        <v>14.54</v>
+        <v>52.01</v>
       </c>
       <c r="H7" t="n">
-        <v>14.11</v>
+        <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>-11.36</v>
+        <v>-3.7</v>
       </c>
       <c r="J7" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>14.54</v>
+        <v>44</v>
       </c>
       <c r="L7" t="n">
-        <v>15.68</v>
+        <v>53.95</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1270,61 +1266,57 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>2359660</v>
+        <v>36571</v>
       </c>
       <c r="P7" t="n">
-        <v>3.65</v>
+        <v>3.41</v>
       </c>
       <c r="Q7" t="n">
-        <v>15.3</v>
+        <v>54.51</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>16.22</v>
+        <v>57.99</v>
       </c>
       <c r="T7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>1.88</v>
+        <v>7.39</v>
       </c>
       <c r="W7" t="n">
-        <v>-3.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="2" t="n">
-        <v>45362.41666666666</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>45362.41666666666</v>
+        <v>45599.41666666666</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD7" t="n">
-        <v>14.54</v>
+        <v>52.01</v>
       </c>
       <c r="AE7" t="n">
-        <v>16.22</v>
+        <v>57.99</v>
       </c>
       <c r="AF7" t="n">
-        <v>8.69</v>
+        <v>3.69</v>
       </c>
       <c r="AG7" t="n">
-        <v>1.91</v>
+        <v>7.39</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1332,7 +1324,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.22</v>
+        <v>2</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1340,7 +1332,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1352,31 +1344,31 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45603.41666666666</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45400.41666666666</v>
+        <v>45608.41666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>13.08</v>
+        <v>54.34</v>
       </c>
       <c r="G8" t="n">
-        <v>12.76</v>
+        <v>52.65</v>
       </c>
       <c r="H8" t="n">
-        <v>12.39</v>
+        <v>51.7</v>
       </c>
       <c r="I8" t="n">
-        <v>-5.26</v>
+        <v>-4.86</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>12.22</v>
+        <v>51.6</v>
       </c>
       <c r="L8" t="n">
-        <v>13.04</v>
+        <v>54.24</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1389,19 +1381,19 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>5618577</v>
+        <v>18287</v>
       </c>
       <c r="P8" t="n">
-        <v>2.06</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.72</v>
+        <v>53.58</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>14.15</v>
+        <v>57.84</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
@@ -1410,10 +1402,10 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>8.18</v>
+        <v>6.44</v>
       </c>
       <c r="W8" t="n">
-        <v>-2.75</v>
+        <v>-1.4</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1424,22 +1416,22 @@
         <v>1</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>45398.41666666666</v>
+        <v>45603.41666666666</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>12.76</v>
+        <v>52.65</v>
       </c>
       <c r="AE8" t="n">
-        <v>14.15</v>
+        <v>57.84</v>
       </c>
       <c r="AF8" t="n">
-        <v>2.45</v>
+        <v>3.11</v>
       </c>
       <c r="AG8" t="n">
-        <v>8.199999999999999</v>
+        <v>6.44</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1447,7 +1439,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>3.35</v>
+        <v>2.07</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
@@ -1455,7 +1447,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1467,31 +1459,31 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>45411.41666666666</v>
+        <v>45624.41666666666</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45424.41666666666</v>
+        <v>45669.41666666666</v>
       </c>
       <c r="F9" t="n">
-        <v>11.44</v>
+        <v>49.88</v>
       </c>
       <c r="G9" t="n">
-        <v>10.23</v>
+        <v>47.93</v>
       </c>
       <c r="H9" t="n">
-        <v>11.76</v>
+        <v>55</v>
       </c>
       <c r="I9" t="n">
-        <v>2.8</v>
+        <v>10.26</v>
       </c>
       <c r="J9" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>10.01</v>
+        <v>48</v>
       </c>
       <c r="L9" t="n">
-        <v>11.2</v>
+        <v>49.58</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1504,19 +1496,19 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>3697242</v>
+        <v>431</v>
       </c>
       <c r="P9" t="n">
-        <v>10</v>
+        <v>1.14</v>
       </c>
       <c r="Q9" t="n">
-        <v>13.1</v>
+        <v>51.55</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>13.42</v>
+        <v>51.55</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1525,32 +1517,40 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>17.31</v>
+        <v>3.35</v>
       </c>
       <c r="W9" t="n">
-        <v>14.51</v>
+        <v>3.35</v>
       </c>
       <c r="X9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>45631.41666666666</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>5</v>
+      </c>
       <c r="AA9" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2" t="n">
+        <v>45631.41666666666</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>5</v>
+      </c>
       <c r="AD9" t="n">
-        <v>10.23</v>
+        <v>47.93</v>
       </c>
       <c r="AE9" t="n">
-        <v>13.42</v>
+        <v>51.55</v>
       </c>
       <c r="AF9" t="n">
-        <v>10.56</v>
+        <v>3.91</v>
       </c>
       <c r="AG9" t="n">
-        <v>17.34</v>
+        <v>3.35</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>1.64</v>
+        <v>0.86</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1566,7 +1566,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1578,31 +1578,31 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>45425.41666666666</v>
+        <v>45704.41666666666</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45434.41666666666</v>
+        <v>45714.41666666666</v>
       </c>
       <c r="F10" t="n">
-        <v>12.1</v>
+        <v>47.99</v>
       </c>
       <c r="G10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="H10" t="n">
-        <v>12.4</v>
+        <v>45.81</v>
       </c>
       <c r="I10" t="n">
-        <v>2.51</v>
+        <v>-4.54</v>
       </c>
       <c r="J10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="L10" t="n">
-        <v>12.08</v>
+        <v>47.97</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1615,19 +1615,19 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>719120</v>
+        <v>6897</v>
       </c>
       <c r="P10" t="n">
-        <v>2.86</v>
+        <v>3.61</v>
       </c>
       <c r="Q10" t="n">
-        <v>11.92</v>
+        <v>48.54</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>12.39</v>
+        <v>50.25</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1636,40 +1636,32 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>2.43</v>
+        <v>4.71</v>
       </c>
       <c r="W10" t="n">
-        <v>-1.46</v>
+        <v>1.15</v>
       </c>
       <c r="X10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="2" t="n">
-        <v>45426.41666666666</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB10" s="2" t="n">
-        <v>45425.41666666666</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
-        <v>11.68</v>
+        <v>46</v>
       </c>
       <c r="AE10" t="n">
-        <v>12.39</v>
+        <v>50.25</v>
       </c>
       <c r="AF10" t="n">
-        <v>3.44</v>
+        <v>4.15</v>
       </c>
       <c r="AG10" t="n">
-        <v>2.45</v>
+        <v>4.71</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -1677,7 +1669,7 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.71</v>
+        <v>1.13</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1685,7 +1677,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1697,31 +1689,31 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45495.41666666666</v>
+        <v>45727.41666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>13.23</v>
+        <v>47.51</v>
       </c>
       <c r="G11" t="n">
-        <v>12.37</v>
+        <v>45.8</v>
       </c>
       <c r="H11" t="n">
-        <v>15.11</v>
+        <v>45.63</v>
       </c>
       <c r="I11" t="n">
-        <v>14.21</v>
+        <v>-3.96</v>
       </c>
       <c r="J11" t="n">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="K11" t="n">
-        <v>12.37</v>
+        <v>45.81</v>
       </c>
       <c r="L11" t="n">
-        <v>12.68</v>
+        <v>46.58</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1734,19 +1726,19 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>2872871</v>
+        <v>31257</v>
       </c>
       <c r="P11" t="n">
-        <v>4.75</v>
+        <v>3.04</v>
       </c>
       <c r="Q11" t="n">
-        <v>12.61</v>
+        <v>46.46</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>13.12</v>
+        <v>46.7</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -1755,40 +1747,40 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>-0.85</v>
+        <v>-1.7</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.7</v>
+        <v>-2.21</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45454.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>45439.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>12.37</v>
+        <v>45.8</v>
       </c>
       <c r="AE11" t="n">
-        <v>13.98</v>
+        <v>48.4</v>
       </c>
       <c r="AF11" t="n">
-        <v>6.53</v>
+        <v>3.6</v>
       </c>
       <c r="AG11" t="n">
-        <v>5.68</v>
+        <v>1.87</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -1796,7 +1788,7 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.87</v>
+        <v>0.52</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1804,7 +1796,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>JUFO</t>
+          <t>AALR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1816,31 +1808,31 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45526.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>17.1</v>
+        <v>48.44</v>
       </c>
       <c r="G12" t="n">
-        <v>14.96</v>
+        <v>45.88</v>
       </c>
       <c r="H12" t="n">
-        <v>19.46</v>
+        <v>45.51</v>
       </c>
       <c r="I12" t="n">
-        <v>13.85</v>
+        <v>-6.05</v>
       </c>
       <c r="J12" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K12" t="n">
-        <v>14.96</v>
+        <v>45.6</v>
       </c>
       <c r="L12" t="n">
-        <v>15.28</v>
+        <v>46.75</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1853,19 +1845,19 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>2885185</v>
+        <v>49292</v>
       </c>
       <c r="P12" t="n">
-        <v>13.79</v>
+        <v>5.14</v>
       </c>
       <c r="Q12" t="n">
-        <v>15.44</v>
+        <v>46.73</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>15.5</v>
+        <v>46.75</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1874,40 +1866,40 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-9.34</v>
+        <v>-3.49</v>
       </c>
       <c r="W12" t="n">
-        <v>-9.69</v>
+        <v>-3.53</v>
       </c>
       <c r="X12" t="b">
         <v>1</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45734.41666666666</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>45503.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>14.96</v>
+        <v>45.88</v>
       </c>
       <c r="AE12" t="n">
-        <v>17.64</v>
+        <v>49.59</v>
       </c>
       <c r="AF12" t="n">
-        <v>12.49</v>
+        <v>5.28</v>
       </c>
       <c r="AG12" t="n">
-        <v>3.18</v>
+        <v>2.37</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1915,7 +1907,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.25</v>
+        <v>0.45</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1932,34 +1924,34 @@
         </is>
       </c>
       <c r="C13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45715.41666666666</v>
+        <v>45322.41666666666</v>
       </c>
       <c r="F13" t="n">
-        <v>20.68</v>
+        <v>13.43</v>
       </c>
       <c r="G13" t="n">
-        <v>18.4</v>
+        <v>12.66</v>
       </c>
       <c r="H13" t="n">
-        <v>28.62</v>
+        <v>13.26</v>
       </c>
       <c r="I13" t="n">
-        <v>38.41</v>
+        <v>-1.25</v>
       </c>
       <c r="J13" t="n">
-        <v>185</v>
+        <v>21</v>
       </c>
       <c r="K13" t="n">
-        <v>18.4</v>
+        <v>12.54</v>
       </c>
       <c r="L13" t="n">
-        <v>20.24</v>
+        <v>13.42</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1972,69 +1964,69 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>807277</v>
+        <v>3180532</v>
       </c>
       <c r="P13" t="n">
-        <v>2.17</v>
+        <v>3.32</v>
       </c>
       <c r="Q13" t="n">
-        <v>20.54</v>
+        <v>12.98</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>23.04</v>
+        <v>13.42</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>11.41</v>
+        <v>-0.09</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.68</v>
+        <v>-3.37</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45572.41666666666</v>
+        <v>45313.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45530.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>18.4</v>
+        <v>12.66</v>
       </c>
       <c r="AE13" t="n">
-        <v>23.04</v>
+        <v>14.32</v>
       </c>
       <c r="AF13" t="n">
-        <v>11.03</v>
+        <v>5.78</v>
       </c>
       <c r="AG13" t="n">
-        <v>11.41</v>
+        <v>6.61</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.03</v>
+        <v>1.14</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2051,34 +2043,34 @@
         </is>
       </c>
       <c r="C14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45733.41666666666</v>
+        <v>45351.41666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>28.64</v>
+        <v>15.59</v>
       </c>
       <c r="G14" t="n">
-        <v>28.08</v>
+        <v>13.66</v>
       </c>
       <c r="H14" t="n">
-        <v>27.22</v>
+        <v>16</v>
       </c>
       <c r="I14" t="n">
-        <v>-4.97</v>
+        <v>2.62</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="K14" t="n">
-        <v>28</v>
+        <v>12.64</v>
       </c>
       <c r="L14" t="n">
-        <v>28.48</v>
+        <v>14.56</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2091,69 +2083,69 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>1546271</v>
+        <v>708583</v>
       </c>
       <c r="P14" t="n">
-        <v>1.79</v>
+        <v>10.05</v>
       </c>
       <c r="Q14" t="n">
-        <v>28.16</v>
+        <v>13.78</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>29</v>
+        <v>15.04</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>1.26</v>
+        <v>-3.54</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.68</v>
+        <v>-11.62</v>
       </c>
       <c r="X14" t="b">
         <v>1</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>45729.41666666666</v>
+        <v>45336.41666666666</v>
       </c>
       <c r="Z14" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>45728.41666666666</v>
+        <v>45326.41666666666</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>28.08</v>
+        <v>13.66</v>
       </c>
       <c r="AE14" t="n">
-        <v>29</v>
+        <v>17.99</v>
       </c>
       <c r="AF14" t="n">
-        <v>1.96</v>
+        <v>12.37</v>
       </c>
       <c r="AG14" t="n">
-        <v>1.26</v>
+        <v>15.39</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.64</v>
+        <v>1.24</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2173,31 +2165,31 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45741.41666666666</v>
+        <v>45362.41666666666</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45756.41666666666</v>
+        <v>45379.41666666666</v>
       </c>
       <c r="F15" t="n">
-        <v>25.97</v>
+        <v>15.92</v>
       </c>
       <c r="G15" t="n">
-        <v>24.72</v>
+        <v>14.54</v>
       </c>
       <c r="H15" t="n">
-        <v>24.16</v>
+        <v>14.11</v>
       </c>
       <c r="I15" t="n">
-        <v>-6.96</v>
+        <v>-11.36</v>
       </c>
       <c r="J15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K15" t="n">
-        <v>24.68</v>
+        <v>14.54</v>
       </c>
       <c r="L15" t="n">
-        <v>25.51</v>
+        <v>15.68</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2210,53 +2202,61 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>767605</v>
+        <v>2359660</v>
       </c>
       <c r="P15" t="n">
-        <v>4.04</v>
+        <v>3.65</v>
       </c>
       <c r="Q15" t="n">
-        <v>27.46</v>
+        <v>15.3</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>29.03</v>
+        <v>16.22</v>
       </c>
       <c r="T15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U15" t="b">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>11.79</v>
+        <v>1.88</v>
       </c>
       <c r="W15" t="n">
-        <v>5.75</v>
+        <v>-3.89</v>
       </c>
       <c r="X15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y15" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
       <c r="AA15" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB15" s="2" t="n">
+        <v>45362.41666666666</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0</v>
+      </c>
       <c r="AD15" t="n">
-        <v>24.72</v>
+        <v>14.54</v>
       </c>
       <c r="AE15" t="n">
-        <v>29.03</v>
+        <v>16.22</v>
       </c>
       <c r="AF15" t="n">
-        <v>4.81</v>
+        <v>8.69</v>
       </c>
       <c r="AG15" t="n">
-        <v>11.8</v>
+        <v>1.91</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>2.45</v>
+        <v>0.22</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2284,31 +2284,31 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45760.41666666666</v>
+        <v>45398.41666666666</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45783.41666666666</v>
+        <v>45400.41666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>25.32</v>
+        <v>13.08</v>
       </c>
       <c r="G16" t="n">
-        <v>24.12</v>
+        <v>12.76</v>
       </c>
       <c r="H16" t="n">
-        <v>23.99</v>
+        <v>12.39</v>
       </c>
       <c r="I16" t="n">
-        <v>-5.24</v>
+        <v>-5.26</v>
       </c>
       <c r="J16" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>24.12</v>
+        <v>12.22</v>
       </c>
       <c r="L16" t="n">
-        <v>25.26</v>
+        <v>13.04</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>623052</v>
+        <v>5618577</v>
       </c>
       <c r="P16" t="n">
-        <v>0.96</v>
+        <v>2.06</v>
       </c>
       <c r="Q16" t="n">
-        <v>26.96</v>
+        <v>12.72</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>26.96</v>
+        <v>14.15</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2342,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>6.48</v>
+        <v>8.18</v>
       </c>
       <c r="W16" t="n">
-        <v>6.48</v>
+        <v>-2.75</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -2353,21 +2353,25 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB16" s="2" t="n">
+        <v>45398.41666666666</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
       <c r="AD16" t="n">
-        <v>24.12</v>
+        <v>12.76</v>
       </c>
       <c r="AE16" t="n">
-        <v>26.96</v>
+        <v>14.15</v>
       </c>
       <c r="AF16" t="n">
-        <v>4.74</v>
+        <v>2.45</v>
       </c>
       <c r="AG16" t="n">
-        <v>6.48</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2375,7 +2379,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>1.37</v>
+        <v>3.35</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2395,31 +2399,31 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45792.41666666666</v>
+        <v>45411.41666666666</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45809.41666666666</v>
+        <v>45424.41666666666</v>
       </c>
       <c r="F17" t="n">
-        <v>22.75</v>
+        <v>11.44</v>
       </c>
       <c r="G17" t="n">
-        <v>21.66</v>
+        <v>10.23</v>
       </c>
       <c r="H17" t="n">
-        <v>21.65</v>
+        <v>11.76</v>
       </c>
       <c r="I17" t="n">
-        <v>-4.85</v>
+        <v>2.8</v>
       </c>
       <c r="J17" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
-        <v>21.66</v>
+        <v>10.01</v>
       </c>
       <c r="L17" t="n">
-        <v>22.2</v>
+        <v>11.2</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2432,19 +2436,19 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>13689820</v>
+        <v>3697242</v>
       </c>
       <c r="P17" t="n">
-        <v>4.94</v>
+        <v>10</v>
       </c>
       <c r="Q17" t="n">
-        <v>23.7</v>
+        <v>13.1</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>25.75</v>
+        <v>13.42</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -2453,10 +2457,10 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>13.18</v>
+        <v>17.31</v>
       </c>
       <c r="W17" t="n">
-        <v>4.17</v>
+        <v>14.51</v>
       </c>
       <c r="X17" t="b">
         <v>0</v>
@@ -2469,16 +2473,16 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="n">
-        <v>21.66</v>
+        <v>10.23</v>
       </c>
       <c r="AE17" t="n">
-        <v>25.75</v>
+        <v>13.42</v>
       </c>
       <c r="AF17" t="n">
-        <v>4.78</v>
+        <v>10.56</v>
       </c>
       <c r="AG17" t="n">
-        <v>13.19</v>
+        <v>17.34</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2486,7 +2490,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>2.76</v>
+        <v>1.64</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2506,31 +2510,31 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45823.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="F18" t="n">
-        <v>21.88</v>
+        <v>12.1</v>
       </c>
       <c r="G18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="H18" t="n">
-        <v>20.53</v>
+        <v>12.4</v>
       </c>
       <c r="I18" t="n">
-        <v>-6.18</v>
+        <v>2.51</v>
       </c>
       <c r="J18" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="L18" t="n">
-        <v>21.78</v>
+        <v>12.08</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2543,19 +2547,19 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>1476660</v>
+        <v>719120</v>
       </c>
       <c r="P18" t="n">
-        <v>1.3</v>
+        <v>2.86</v>
       </c>
       <c r="Q18" t="n">
-        <v>21.54</v>
+        <v>11.92</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>22.52</v>
+        <v>12.39</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -2564,40 +2568,40 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>2.93</v>
+        <v>2.43</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.55</v>
+        <v>-1.46</v>
       </c>
       <c r="X18" t="b">
         <v>1</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>45818.41666666666</v>
+        <v>45426.41666666666</v>
       </c>
       <c r="Z18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>45811.41666666666</v>
+        <v>45425.41666666666</v>
       </c>
       <c r="AC18" t="n">
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>21.35</v>
+        <v>11.68</v>
       </c>
       <c r="AE18" t="n">
-        <v>22.52</v>
+        <v>12.39</v>
       </c>
       <c r="AF18" t="n">
-        <v>2.41</v>
+        <v>3.44</v>
       </c>
       <c r="AG18" t="n">
-        <v>2.93</v>
+        <v>2.45</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -2605,7 +2609,7 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>1.22</v>
+        <v>0.71</v>
       </c>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
@@ -2625,31 +2629,31 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>45831.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45839.41666666666</v>
+        <v>45495.41666666666</v>
       </c>
       <c r="F19" t="n">
-        <v>21.16</v>
+        <v>13.23</v>
       </c>
       <c r="G19" t="n">
-        <v>19.2</v>
+        <v>12.37</v>
       </c>
       <c r="H19" t="n">
-        <v>21.32</v>
+        <v>15.11</v>
       </c>
       <c r="I19" t="n">
-        <v>0.76</v>
+        <v>14.21</v>
       </c>
       <c r="J19" t="n">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="K19" t="n">
-        <v>19.92</v>
+        <v>12.37</v>
       </c>
       <c r="L19" t="n">
-        <v>20.64</v>
+        <v>12.68</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2662,65 +2666,69 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>5666121</v>
+        <v>2872871</v>
       </c>
       <c r="P19" t="n">
         <v>4.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>22.02</v>
+        <v>12.61</v>
       </c>
       <c r="R19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>22.52</v>
+        <v>13.12</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
       </c>
       <c r="U19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" t="n">
-        <v>6.43</v>
+        <v>-0.85</v>
       </c>
       <c r="W19" t="n">
-        <v>4.06</v>
+        <v>-4.7</v>
       </c>
       <c r="X19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y19" s="2" t="n">
+        <v>45454.41666666666</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>11</v>
+      </c>
       <c r="AA19" t="b">
         <v>1</v>
       </c>
       <c r="AB19" s="2" t="n">
-        <v>45833.41666666666</v>
+        <v>45439.41666666666</v>
       </c>
       <c r="AC19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD19" t="n">
-        <v>19.2</v>
+        <v>12.37</v>
       </c>
       <c r="AE19" t="n">
-        <v>22.52</v>
+        <v>13.98</v>
       </c>
       <c r="AF19" t="n">
-        <v>9.26</v>
+        <v>6.53</v>
       </c>
       <c r="AG19" t="n">
-        <v>6.43</v>
+        <v>5.68</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.87</v>
       </c>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
@@ -2740,31 +2748,31 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>45845.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45860.41666666666</v>
+        <v>45526.41666666666</v>
       </c>
       <c r="F20" t="n">
-        <v>21.91</v>
+        <v>17.1</v>
       </c>
       <c r="G20" t="n">
-        <v>21.28</v>
+        <v>14.96</v>
       </c>
       <c r="H20" t="n">
-        <v>22.48</v>
+        <v>19.46</v>
       </c>
       <c r="I20" t="n">
-        <v>2.59</v>
+        <v>13.85</v>
       </c>
       <c r="J20" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="K20" t="n">
-        <v>21.29</v>
+        <v>14.96</v>
       </c>
       <c r="L20" t="n">
-        <v>21.84</v>
+        <v>15.28</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2777,69 +2785,69 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>1366828</v>
+        <v>2885185</v>
       </c>
       <c r="P20" t="n">
-        <v>1.44</v>
+        <v>13.79</v>
       </c>
       <c r="Q20" t="n">
-        <v>22.06</v>
+        <v>15.44</v>
       </c>
       <c r="R20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>22.44</v>
+        <v>15.5</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
       </c>
       <c r="U20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
-        <v>2.41</v>
+        <v>-9.34</v>
       </c>
       <c r="W20" t="n">
-        <v>0.68</v>
+        <v>-9.69</v>
       </c>
       <c r="X20" t="b">
         <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>45847.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="Z20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>45847.41666666666</v>
+        <v>45503.41666666666</v>
       </c>
       <c r="AC20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD20" t="n">
-        <v>21.28</v>
+        <v>14.96</v>
       </c>
       <c r="AE20" t="n">
-        <v>22.44</v>
+        <v>17.64</v>
       </c>
       <c r="AF20" t="n">
-        <v>2.88</v>
+        <v>12.49</v>
       </c>
       <c r="AG20" t="n">
-        <v>2.41</v>
+        <v>3.18</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.84</v>
+        <v>0.25</v>
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
@@ -2859,31 +2867,31 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45887.41666666666</v>
+        <v>45715.41666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>23.36</v>
+        <v>20.68</v>
       </c>
       <c r="G21" t="n">
-        <v>22.64</v>
+        <v>18.4</v>
       </c>
       <c r="H21" t="n">
-        <v>22.81</v>
+        <v>28.62</v>
       </c>
       <c r="I21" t="n">
-        <v>-2.36</v>
+        <v>38.41</v>
       </c>
       <c r="J21" t="n">
-        <v>15</v>
+        <v>185</v>
       </c>
       <c r="K21" t="n">
-        <v>22.39</v>
+        <v>18.4</v>
       </c>
       <c r="L21" t="n">
-        <v>23.18</v>
+        <v>20.24</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2896,19 +2904,19 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>1011332</v>
+        <v>807277</v>
       </c>
       <c r="P21" t="n">
-        <v>1.74</v>
+        <v>2.17</v>
       </c>
       <c r="Q21" t="n">
-        <v>23.12</v>
+        <v>20.54</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>23.48</v>
+        <v>23.04</v>
       </c>
       <c r="T21" t="b">
         <v>0</v>
@@ -2917,40 +2925,40 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>0.51</v>
+        <v>11.41</v>
       </c>
       <c r="W21" t="n">
-        <v>-1.03</v>
+        <v>-0.68</v>
       </c>
       <c r="X21" t="b">
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>45873.41666666666</v>
+        <v>45572.41666666666</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
       </c>
       <c r="AB21" s="2" t="n">
-        <v>45872.41666666666</v>
+        <v>45530.41666666666</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>22.64</v>
+        <v>18.4</v>
       </c>
       <c r="AE21" t="n">
-        <v>23.48</v>
+        <v>23.04</v>
       </c>
       <c r="AF21" t="n">
-        <v>3.08</v>
+        <v>11.03</v>
       </c>
       <c r="AG21" t="n">
-        <v>0.51</v>
+        <v>11.41</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
@@ -2958,7 +2966,7 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.17</v>
+        <v>1.03</v>
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
@@ -2978,31 +2986,31 @@
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45900.41666666666</v>
+        <v>45733.41666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>21.7</v>
+        <v>28.64</v>
       </c>
       <c r="G22" t="n">
-        <v>21.06</v>
+        <v>28.08</v>
       </c>
       <c r="H22" t="n">
-        <v>21.02</v>
+        <v>27.22</v>
       </c>
       <c r="I22" t="n">
-        <v>-3.13</v>
+        <v>-4.97</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>21.02</v>
+        <v>28</v>
       </c>
       <c r="L22" t="n">
-        <v>21.26</v>
+        <v>28.48</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3015,19 +3023,19 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>811883</v>
+        <v>1546271</v>
       </c>
       <c r="P22" t="n">
-        <v>2.81</v>
+        <v>1.79</v>
       </c>
       <c r="Q22" t="n">
-        <v>21.61</v>
+        <v>28.16</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>21.83</v>
+        <v>29</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
@@ -3036,16 +3044,16 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>0.62</v>
+        <v>1.26</v>
       </c>
       <c r="W22" t="n">
-        <v>-0.4</v>
+        <v>-1.68</v>
       </c>
       <c r="X22" t="b">
         <v>1</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>45900.41666666666</v>
+        <v>45729.41666666666</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -3054,22 +3062,22 @@
         <v>1</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>45897.41666666666</v>
+        <v>45728.41666666666</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>21.06</v>
+        <v>28.08</v>
       </c>
       <c r="AE22" t="n">
-        <v>21.83</v>
+        <v>29</v>
       </c>
       <c r="AF22" t="n">
-        <v>2.95</v>
+        <v>1.96</v>
       </c>
       <c r="AG22" t="n">
-        <v>0.63</v>
+        <v>1.26</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
@@ -3077,7 +3085,7 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.21</v>
+        <v>0.64</v>
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
@@ -3097,31 +3105,31 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>45911.41666666666</v>
+        <v>45741.41666666666</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45972.41666666666</v>
+        <v>45754.41666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>21.51</v>
+        <v>25.97</v>
       </c>
       <c r="G23" t="n">
-        <v>20.27</v>
+        <v>24.72</v>
       </c>
       <c r="H23" t="n">
-        <v>24.94</v>
+        <v>25.2</v>
       </c>
       <c r="I23" t="n">
-        <v>15.94</v>
+        <v>-2.96</v>
       </c>
       <c r="J23" t="n">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="K23" t="n">
-        <v>20.28</v>
+        <v>24.68</v>
       </c>
       <c r="L23" t="n">
-        <v>20.96</v>
+        <v>25.51</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3134,69 +3142,61 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>2694406</v>
+        <v>767605</v>
       </c>
       <c r="P23" t="n">
-        <v>3.42</v>
+        <v>4.04</v>
       </c>
       <c r="Q23" t="n">
-        <v>20.96</v>
+        <v>27.46</v>
       </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>20.96</v>
+        <v>29.03</v>
       </c>
       <c r="T23" t="b">
         <v>0</v>
       </c>
       <c r="U23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>-2.57</v>
+        <v>11.79</v>
       </c>
       <c r="W23" t="n">
-        <v>-2.57</v>
+        <v>5.75</v>
       </c>
       <c r="X23" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y23" s="2" t="n">
-        <v>45923.41666666666</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB23" s="2" t="n">
-        <v>45911.41666666666</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="n">
-        <v>20.27</v>
+        <v>24.72</v>
       </c>
       <c r="AE23" t="n">
-        <v>22.19</v>
+        <v>29.03</v>
       </c>
       <c r="AF23" t="n">
-        <v>5.76</v>
+        <v>4.81</v>
       </c>
       <c r="AG23" t="n">
-        <v>3.16</v>
+        <v>11.8</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.55</v>
+        <v>2.45</v>
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
@@ -3216,31 +3216,31 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>45994.41666666666</v>
+        <v>45760.41666666666</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>46002.41666666666</v>
+        <v>45783.41666666666</v>
       </c>
       <c r="F24" t="n">
-        <v>23.44</v>
+        <v>25.32</v>
       </c>
       <c r="G24" t="n">
-        <v>22.68</v>
+        <v>24.12</v>
       </c>
       <c r="H24" t="n">
-        <v>23.56</v>
+        <v>23.99</v>
       </c>
       <c r="I24" t="n">
-        <v>0.51</v>
+        <v>-5.24</v>
       </c>
       <c r="J24" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="K24" t="n">
-        <v>22.51</v>
+        <v>24.12</v>
       </c>
       <c r="L24" t="n">
-        <v>23.43</v>
+        <v>25.26</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>2183354</v>
+        <v>623052</v>
       </c>
       <c r="P24" t="n">
-        <v>1.78</v>
+        <v>0.96</v>
       </c>
       <c r="Q24" t="n">
-        <v>23.05</v>
+        <v>26.96</v>
       </c>
       <c r="R24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>24.98</v>
+        <v>26.96</v>
       </c>
       <c r="T24" t="b">
         <v>0</v>
@@ -3274,10 +3274,10 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>6.57</v>
+        <v>6.48</v>
       </c>
       <c r="W24" t="n">
-        <v>-1.66</v>
+        <v>6.48</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -3285,25 +3285,21 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB24" s="2" t="n">
-        <v>45994.41666666666</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="n">
-        <v>22.68</v>
+        <v>24.12</v>
       </c>
       <c r="AE24" t="n">
-        <v>24.98</v>
+        <v>26.96</v>
       </c>
       <c r="AF24" t="n">
-        <v>3.24</v>
+        <v>4.74</v>
       </c>
       <c r="AG24" t="n">
-        <v>6.57</v>
+        <v>6.48</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
@@ -3311,7 +3307,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>2.03</v>
+        <v>1.37</v>
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
@@ -3331,31 +3327,31 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>46016.41666666666</v>
+        <v>45792.41666666666</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>46027.41666666666</v>
+        <v>45809.41666666666</v>
       </c>
       <c r="F25" t="n">
-        <v>24.6</v>
+        <v>22.75</v>
       </c>
       <c r="G25" t="n">
-        <v>23.75</v>
+        <v>21.66</v>
       </c>
       <c r="H25" t="n">
-        <v>24.41</v>
+        <v>21.65</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.77</v>
+        <v>-4.85</v>
       </c>
       <c r="J25" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="K25" t="n">
-        <v>23.41</v>
+        <v>21.66</v>
       </c>
       <c r="L25" t="n">
-        <v>24.09</v>
+        <v>22.2</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3368,31 +3364,31 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>2756109</v>
+        <v>13689820</v>
       </c>
       <c r="P25" t="n">
-        <v>3.54</v>
+        <v>4.94</v>
       </c>
       <c r="Q25" t="n">
-        <v>24.08</v>
+        <v>23.7</v>
       </c>
       <c r="R25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>24.5</v>
+        <v>25.75</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
       </c>
       <c r="U25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>-0.41</v>
+        <v>13.18</v>
       </c>
       <c r="W25" t="n">
-        <v>-2.11</v>
+        <v>4.17</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -3400,33 +3396,29 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB25" s="2" t="n">
-        <v>46016.41666666666</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="n">
-        <v>23.75</v>
+        <v>21.66</v>
       </c>
       <c r="AE25" t="n">
-        <v>25.69</v>
+        <v>25.75</v>
       </c>
       <c r="AF25" t="n">
-        <v>3.46</v>
+        <v>4.78</v>
       </c>
       <c r="AG25" t="n">
-        <v>4.43</v>
+        <v>13.19</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>1.28</v>
+        <v>2.76</v>
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
@@ -3446,31 +3438,31 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>46069.41666666666</v>
+        <v>45823.41666666666</v>
       </c>
       <c r="F26" t="n">
-        <v>26</v>
+        <v>21.88</v>
       </c>
       <c r="G26" t="n">
-        <v>24.3</v>
+        <v>21.35</v>
       </c>
       <c r="H26" t="n">
-        <v>28.5</v>
+        <v>20.53</v>
       </c>
       <c r="I26" t="n">
-        <v>9.619999999999999</v>
+        <v>-6.18</v>
       </c>
       <c r="J26" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="K26" t="n">
-        <v>24.01</v>
+        <v>21.35</v>
       </c>
       <c r="L26" t="n">
-        <v>25.42</v>
+        <v>21.78</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3483,37 +3475,37 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>2965366</v>
+        <v>1476660</v>
       </c>
       <c r="P26" t="n">
-        <v>6.51</v>
+        <v>1.3</v>
       </c>
       <c r="Q26" t="n">
-        <v>25.42</v>
+        <v>21.54</v>
       </c>
       <c r="R26" t="b">
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>25.42</v>
+        <v>22.52</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
       </c>
       <c r="U26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>-2.23</v>
+        <v>2.93</v>
       </c>
       <c r="W26" t="n">
-        <v>-2.23</v>
+        <v>-1.55</v>
       </c>
       <c r="X26" t="b">
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>46033.41666666666</v>
+        <v>45818.41666666666</v>
       </c>
       <c r="Z26" t="n">
         <v>2</v>
@@ -3522,30 +3514,30 @@
         <v>1</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>46028.41666666666</v>
+        <v>45811.41666666666</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>24.3</v>
+        <v>21.35</v>
       </c>
       <c r="AE26" t="n">
-        <v>27.41</v>
+        <v>22.52</v>
       </c>
       <c r="AF26" t="n">
-        <v>6.54</v>
+        <v>2.41</v>
       </c>
       <c r="AG26" t="n">
-        <v>5.42</v>
+        <v>2.93</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>0.83</v>
+        <v>1.22</v>
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
@@ -3565,31 +3557,31 @@
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>46120.41666666666</v>
+        <v>45831.41666666666</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>46139.41666666666</v>
+        <v>45839.41666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>26.61</v>
+        <v>21.16</v>
       </c>
       <c r="G27" t="n">
-        <v>25.21</v>
+        <v>19.2</v>
       </c>
       <c r="H27" t="n">
-        <v>28.7</v>
+        <v>21.32</v>
       </c>
       <c r="I27" t="n">
-        <v>7.85</v>
+        <v>0.76</v>
       </c>
       <c r="J27" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="K27" t="n">
-        <v>23.8</v>
+        <v>19.92</v>
       </c>
       <c r="L27" t="n">
-        <v>25.7</v>
+        <v>20.64</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3602,61 +3594,57 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>2499912</v>
+        <v>5666121</v>
       </c>
       <c r="P27" t="n">
-        <v>4.31</v>
+        <v>4.75</v>
       </c>
       <c r="Q27" t="n">
-        <v>26.8</v>
+        <v>22.02</v>
       </c>
       <c r="R27" t="b">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>26.8</v>
+        <v>22.52</v>
       </c>
       <c r="T27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U27" t="b">
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>0.71</v>
+        <v>6.43</v>
       </c>
       <c r="W27" t="n">
-        <v>0.71</v>
+        <v>4.06</v>
       </c>
       <c r="X27" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y27" s="2" t="n">
-        <v>46120.41666666666</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="b">
         <v>1</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>46127.41666666666</v>
+        <v>45833.41666666666</v>
       </c>
       <c r="AC27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD27" t="n">
-        <v>25.21</v>
+        <v>19.2</v>
       </c>
       <c r="AE27" t="n">
-        <v>26.8</v>
+        <v>22.52</v>
       </c>
       <c r="AF27" t="n">
-        <v>5.26</v>
+        <v>9.26</v>
       </c>
       <c r="AG27" t="n">
-        <v>0.71</v>
+        <v>6.43</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -3664,10 +3652,954 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.13</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C28" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>45845.41666666666</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>45860.41666666666</v>
+      </c>
+      <c r="F28" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="G28" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="H28" t="n">
+        <v>22.48</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="J28" t="n">
+        <v>15</v>
+      </c>
+      <c r="K28" t="n">
+        <v>21.29</v>
+      </c>
+      <c r="L28" t="n">
+        <v>21.84</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>1366828</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>22.06</v>
+      </c>
+      <c r="R28" t="b">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="T28" t="b">
+        <v>0</v>
+      </c>
+      <c r="U28" t="b">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="X28" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y28" s="2" t="n">
+        <v>45847.41666666666</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB28" s="2" t="n">
+        <v>45847.41666666666</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C29" t="b">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>45872.41666666666</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>45887.41666666666</v>
+      </c>
+      <c r="F29" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="G29" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="H29" t="n">
+        <v>22.81</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-2.36</v>
+      </c>
+      <c r="J29" t="n">
+        <v>15</v>
+      </c>
+      <c r="K29" t="n">
+        <v>22.39</v>
+      </c>
+      <c r="L29" t="n">
+        <v>23.18</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>1011332</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="T29" t="b">
+        <v>0</v>
+      </c>
+      <c r="U29" t="b">
+        <v>0</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="W29" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="X29" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y29" s="2" t="n">
+        <v>45873.41666666666</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA29" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB29" s="2" t="n">
+        <v>45872.41666666666</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AJ29" t="inlineStr"/>
+      <c r="AK29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C30" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>45897.41666666666</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="F30" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="G30" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="H30" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-3.13</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="L30" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>811883</v>
+      </c>
+      <c r="P30" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="T30" t="b">
+        <v>0</v>
+      </c>
+      <c r="U30" t="b">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="W30" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="X30" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y30" s="2" t="n">
+        <v>45900.41666666666</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA30" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB30" s="2" t="n">
+        <v>45897.41666666666</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C31" t="b">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>45972.41666666666</v>
+      </c>
+      <c r="F31" t="n">
+        <v>21.51</v>
+      </c>
+      <c r="G31" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="H31" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="I31" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="J31" t="n">
+        <v>61</v>
+      </c>
+      <c r="K31" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="L31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>2694406</v>
+      </c>
+      <c r="P31" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="T31" t="b">
+        <v>0</v>
+      </c>
+      <c r="U31" t="b">
+        <v>1</v>
+      </c>
+      <c r="V31" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="W31" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="X31" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="2" t="n">
+        <v>45923.41666666666</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA31" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB31" s="2" t="n">
+        <v>45911.41666666666</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ31" t="inlineStr"/>
+      <c r="AK31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>46002.41666666666</v>
+      </c>
+      <c r="F32" t="n">
+        <v>23.44</v>
+      </c>
+      <c r="G32" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="H32" t="n">
+        <v>23.56</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J32" t="n">
+        <v>8</v>
+      </c>
+      <c r="K32" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="L32" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>2183354</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>22.87</v>
+      </c>
+      <c r="R32" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="T32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V32" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="W32" t="n">
+        <v>-2.43</v>
+      </c>
+      <c r="X32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB32" s="2" t="n">
+        <v>45994.41666666666</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AJ32" t="inlineStr"/>
+      <c r="AK32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C33" t="b">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>46027.41666666666</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G33" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="H33" t="n">
+        <v>24.41</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="J33" t="n">
+        <v>11</v>
+      </c>
+      <c r="K33" t="n">
+        <v>23.41</v>
+      </c>
+      <c r="L33" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O33" t="n">
+        <v>2756109</v>
+      </c>
+      <c r="P33" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>24.08</v>
+      </c>
+      <c r="R33" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="T33" t="b">
+        <v>0</v>
+      </c>
+      <c r="U33" t="b">
+        <v>1</v>
+      </c>
+      <c r="V33" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="W33" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="X33" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB33" s="2" t="n">
+        <v>46016.41666666666</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="AJ33" t="inlineStr"/>
+      <c r="AK33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>46069.41666666666</v>
+      </c>
+      <c r="F34" t="n">
+        <v>26</v>
+      </c>
+      <c r="G34" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I34" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="J34" t="n">
+        <v>41</v>
+      </c>
+      <c r="K34" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="L34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>2965366</v>
+      </c>
+      <c r="P34" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="R34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S34" t="n">
+        <v>25.42</v>
+      </c>
+      <c r="T34" t="b">
+        <v>0</v>
+      </c>
+      <c r="U34" t="b">
+        <v>1</v>
+      </c>
+      <c r="V34" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="W34" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="X34" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="2" t="n">
+        <v>46033.41666666666</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA34" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="2" t="n">
+        <v>46028.41666666666</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>RANGE</t>
+        </is>
+      </c>
+      <c r="AI34" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AJ34" t="inlineStr"/>
+      <c r="AK34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>JUFO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKOUT</t>
+        </is>
+      </c>
+      <c r="C35" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>46139.41666666666</v>
+      </c>
+      <c r="F35" t="n">
+        <v>26.61</v>
+      </c>
+      <c r="G35" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="I35" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="J35" t="n">
+        <v>19</v>
+      </c>
+      <c r="K35" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="L35" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>RANGE_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>2499912</v>
+      </c>
+      <c r="P35" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>25.73</v>
+      </c>
+      <c r="R35" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="T35" t="b">
+        <v>1</v>
+      </c>
+      <c r="U35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="W35" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="X35" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB35" s="2" t="n">
+        <v>46120.41666666666</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>ANCHOR</t>
+        </is>
+      </c>
+      <c r="AI35" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3885,31 +4817,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>46139.41666666666</v>
       </c>
       <c r="F2" t="n">
-        <v>53.91</v>
+        <v>47.87</v>
       </c>
       <c r="G2" t="n">
-        <v>43.72</v>
+        <v>46</v>
       </c>
       <c r="H2" t="n">
         <v>181</v>
       </c>
       <c r="I2" t="n">
-        <v>235.74</v>
+        <v>278.11</v>
       </c>
       <c r="J2" t="n">
-        <v>593</v>
+        <v>384</v>
       </c>
       <c r="K2" t="n">
-        <v>43.03</v>
+        <v>45</v>
       </c>
       <c r="L2" t="n">
-        <v>45.91</v>
+        <v>46.89</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -3922,69 +4854,69 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>128396</v>
+        <v>47815</v>
       </c>
       <c r="P2" t="n">
-        <v>19.99</v>
+        <v>2.73</v>
       </c>
       <c r="Q2" t="n">
-        <v>45.33</v>
+        <v>46.62</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>48.75</v>
+        <v>51</v>
       </c>
       <c r="T2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>-9.57</v>
+        <v>6.54</v>
       </c>
       <c r="W2" t="n">
-        <v>-15.92</v>
+        <v>-2.61</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45547.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="Z2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>45546.41666666666</v>
+        <v>45755.41666666666</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>43.72</v>
+        <v>46</v>
       </c>
       <c r="AE2" t="n">
-        <v>59.63</v>
+        <v>51</v>
       </c>
       <c r="AF2" t="n">
-        <v>18.9</v>
+        <v>3.91</v>
       </c>
       <c r="AG2" t="n">
-        <v>10.61</v>
+        <v>6.54</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.67</v>
       </c>
       <c r="AJ2" t="n">
         <v>181</v>
@@ -4126,25 +5058,25 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>66.67</v>
+        <v>27.27</v>
       </c>
       <c r="G2" t="n">
-        <v>1.19</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.58</v>
+        <v>-25.44</v>
       </c>
       <c r="J2" t="n">
         <v>12.48</v>
@@ -4153,28 +5085,28 @@
         <v>-14.25</v>
       </c>
       <c r="L2" t="n">
-        <v>13.42</v>
+        <v>7.68</v>
       </c>
       <c r="M2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="N2" t="n">
-        <v>6.84</v>
+        <v>7.98</v>
       </c>
       <c r="O2" t="n">
-        <v>14.25</v>
+        <v>6.17</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.2320120319001387</v>
+        <v>0.1209768433179723</v>
       </c>
       <c r="R2" t="n">
-        <v>0.09086</v>
+        <v>-0.09292000000000003</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1473208127600555</v>
+        <v>-0.007361262672811078</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -4182,7 +5114,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.1473208127600555</v>
+        <v>-0.007361262672811078</v>
       </c>
     </row>
     <row r="3">
@@ -4212,10 +5144,10 @@
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
       <c r="I3" t="n">
-        <v>59.34</v>
+        <v>63.34</v>
       </c>
       <c r="J3" t="n">
         <v>38.41</v>
@@ -4224,28 +5156,28 @@
         <v>-11.36</v>
       </c>
       <c r="L3" t="n">
-        <v>10.64</v>
+        <v>10.51</v>
       </c>
       <c r="M3" t="n">
-        <v>2.13</v>
+        <v>2.31</v>
       </c>
       <c r="N3" t="n">
         <v>9.31</v>
       </c>
       <c r="O3" t="n">
-        <v>4.76</v>
+        <v>4.39</v>
       </c>
       <c r="P3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5084026632302405</v>
+        <v>0.5176452432667247</v>
       </c>
       <c r="R3" t="n">
-        <v>0.49842</v>
+        <v>0.51042</v>
       </c>
       <c r="S3" t="n">
-        <v>0.5024130652920962</v>
+        <v>0.5133100973066899</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -4253,7 +5185,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.5024130652920962</v>
+        <v>0.5133100973066899</v>
       </c>
     </row>
   </sheetData>
@@ -4324,22 +5256,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.15</v>
+        <v>-0.01</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>66.67</v>
+        <v>27.27</v>
       </c>
       <c r="F2" t="n">
-        <v>0.96</v>
+        <v>0.48</v>
       </c>
       <c r="G2" t="n">
-        <v>1.19</v>
+        <v>-4.54</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.19</v>
+        <v>-2.31</v>
       </c>
     </row>
     <row r="3">
@@ -4354,7 +5286,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="D3" t="n">
         <v>23</v>
@@ -4363,13 +5295,13 @@
         <v>52.17</v>
       </c>
       <c r="F3" t="n">
-        <v>2.13</v>
+        <v>2.31</v>
       </c>
       <c r="G3" t="n">
         <v>0.51</v>
       </c>
       <c r="H3" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-29 19:57:32.310597
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -687,16 +687,16 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>0.76</v>
+        <v>0.65</v>
       </c>
       <c r="T2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>1.33</v>
+        <v>-13.33</v>
       </c>
       <c r="W2" t="n">
         <v>-13.33</v>
@@ -705,10 +705,10 @@
         <v>1</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>45300.41666666666</v>
+        <v>45301.41666666666</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -723,21 +723,21 @@
         <v>0.63</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="AF2" t="n">
         <v>15.47</v>
       </c>
       <c r="AG2" t="n">
-        <v>1.87</v>
+        <v>3.73</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>0.12</v>
+        <v>0.24</v>
       </c>
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
@@ -800,55 +800,47 @@
         <v>7.93</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.04</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.72</v>
+        <v>1.04</v>
       </c>
       <c r="T3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U3" t="b">
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>1.69</v>
+        <v>46.89</v>
       </c>
       <c r="W3" t="n">
-        <v>-2.54</v>
+        <v>46.89</v>
       </c>
       <c r="X3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y3" s="2" t="n">
-        <v>45371.41666666666</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB3" s="2" t="n">
-        <v>45371.41666666666</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="n">
         <v>0.63</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.72</v>
+        <v>1.04</v>
       </c>
       <c r="AF3" t="n">
         <v>11.58</v>
       </c>
       <c r="AG3" t="n">
-        <v>1.41</v>
+        <v>46.89</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
@@ -856,7 +848,7 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0.12</v>
+        <v>4.05</v>
       </c>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr"/>
@@ -919,7 +911,7 @@
         <v>8.630000000000001</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
@@ -928,25 +920,25 @@
         <v>0.73</v>
       </c>
       <c r="T4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V4" t="n">
         <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>-4.11</v>
+        <v>-5.48</v>
       </c>
       <c r="X4" t="b">
         <v>1</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>45386.41666666666</v>
+        <v>45399.41666666666</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -961,21 +953,21 @@
         <v>0.67</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.73</v>
+        <v>0.8</v>
       </c>
       <c r="AF4" t="n">
         <v>8.77</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.55</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.06</v>
+        <v>1.12</v>
       </c>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
@@ -1044,16 +1036,16 @@
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="T5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>1.58</v>
+        <v>-1.06</v>
       </c>
       <c r="W5" t="n">
         <v>-1.06</v>
@@ -1062,10 +1054,10 @@
         <v>1</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>45428.41666666666</v>
+        <v>45434.41666666666</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1080,21 +1072,21 @@
         <v>0.66</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.77</v>
+        <v>0.86</v>
       </c>
       <c r="AF5" t="n">
         <v>12.66</v>
       </c>
       <c r="AG5" t="n">
-        <v>1.58</v>
+        <v>13.98</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.12</v>
+        <v>1.1</v>
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
@@ -1157,34 +1149,34 @@
         <v>12.2</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>0.95</v>
+        <v>0.87</v>
       </c>
       <c r="T6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>1.28</v>
+        <v>-7.25</v>
       </c>
       <c r="W6" t="n">
-        <v>-10.45</v>
+        <v>-9.380000000000001</v>
       </c>
       <c r="X6" t="b">
         <v>1</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>45454.41666666666</v>
+        <v>45466.41666666666</v>
       </c>
       <c r="Z6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1199,21 +1191,21 @@
         <v>0.8</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.95</v>
+        <v>1.02</v>
       </c>
       <c r="AF6" t="n">
         <v>15.14</v>
       </c>
       <c r="AG6" t="n">
-        <v>1.71</v>
+        <v>8.74</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.11</v>
+        <v>0.58</v>
       </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
@@ -1276,7 +1268,7 @@
         <v>1.23</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
@@ -1285,7 +1277,7 @@
         <v>1.16</v>
       </c>
       <c r="T7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U7" t="b">
         <v>0</v>
@@ -1294,17 +1286,13 @@
         <v>0.35</v>
       </c>
       <c r="W7" t="n">
-        <v>-0.52</v>
+        <v>-1.38</v>
       </c>
       <c r="X7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="2" t="n">
-        <v>45502.41666666666</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
@@ -1318,21 +1306,21 @@
         <v>1.14</v>
       </c>
       <c r="AE7" t="n">
-        <v>1.16</v>
+        <v>1.27</v>
       </c>
       <c r="AF7" t="n">
         <v>1.73</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.35</v>
+        <v>10.03</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.2</v>
+        <v>5.8</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -1401,29 +1389,25 @@
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>1.2</v>
+        <v>1.17</v>
       </c>
       <c r="T8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V8" t="n">
-        <v>0.67</v>
+        <v>-1.85</v>
       </c>
       <c r="W8" t="n">
         <v>-1.85</v>
       </c>
       <c r="X8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y8" s="2" t="n">
-        <v>45512.41666666666</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="b">
         <v>1</v>
       </c>
@@ -1437,21 +1421,21 @@
         <v>1.05</v>
       </c>
       <c r="AE8" t="n">
-        <v>1.2</v>
+        <v>1.41</v>
       </c>
       <c r="AF8" t="n">
         <v>11.91</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.5</v>
+        <v>18.46</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>0.04</v>
+        <v>1.55</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
@@ -1514,13 +1498,13 @@
         <v>1.85</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.32</v>
+        <v>1.1</v>
       </c>
       <c r="R9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>1.11</v>
+        <v>1.19</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -1529,36 +1513,36 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>0.91</v>
+        <v>8.18</v>
       </c>
       <c r="W9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="X9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="2" t="n">
-        <v>45557.41666666666</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2" t="n">
+        <v>45554.41666666666</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0</v>
+      </c>
       <c r="AD9" t="n">
         <v>1.07</v>
       </c>
       <c r="AE9" t="n">
-        <v>1.11</v>
+        <v>1.19</v>
       </c>
       <c r="AF9" t="n">
         <v>2.91</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.55</v>
+        <v>7.82</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -1566,7 +1550,7 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.19</v>
+        <v>2.69</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1635,29 +1619,25 @@
         <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="T10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V10" t="n">
-        <v>1.1</v>
+        <v>-0.74</v>
       </c>
       <c r="W10" t="n">
         <v>-0.74</v>
       </c>
       <c r="X10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="2" t="n">
-        <v>45592.41666666666</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="b">
         <v>1</v>
       </c>
@@ -1671,21 +1651,21 @@
         <v>1.06</v>
       </c>
       <c r="AE10" t="n">
-        <v>1.1</v>
+        <v>1.19</v>
       </c>
       <c r="AF10" t="n">
         <v>2.39</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.74</v>
+        <v>9.74</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.31</v>
+        <v>4.08</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -1748,7 +1728,7 @@
         <v>3.57</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
@@ -1757,7 +1737,7 @@
         <v>0.87</v>
       </c>
       <c r="T11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U11" t="b">
         <v>0</v>
@@ -1766,16 +1746,16 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.3</v>
+        <v>-3.45</v>
       </c>
       <c r="X11" t="b">
         <v>1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>45659.41666666666</v>
+        <v>45673.41666666666</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1790,21 +1770,21 @@
         <v>0.82</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.87</v>
+        <v>0.92</v>
       </c>
       <c r="AF11" t="n">
         <v>6.21</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.46</v>
+        <v>6.21</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.07000000000000001</v>
+        <v>1</v>
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
@@ -1867,35 +1847,31 @@
         <v>7.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.21</v>
+        <v>1.22</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>1.31</v>
+        <v>1.22</v>
       </c>
       <c r="T12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>3.64</v>
+        <v>-3.48</v>
       </c>
       <c r="W12" t="n">
-        <v>-4.27</v>
+        <v>-3.48</v>
       </c>
       <c r="X12" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y12" s="2" t="n">
-        <v>45761.41666666666</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
@@ -1909,21 +1885,21 @@
         <v>1.16</v>
       </c>
       <c r="AE12" t="n">
-        <v>1.31</v>
+        <v>1.48</v>
       </c>
       <c r="AF12" t="n">
         <v>8.539999999999999</v>
       </c>
       <c r="AG12" t="n">
-        <v>3.64</v>
+        <v>16.93</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.43</v>
+        <v>1.98</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1986,13 +1962,13 @@
         <v>2</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.42</v>
+        <v>1.44</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>1.48</v>
+        <v>1.44</v>
       </c>
       <c r="T13" t="b">
         <v>1</v>
@@ -2001,10 +1977,10 @@
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>3.79</v>
+        <v>0.98</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.42</v>
+        <v>0.98</v>
       </c>
       <c r="X13" t="b">
         <v>1</v>
@@ -2019,22 +1995,22 @@
         <v>1</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>45837.41666666666</v>
+        <v>45838.41666666666</v>
       </c>
       <c r="AC13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD13" t="n">
         <v>1.38</v>
       </c>
       <c r="AE13" t="n">
-        <v>1.48</v>
+        <v>1.44</v>
       </c>
       <c r="AF13" t="n">
         <v>2.95</v>
       </c>
       <c r="AG13" t="n">
-        <v>3.79</v>
+        <v>0.98</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
@@ -2042,7 +2018,7 @@
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>1.28</v>
+        <v>0.33</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2111,29 +2087,25 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>1.44</v>
+        <v>1.42</v>
       </c>
       <c r="T14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>0.42</v>
+        <v>-0.98</v>
       </c>
       <c r="W14" t="n">
         <v>-0.98</v>
       </c>
       <c r="X14" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y14" s="2" t="n">
-        <v>45882.41666666666</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="b">
         <v>1</v>
       </c>
@@ -2147,21 +2119,21 @@
         <v>1.39</v>
       </c>
       <c r="AE14" t="n">
-        <v>1.44</v>
+        <v>1.5</v>
       </c>
       <c r="AF14" t="n">
         <v>3.07</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.14</v>
+        <v>4.32</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.05</v>
+        <v>1.41</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2224,34 +2196,34 @@
         <v>7.35</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.4</v>
+        <v>1.39</v>
       </c>
       <c r="R15" t="b">
         <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>1.6</v>
+        <v>1.41</v>
       </c>
       <c r="T15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V15" t="n">
-        <v>9.59</v>
+        <v>-3.42</v>
       </c>
       <c r="W15" t="n">
-        <v>-4.11</v>
+        <v>-4.79</v>
       </c>
       <c r="X15" t="b">
         <v>1</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>45929.41666666666</v>
+        <v>45937.41666666666</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -2266,21 +2238,21 @@
         <v>1.33</v>
       </c>
       <c r="AE15" t="n">
-        <v>1.6</v>
+        <v>1.61</v>
       </c>
       <c r="AF15" t="n">
         <v>8.9</v>
       </c>
       <c r="AG15" t="n">
-        <v>9.59</v>
+        <v>10.41</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>1.08</v>
+        <v>1.17</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2343,10 +2315,10 @@
         <v>4.04</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>1.05</v>
@@ -2361,7 +2333,7 @@
         <v>1.94</v>
       </c>
       <c r="W16" t="n">
-        <v>-1.94</v>
+        <v>0</v>
       </c>
       <c r="X16" t="b">
         <v>1</v>
@@ -2462,34 +2434,34 @@
         <v>7.32</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="R17" t="b">
         <v>1</v>
       </c>
       <c r="S17" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="T17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U17" t="b">
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>0.89</v>
+        <v>3.86</v>
       </c>
       <c r="W17" t="n">
-        <v>-5.04</v>
+        <v>-1.09</v>
       </c>
       <c r="X17" t="b">
         <v>1</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>45993.41666666666</v>
+        <v>46002.41666666666</v>
       </c>
       <c r="Z17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -2504,13 +2476,13 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="AE17" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="AF17" t="n">
         <v>7.02</v>
       </c>
       <c r="AG17" t="n">
-        <v>0.89</v>
+        <v>3.86</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
@@ -2518,7 +2490,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.13</v>
+        <v>0.55</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>
@@ -2782,35 +2754,31 @@
         <v>2.11</v>
       </c>
       <c r="Q2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S2" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="R2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.84</v>
-      </c>
       <c r="T2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>2.31</v>
+        <v>-1.34</v>
       </c>
       <c r="W2" t="n">
-        <v>-1.34</v>
+        <v>-0.12</v>
       </c>
       <c r="X2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y2" s="2" t="n">
-        <v>46141.41666666666</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
@@ -2824,27 +2792,27 @@
         <v>0.8</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.84</v>
+        <v>0.9</v>
       </c>
       <c r="AF2" t="n">
         <v>2.56</v>
       </c>
       <c r="AG2" t="n">
-        <v>2.31</v>
+        <v>9.5</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>0.9</v>
+        <v>3.71</v>
       </c>
       <c r="AJ2" t="n">
         <v>0.82</v>
       </c>
       <c r="AK2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update trading data 2026-04-29 20:23:01.035976
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -681,7 +681,7 @@
         <v>17.55</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
@@ -699,7 +699,7 @@
         <v>-13.33</v>
       </c>
       <c r="W2" t="n">
-        <v>-13.33</v>
+        <v>-14.67</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
@@ -800,13 +800,13 @@
         <v>7.93</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.04</v>
+        <v>0.73</v>
       </c>
       <c r="R3" t="b">
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>1.04</v>
+        <v>0.84</v>
       </c>
       <c r="T3" t="b">
         <v>0</v>
@@ -815,10 +815,10 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>46.89</v>
+        <v>18.64</v>
       </c>
       <c r="W3" t="n">
-        <v>46.89</v>
+        <v>3.11</v>
       </c>
       <c r="X3" t="b">
         <v>0</v>
@@ -826,21 +826,25 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB3" s="2" t="n">
+        <v>45372.41666666666</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>1</v>
+      </c>
       <c r="AD3" t="n">
         <v>0.63</v>
       </c>
       <c r="AE3" t="n">
-        <v>1.04</v>
+        <v>0.84</v>
       </c>
       <c r="AF3" t="n">
         <v>11.58</v>
       </c>
       <c r="AG3" t="n">
-        <v>46.89</v>
+        <v>18.64</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
@@ -848,7 +852,7 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>4.05</v>
+        <v>1.61</v>
       </c>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr"/>
@@ -917,7 +921,7 @@
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>0.73</v>
+        <v>0.7</v>
       </c>
       <c r="T4" t="b">
         <v>0</v>
@@ -926,7 +930,7 @@
         <v>1</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>-4.11</v>
       </c>
       <c r="W4" t="n">
         <v>-5.48</v>
@@ -935,10 +939,10 @@
         <v>1</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>45399.41666666666</v>
+        <v>45389.41666666666</v>
       </c>
       <c r="Z4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -953,13 +957,13 @@
         <v>0.67</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="AF4" t="n">
         <v>8.77</v>
       </c>
       <c r="AG4" t="n">
-        <v>9.859999999999999</v>
+        <v>6.03</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
@@ -967,7 +971,7 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>1.12</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
@@ -1030,7 +1034,7 @@
         <v>12.8</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
@@ -1048,7 +1052,7 @@
         <v>-1.06</v>
       </c>
       <c r="W5" t="n">
-        <v>-1.06</v>
+        <v>-14.25</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
@@ -1383,7 +1387,7 @@
         <v>10.17</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.17</v>
+        <v>1.11</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
@@ -1401,7 +1405,7 @@
         <v>-1.85</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.85</v>
+        <v>-6.88</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1498,25 +1502,25 @@
         <v>1.85</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="R9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>1.19</v>
+        <v>1.08</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
       </c>
       <c r="U9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" t="n">
-        <v>8.18</v>
+        <v>-1.82</v>
       </c>
       <c r="W9" t="n">
-        <v>0</v>
+        <v>0.91</v>
       </c>
       <c r="X9" t="b">
         <v>0</v>
@@ -1527,30 +1531,30 @@
         <v>1</v>
       </c>
       <c r="AB9" s="2" t="n">
-        <v>45554.41666666666</v>
+        <v>45557.41666666666</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD9" t="n">
         <v>1.07</v>
       </c>
       <c r="AE9" t="n">
-        <v>1.19</v>
+        <v>1.14</v>
       </c>
       <c r="AF9" t="n">
         <v>2.91</v>
       </c>
       <c r="AG9" t="n">
-        <v>7.82</v>
+        <v>3.64</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>2.69</v>
+        <v>1.25</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1847,13 +1851,13 @@
         <v>7.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1862,16 +1866,20 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.48</v>
+        <v>-4.27</v>
       </c>
       <c r="W12" t="n">
-        <v>-3.48</v>
+        <v>-5.06</v>
       </c>
       <c r="X12" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y12" s="2" t="n">
+        <v>45763.41666666666</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>2</v>
+      </c>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
@@ -1885,13 +1893,13 @@
         <v>1.16</v>
       </c>
       <c r="AE12" t="n">
-        <v>1.48</v>
+        <v>1.47</v>
       </c>
       <c r="AF12" t="n">
         <v>8.539999999999999</v>
       </c>
       <c r="AG12" t="n">
-        <v>16.93</v>
+        <v>15.98</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1899,7 +1907,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>1.98</v>
+        <v>1.87</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1968,16 +1976,16 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>1.44</v>
+        <v>1.42</v>
       </c>
       <c r="T13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>0.98</v>
+        <v>-0.42</v>
       </c>
       <c r="W13" t="n">
         <v>0.98</v>
@@ -1986,10 +1994,10 @@
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45837.41666666666</v>
+        <v>45851.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -2004,21 +2012,21 @@
         <v>1.38</v>
       </c>
       <c r="AE13" t="n">
-        <v>1.44</v>
+        <v>1.52</v>
       </c>
       <c r="AF13" t="n">
         <v>2.95</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.98</v>
+        <v>6.45</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>0.33</v>
+        <v>2.19</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2202,7 +2210,7 @@
         <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>1.41</v>
+        <v>1.4</v>
       </c>
       <c r="T15" t="b">
         <v>0</v>
@@ -2211,7 +2219,7 @@
         <v>1</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.42</v>
+        <v>-4.11</v>
       </c>
       <c r="W15" t="n">
         <v>-4.79</v>
@@ -2220,10 +2228,10 @@
         <v>1</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>45937.41666666666</v>
+        <v>45929.41666666666</v>
       </c>
       <c r="Z15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -2238,13 +2246,13 @@
         <v>1.33</v>
       </c>
       <c r="AE15" t="n">
-        <v>1.61</v>
+        <v>1.6</v>
       </c>
       <c r="AF15" t="n">
         <v>8.9</v>
       </c>
       <c r="AG15" t="n">
-        <v>10.41</v>
+        <v>9.73</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2252,7 +2260,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>1.17</v>
+        <v>1.09</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2315,13 +2323,13 @@
         <v>4.04</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.03</v>
+        <v>0.98</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="T16" t="b">
         <v>1</v>
@@ -2330,10 +2338,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>1.94</v>
+        <v>0.97</v>
       </c>
       <c r="W16" t="n">
-        <v>0</v>
+        <v>-4.85</v>
       </c>
       <c r="X16" t="b">
         <v>1</v>
@@ -2357,13 +2365,13 @@
         <v>0.98</v>
       </c>
       <c r="AE16" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="AF16" t="n">
         <v>4.85</v>
       </c>
       <c r="AG16" t="n">
-        <v>1.94</v>
+        <v>0.97</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2371,7 +2379,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2434,25 +2442,25 @@
         <v>7.32</v>
       </c>
       <c r="Q17" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="R17" t="b">
         <v>1</v>
       </c>
       <c r="S17" t="n">
-        <v>1.05</v>
+        <v>0.98</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
       </c>
       <c r="U17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V17" t="n">
-        <v>3.86</v>
+        <v>-3.07</v>
       </c>
       <c r="W17" t="n">
-        <v>-1.09</v>
+        <v>-6.03</v>
       </c>
       <c r="X17" t="b">
         <v>1</v>
@@ -2482,15 +2490,15 @@
         <v>7.02</v>
       </c>
       <c r="AG17" t="n">
-        <v>3.86</v>
+        <v>3.46</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>ANCHOR</t>
+          <t>RANGE</t>
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.55</v>
+        <v>0.49</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-29 20:24:33.466447
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -681,7 +681,7 @@
         <v>17.55</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
@@ -699,7 +699,7 @@
         <v>-13.33</v>
       </c>
       <c r="W2" t="n">
-        <v>-14.67</v>
+        <v>-13.33</v>
       </c>
       <c r="X2" t="b">
         <v>1</v>
@@ -800,13 +800,13 @@
         <v>7.93</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.73</v>
+        <v>1.04</v>
       </c>
       <c r="R3" t="b">
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.84</v>
+        <v>1.04</v>
       </c>
       <c r="T3" t="b">
         <v>0</v>
@@ -815,10 +815,10 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>18.64</v>
+        <v>46.89</v>
       </c>
       <c r="W3" t="n">
-        <v>3.11</v>
+        <v>46.89</v>
       </c>
       <c r="X3" t="b">
         <v>0</v>
@@ -826,25 +826,21 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB3" s="2" t="n">
-        <v>45372.41666666666</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="n">
         <v>0.63</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.84</v>
+        <v>1.04</v>
       </c>
       <c r="AF3" t="n">
         <v>11.58</v>
       </c>
       <c r="AG3" t="n">
-        <v>18.64</v>
+        <v>46.89</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
@@ -852,7 +848,7 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>1.61</v>
+        <v>4.05</v>
       </c>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr"/>
@@ -921,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="T4" t="b">
         <v>0</v>
@@ -930,7 +926,7 @@
         <v>1</v>
       </c>
       <c r="V4" t="n">
-        <v>-4.11</v>
+        <v>0</v>
       </c>
       <c r="W4" t="n">
         <v>-5.48</v>
@@ -939,10 +935,10 @@
         <v>1</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>45389.41666666666</v>
+        <v>45399.41666666666</v>
       </c>
       <c r="Z4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -957,13 +953,13 @@
         <v>0.67</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="AF4" t="n">
         <v>8.77</v>
       </c>
       <c r="AG4" t="n">
-        <v>6.03</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
@@ -971,7 +967,7 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.12</v>
       </c>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
@@ -1034,7 +1030,7 @@
         <v>12.8</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
@@ -1052,7 +1048,7 @@
         <v>-1.06</v>
       </c>
       <c r="W5" t="n">
-        <v>-14.25</v>
+        <v>-1.06</v>
       </c>
       <c r="X5" t="b">
         <v>1</v>
@@ -1387,7 +1383,7 @@
         <v>10.17</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.11</v>
+        <v>1.17</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
@@ -1405,7 +1401,7 @@
         <v>-1.85</v>
       </c>
       <c r="W8" t="n">
-        <v>-6.88</v>
+        <v>-1.85</v>
       </c>
       <c r="X8" t="b">
         <v>0</v>
@@ -1502,25 +1498,25 @@
         <v>1.85</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="R9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>1.08</v>
+        <v>1.19</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
       </c>
       <c r="U9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>-1.82</v>
+        <v>8.18</v>
       </c>
       <c r="W9" t="n">
-        <v>0.91</v>
+        <v>0</v>
       </c>
       <c r="X9" t="b">
         <v>0</v>
@@ -1531,30 +1527,30 @@
         <v>1</v>
       </c>
       <c r="AB9" s="2" t="n">
-        <v>45557.41666666666</v>
+        <v>45554.41666666666</v>
       </c>
       <c r="AC9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD9" t="n">
         <v>1.07</v>
       </c>
       <c r="AE9" t="n">
-        <v>1.14</v>
+        <v>1.19</v>
       </c>
       <c r="AF9" t="n">
         <v>2.91</v>
       </c>
       <c r="AG9" t="n">
-        <v>3.64</v>
+        <v>7.82</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>1.25</v>
+        <v>2.69</v>
       </c>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
@@ -1851,13 +1847,13 @@
         <v>7.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.2</v>
+        <v>1.22</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>1.21</v>
+        <v>1.22</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -1866,20 +1862,16 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>-4.27</v>
+        <v>-3.48</v>
       </c>
       <c r="W12" t="n">
-        <v>-5.06</v>
+        <v>-3.48</v>
       </c>
       <c r="X12" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y12" s="2" t="n">
-        <v>45763.41666666666</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="b">
         <v>1</v>
       </c>
@@ -1893,13 +1885,13 @@
         <v>1.16</v>
       </c>
       <c r="AE12" t="n">
-        <v>1.47</v>
+        <v>1.48</v>
       </c>
       <c r="AF12" t="n">
         <v>8.539999999999999</v>
       </c>
       <c r="AG12" t="n">
-        <v>15.98</v>
+        <v>16.93</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -1907,7 +1899,7 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>1.87</v>
+        <v>1.98</v>
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
@@ -1976,16 +1968,16 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>1.42</v>
+        <v>1.44</v>
       </c>
       <c r="T13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.42</v>
+        <v>0.98</v>
       </c>
       <c r="W13" t="n">
         <v>0.98</v>
@@ -1994,10 +1986,10 @@
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>45851.41666666666</v>
+        <v>45837.41666666666</v>
       </c>
       <c r="Z13" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -2012,21 +2004,21 @@
         <v>1.38</v>
       </c>
       <c r="AE13" t="n">
-        <v>1.52</v>
+        <v>1.44</v>
       </c>
       <c r="AF13" t="n">
         <v>2.95</v>
       </c>
       <c r="AG13" t="n">
-        <v>6.45</v>
+        <v>0.98</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>2.19</v>
+        <v>0.33</v>
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
@@ -2210,7 +2202,7 @@
         <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>1.4</v>
+        <v>1.41</v>
       </c>
       <c r="T15" t="b">
         <v>0</v>
@@ -2219,7 +2211,7 @@
         <v>1</v>
       </c>
       <c r="V15" t="n">
-        <v>-4.11</v>
+        <v>-3.42</v>
       </c>
       <c r="W15" t="n">
         <v>-4.79</v>
@@ -2228,10 +2220,10 @@
         <v>1</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>45929.41666666666</v>
+        <v>45937.41666666666</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -2246,13 +2238,13 @@
         <v>1.33</v>
       </c>
       <c r="AE15" t="n">
-        <v>1.6</v>
+        <v>1.61</v>
       </c>
       <c r="AF15" t="n">
         <v>8.9</v>
       </c>
       <c r="AG15" t="n">
-        <v>9.73</v>
+        <v>10.41</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
@@ -2260,7 +2252,7 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>1.09</v>
+        <v>1.17</v>
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
@@ -2323,13 +2315,13 @@
         <v>4.04</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.98</v>
+        <v>1.03</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="T16" t="b">
         <v>1</v>
@@ -2338,10 +2330,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>0.97</v>
+        <v>1.94</v>
       </c>
       <c r="W16" t="n">
-        <v>-4.85</v>
+        <v>0</v>
       </c>
       <c r="X16" t="b">
         <v>1</v>
@@ -2365,13 +2357,13 @@
         <v>0.98</v>
       </c>
       <c r="AE16" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="AF16" t="n">
         <v>4.85</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.97</v>
+        <v>1.94</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
@@ -2379,7 +2371,7 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
@@ -2442,25 +2434,25 @@
         <v>7.32</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="R17" t="b">
         <v>1</v>
       </c>
       <c r="S17" t="n">
-        <v>0.98</v>
+        <v>1.05</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
       </c>
       <c r="U17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>-3.07</v>
+        <v>3.86</v>
       </c>
       <c r="W17" t="n">
-        <v>-6.03</v>
+        <v>-1.09</v>
       </c>
       <c r="X17" t="b">
         <v>1</v>
@@ -2490,15 +2482,15 @@
         <v>7.02</v>
       </c>
       <c r="AG17" t="n">
-        <v>3.46</v>
+        <v>3.86</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.49</v>
+        <v>0.55</v>
       </c>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr"/>

</xml_diff>

<commit_message>
Update trading data 2026-04-29 20:36:05.928275
</commit_message>
<xml_diff>
--- a/Complete_Trades_Metrics.xlsx
+++ b/Complete_Trades_Metrics.xlsx
@@ -1268,13 +1268,13 @@
         <v>1.23</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.14</v>
+        <v>1.17</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="T7" t="b">
         <v>0</v>
@@ -1283,44 +1283,44 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>0.35</v>
+        <v>1.21</v>
       </c>
       <c r="W7" t="n">
-        <v>-1.38</v>
+        <v>1.21</v>
       </c>
       <c r="X7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>45503.41666666666</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>1</v>
+      </c>
       <c r="AA7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB7" s="2" t="n">
-        <v>45502.41666666666</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="n">
         <v>1.14</v>
       </c>
       <c r="AE7" t="n">
-        <v>1.27</v>
+        <v>1.17</v>
       </c>
       <c r="AF7" t="n">
         <v>1.73</v>
       </c>
       <c r="AG7" t="n">
-        <v>10.03</v>
+        <v>0.87</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>5.8</v>
+        <v>0.5</v>
       </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
@@ -2087,16 +2087,16 @@
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>1.42</v>
+        <v>1.44</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.98</v>
+        <v>0.42</v>
       </c>
       <c r="W14" t="n">
         <v>-0.98</v>
@@ -2119,21 +2119,21 @@
         <v>1.39</v>
       </c>
       <c r="AE14" t="n">
-        <v>1.5</v>
+        <v>1.44</v>
       </c>
       <c r="AF14" t="n">
         <v>3.07</v>
       </c>
       <c r="AG14" t="n">
-        <v>4.32</v>
+        <v>0.28</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>1.41</v>
+        <v>0.09</v>
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
@@ -2760,16 +2760,16 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="T2" t="b">
         <v>0</v>
       </c>
       <c r="U2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>-1.34</v>
+        <v>3.53</v>
       </c>
       <c r="W2" t="n">
         <v>-0.12</v>
@@ -2792,27 +2792,27 @@
         <v>0.8</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="AF2" t="n">
         <v>2.56</v>
       </c>
       <c r="AG2" t="n">
-        <v>9.5</v>
+        <v>4.02</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>RANGE</t>
+          <t>ANCHOR</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>3.71</v>
+        <v>1.57</v>
       </c>
       <c r="AJ2" t="n">
         <v>0.82</v>
       </c>
       <c r="AK2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>